<commit_message>
fix: improve code readability and update comments in Python notebooks for better understanding
</commit_message>
<xml_diff>
--- a/04_bverfg_rag/bverfg_urteil.xlsx
+++ b/04_bverfg_rag/bverfg_urteil.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D240"/>
+  <dimension ref="A1:D165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Die abstrakte Normenkontrolle von 216 Mitgliedern des 19. Deutschen Bundestages der Fraktionen BÜNDNIS 90/DIE GRÜNEN, DIE LINKE und FDP wendet sich gegen Art. 1 Nr. 3 bis 5 des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 (BGBl I S. 2395 &lt;BWahlGÄndG&gt;). Durch die zur Überprüfung gestellten Bestimmungen wurden insbesondere das Verfahren der Sitzzuteilung bei der Bundestagswahl sowie die Regelung für die Berufung von Listennachfolgern geändert.</t>
+          <t>Die Verfassungsbeschwerde betrifft die Fragen, ob die Wiederaufnahme eines Strafverfahrens zuungunsten eines rechtskräftig Freigesprochenen aufgrund neuer Tatsachen oder Beweismittel mit Art. 103 Abs. 3 GG vereinbar und ob die neue Regelung rückwirkend anwendbar ist.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -462,14 +462,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Das Verfahren über die Verteilung der Sitze im Deutschen Bundestag war vor der verfahrensgegenständlichen Änderung zuletzt mit dem Zweiundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 3. Mai 2013 (BGBl I S. 1082 &lt;BWahlG 2013&gt;) geändert worden. Veranlasst war diese Änderung durch die Entscheidung des Bundesverfassungsgerichts vom 25. Juli 2012 (BVerfGE 131, 316), mit der § 6 Abs. 1 Satz 1 und Abs. 2a Bundeswahlgesetz in der Fassung des Art. 1 des Neunzehnten Gesetzes zur Änderung des Bundeswahlgesetzes vom 25. November 2011 (BGBl I S. 2313 &lt;BWahlG 2011&gt;) für mit Art. 21 Abs. 1 und Art. 38 Abs. 1 Satz 1 GG unvereinbar und nichtig erklärt sowie festgestellt worden war, dass § 6 Abs. 5 BWahlG 2011 nach Maßgabe der Urteilsgründe mit diesen Verfassungsbestimmungen unvereinbar ist. In der Folge wurde das Sitzzuteilungsverfahren wie folgt gefasst:</t>
+          <t>1. Die Wiederaufnahme eines Strafverfahrens zuungunsten eines Angeklagten ist in § 362 StPO geregelt. Mit dem Gesetz zur Änderung der Strafprozessordnung – Erweiterung der Wiederaufnahmemöglichkeiten zuungunsten des Verurteilten gemäß § 362 StPO und zur Änderung der zivilrechtlichen Verjährung (Gesetz zur Herstellung materieller Gerechtigkeit) vom 21. Dezember 2021 (BGBl I S. 5252) wurde die Norm um eine weitere Fallgruppe (Nr. 5) ergänzt. Die Vorschrift lautet seither:</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -478,14 +478,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>a) In einer ersten – rein rechnerischen – Verteilung wurde die Gesamtzahl der 598 Sitze (§ 1 Abs. 1 Satz 1 BWahlG 2013) nach dem Divisorverfahren mit Standardrundung nach Sainte-Laguë/Schepers (§ 6 Abs. 2 Satz 2 bis 7 BWahlG 2013; vgl. dazu BTDrucks 16/7461, S. 9 ff.) den Ländern nicht mehr nach der Wählerzahl, sondern nach ihrem Bevölkerungsanteil zugeordnet (§ 6 Abs. 2 Satz 1 BWahlG 2013). Sodann wurden die Sitze eines Landes im Rahmen einer Unterverteilung auf die jeweils in dem Land angetretenen Landeslisten nach dem Zweitstimmenanteil verteilt (mit Ausnahme der nach den Vorgaben des § 6 Abs. 1 Satz 3 BWahlG 2013 abgezogenen Sitze, § 6 Abs. 2 Satz 1 BWahlG 2013). Dabei griffen die Sperr- und die Grundmandatsklausel, wonach bei der Verteilung auf die Landeslisten nur Parteien berücksichtigt wurden, die mindestens fünf Prozent der im Wahlgebiet abgegebenen gültigen Zweitstimmen erhalten oder in mindestens drei Wahlkreisen einen Sitz errungen hatten (§ 6 Abs. 3 Satz 1 BWahlG 2013), es sei denn, es handelte sich um Listen von Parteien nationaler Minderheiten (§ 6 Abs. 3 Satz 2 BWahlG 2013). Von der auf diese Weise für jede Landesliste ermittelten Sitzzahl wurde die Zahl der Wahlkreismandate abgerechnet; erzielte Wahlkreismandate verblieben der Landesliste auch dann, wenn sie die für diese ermittelte Sitzzahl überstiegen (§ 6 Abs. 4 Satz 1 und 2 BWahlG 2013). Da derartige, nicht vom Zweitstimmenanteil gedeckte Mandate ausschließlich in der fiktiven ersten Verteilung auftreten konnten, wurden sie als „Quasi-Überhangmandate“ bezeichnet (vgl. Behnke, ZParl 2014, S. 17 &lt;20&gt;). Bei der Summe der so für die Landeslisten einer Partei errechneten Mandate handelte es sich um die Mindestsitzzahl, die dieser Partei in der zweiten – tatsächlichen – Verteilung mindestens zugeteilt wurde (vgl. Strelen, in: Schreiber, BWahlG, 10. Aufl. 2017, § 6 Rn. 26c).</t>
+          <t>2. Die ersten vier Wiederaufnahmegründe und damit die vorausgehende Fassung des § 362 StPO lassen sich auf die Reichsstrafprozessordnung vom 1. Februar 1877 (RGBl S. 253 ff.) zurückführen.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -494,14 +494,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>b) Gemäß § 6 Abs. 5 BWahlG 2013 wurde sodann die Zahl der nach § 6 Abs. 1 Satz 3 BWahlG 2013 verbleibenden Sitze erhöht, bis jede Partei bei der zweiten Verteilung nach § 6 Abs. 6 Satz 1 BWahlG 2013 mindestens die für sie ermittelte Mindestsitzzahl erhielt (§ 6 Abs. 5 Satz 1 BWahlG 2013). Die Gesamtzahl von 598 Sitzen erhöhte sich um die Unterschiedszahl (§ 6 Abs. 5 Satz 2 BWahlG 2013). Die Regelung des § 6 Abs. 5 BWahlG 2013 zielte auf einen vollständigen Ausgleich der rechnerisch anfallenden Überhangmandate (vgl. BTDrucks 17/11819, S. 5), das heißt derjenigen Mandate, um die die Zahl der von einer Partei in einem Land erzielten Wahlkreismandate die Zahl der für die jeweilige Landesliste ermittelten Sitze überstieg.</t>
+          <t>a) Die Regelung in der Reichsstrafprozessordnung bildete anknüpfend an die uneinheitliche Rechtslage in den deutschen Partikularstaaten des 19. Jahrhunderts einen Mittelweg zwischen einem akkusatorischen und einem inquisitorischen Strafverfahren ab (vgl. Motive zu dem Entwurf einer Deutschen Strafprozessordnung nach den Beschlüssen der von dem Bundesrath eingesetzten Kommission, 1873, S. 173 f.; Motive zum Entwurf einer Strafprozessordnung von 1874, abgedruckt in: Hahn, Die gesammten Materialien zu den Reichs-Justizgesetzen, Bd. 3, Erste Abteilung, 1880, S. 264 f.).</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -510,14 +510,14 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>c) Diese erhöhte Gesamtsitzzahl des Deutschen Bundestages wurde in der zweiten – tatsächlichen – Verteilung nach § 6 Abs. 6 BWahlG 2013 zunächst in einer Oberverteilung bundesweit nach der Zweitstimmenzahl im Divisorverfahren mit Standardrundung nach Sainte-Laguë/Schepers auf die zu berücksichtigenden Parteien verteilt (§ 6 Abs. 6 Satz 1 BWahlG 2013). Sodann erfolgte eine Unterverteilung innerhalb der Parteien auf deren Landeslisten (§ 6 Abs. 6 Satz 2 BWahlG 2013). An diese schloss sich die konkrete Mandatsvergabe unter vorrangiger Berücksichtigung der erfolgreichen Wahlkreisbewerber an (§ 6 Abs. 6 Satz 3 bis 6 BWahlG 2013).</t>
+          <t>Der Grundsatz ne bis in idem wird auf das kontradiktorische Verfahren im römischen Recht zurückgeführt. Demgegenüber oblag nach dem gemeinrechtlichen und teils auch kodifizierten Inquisitionsverfahren die Aufgabe der Strafverfolgung ausschließlich dem Staat, der im Interesse der Allgemeinheit und der Gerechtigkeit die Wahrheit zu erkennen und durchzusetzen hatte. Dem Verfahrensziel, die objektive Wahrheit zu erlangen, entsprach es, auch nach Abschluss eines Verfahrens ein und dieselbe Tat erneut zu untersuchen und gegebenenfalls erneut zu bestrafen, wenn neue Verdachtsgründe oder Beweismittel zutage traten. Dies wurde durch die sogenannte Lossprechung von der Instanz (absolutio ab instantia) ermöglicht, wenn nach den gesetzlichen Beweisregeln des Inquisitionsverfahrens weder die Schuld noch die Unschuld festgestellt werden konnte (vgl. Grünewald, ZStW 120 &lt;2008&gt;, S. 545 &lt;549&gt;; Frank, Die Wiederaufnahme zuungunsten des Angeklagten im Strafverfahren, 2022, S. 11 ff. m.w.N.).</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -526,14 +526,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2. a) Für den Fall des Ausscheidens eines direkt gewählten Abgeordneten hatte das Wahlgesetz zum ersten Bundestag und zur ersten Bundesversammlung vom 15. Juni 1949 (BGBl S. 21 &lt;BWahlG 1949&gt;) noch eine Ersatzwahl vorgesehen; lediglich für ausscheidende Abgeordnete, die auf der Grundlage eines Listenvorschlags gewählt worden waren, galt das Prinzip der Listennachfolge (§ 15 BWahlG 1949). Das Wahlgesetz zum zweiten Bundestag und zur Bundesversammlung vom 8. Juli 1953 (BGBl I S. 470 &lt;BWahlG 1953&gt;) erstreckte demgegenüber das Prinzip der Listennachfolge auch auf direkt gewählte Bewerber (§ 54 Abs. 1 BWahlG 1953). Seit dem Bundeswahlgesetz vom 7. Mai 1956 (BGBl I S. 383 &lt;BWahlG 1956&gt;) ist die dahingehende Regelung in § 48 Abs. 1 enthalten. Danach wurde, wenn ein gewählter Bewerber starb oder die Annahme der Wahl ablehnte oder ein Abgeordneter starb oder sonst nachträglich aus dem Bundestag ausschied, der Sitz aus der Landesliste derjenigen Partei besetzt, für die der Ausgeschiedene bei der Wahl aufgetreten war (Satz 1), wobei Listenbewerber unberücksichtigt blieben, wenn sie zwischenzeitlich aus der Partei ausgeschieden waren (Satz 2). War die Liste erschöpft, blieb der Sitz unbesetzt (Satz 3). Die Norm fand auch Anwendung, wenn ein direkt gewählter Abgeordneter aus dem Deutschen Bundestag ausschied, der in einem Land gewählt war, in dem seine Partei über Überhangmandate verfügte (vgl. BVerfGE 97, 317 &lt;321, 329 f.&gt;).</t>
+          <t>Nach Einführung des akkusatorischen Strafverfahrens in Frankreich infolge der Revolution von 1791 wurde der Anklageprozess in zahlreichen deutschen Partikularstaaten rezipiert und auch in § 179 Abs. 1 der Frankfurter Paulskirchenverfassung von 1849 vorgegeben. Als Kern des akkusatorischen Verfahrens galt, dass die Parteien den Prozessstoff zu sammeln und vorzulegen hatten, so dass bewusst oder unbewusst nicht vorgebrachter Prozessstoff unbeachtlich war. Zugleich hielt der Gedanke der Rechtskraft der richterlichen Streitentscheidung Einzug in den Strafprozess. Bei offen gebliebenen Anklagepunkten trat an die Stelle der nur verfahrenseinstellenden absolutio ab instantia der Freispruch als verfahrensbeendendes Sachurteil (vgl. Grünewald, ZStW 120 &lt;2008&gt;, S. 545 &lt;552&gt; m.w.N.; Frank, Die Wiederaufnahme zuungunsten des Angeklagten im Strafverfahren, 2022, S. 19 ff.). Eine Wiederaufnahme wegen neuer Tatsachen oder Beweismittel gab es nicht.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -542,14 +542,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>b) Mit Beschluss vom 26. Februar 1998 (BVerfGE 97, 317) entschied das Bundesverfassungsgericht, dass § 48 Abs. 1 Bundeswahlgesetz in der Fassung der Bekanntmachung vom 23. Juli 1993 (BGBl I S. 1288, berichtigt S. 1595 &lt;BWahlG 1993&gt;) nur anwendbar sei, soweit Sitze wieder zu besetzen seien, die aufgrund des Zweitstimmenergebnisses für die Landesliste ermittelt worden seien. Scheide ein direkt gewählter Wahlkreisabgeordneter aus dem Deutschen Bundestag aus, komme demzufolge eine Listennachfolge nicht in Betracht, solange die Partei, der er angehöre, in dem betroffenen Land über mehr Direktmandate verfüge, als ihr Listensitze zustünden. Zur Begründung verwies der Zweite Senat darauf, dass Überhangmandate nicht durch Zweitstimmen legitimiert seien, da sie nicht im Wege der Anrechnung auf das Sitzkontingent der Liste einen Listensitz verdrängten. Für solche Fälle halte die Landesliste daher mitgewählte Ersatzleute nicht vor (vgl. BVerfGE 97, 317 &lt;328&gt; sowie 3. Leitsatz).</t>
+          <t>In der Weimarer Republik blieben die strafprozessualen Bestimmungen inhaltlich unverändert (vgl. Verordnung vom 4. Januar 1924 zur (Neu-)Bekanntmachung der Reichsstrafprozessordnung, RGBl I S. 299 ff. &lt;358 ff.&gt;). Eine Erweiterung der Wiederaufnahmegründe zulasten des Angeklagten um neue Tatsachen oder Beweismittel wurde 1931 auf dem Deutschen Juristentag kontrovers diskutiert und im Ergebnis abgelehnt (vgl. Verhandlungen des 36. Deutschen Juristentages, Bd. 1, 4. Lieferung, 1931, S. 1141 ff.; Bd. 2, 1932, S. 222 ff.).</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -558,14 +558,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>c) In der Folgezeit wurde der Norm die Auslegung des Bundesverfassungsgerichts zugrunde gelegt (vgl. BT-Plenarprotokoll 13/235, S. 21538). Mit dem Gesetz zur Änderung des Wahl- und Abgeordnetenrechts vom 17. März 2008 (BGBl I S. 394 &lt;BWahlG 2008&gt;) wurde diese Handhabung ausdrücklich geregelt und § 48 Abs. 1 BWahlG um einen neuen Satz 2 ergänzt, nach dem eine Listennachfolge nicht stattfindet, solange die Partei in dem betreffenden Land Überhangmandate innehat (vgl. BTDrucks 16/7461, S. 20). Mit dem Zweiundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 3. Mai 2013 (BGBl I S. 1082), das einen Vollausgleich von rechnerisch anfallenden Überhangmandaten einführte, wurde § 48 Abs. 1 Satz 2 BWahlG gestrichen. Zur Begründung wurde darauf verwiesen, einer Sonderregelung für den Fall, dass eine Partei in einem Land über mehr Direktmandate verfüge, als ihr Listensitze zustünden, bedürfe es nicht mehr. Durch den Vollausgleich werde keiner der Sitze nur von einer Mehrheit der Erststimmen getragen (vgl. BTDrucks 17/11819, S. 7, 11 f.).</t>
+          <t>b) Unter der nationalsozialistischen Herrschaft wurden die Wiederaufnahmegründe zugunsten und zuungunsten des Angeklagten durch die Dritte Verordnung zur Vereinfachung der Strafrechtspflege vom 29. Mai 1943 (RGBl I S. 342 ff.) einander angeglichen. In der Begründung des vorangegangenen Entwurfs hieß es, wichtiger als die – vorwiegend als Schutz des Beschuldigten gedachte – formale Rechtskraft sei das Verlangen der Volksgemeinschaft nach Verwirklichung der materiellen Gerechtigkeit. Diese Gerechtigkeit sei einheitlich und unteilbar und sei die gleiche bei Entscheidungen zugunsten wie zuungunsten des Angeklagten (vgl. Begründung des Entwurfs einer Strafverfahrensordnung vom 1. Mai 1939, abgedruckt in: Schubert/Regge/Rieß/Schmid, Quellen zur Reform des Straf- und Strafprozessrechts, Abteilung III, Bd. 1, 1991, S. 541). Daneben konnte mit der sogenannten Urteilsergänzung die Rechtskraft in denjenigen Fällen durchbrochen werden, in denen das Urteil den „Belangen der Volksgemeinschaft“ widersprach (vgl. Schulze-Fielitz, in: Dreier, GG, Bd. 3, 3. Aufl. 2018, Art. 103 Abs. 3 Rn. 4).</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -574,14 +574,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3. Nachdem der Deutsche Bundestag bei der Wahl 2017 auf 709 Abgeordnete angewachsen war, legten die damaligen Regierungsfraktionen aus CDU/CSU und SPD am 15. September 2020 erneut einen Entwurf zur Änderung des Bundeswahlgesetzes vor (BTDrucks 19/22504).</t>
+          <t>c) Nach dem Ende des Zweiten Weltkriegs wurde zunächst in den Besatzungszonen die Rechtslage im Wesentlichen entsprechend der Reichsstrafprozessordnung in der Fassung der Neubekanntmachung von 1924 wiederhergestellt (vgl. im Einzelnen Ziemba, Die Wiederaufnahme des Verfahrens zuungunsten des Freigesprochenen oder Verurteilten &lt;§§ 362 ff. StPO&gt;, 1974, S. 71 und 143; Bohn, Die Wiederaufnahme des Strafverfahrens zuungunsten des Angeklagten vor dem Hintergrund neuer Beweise, 2016, S. 87 f.).</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -590,14 +590,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>a) Dieser zielte nach der Entwurfsbegründung darauf ab, die ausgleichsbedingte Bundestagsvergrößerung, welche den Deutschen Bundestag an die Grenzen seiner Arbeits- und Handlungsfähigkeit bringen und die Akzeptanz des Parlaments in der Bevölkerung beeinträchtigen könne, zu vermindern (vgl. BTDrucks 19/22504, S. 1, 5). Dies sollte zum einen dadurch erreicht werden, dass mit Wirkung ab dem 1. Januar 2024 bei Beibehaltung der Regelgröße des Deutschen Bundestages von 598 Abgeordneten die Zahl der Wahlkreise auf 280 reduziert wird (vgl. BTDrucks 19/22504, S. 1, 5 f., 8). Zum anderen sah der Entwurf eine unmittelbar mit Inkrafttreten des Gesetzes wirksam werdende Änderung des Sitzzuteilungsverfahrens vor. Demnach sollte mit dem Ausgleich von Überhangmandaten erst nach dem dritten Überhangmandat begonnen und ein weiterer Aufwuchs zudem durch Anrechnung von Wahlkreismandaten auf Listenmandate derselben Partei in anderen Ländern vermieden werden (vgl. BTDrucks 19/22504, S. 1, 5). Da in der Folge erneut Überhangmandate auftreten konnten, sah der Entwurf zudem vor, die zuletzt in § 48 Abs. 1 Satz 2 BWahlG 2008 vorgesehene Regelung zum Ausschluss der Listennachfolge für den Fall, dass die betroffene Partei in dem entsprechenden Land über Überhangmandate verfügt, wiedereinzuführen (vgl. BTDrucks 19/22504, S. 1, 5).</t>
+          <t>Nach Gründung der Bundesrepublik Deutschland galt dies bundeseinheitlich aufgrund des Gesetzes zur Wiederherstellung der Rechtseinheit auf dem Gebiete der Gerichtsverfassung, der bürgerlichen Rechtspflege, des Strafverfahrens und des Kostenrechts vom 20. September 1950 (BGBl S. 455). In der Folgezeit wurde eine Reform des Wiederaufnahmerechts im Schrifttum diskutiert (vgl. nur Peters, Fehlerquellen im Strafprozeß, Bd. 2, 1972, S. 321; Ziemba, Die Wiederaufnahme des Verfahrens zuungunsten des Freigesprochenen oder Verurteilten &lt;§§ 362 ff. StPO&gt;, 1974; BRAK, Denkschrift zur Reform des Rechtsmittelrechts und der Wiederaufnahme des Verfahrens im Strafprozess, 1971, S. 76; Meyer, Wiederaufnahmereform, 1977, S. 158; Deml, Zur Reform der Wiederaufnahme des Strafverfahrens, 1979, S. 142), ohne dass es zu Änderungen zuungunsten des Angeklagten kam.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -606,14 +606,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>b) Der Entwurf der Regierungsfraktionen wurde in der 177. Sitzung des 19. Deutschen Bundestages am 18. September 2020 in erster Lesung beraten und sodann federführend an den Ausschuss für Inneres und Heimat überwiesen (vgl. BT-Plenarprotokoll 19/177, S. 22326 ff.). Nachdem der Ausschuss am 5. Oktober 2020 auf Grundlage schriftlicher Stellungnahmen (vgl. BTAusschussdrucks 19&lt;4&gt;584 A-F) eine Sachverständigenanhörung zu dem Gesetzentwurf durchgeführt hatte (vgl. Ausschuss für Inneres und Heimat, Protokoll Nr. 19/100), empfahl er die Annahme des Entwurfs in unveränderter Fassung (vgl. BTDrucks 19/23187, S. 2, 6). Hinsichtlich der konkurrierenden Entwürfe der Fraktionen von FDP, DIE LINKE und BÜNDNIS 90/DIE GRÜNEN einerseits (BTDrucks 19/14672) sowie von Abgeordneten und der Fraktion der AfD andererseits (BTDrucks 19/22894) empfahl er die Ablehnung (vgl. BTDrucks 19/23187, S. 2, 6).</t>
+          <t>Im Gegensatz dazu wurde in der Deutschen Demokratischen Republik die Wiederaufnahme zuungunsten des Angeklagten aus denselben Gründen zugelassen wie zugunsten des Verurteilten; die ungünstige Wiederaufnahme war aber nur innerhalb von fünf Jahren seit Rechtskraft des Urteils möglich (§ 328 der Strafprozessordnung vom 12. Januar 1968 &lt;GBl DDR 1968 I S. 49&gt;).</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -622,14 +622,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>c) Der Gesetzentwurf der Regierungsfraktionen wurde gemeinsam mit den konkurrierenden Gesetzentwürfen in der 183. Sitzung des 19. Deutschen Bundestages am 8. Oktober 2020 in zweiter und dritter Lesung beraten; die Entwürfe der Opposition wurden abgelehnt und der Entwurf der Regierungsfraktionen wurde in unveränderter Fassung angenommen (vgl. BT-Plenarprotokoll 19/183, S. 23041 ff., 23052, 23061 ff.).</t>
+          <t>3. Der Einführung des § 362 Nr. 5 StPO gingen mehrere, jeweils durch Einzelfälle angestoßene Reformversuche voraus.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -638,14 +638,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4. a) Art. 1 Nr. 3 BWahlGÄndG fasste § 6 Abs. 5 BWahlG 2013 gänzlich und § 6 Abs. 6 BWahlG 2013 teilweise neu. § 6 Bundeswahlgesetz in der Fassung des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 lautet wie folgt:</t>
+          <t>a) Ende 1992 scheiterte im Fall des 1938 in einem Konzentrationslager verstorbenen Journalisten Carl von Ossietzky die von dessen Tochter beantragte Wiederaufnahme des Strafverfahrens, das 1931 mit einer Verurteilung von Ossietzkys durch das Reichsgericht wegen Landesverrats geendet hatte (vgl. BGHSt 39, 75). Daraufhin brachte die SPD-Bundestagsfraktion 1993 und erneut 1996 einen Gesetzentwurf zur umfassenden Reform des Wiederaufnahmerechts in den Bundestag ein. Mit Blick auf die Wiederaufnahme zuungunsten des Angeklagten wurde „wegen des verfassungsrechtlichen Grundsatzes des ‚ne bis in idem‘ (Artikel 103 Abs. 3 GG) nach dem Vorbild ausländischer Rechtsordnungen“ vorgeschlagen, die Wiederaufnahme zuzulassen, „wenn neue Tatsachen oder Beweismittel beigebracht werden, die allein oder in Verbindung mit den früher erhobenen Beweisen jeden begründeten Zweifel ausschließen, dass der Angeklagte in einer neuen Hauptverhandlung der Begehung eines Mordes (§ 211 StGB) oder Völkermordes (§ 220a StGB) überführt werden wird“ (vgl. BTDrucks 12/6219, S. 1, 3). Nach kontroverser Debatte sah der Rechtsausschuss des 13. Deutschen Bundestages keinen umfassenden Reformbedarf (vgl. BTDrucks 13/10333, S. 4), und § 362 StPO blieb unverändert.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -654,14 +654,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>b) § 48 Abs. 1 Satz 1 und 2 BWahlG wurden durch Art. 1 Nr. 5 BWahlGÄndG wie folgt gefasst:</t>
+          <t>b) Im September 2007 brachten das Land Nordrhein-Westfalen und die Freie und Hansestadt Hamburg einen Gesetzentwurf in den Bundesrat ein, nach dem in Fällen des vollendeten Mordes und einiger Verbrechen nach dem Völkerstrafgesetzbuch eine Wiederaufnahme zulasten des Angeklagten zulässig sein sollte, „wenn auf der Grundlage neuer, wissenschaftlich anerkannter technischer Untersuchungsmethoden, die bei Erlass des Urteils […] nicht zur Verfügung standen, neue Tatsachen oder Beweismittel beigebracht werden“ (vgl. BRDrucks 655/07, S. 1; BTDrucks 16/7957, S. 5). Anlass für diese Initiative war ein Fall, in dem 1993 die Angestellte einer Videothek bei einem Raubüberfall getötet worden war und 2004 durch die Untersuchung von auf Asservaten sichergestellten Hautpartikeln diese dem zuvor mangels Beweisen Freigesprochenen zugeordnet werden konnten (vgl. BRPlenProt 837, S. 341 &lt;C&gt;-&lt;D&gt;). Auch hier kam es letztlich nicht zu einer Gesetzesänderung (vgl. Mitteilung des Rechtsausschusses des Deutschen Bundestages vom 12. März 2009 zur 130. Sitzung; BRDrucks 222/10 und BRPlenProt 869, S. 123 &lt;A&gt;, 156 &lt;D&gt;; BMJV, Abschlussbericht der StPO-Expertenkommission, 2015, S. 168 und hierzu Anlagenband I, Gutachten, S. 660; BRPlenProt 967, S. 131 &lt;C&gt; und 138 &lt;A&gt;).</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -670,14 +670,14 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>c) Art. 1 Nr. 4 BWahlGÄndG passte § 46 Abs. 2 BWahlG an die Neuformulierung des § 6 Abs. 6 BWahlG an.</t>
+          <t>c) Die Einfügung des § 362 Nr. 5 StPO durch das Gesetz zur Herstellung materieller Gerechtigkeit vom 21. Dezember 2021 ist ebenfalls durch einen Einzelfall – den hier verfahrensgegenständlichen – veranlasst (vgl. BVerfGE 162, 358 &lt;361 Rn. 7&gt; – Wiederaufnahme zuungunsten des Freigesprochenen-eA). Dazu heißt es in der Gesetzesbegründung (vgl. BTDrucks 19/30399, S. 9 f.):</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -686,14 +686,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5. Der Termin für die Wahl zum 20. Deutschen Bundestag wurde gemäß § 16 BWahlG mit Anordnung vom 8. Dezember 2020 (BGBl I S. 2769) auf den 26. September 2021 bestimmt.</t>
+          <t>4. Nach einer Auswertung des Statistischen Bundesamtes gingen im Jahr 2020 von den 13.819 vor den Landgerichten erledigten Verfahren 19 auf einen Antrag auf Wiederaufnahme zuungunsten des Angeklagten zurück (Statistisches Bundesamt, Fachserie 10, Reihe 2.3, 2020, S. 62).</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -702,14 +702,14 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6. a) Mit Beschluss vom 20. Juli 2021 (2 BvF 1/21 – Normenkontrolle Bundeswahl- recht - eA) lehnte das Bundesverfassungsgericht den Antrag der Antragstellerinnen und Antragsteller ab, im Wege der vorläufigen Regelung anzuordnen, dass Art. 1 Nr. 3 bis 5 BWahlGÄndG bei der Wahl zum 20. Deutschen Bundestag nicht anzuwenden ist.</t>
+          <t>In den zurückliegenden Jahren wurden pro Kalenderjahr knapp 10 Verfahren mit einem Freispruch vom Tatvorwurf des Mordes abgeschlossen (vgl. für 2003 und 2004: BTDrucks 16/7957, S. 2; für 2010-2019: BTDrucks 19/30798, S. 47 f.; für 2020: Statistisches Bundesamt, Fachserie 10, Reihe 3, 2020, S. 24, 50 f. und 71). Ein Freispruch vom Tatvorwurf des Völkermordes erfolgte einmal im Jahr 2011 (BTDrucks 19/30798, S. 47 f.).</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -718,14 +718,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>b) Am 26. September 2021 wurde der 20. Deutsche Bundestag gewählt. Die Sitzzuteilung fand erstmals auf Grundlage der vorliegend zur Überprüfung gestellten Bestimmungen statt. Der 20. Deutsche Bundestag zählt 736 Abgeordnete, von denen nach dem Sitzzuteilungsverfahren 206 Sitze auf die SPD, 152 auf die CDU, 118 auf BÜNDNIS 90/DIE GRÜNEN, 92 auf die FDP, 83 auf die AfD, 45 auf die CSU, 39 auf DIE LINKE sowie ein Sitz auf den Südschleswigschen Wählerverband (SSW) entfielen (vgl. Bundeswahlleiter, Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 421). Im Rahmen der ersten – fiktiven – Verteilung ergaben sich insgesamt 34 Quasi-Überhangmandate (vgl. Bundeswahlleiter, Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 417 ff.), die bei der anschließenden Erhöhung der Sitzzahl nach § 6 Abs. 5 BWahlG mit Ausnahme von drei Mandaten ausgeglichen wurden. Bei der – tatsächlichen – zweiten Sitzverteilung wurden diese als verbleibende Überhangmandate der CSU zugeordnet (vgl. Bundeswahlleiter, Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 421).</t>
+          <t>5. In Art. 4 des 7. Zusatzprotokolls zur Europäischen Menschenrechtskonvention (nachfolgend: 7. ZP-EMRK), das die Bundesrepublik Deutschland nicht ratifiziert hat, ist der Grundsatz ne bis in idem verankert, der nur für Strafverfahren innerhalb eines Staates, nicht für Strafverfahren in verschiedenen Staaten gilt (vgl. EGMR, Amrollahi v. Denmark, Entscheidung vom 28. Juni 2001, Nr. 56811/00, § 1; Trabelsi v. Belgium, Urteil vom 4. September 2014, Nr. 140/10, § 164). Dies schließt nach Absatz 2 die Wiederaufnahme des Verfahrens nach dem Gesetz und dem Strafverfahrensrecht des betreffenden Staates nicht aus, falls neue oder neu bekannt gewordene Tatsachen vorliegen oder das vorausgegangene Verfahren schwere, den Ausgang des Verfahrens berührende Mängel aufweist. Auch nach Art. 14 Abs. 7 des Internationalen Paktes über bürgerliche und politische Rechte vom 19. Dezember 1966 (BGBl II 1973 S. 1553) darf niemand wegen einer strafbaren Handlung, wegen der er bereits nach dem Gesetz und dem Strafverfahrensrecht des jeweiligen Landes rechtskräftig verurteilt oder freigesprochen worden ist, erneut verfolgt oder bestraft werden. Art. 20 des Römischen Statuts des Internationalen Strafgerichtshofes (BGBl I 2002 S. 2144) bietet Schutz vor wiederholter strafrechtlicher Verfolgung im Zusammenhang mit vor dem Strafgerichtshof geführten oder zu führenden Verfahren.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -734,14 +734,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7. a) Am 24. Januar 2023 legten die Fraktionen von SPD, BÜNDNIS 90/DIE GRÜNEN und FDP den Entwurf eines Gesetzes zur Änderung des Bundeswahlgesetzes und des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes (BTDrucks 20/5370 &lt;BWahlGÄndG 2023&gt;) vor, welches insbesondere das Sitzzuteilungsverfahren für die Wahl des Deutschen Bundestages gemäß § 6 BWahlG neu regelt. Der Gesetzentwurf wurde in der 92. Sitzung des 20. Deutschen Bundestages am 17. März 2023 in zweiter und dritter Lesung beraten und in der Fassung der Beschlussempfehlung des Ausschusses für Inneres und Heimat (BTDrucks 20/6015) beschlossen (vgl. BT-Plenarprotokoll 20/92 &lt;neu&gt;, S. 11015 ff., 11050 ff.). Der Bundesrat entschied in seiner 1033. Sitzung am 12. Mai 2023, zu dem Gesetz keinen Antrag gemäß Art. 77 Abs. 2 GG zu stellen (vgl. BRDrucks 160/23 &lt;Beschluss&gt;). Das Gesetz zur Änderung des Bundeswahlgesetzes und des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes wurde am 8. Juni 2023 durch den Bundespräsidenten ausgefertigt und am 13. Juni 2023 im Bundesgesetzblatt verkündet (BGBl I Nr. 147). Seine wesentlichen Vorschriften traten am 14. Juni 2023 in Kraft (Art. 3 BWahlGÄndG 2023).</t>
+          <t>Für die Europäische Union entfaltet das Doppelbestrafungsverbot des Art. 54 des Schengener Durchführungsübereinkommens (vom 19. Juni 1990, ABl EU Nr. L 239 vom 22. September 2000, S. 19, zuletzt geändert durch Art. 64 ÄndVO &lt;EU&gt; 2018/1861 vom 28. November 2018, ABl EU Nr. L 312 vom 7. Dezember 2018, S. 14; nachfolgend: SDÜ) transnationale Wirkung. Es findet seine Verankerung zudem in Art. 50 der Grundrechtecharta der Europäischen Union (nachfolgend: GRCh), der eine erneute Verfolgung oder Bestrafung wegen einer Straftat verbietet, deretwegen der Betroffene bereits in der Union rechtskräftig verurteilt oder freigesprochen worden ist (vgl. EuGH, Urteil vom 26. Februar 2013, Åkerberg Fransson, C-617/10, EU:C:2013:105, Rn. 33 f.; Urteil vom 5. Juni 2014, M, C-398/12, EU:C:2014:1057, Rn. 35; Urteil vom 28. Oktober 2022, PPU, C-435/22, EU:C:2022:852, Rn. 64 ff.; BVerfG, Beschluss der 1. Kammer des Zweiten Senats vom 19. Mai 2022 - 2 BvR 1110/21 -, Rn. 40 ff.).</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -750,14 +750,14 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>b) Mit Blick auf das Gesetzgebungsverfahren zur erneuten Änderung des Sitzzuteilungsverfahrens für die Wahl zum Deutschen Bundestag haben die Antragstellerinnen und Antragsteller am 13. März 2023 beantragt, das Ruhen des Verfahrens anzuordnen. Diesen Antrag hat der Zweite Senat mit Beschluss vom 22. März 2023 (2 BvF 1/21 – Normenkontrolle Bundeswahlrecht - Antrag auf Ruhen des Verfahrens) unter Verweis auf das öffentliche Interesse an der Fortführung des Verfahrens abgelehnt.</t>
+          <t>6. Eine Anfrage des Bundesverfassungsgerichts an die Europäische Kommission für Demokratie durch Recht (Venedig-Kommission) zur Rechtslage betreffend den Grundsatz ne bis in idem und die Wiederaufnahme von Strafverfahren hat ergeben, dass in den meisten derjenigen Staaten, die eine Stellungnahme abgegeben haben, der Grundsatz ne bis in idem jedenfalls aufgrund von Art. 4 des 7. ZP-EMRK eine verfassungsrechtliche Verankerung erfahren hat. Zur Zulässigkeit der Wiederaufnahme ergaben die Antworten ein heterogenes Bild nicht zuletzt deswegen, weil in den verschiedenen Rechtsordnungen unterschiedlich zwischen strafrechtlichen und ordnungs- beziehungsweise disziplinarrechtlichen Sanktionen oder unterschiedlichen Arten der Verfahrensbeendigung differenziert wird. Außerdem bestehen unterschiedliche Fristen für eine Wiederaufnahme, entweder durch den Eintritt der Verjährung der verfolgten Straftat oder anknüpfend an die Rechtskraft des Urteils; soweit eine Wiederaufnahme aufgrund neuer Tatsachen oder Beweise (propter nova) möglich ist, ist teilweise eine Frist ab Kenntniserlangung zu beachten.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -766,14 +766,14 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Die Antragstellerinnen und Antragsteller rügen einen Verstoß von Art. 1 Nr. 3 bis 5 BWahlGÄndG gegen Art. 20 Abs. 3 GG, Art. 20 Abs. 1 und 2 GG, Art. 38 Abs. 1 Satz 1 GG sowie Art. 21 Abs. 1 GG.</t>
+          <t>Eine Wiederaufnahme zuungunsten der betroffenen Person ist in sieben der ausgewerteten Staaten (vgl. auch Wissenschaftliche Dienste des Bundestages, WD 7 – 3000 – 262/18 und WD 7 – 3000 – 007/22) insgesamt unzulässig. In weiteren sieben Staaten ist sie beschränkt auf gefälschte Beweismittel, Falschaussagen oder andere Verfahrensfehler wie Korruption, Bestechung oder Amtsmissbrauch (propter falsa) vorgesehen. In 17 Staaten ist dagegen mit Unterschieden im Einzelnen eine ungünstige Wiederaufnahme auch aufgrund neuer Tatsachen oder Beweismittel (propter nova) möglich.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -782,14 +782,14 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1. Die zur Überprüfung gestellten Normen verstießen gegen das aus dem Rechtsstaatsprinzip gemäß Art. 20 Abs. 3 GG folgende Gebot der Normenklarheit, das im Bereich des Wahlrechts durch das Demokratieprinzip aus Art. 20 Abs. 2 GG konkretisiert werde.</t>
+          <t>1. Der Beschwerdeführer wurde mit seit dem 21. Mai 1983 rechtskräftigem Urteil des Landgerichts Stade vom 13. Mai 1983 vom Vorwurf der Vergewaltigung und des Mordes freigesprochen. Nach Einführung des § 362 Nr. 5 StPO stellte die zuständige Staatsanwaltschaft im Februar 2022 beim Landgericht Verden (nachfolgend: Landgericht) einen Antrag auf Wiederaufnahme des Strafverfahrens nach dieser Vorschrift und auf Erlass eines Haftbefehls. Das Landgericht erklärte den Wiederaufnahmeantrag mit Beschluss vom 25. Februar 2022 für zulässig und ordnete Untersuchungshaft gegen den Beschwerdeführer an. Die hiergegen gerichtete Beschwerde verwarf das Oberlandesgericht Celle (nachfolgend: Oberlandesgericht) mit Beschluss vom 20. April 2022 (vgl. im Einzelnen BVerfGE 162, 358 &lt;360 ff. Rn. 2 ff.&gt;).</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -798,14 +798,14 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>a) Der Gesetzgeber sei nach dem Rechtsstaatsprinzip gehalten, Gesetze hinreichend bestimmt zu fassen. Der Wille der an der Gesetzgebung beteiligten Verfassungsorgane müsse zurechenbar festgestellt werden können, damit eine demokratisch legitimierte Entscheidung vorliege. Darüber hinaus erfordere das Rechtsstaatsprinzip eine hinreichende Klarheit gesetzlicher Regelungen im Hinblick auf die Normunterworfenen; sie müssten die Rechtslage so konkret erkennen können, dass sie ihr Verhalten danach ausrichten könnten. Die Anforderungen an die Normenklarheit seien erhöht, wenn die Unsicherheit bei der Beurteilung der Gesetzeslage die Betätigung von Grundrechten erschwere. Dies gelte nicht nur bei Eingriffen in die Freiheitssphäre des Einzelnen und bei der Gewährung von Leistungen, sondern auch, wenn grundrechtsgleiche Rechte wie das Wahlrecht aus Art. 38 Abs. 1 Satz 1 GG betroffen seien. Das Bundeswahlgesetz müsse so bestimmt sein, dass für den Bürger erkennbar sei, in welcher Weise sich seine Stimmabgabe auf die Zusammensetzung des von ihm gewählten Parlaments auswirke. Diese Anforderungen würden durch das Demokratieprinzip des Art. 20 Abs. 1 und 2 GG verschärft. Die Sicherung der Integrationsfunktion der Wahl setze voraus, dass das Wahlrecht so verständlich sei, dass die Wählerinnen und Wähler den Wahlakt als einen Vorgang erlebten, in dem sie Einfluss auf die Ausübung von Staatsgewalt nehmen könnten. Darüber hinaus fordere die aus dem Demokratieprinzip folgende Wesentlichkeitslehre, dass das Wahlverfahren als für den demokratischen Prozess wesentlichste Frage durch den Gesetzgeber in einem transparenten Verfahren unter Beteiligung der parlamentarischen Opposition entschieden werde. Das Bundesverfassungsgericht habe mehrfach betont, dass im Wahlrecht hohe Anforderungen an die Rechtsklarheit zu stellen seien.</t>
+          <t>2. Mit seiner unmittelbar gegen die Beschlüsse des Oberlandesgerichts und des Landgerichts sowie mittelbar gegen § 362 Nr. 5 StPO gerichteten Verfassungsbeschwerde rügt der Beschwerdeführer eine Verletzung seiner Rechte aus Art. 103 Abs. 3 GG sowie aus Art. 2 Abs. 1 in Verbindung mit Art. 20 Abs. 3 GG.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -814,14 +814,14 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>b) Diesen Anforderungen werde die Neuregelung des Bundeswahlgesetzes in Art. 1 Nr. 3 bis 5 BWahlGÄndG nicht gerecht. Der Gesetzestext sei an zahlreichen Stellen unvollständig und weise systematische Brüche auf, die eine methodengeleitete Auslegung unmöglich machten. Dies führe dazu, dass wesentliche Fragen vom Bundeswahlleiter beantwortet werden müssten, dem damit unmittelbarer Einfluss auf die Umrechnung des Wahlergebnisses in Bundestagsmandate zukomme.</t>
+          <t>§ 362 Nr. 5 StPO sei verfassungswidrig und könne auch nicht verfassungskonform ausgelegt werden. Die Norm stelle keine bloße Grenzkorrektur des Art. 103 Abs. 3 GG dar. Die neue Vorschrift sei gegenüber den bisherigen Wiederaufnahmegründen wesensverschieden. Anlass für ihre Einführung seien nicht etwa aufgekommene Zweifelsfragen im Zusammenhang mit einem der bisherigen Wiederaufnahmegründe. Auch stelle die Neuregelung keine Fortschreibung der bisherigen Wiederaufnahmegründe des § 362 StPO dar; diese beträfen die Manipulation der Beweisführung (Nr. 1–3) beziehungsweise stammten aus der Sphäre des Täters (Nr. 4), der durch das Geständnis auf den Schutz durch das Doppelverfolgungsverbot verzichte.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -830,14 +830,14 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>aa) § 6 Abs. 5 Satz 1 BWahlG arbeite mit einem Zirkelverweis auf § 6 Abs. 6 BWahlG. § 6 Abs. 6 BWahlG setze nach seinem Wortlaut voraus, dass die Anzahl der zu vergebenden Sitze bereits nach § 6 Abs. 5 BWahlG berechnet worden sei. § 6 Abs. 5 BWahlG setze wiederum voraus, dass parallel eine Berechnung nach § 6 Abs. 6 BWahlG stattfinde. Bei strenger Beachtung des Wortlauts sei die Rechenoperation nicht durchführbar. Nur unter Zuhilfenahme der Entwurfsbegründung lasse sich die Bestimmung dahingehend auslegen, dass ein stufenweises Verfahren durchzuführen sei, bei dem die Sitzzahl schrittweise erhöht werde.</t>
+          <t>Die Wertung des Gesetzgebers, dass durch einen erwiesenermaßen ungerechtfertigten Freispruch der Rechtsfrieden und das Gerechtigkeitsgefühl der Bevölkerung in mindestens ebenso starkem Maße beeinträchtigt werde wie durch die Verurteilung eines unschuldigen Angeklagten (vgl. BTDrucks 19/30399, S. 9 f.), missachte die Funktion des Strafverfahrens. Zu seinen verfahrensrechtlichen Vorkehrungen gehöre, dass nur der Verurteilte nach § 359 Nr. 5 StPO neue Tatsachen oder Beweismittel geltend machen könne. Diese Besserstellung sei von Verfassungs wegen geboten und dürfe nicht durch eine gleichgewichtige Urteilskorrektur zur Durchsetzung des staatlichen Strafanspruchs ausgehöhlt werden. Der in den Gesetzesmaterialien angeführte Begriff der Unerträglichkeit sei emotionalisiert und unbestimmt und daher nicht geeignet, als rechtssicheres Kriterium für die Kodifizierung von Ausnahmen vom Grundsatz ne bis in idem zu dienen. Die dort zum Ausdruck kommende Annahme, die „sehr hohe Schwelle“ der dringenden Gründe für eine Verurteilung sichere die Verhältnismäßigkeit der Gesamtregelung ab, verfehle die Verdachtslage bei der Wiederaufnahme. Denn allen Urteilen liege ein Eröffnungsbeschluss und damit die Annahme des hinreichenden Tatverdachts zugrunde. Es sei rational nicht vermittelbar, dass dieser eine mindere Intensität aufweise als der dringende Tatverdacht nach § 114 Abs. 2 Nr. 4 StPO. Daher sei nicht sichergestellt, dass eine Verurteilung mit ganz überwiegender Wahrscheinlichkeit zu erwarten sei. Schließlich verstoße die Beseitigung der Rechtskraft des freisprechenden Urteils gegen das aus dem Rechtsstaatsprinzip folgende Rückwirkungsverbot.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -846,14 +846,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>bb) § 6 Abs. 5 Satz 4 BWahlG sei normenunklar. Aus dem Text lasse sich keine Rechenoperation ableiten, die es ermögliche, das nach der Entwurfsbegründung verfolgte Ziel der Entstehung von bis zu drei unausgeglichenen Überhangmandaten zu erreichen. Auslegungsmöglichkeiten, die dazu führten, dass der Norm eine eindeutige Rechenoperation entnommen werden könne, fehlten.</t>
+          <t>Auf den Antrag des Beschwerdeführers auf Erlass einer einstweiligen Anordnung hat der Senat den Vollzug des Haftbefehls des Landgerichts vom 25. Februar 2022 mit Beschluss vom 14. Juli 2022 (BVerfGE 162, 358), wiederholt mit Beschluss vom 20. Dezember 2022, unter Auflagen ausgesetzt. Mit Beschluss vom 16. Juni 2023 wurde die einstweilige Anordnung ohne Auflagen verlängert.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -862,14 +862,14 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>(1) Bezüglich der Formulierung „bis zu einer Zahl von drei“ seien drei verschiedene Auslegungen denkbar: drei Sitze pro Landesliste, drei Sitze pro Partei oder drei Sitze insgesamt. Der Wortlaut lege nahe, von bis zu drei Sitzen pro Landesliste einer Partei auszugehen, denn § 6 Abs. 5 Satz 4 BWahlG verwende bei dem Verweis auf § 6 Abs. 4 Satz 1 BWahlG das Wort Landesliste in der Einzahl. Dafür, dass bis zu drei Sitze pro Partei insgesamt unberücksichtigt bleiben sollten, spreche demgegenüber der systematische Zusammenhang von § 6 Abs. 5 Satz 4 mit § 6 Abs. 5 Satz 1 und 3 BWahlG, die jeweils auf die Gesamtzahl der den Landeslisten oder Parteien zugeordneten Sitze verwiesen. Die Sachverständigen Pukelsheim und Behnke seien davon ausgegangen, dass § 6 Abs. 5 Satz 4 BWahlG bis zu drei Sitze bezogen auf alle Parteien in allen Bundesländern meine. Dafür spreche auch die Begründung des Gesetzentwurfs, wonach im Ergebnis bis zu drei Überhangmandate entstehen sollten. Allerdings beziehe sich die Begründung insofern auf die Neuregelung in § 6 Abs. 6 BWahlG. Zudem sei der Wert der Entwurfsbegründung als Auslegungshilfe beschränkt. Im Gesetzgebungsverfahren sei mehrfach auf die missverständliche Formulierung hingewiesen worden, ohne dass der Gesetzgeber eine Klarstellung vorgenommen habe. Die Aussagekraft der Gesetzesmaterialien sinke, wenn das Gesetz – wie vorliegend – sehr umstritten und nur das Ergebnis eines Formelkompromisses sei. Jedenfalls stehe einer Auslegung im Sinne von drei Mandaten insgesamt entgegen, dass aus dem Wortlaut nicht hervorgehe, wie diese drei Mandate zu bestimmen seien.</t>
+          <t>Der Bundestag, der Bundesrat, das Bundeskanzleramt, das Bundesministerium des Innern und für Heimat, das Bundesministerium der Justiz, die Landesregierungen, der Bundesgerichtshof, die Nebenklägerin im fachgerichtlichen Verfahren, der Generalbundesanwalt beim Bundesgerichtshof, die Direktorin der Abteilung Strafrecht am Max-Planck-Institut zur Erforschung von Kriminalität, Sicherheit und Recht in Freiburg, die Bundesrechtsanwaltskammer, der Deutsche Anwaltverein e.V., der Deutsche Richterbund e.V., die Neue Richtervereinigung e.V., das Organisationsbüro der Strafverteidigervereinigungen sowie der Arbeitskreis deutscher, österreichischer und schweizerischer Strafrechtslehrer (Arbeitskreis Alternativ-Entwurf) haben Gelegenheit zur Stellungnahme erhalten.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -878,14 +878,14 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>(2) Der vagen Formulierung „unberücksichtigt bleiben“ könne eine exakte Rechenoperation nicht entnommen werden. Wie das Tatbestandsmerkmal zu verstehen sei, hänge von der Auslegung der Formulierung „bis zu einer Zahl von drei“ ab. Werde diese so verstanden, dass sie eine vorab identifizierbare Zahl von Sitzen bezeichne, lasse sich das Tatbestandsmerkmal dahin verstehen, dass die nicht zu berücksichtigenden Sitze nach dem Ausgleich von der errechneten Gesamtmandatszahl abgezogen würden. Dies führe dazu, dass sich die Bundestagsgröße um bis zu drei Mandate verringere. Naheliegender sei es, bei der Berechnung der Erhöhung anzusetzen. Das „Unberücksichtigt-Bleiben“ beziehe sich in diesem Fall auf § 6 Abs. 5 Satz 1 BWahlG. Es sei indes nicht möglich, drei Mandate bei der Berechnung „unberücksichtigt“ zu lassen, wenn man diese nicht einer bestimmten Partei zuordnen könne. Die Sachverständigen Pukelsheim und Behnke hätten insofern ein Rechenverfahren eingesetzt, wonach die Zahl der Sitze so lange erhöht werde, bis denjenigen Parteien, denen Sitze nach § 6 Abs. 5 Satz 4 BWahlG zustünden, eine Sitzzahl zugeordnet werde, die die Summe der allen Landeslisten nach § 6 Abs. 5 Satz 2 und 3 BWahlG zugeordneten Sitze nicht um mehr als drei unterschreite, und gleichzeitig jede Partei mindestens die Gesamtzahl der ihren Landeslisten nach § 6 Abs. 5 Satz 2 und 3 BWahlG zugeordneten Sitze erhalte. Für diese Rechenoperation finde sich im Wortlaut der Norm kein Anhaltspunkt.</t>
+          <t>1. Aus dem Deutschen Bundestag haben die Fraktionen von BÜNDNIS 90/DIE GRÜNEN und der FDP gemeinsam (a) und die Fraktionen der SPD (b) sowie der CDU/CSU (c) jeweils gesondert Stellung genommen.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -894,14 +894,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>cc) Soweit § 6 Abs. 5 Satz 5 BWahlG bestimme, dass sich die Gesamtzahl der Sitze um die Unterschiedszahl erhöhe, sei unklar, welche Unterschiedszahl gemeint sei, da in den Sätzen zuvor drei verschiedene Größen (Regelgröße des Bundestages, Zahl der „nicht zu berücksichtigenden Mandate“, erhöhte Sitzzahl ohne Überhangmandate) in Bezug genommen würden. Gemeint sei vermutlich die Differenz zwischen der gesetzlichen Regelgröße des Bundestages und der erhöhten Zahl der Mandate ohne die Überhangmandate. Aus dem Wortlaut sei dies jedoch nicht erkennbar.</t>
+          <t>a) Nach der gemeinsamen Stellungnahme der Fraktionen von BÜNDNIS 90/DIE GRÜNEN und der FDP ist § 362 Nr. 5 StPO wegen Verstoßes gegen Art. 103 Abs. 3 GG und das in Art. 2 Abs. 1 in Verbindung mit Art. 20 Abs. 3 GG wurzelnde Rückwirkungsverbot verfassungswidrig.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -910,14 +910,14 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>dd) Die Unklarheiten setzten sich in § 6 Abs. 6 BWahlG fort, der die endgültige Sitzverteilung regele. In § 6 Abs. 6 Satz 1 BWahlG bleibe offen, was genau „die nach Absatz 5 zu vergebenden Sitze“ seien. In Betracht komme die erhöhte Zahl der Sitze mit oder ohne die nicht ausgeglichenen Überhangmandate. Da die Überhangmandate nicht proportional nach dem Zweitstimmenergebnis verteilt würden, könne nur die Zahl der Sitze ohne die Überhangmandate gemeint sein. Diese Auslegung führe allerdings zu einem unauflösbaren Widerspruch mit § 6 Abs. 6 Satz 2 BWahlG, wonach in den Parteien die Sitze nach der Zahl der zu berücksichtigenden Zweitstimmen auf die Landeslisten verteilt würden und jeder Landesliste mindestens die nach § 6 Abs. 5 Satz 2 BWahlG für sie ermittelte Sitzzahl zustehe. Gehe man davon aus, dass nach § 6 Abs. 6 Satz 1 BWahlG die Gesamtzahl der Sitze ohne Berücksichtigung der Überhangmandate verteilt werde, sei es unmöglich, diese Sitze nach Maßgabe des § 6 Abs. 6 Satz 2 BWahlG zu verteilen, da dies eine Einbeziehung der Überhangmandate voraussetze. Dieser Widerspruch lasse sich nicht ohne Bruch auflösen. Jedenfalls werde die notwendige Berechnung durch den Gesetzestext nicht so beschrieben, dass sie durch die zuständige Behörde vollzogen werden könne. § 6 Abs. 6 Satz 2 BWahlG verweise auf das in § 6 Abs. 2 Satz 2 bis 7 BWahlG beschriebene Berechnungsverfahren, welches eine rein proportionale Verteilung nach Zweitstimmen vorsehe. Die Gesetzesänderung nehme aber eine innerparteiliche föderale Proporzverzerrung hin. Es sei folglich eine Modifizierung des Berechnungsverfahrens erforderlich, die aus dem Gesetz nicht erkennbar sei. Schließlich scheine sich in § 6 Abs. 6 Satz 3 bis 5 BWahlG die Bezugsgröße der Berechnung mehrfach zu ändern. Satz 3 nehme auf die für jede Landesliste ermittelte Zahl von Sitzen Bezug. Demgegenüber stelle Satz 4 nicht auf diese Größe, sondern auf die Differenz zwischen der Zahl der gewonnenen Wahlkreismandate und der „nach Satz 1 ermittelten Zahl“ an Sitzen ab.</t>
+          <t>Art. 103 Abs. 3 GG verbürge die Einmaligkeit des Strafverfahrens und gewähre einen Ausgleich für die mit einem Strafverfahren verbundenen erheblichen Belastungen. In den Fällen des § 362 Nr. 5 StPO seien diese noch deutlich härter, weil mit erneuter Berichterstattung, vor allem aber mit erneuter Untersuchungshaft zu rechnen sei. Um das dem Strafprozess immanente Ungleichgewicht zwischen dem Angeklagten und den Strafverfolgungsbehörden auszugleichen, müsse die Wiederaufnahme zulasten des Angeklagten wesentlich höheren Voraussetzungen unterliegen als die Wiederaufnahme zu seinen Gunsten. Darin liege ein wesentlicher Unterschied zum Inquisitionsverfahren des gemeinen Rechts, das der materiellen Gerechtigkeit Vorrang gegenüber der Rechtskraft einräume und insbesondere Strafverfahren aus Mangel an Beweisen mit dem Institut der Lossprechung von der Instanz (absolutio ab instantia) nur vorläufig beende. Die Reichsstrafprozessordnung habe bewusst auf eine ungünstige Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel verzichtet, einerseits, um den Rechtskraftgedanken durchzusetzen, und andererseits, weil nunmehr die Staatsanwaltschaft als Herrin des Ermittlungsverfahrens berufen sei, dieses bei unsicherer Beweislage einzustellen (vgl. § 170 Abs. 2 StPO).</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -926,14 +926,14 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ee) Die Unmöglichkeit, einen Zusammenhang zwischen § 6 Abs. 6 Satz 2 und 4 BWahlG herzustellen, schlage auch auf § 48 Abs. 1 BWahlG durch. Nach § 48 Abs. 1 Satz 2 BWahlG gelte die Listennachfolge nicht, solange die Partei in dem betreffenden Land Mandate nach § 6 Abs. 6 Satz 4 BWahlG innehabe. Durch die Unverständlichkeit von § 6 Abs. 6 Satz 4 BWahlG sei nicht klar zu ermitteln, um welche Mandate es sich handele. Soweit sich aus Sinn und Zweck der Regelung schließen lasse, dass es sich vermutlich um die bis zu drei ausgleichslosen Überhangmandate handele, fehle der Regelung die erforderliche Bestimmtheit. Sie spreche von Mandaten „in dem betreffenden Land“, jedoch ordneten weder § 6 Abs. 5 Satz 4 BWahlG noch § 6 Abs. 6 Satz 4 BWahlG die Mandate einem konkreten Land zu. Im Gesetzgebungsverfahren seien unterschiedliche Auslegungs- und Berechnungsvarianten zur Bestimmung der Überhangmandate vertreten worden; weitere seien denkbar. Dies zeige, dass ein Vollzug der Vorschrift durch die zuständige Behörde nicht möglich sei.</t>
+          <t>Auch aus dem historischen Hintergrund des Art. 103 Abs. 3 GG folge, dass der Gesetzgeber die Wiederaufnahme zulasten des Angeklagten nicht um den Grund neuer Tatsachen oder Beweise erweitern dürfe. Mit den grundgesetzlichen Garantien betreffend die Strafrechtspflege habe der Verfassungsgeber als Reaktion auf die Erfahrungen in der Zeit der nationalsozialistischen Willkürherrschaft ausschließen wollen, dass die Justiz für justizfremde Zwecke missbraucht werden könne. Die zur Zeit des Nationalsozialismus eingeführten Wiederaufnahmemöglichkeiten hätten aus Sicht der Rechtswissenschaft der unmittelbaren Nachkriegszeit trotz ihrer Begrenzungen mangels klarer Entscheidungsmaßstäbe bewirkt, dass „der Freispruch des Richters dem Freigesprochenen die Freiheit nicht mehr verschaffte“ (unter Verweis auf Bader, Die deutschen Juristen, 1947, S. 14). Dasselbe gelte für § 362 Nr. 5 StPO.</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -942,14 +942,14 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2. Die zur Überprüfung gestellten Normen verstießen darüber hinaus gegen die Grundsätze der Wahlgleichheit (Art. 38 Abs. 1 Satz 1 GG) und der Chancengleichheit der Parteien (Art. 21 Abs. 1 GG).</t>
+          <t>Die Neuregelung stelle auch keine bloße Grenzkorrektur im Randbereich des Art. 103 Abs. 3 GG dar. Die Entscheidung des Bundesverfassungsgerichts BVerfGE 56, 22 gebe nichts dafür her, dass der Gesetzgeber nach Belieben neue Wiederaufnahmegründe ergänzen dürfe. Neue Tatsachen oder Beweismittel seien kein für die Prozessrechtswissenschaft und Literatur neu auftauchender Gesichtspunkt. Dies gelte auch für neue kriminalistische Methoden. Das Wiederaufnahmerecht dürfe nicht dazu dienen, Mängel auszugleichen, die in der Struktur des gesetzlichen Verfahrens selbst wurzelten. Genau darum gehe es aber bei § 362 Nr. 5 StPO, da jedes Strafverfahren denknotwendig zeitgebunden sei, weil jedes Gericht nur auf die zum Verfahrenszeitpunkt verfügbaren Erkenntnismittel zurückgreifen könne. § 362 Nr. 5 StPO sei außerdem ein Fremdkörper im bestehenden Recht der ungünstigen Wiederaufnahme; die herkömmlichen Gründe verfolgten mitnichten Belange der materiellen Gerechtigkeit um ihrer selbst willen, sondern nähmen Angriffe auf die materielle Gerechtigkeit durch menschliches Verhalten zum Anlass für eine Wiederaufnahme. Zudem grenze § 362 Nr. 5 StPO die zur Wiederaufnahme berechtigenden neuen Tatsachen oder Beweismittel nicht ein. Damit werde für Freigesprochene die Gefahr repetitiver Strafverfolgung real. Freisprechende Urteile verlören an Autorität und könnten ihre rechtsfriedenstiftende Funktion nicht erfüllen, weil sie in den Augen der Öffentlichkeit nicht mehr als das letzte Wort gelten könnten.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -958,14 +958,14 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>a) Die Wahlgleichheit aus Art. 38 Abs. 1 Satz 1 GG fordere, dass alle Bürger ihr Wahlrecht in formal gleicher Weise ausüben könnten. Mit der Entscheidung für ein Verhältniswahlsystem habe sich der Gesetzgeber dem Gebot des gleichen Erfolgswertes jeder Stimme unterworfen. Abweichungen hiervon bedürften einer jeweils eigenständigen verfassungsrechtlichen Rechtfertigung. Das Bundesverfassungsgericht habe zudem der Möglichkeit des Gesetzgebers, ausgleichslose Überhangmandate zuzulassen, eine klare Grenze gesetzt. Überhangmandate seien schon begrifflich nur solche Mandate, die aufgrund eines nicht vollständig durchgeführten Verrechnungsverfahrens entstünden. Dies treffe auf Mandate, die aufgrund einer gesetzgeberischen Entscheidung bewusst in proporzverzerrender Weise erzwungen würden, nicht zu. Die Gewährleistungen der Wahlgleichheit würden verstärkt durch die Chancengleichheit der Parteien aus Art. 21 Abs. 1 GG. Durch eine ungleiche Gewichtung der auf die Parteien entfallenden Stimmen werde auch die Gleichheit der Parteien in der Wahl als Wettbewerbsprozess berührt.</t>
+          <t>Dass die Wiederaufnahme der materiellen Gerechtigkeit zum Durchbruch verhelfe, könne nicht als rechtfertigender Belang herangezogen werden. Naturgemäß könne erst nach dem erneuten Strafverfahren beantwortet werden, ob ein Freispruch ungerechtfertigt sei. Davor bestehe nur ein dringender Verdacht, an dem auch ein hoher Verdachtsgrad nichts ändern könne. Insbesondere bei Mordverdacht sei die Freispruchquote deutlich höher als bei dem Gesamtaufkommen aller Straftaten, wegen derer Untersuchungshaft angeordnet werde. Wiederaufgenommene Prozesse dürften zudem häufig mit einem Freispruch enden, weil durch den Zeitverlauf weitere, neben den neuen Tatsachen oder Beweismitteln erforderliche Erkenntnismittel verloren gingen, ihre Qualität abnehme oder sie nicht mehr verwertbar seien. Der Gesetzgeber habe auch versäumt, den Widerspruch zwischen § 362 Nr. 5 StPO und § 373 Abs. 1 StPO zu klären, so dass unklar bleibe, ob das Gericht nach erneuter Hauptverhandlung auf eine Verurteilung wegen der in § 362 Nr. 5 StPO genannten Delikte beschränkt wäre.</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -974,14 +974,14 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>b) Das geänderte Wahlgesetz verstoße gegen diese Vorgaben. Die Überhangmandate seien nicht mehr Systemfolge der personalisierten Verhältniswahl, sondern würden vom Gesetzgeber erzwungen. Davon ausgehend könne die mit den Überhangmandaten verbundene Proporzverzerrung nicht durch das besondere Anliegen der Personalisierung gerechtfertigt werden. Diesem sei mit einem Vollausgleich von Überhangmandaten in gleicher Weise gedient. Jedenfalls sei die Grenze des Erforderlichen überschritten. Das Ziel, die Vergrößerung des Bundestages zu dämpfen, werde durch den Nichtausgleich von bis zu drei Überhangmandaten in derart geringer Weise gefördert, dass es den damit verbundenen Eingriff in die Wahlgleichheit und die Chancengleichheit der Parteien nicht legitimieren könne.</t>
+          <t>b) Die Fraktion der SPD hält die Verfassungsbeschwerde für unbegründet. § 362 Nr. 5 StPO sei verfassungsgemäß.</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -990,14 +990,14 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Der Deutsche Bundestag, der Bundesrat, die Bundesregierung sowie die Landesregierungen haben gemäß § 77 Nr. 1 BVerfGG Gelegenheit zur Äußerung erhalten. Von dieser haben der Deutsche Bundestag (1.) und die Bundesregierung (2.) Gebrauch gemacht.</t>
+          <t>Art. 103 Abs. 3 GG sei nicht verletzt. Die Norm beinhalte nach ihrem eindeutigen Wortlaut schon kein Mehrfachverfolgungs-, sondern nur ein Mehrfachbestrafungsverbot. Dieses greife bei § 362 Nr. 5 StPO mangels Bestrafung im Erstverfahren nicht. Aus der Entstehungsgeschichte ergebe sich nichts anderes. In den Beratungen des Parlamentarischen Rates fänden sich keine Hinweise darauf, dass neben der wiederholten Bestrafung auch die erneute Strafverfolgung habe erfasst werden sollen. Die gegenteilige Auffassung des Bundesgerichtshofs beruhe auf einer grundlegend falschen Prämisse, da die rechtsstaatlichen Grundlagen des Mehrfachverfolgungsverbots nicht mit denen des Doppelbestrafungsverbots identisch seien. Das Mehrfachverfolgungsverbot sei als Bestandteil des Rechtsstaatsprinzips in Art. 20 Abs. 3 GG zu verorten. Eine Abwägung mit anderen Grundsätzen des Rechtsstaats, hier der materiellen Gerechtigkeit, sei dann möglich.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1006,14 +1006,14 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1. Der Deutsche Bundestag hält den Antrag für unbegründet.</t>
+          <t>Ungeachtet dessen sei auch Art. 103 Abs. 3 GG nicht abwägungsfest, sondern verlange nur den Ausnahmecharakter der Wiederaufnahme. Verfassungsrechtlich ausgeschlossen sei eine routinemäßige Überprüfung rechtskräftiger Freisprüche oder eine Wiederaufnahme allein aufgrund einer Neubewertung bereits vorhandener Beweismittel. § 362 Nr. 5 StPO normiere hingegen einen exzeptionellen Vorbehalt zugunsten der materiellen Gerechtigkeit in Fällen, in denen die Rechtskraft des Urteils keine Befriedungsfunktion mehr entfalte.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1022,14 +1022,14 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>a) aa) Das Entstehen von bis zu drei ausgleichslosen Überhangmandaten nach § 6 Abs. 5 Satz 4 BWahlG sei mit der Wahlgleichheit sowie der Chancengleichheit der Parteien vereinbar. Nach der Rechtsprechung des Bundesverfassungsgerichts sei die mit Überhangmandaten einhergehende Beeinträchtigung des Zweitstimmenproporzes durch die Zielsetzung der personalisierten Verhältniswahl gerechtfertigt, solange dadurch der Grundcharakter der Bundestagswahl als Verhältniswahl nicht aufgehoben werde. Davon könne erst ausgegangen werden, wenn die Zahl der Überhangmandate etwa die Hälfte der für die Bildung einer Fraktion erforderlichen Zahl überschreite. Dem trage § 6 Abs. 5 Satz 4 BWahlG Rechnung, da nur bis zu drei ausgleichslose Überhangmandate zugelassen würden.</t>
+          <t>Die Neuregelung sei auch verhältnismäßig, da sie eine Vielzahl materieller und prozessualer Einschränkungen enthalte, die den Ausnahmecharakter der Wiederaufnahme gewährleisteten. Dies seien insbesondere die dringenden Gründe für eine Verurteilung und die Begrenzung auf besonders schwere Straftaten. Die Annäherung an die materielle Wahrheit sei ein wesentliches Instrument des deutschen Strafverfahrensrechts. Es sei hingegen nicht wie das adversatorische Verfahrensmodell von Elementen des Wettstreits und insbesondere der Vorstellung geprägt, dass der Staat nur einen Versuch zur Überführung des Täters habe. Das gegen die Neuregelung angeführte Dammbruch-Argument sei nicht auf eine valide Risikoabschätzung gestützt.</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1038,14 +1038,14 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>bb) Die Behauptung, der Gesetzgeber dürfe ausgleichslose Überhangmandate nicht als Gestaltungsinstrument einsetzen, finde in der Rechtsprechung des Bundesverfassungsgerichts keinen Niederschlag. Außerdem erzwinge die Gesetzesänderung keine Überhangmandate. Sie lasse lediglich zu, dass bis zu drei ausgleichslose Überhangmandate entstehen könnten. Einen Zwang zum Vollausgleich habe das Bundesverfassungsgericht nicht angenommen.</t>
+          <t>Ein Verstoß gegen das Rückwirkungsverbot sei ebenfalls nicht gegeben. Die überragenden Ziele des Gemeinwohls, die der Gesetzgeber mit § 362 Nr. 5 StPO verfolge, könnten nur erreicht werden, wenn die Vorschrift auch auf Fälle angewendet werde, in denen die Betroffenen bereits vor Inkrafttreten der Neuregelung rechtskräftig freigesprochen worden seien. Das Bundesverfassungsgericht habe 1999 eine echte Rückwirkung gebilligt, wenn die Gesetzesänderung ein zentrales Gebot der Gerechtigkeit darstelle (unter Verweis auf BVerfGE 101, 239 &lt;268 f.&gt;). Im Jahr 2021 habe es für die Fälle nachträglicher Vermögensabschöpfung entschieden, dass eine echte Rückwirkung zur Erweisung der Gerechtigkeit und Unverbrüchlichkeit der Rechtsordnung gerechtfertigt sein könne; es habe als überragenden Gemeinwohlbelang die Notwendigkeit anerkannt, einem für die Rechtstreue der Bevölkerung abträglichen Eindruck eines erheblichen Vollzugsdefizits entgegenzuwirken (unter Verweis auf BVerfGE 156, 354 &lt;410 f. Rn. 151 f.&gt;). Dies müsse erst recht für eine unterlassene Wiederaufnahme in einem Mordfall trotz gravierender neuer Beweise gelten.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1054,14 +1054,14 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cc) Die Annahme, die Zulassung von bis zu drei ausgleichslosen Überhangmandaten habe auf die Größe des Bundestages nur geringen Einfluss, beruhe auf nur einer Modellrechnung mit Daten nur eines Zeitpunktes. Dies erlaube keinen generellen Rückschluss auf die Dämpfungswirkungen der Regelung. Außerdem liege die verfassungsrechtliche Rechtfertigung der Überhangmandate nicht in der Reduzierung der Größe des Bundestages, sondern darin, dem Wähler im Rahmen der Verhältniswahl die Wahl von Persönlichkeiten zu ermöglichen.</t>
+          <t>c) Die Fraktion der CDU/CSU hält die Verfassungsbeschwerde ebenfalls für unbegründet und § 362 Nr. 5 StPO für verfassungskonform.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -1070,14 +1070,14 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>b) Die Regelungen des Sitzzuteilungsverfahrens seien hinreichend bestimmt.</t>
+          <t>Der Verfassungsgeber habe sich für eine enge Fassung des Art. 103 Abs. 3 GG entschieden. Seine Kerngewährleistung verbiete eine doppelte Bestrafung und eine Strafverfolgung zum Zweck einer doppelten Bestrafung. Er umfasse jedoch kein generelles Verbot mehrfacher Strafverfolgung. Faktisch und grundrechtsdogmatisch unterscheide sich eine doppelte Bestrafung gravierend von einer erneuten Strafverfolgung. Bei ersterer gehe es um Eingriffe in Art. 2 Abs. 2 Satz 2, Art. 14 Abs. 1 und Art. 1 Abs. 1 in Verbindung mit Art. 2 Abs. 1 GG, bei letzterer für sich betrachtet um den Verlust an Rechtssicherheit und den Schutz des individuellen Rechtsfriedens.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1086,14 +1086,14 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>aa) Der Normgehalt könne durch methodengerechte Auslegung ermittelt werden. Für das gebotene Maß an Bestimmtheit sei auf die Eigenart des Regelungsgegenstands und den Normzweck abzustellen. Demgemäß müssten die Regelungen des Sitzzuteilungsverfahrens der Bundestagswahl komplex sein, da sie unterschiedliche und zum Teil gegenläufige Prinzipien und Wahlrechtsgrundsätze beachten müssten. Erhöhte man entsprechend dem Antragsvorbringen die Bestimmtheitsanforderungen an wahlrechtliche Sitzzuteilungsregelungen, könnte der Gesetzgeber seinen Gestaltungsspielraum nicht mehr wahrnehmen. Auch aus der Integrationsfunktion der Wahl und dem Gesichtspunkt demokratischer Wesentlichkeit folgten keine eigenständigen oder erhöhten Anforderungen an die Bestimmtheit wahlrechtlicher Sitzzuteilungsregeln.</t>
+          <t>Da strafprozess- und verfassungsrechtlich anerkannte Gründe für eine erneute Verfolgung existierten, könne Art. 103 Abs. 3 GG kein absolutes Verbot der Mehrfachverfolgung statuieren. Der Gewährleistungsumfang des Art. 103 Abs. 3 GG sei auch nicht mit der vorkonstitutionellen Rechtslage deckungsgleich, so dass eine Erweiterung des § 362 StPO um andere Tatsachen oder Beweismittel als das Geständnis (§ 362 Nr. 4 StPO) möglich sei. Zwar sei die Kerngewährleistung des Art. 103 Abs. 3 GG abwägungsfest. Jedoch lasse sich weder aus der Verfassung noch aus der Rechtsprechung des Bundesverfassungsgerichts unmittelbar ableiten, dass zum Kern des von Art. 103 Abs. 3 GG verbotenen staatlichen Handelns die Wiederaufnahme aufgrund neuer Tatsachen gehöre.</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -1102,14 +1102,14 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>bb) § 6 Abs. 5 Satz 1 und Abs. 6 Satz 1 BWahlG ließen hinreichend erkennen, dass die Sitzzahl iterativ zu erhöhen sei. Dieser Prozess habe stattzufinden, bis („so lange“) das vorgegebene Ziel erreicht sei, dass die Parteien bei der zweiten Verteilung mindestens die Gesamtzahl der ihren Landeslisten nach den Sätzen 2 und 3 zugeordneten Sitze erhielten. Ein Zirkelverweis liege nicht vor.</t>
+          <t>Für die Verhältnismäßigkeitsprüfung existiere kein Sondermaßstab wie eine Beschränkung auf Grenzkorrekturen oder ein Unerträglichkeitserfordernis. Es sei Zurückhaltung bei der verfassungsrechtlichen Maßstabsbildung geboten; insbesondere dürfe keine umstrittene strafprozessrechtsdogmatische Frage verfassungsgerichtlich entschieden werden. Das Interesse der Allgemeinheit und insbesondere der Opfer an einer als legitimes Verfassungsziel anerkannten effektiven Strafverfolgung ende nicht per se mit Eintritt der Rechtskraft. Vielmehr könnten neben den auflösenden Bedingungen der Rechtskraft nach § 362 StPO a.F. auch neue Tatsachen oder Beweismittel einen Freispruch entkräften, und das Interesse an einer wirksamen Strafverfolgung könne wiederaufleben. § 362 Nr. 5 StPO sei auf Taten mit einem exzeptionellen Unrechtsgehalt beschränkt und trage dafür Sorge, dass die Befriedungsfunktion des Strafrechts nicht dadurch Schaden nehme, dass einem dringenden Verdacht nicht nachgegangen werden könne. § 362 Nr. 5 StPO sei zudem geeignet und erforderlich sowie angemessen.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1118,14 +1118,14 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>cc) Soweit § 6 Abs. 5 Satz 4 BWahlG bei der Berechnung der zum Ausgleich erhöhten Sitzzahl bestimme, dass bis zu drei potenzielle Überhangmandate unberücksichtigt blieben, sei Bezugspunkt die „Erhöhung der Sitzzahl“ nach § 6 Abs. 5 Satz 1 BWahlG. Diese umfasse alle Länder und alle Parteien. Demgemäß gehe es um insgesamt bis zu drei Überhangmandate. Die in der Antragsschrift aufgeführten weiteren Auslegungsansätze – bis zu drei Sitze pro Landesliste oder Partei – verfehlten Wortlaut, Systematik und Sinngehalt der Regelung. Soweit die Antragsschrift behaupte, es sei nicht bestimmbar, welches Mandat ein Überhangmandat sei, werde verkannt, dass es lediglich um eine Rechengröße gehe.</t>
+          <t>Auch die rückwirkende Anwendung des § 362 Nr. 5 StPO sei zulässig. Im Vergleich mit sachnahen Judikaten, namentlich der Entscheidung zur Vermögensabschöpfung (mit Verweis auf BVerfGE 156, 354), gerate die Wiederaufnahme nicht mit dem Rückwirkungsverbot in Konflikt.</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1134,14 +1134,14 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>dd) Auch § 6 Abs. 5 Satz 5 BWahlG sei hinreichend bestimmt. Die in der Norm benannte „Unterschiedszahl“ beziehe sich auf die Differenz zwischen der gesetzlichen Regelgröße des Deutschen Bundestages und der erhöhten Gesamtzahl der Mandate.</t>
+          <t>2. Die Landesregierungen des Landes Niedersachsen, des Freistaats Bayern und der Länder Brandenburg und Hessen halten § 362 Nr. 5 StPO mit vergleichbaren Erwägungen für verfassungskonform und die Verfassungsbeschwerde für unbegründet. Die Landesregierung des Freistaats Thüringen erachtet § 362 Nr. 5 StPO wegen Verstoßes gegen Art. 103 Abs. 3 GG für verfassungswidrig.</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -1150,14 +1150,14 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ee) § 6 Abs. 6 Satz 1 BWahlG beziehe sich auf die Zahl der Sitze ohne Überhangmandate, da nur diese die „nach Absatz 5 zu vergebenden Sitze“ darstellten. Die nach § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG zu verteilende Sitzzahl schließe dagegen die ausgleichslosen Überhangmandate ein, wodurch die Zahl um bis zu drei Mandate höher ausfallen könne als nach Satz 1. Die Bewältigung der möglichen Differenz habe der Gesetzgeber einer Regelung zugeführt: Nach § 6 Abs. 6 Satz 5 BWahlG werde die Gesamtzahl der Sitze um die Unterschiedszahl erhöht, ohne dass eine erneute Proportionalverteilung stattfinde.</t>
+          <t>3. Die sowohl für als auch gegen die Neuregelung vorgebrachten Gesichtspunkte sind in den Stellungnahmen des Arbeitskreises Alternativ-Entwurf (a), des Deutschen Anwaltvereins e.V. und des Organisationsbüros der Strafverteidigervereinigungen (b) sowie der Direktorin des Max-Planck-Instituts zur Erforschung von Kriminalität, Sicherheit und Recht in Freiburg (c) bestätigt und vertieft worden.</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -1166,14 +1166,14 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ff) Schließlich sei auch § 48 Abs. 1 Satz 2 BWahlG hinreichend bestimmt. Die in Bezug genommenen Mandate gemäß § 6 Abs. 6 Satz 4 BWahlG seien die ausgleichslosen Überhangmandate. Ein Überhang liege in einem Land vor, wenn sich dort ein Sitz nur durch die Garantie aller Wahlkreismandate gemäß § 6 Abs. 5 Satz 2 BWahlG ergebe. Um dies zu ermitteln, seien die Verteilung bei abgesenkter Sitzzahl (§ 6 Abs. 6 Satz 1 i.V.m. Abs. 5 Satz 4 BWahlG) und die Verteilung mit Garantie aller Direktmandate (§ 6 Abs. 6 Satz 2 i.V.m. Abs. 5 Satz 2 BWahlG) miteinander zu vergleichen. Die Berechnung sei iterativ nach dem Divisorverfahren mit Standardrundung vorzunehmen. Dort, wo bei der ersten Berechnung weniger Sitze anfielen als bei der zweiten, fielen die Überhangmandate an. Das Berechnungsverfahren ergebe sich aus dem Normzweck des § 48 Abs. 1 Satz 2 BWahlG und der Genese des Gesetzes.</t>
+          <t>a) Der Arbeitskreis Alternativ-Entwurf hält zum Verständnis des § 362 Nr. 5 StPO fest, dass der frühere Anklagevorwurf nicht notwendig eine Katalogtat oder überhaupt eine Straftat gegen das Leben umfassen müsse. Der Maßstab, wann eine Tatsache oder ein Beweismittel als neu anzusehen sei, könne trotz einheitlicher Formulierung in § 359 Nr. 5 und § 373a StPO nicht einheitlich bestimmt werden und sollte in § 362 Nr. 5 StPO enger gefasst werden als in § 359 Nr. 5 StPO. Das Merkmal „dringende Gründe“ könne entgegen der Begründung des Gesetzentwurfs nicht sachgerecht dem dringenden Tatverdacht als Voraussetzung für den Erlass eines Haftbefehls entsprechen, sondern müsse bei aller Schwierigkeit der Quantifizierung als „große Wahrscheinlichkeit für die Verurteilung“ interpretiert werden. Fragwürdig sei, ob allein die vollendete Tat und allein die täterschaftliche Begehung erfasst seien, zumal die Anstiftung ebenso wenig verjähre wie der Versuch. Nicht stimmig erscheine die Auswahl der fünf Straftatbestände, denn die Unverjährbarkeit sei kein eindeutiger Indikator für die Unrechtsschwere. Im Fall des Mordes sei sie der zum Zeitpunkt der Gesetzesänderung drohenden Verjährung von NS-Mordtaten geschuldet gewesen; die Unverjährbarkeit „gewöhnlicher“, nicht im Kontext von Makrokriminalität begangener Mordtaten sei ein unbeabsichtigter Nebeneffekt. Für Völkerstraftaten beruhe die Unverjährbarkeit auf Völkergewohnheitsrecht und erstrecke sich gemäß § 5 VStGB auf Taten recht unterschiedlichen Unrechtsgewichts. Es erscheine auch fraglich, ob es ein praktisches Bedürfnis für die Wiederaufnahme von Verfahren wegen Völkerstraftaten zur Vermeidung unerträglicher Ergebnisse gebe, da in den Verfahrensordnungen der internationalen Strafgerichte die ungünstige Wiederaufnahme propter nova wegen core crimes zumeist entweder nur eingeschränkt binnen eines Jahres nach Rechtskraft oder wie beim Internationalen Strafgerichtshof gar nicht zugelassen sei. Mit Blick auf die Rechtsfolgen sei festzuhalten, dass § 362 Nr. 5 StPO mangels einschränkender Bedingungen theoretisch zur Beseitigung jeglichen Freispruchs und zur Verurteilung wegen jeglichen Straftatbestands führen könne, sofern sich ex post der Verdacht einer Katalogtat ergebe.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1182,14 +1182,14 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>c) Jedenfalls sei eine verfassungskonforme Auslegung der angegriffenen Regelungen möglich. Sollten die Regelungen des Sitzzuteilungsverfahrens hinsichtlich der ausgleichslosen Überhangmandate verfassungswidrig sein, sei zu beachten, dass sie integraler Teil einer Reform des Bundestagswahlrechts seien. Würden sie für nichtig erklärt, führten die verbleibenden Teile der Neuregelung einseitig zu einer Stärkung des Verhältniselements der Bundestagswahl, was dem Willen des Gesetzgebers entgegenliefe.</t>
+          <t>Die Annahme des Gesetzgebers, es entspreche der herrschenden Meinung, dass eine Erweiterung des § 362 StPO verfassungsrechtlich zulässig sei, treffe nicht zu. Die Vereinbarkeit der Neuregelung mit Art. 103 Abs. 3 GG erscheine auch mit Blick auf die Rechtsprechung des Bundesverfassungsgerichts als zweifelhaft. Eine Unterbindung neuer Verfahren, wenn sich die Rechtslage ändere oder neue Tatsachen oder Beweismittel bekannt würden, sei keine Nebenfolge, sondern der Hauptzweck der materiellen Rechtskraft. Dies erschließe sich aus der Entwicklung des Instituts der Rechtskraft im römischen Recht und gelte sowohl bei Verurteilung wie bei Freispruch. Von Bedeutung für die deutsche Rechtsentwicklung sei zudem die Einführung des Anklageprozesses nach englischem Vorbild im Zuge der französischen Revolution. Nachdem sich die Paulskirchenverfassung 1849 zum Anklageprozess bekannt habe, habe sich dieser zunehmend durchgesetzt, wenn auch das Partikularrecht bei Schaffung der Reichsstrafprozessordnung ein inhomogenes Bild geboten habe.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1198,14 +1198,14 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2. Auch die Bundesregierung hält den Normenkontrollantrag für unbegründet.</t>
+          <t>Wegen der Beschränkung auf Fälle des Freispruchs und der Auswahl der Straftatbestände verstoße § 362 Nr. 5 StPO insgesamt auch gegen Art. 3 Abs. 1 GG.</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1214,14 +1214,14 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>a) Die Zulassung von bis zu drei Überhangmandaten verstoße nicht gegen die Gleichheit oder die Unmittelbarkeit der Wahl aus Art. 38 Abs. 1 Satz 1 GG oder die Chancengleichheit der Parteien aus Art. 21 Abs. 1 Satz 1 GG.</t>
+          <t>b) Der Deutsche Anwaltverein e.V. und das Organisationsbüro der Strafverteidigervereinigungen sehen in der Neuregelung einen Verstoß gegen Art. 103 Abs. 3 GG und das allgemeine Rückwirkungsverbot. Das Bundesverfassungsgericht habe mit den Entscheidungen BVerfGE 2, 380 und 3, 248 klargestellt, dass die vorkonstitutionellen Wiederaufnahmegründe zuungunsten des Angeklagten einen abschließenden Kanon bildeten, dessen Erweiterung um neue Wiederaufnahmegründe Art. 103 Abs. 3 GG entgegenstehe. Dies werde auch nicht durch die Entscheidung BVerfGE 56, 22 infrage gestellt. Dort habe das Bundesverfassungsgericht sich lediglich zum Tatbegriff verhalten und zudem nochmals verdeutlicht, dass Grenzkorrekturen nur innerhalb des bereits bestehenden Kanons der Wiederaufnahmegründe gestattet seien. Ebenso wenig führe die Entscheidung BVerfGE 65, 377 zu einem anderen Befund. In diesem Judikat habe das Gericht lediglich auf die vorkonstitutionell vorgezeichnete Zulässigkeit der Durchbrechung der Rechtskraft von Strafbefehlen abgestellt.</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1230,14 +1230,14 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>aa) Das verfahrensgegenständliche Gesetz entspreche der Rechtsprechung des Bundesverfassungsgerichts zu Überhangmandaten, indem es die Anzahl zulässiger Überhangmandate unterhalb der Grenze von 15 festschreibe. Die These, Überhangmandate dürften nur als „Nebenfolge“ einer wahlrechtlichen Systementscheidung zugelassen werden, überzeuge nicht. Das Bundesverfassungsgericht habe den Anfall ausgleichsloser Überhangmandate als Ausdruck der Systementscheidung für die personalisierte Verhältniswahl angesehen. Sie seien vorhersehbare Folge der besonderen Akzentuierung der Wahlkreismandate, wie sie der personalisierten Verhältniswahl eigen sei. Das Bundesverfassungsgericht habe auch die potenziell mehrheitsbeeinflussende Wirkung von Überhangmandaten akzeptiert.</t>
+          <t>c) Nach Ansicht der Direktorin des Max-Planck-Instituts zur Erforschung von Kriminalität, Sicherheit und Recht ist § 362 Nr. 5 StPO verfassungsgemäß. Das Recht der Opfer müsse stärker in den Vordergrund gerückt werden. Bei der Verhältnismäßigkeitsprüfung stünden dadurch auf beiden Seiten Individualrechte, deren umfassende Berücksichtigung nach dem Prinzip der praktischen Konkordanz erforderlich sei. Vor diesem Hintergrund sei die These eines absoluten, pauschalen Abwägungsverbots auf keinen Fall überzeugend. § 362 Nr. 5 StPO könne unter drei Bedingungen als angemessene Einschränkung des Art. 103 Abs. 3 GG eingestuft werden. Erstens sei durch die angeordnete Beschränkung auf Mord und Völkerrechtsverbrechen gewährleistet, dass wirklich nur Sachverhalte erfasst seien, bei denen auf beiden abzuwägenden Seiten subjektive Rechte stünden. Zweitens bedürften die „dringenden Gründe“ einer verfassungskonformen Auslegung dahin, dass eine sehr hohe Wahrscheinlichkeit der strafrechtlichen Verantwortlichkeit bestehen müsse, was der Fall sei, wenn die neue Tatsache oder das neue Beweismittel die Sachverhaltsrekonstruktion oder Beweislage in grundlegender Weise ändere. Drittens müsse für die schließlich verurteilten Täter als Kompensation für das zweimal zu erduldende Strafverfahren die Strafe gemindert werden.</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -1246,14 +1246,14 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>bb) Entgegen der Ansicht der Antragstellerinnen und Antragsteller sei der Gesetzgeber im Rahmen seiner Gestaltungsfreiheit nach Art. 38 Abs. 3 GG nicht zu einem Vollausgleich aller Überhangmandate verpflichtet. Soweit eine zu geringe Dämpfungswirkung des Verzichts auf einen solchen Vollausgleich kritisiert werde, sei dies verfassungsrechtlich irrelevant. Die Grenze der Funktionsunfähigkeit des Parlaments, aus der sich allenfalls die Notwendigkeit weiterer Maßnahmen zur Mandatszahlbegrenzung ergeben könnte, sei nicht erreicht.</t>
+          <t>Der Senat hat am 24. Mai 2023 eine mündliche Verhandlung durchgeführt, in der die Verfahrensbeteiligten ihr bisheriges Vorbringen ergänzt und vertieft haben. Als sachkundige Auskunftspersonen sind angehört worden: die Direktorin des Max-Planck-Instituts zur Erforschung von Kriminalität, Sicherheit und Recht in Freiburg, Professorin Dr. …, Professor Dr. …, Universität Augsburg, Rechtsanwalt … für das Organisationsbüro der Strafverteidigervereinigungen sowie Professor Dr. … als Mitglied des Bundesvorstands des WEISSER RING e.V.</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -1262,14 +1262,14 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>b) Das Sitzzuteilungsverfahren sei hinreichend bestimmt.</t>
+          <t>Die Verfassungsbeschwerde ist zulässig. Insoweit wird auf die Gründe des Beschlusses des Senats vom 14. Juli 2022 über den Antrag des Beschwerdeführers auf Erlass einer einstweiligen Anordnung verwiesen (vgl. BVerfGE 162, 358 &lt;367 ff. Rn. 31 ff.&gt;).</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -1278,14 +1278,14 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>aa) Nach der Rechtsprechung des Bundesverfassungsgerichts sei es verfassungsrechtlich nicht geboten, dass sich der Aussagegehalt von Regelungen insbesondere des Sitzzuteilungsverfahrens ohne Weiteres aus dem Wortlaut erschließe. Es genüge, wenn der Normgehalt durch Auslegung ermittelt werden könne. Das Bundesverfassungsgericht gehe davon aus, dass der Gesetzgeber eine Vorschrift so fassen dürfe, wie dies nach der Eigenart des zu ordnenden Lebenssachverhalts mit Rücksicht auf den Normzweck möglich sei. Es sei nicht ersichtlich, dass sich mit Blick auf Art. 38 GG ein anderer Bestimmtheitsmaßstab ergebe. Art. 38 Abs. 3 GG eröffne dem Gesetzgeber einen weiten Gestaltungsspielraum, der nicht konterkariert werden dürfe. Mit Blick auf die Integrationsfunktion der Wahl habe das Bundesverfassungsgericht nicht gefordert, dass die Umrechnung von Stimmen in Mandate „einfach“ sein müsse.</t>
+          <t>Die Verfassungsbeschwerde ist auch begründet. Die Wiederaufnahme des Strafverfahrens gegen den Beschwerdeführer ist verfassungswidrig. Ihre Rechtsgrundlage, der mittelbar angegriffene § 362 Nr. 5 StPO, verstößt gegen Art. 103 Abs. 3 GG (I.). Zudem verletzt seine Anwendung auf Freisprüche, die bereits zum Zeitpunkt des Inkrafttretens der Regelung am 30. Dezember 2021 rechtskräftig waren, das Rückwirkungsverbot aus Art. 103 Abs. 3 in Verbindung mit Art. 20 Abs. 3 GG (II.).</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -1294,14 +1294,14 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>bb) § 6 BWahlG sei keine leicht verständliche Vorschrift. Der Grund liege darin, dass die Norm bei der Umwandlung von Stimmen in Mandate den Anforderungen von zwei unterschiedlichen Wahlsystemen (Personen- und Verhältniswahl) genügen müsse. Zudem müsse sie dafür sorgen, dass das System der personalisierten Verhältniswahl in mathematische Handlungsschritte umgesetzt werden könne.</t>
+          <t>§ 362 Nr. 5 StPO verstößt gegen Art. 103 Abs. 3 GG. Dieses grundrechtsgleiche Recht verbietet dem Gesetzgeber die Regelung der Wiederaufnahme eines Strafverfahrens zum Nachteil des Grundrechtsträgers aufgrund neuer Tatsachen oder Beweismittel (1.). Damit ist § 362 Nr. 5 StPO nicht vereinbar (2.).</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -1310,14 +1310,14 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>cc) Dabei genüge zunächst § 6 Abs. 5 BWahlG den Bestimmtheitsanforderungen.</t>
+          <t>1. Art. 103 Abs. 3 GG enthält ein Mehrfachverfolgungsverbot auch gegenüber dem Gesetzgeber (a). Diese verfassungsrechtliche Entscheidung zugunsten der Rechtssicherheit gegenüber der materialen Gerechtigkeit ist abwägungsfest und eröffnet dem Gesetzgeber bei der Regelung der Wiederaufnahme eines Strafverfahrens keinen Spielraum (b). Als abwägungsfestes Verbot ist Art. 103 Abs. 3 GG eng auszulegen; soweit sein Schutzgehalt reicht, verbietet er dem Gesetzgeber die Eröffnung einer Wiederaufnahmemöglichkeit zum Nachteil des Grundrechtsträgers aufgrund neuer Tatsachen oder Beweismittel (c).</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -1326,14 +1326,14 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>(1) Etwas anderes folge nicht daraus, dass die möglichen Überhangmandate nicht konkret identifizierbar seien. Auf der ersten Verteilungsstufe sei ihre Identifizierung nicht notwendig, da es sich nur um eine fiktive Rechnung handele. Soweit die Überhangmandate für die endgültige Sitzzuteilung identifiziert werden müssten, sei dies möglich, indem die Sitzzahl nach der Erhöhung mit dem Mindestsitzanspruch der Parteien verglichen werde. Sei die Mindestsitzzahl der Parteien höher als die erhöhte Sitzzahl, handele es sich um Überhangmandate.</t>
+          <t>a) Art. 103 Abs. 3 GG gewährt einem Verurteilten oder Freigesprochenen ein subjektives grundrechtsgleiches Recht, das zunächst unmittelbar an die Strafgerichte und Strafverfolgungsorgane gerichtet ist (aa). Die gleiche Wirkung entfaltet Art. 103 Abs. 3 GG gegenüber dem Gesetzgeber, wenn dieser die gesetzlichen Voraussetzungen für eine erneute Strafverfolgung durch die Wiederaufnahme eines Strafverfahrens schafft (bb).</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -1342,14 +1342,14 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>(2) Soweit die Antragstellerinnen und Antragsteller meinten, die Formulierung in § 6 Abs. 5 Satz 4 BWahlG („bis zu einer Zahl von drei unberücksichtigt“) erlaube mehrere Auslegungen, beruhe dies auf einem dekonstruktivistischen Zugriff, der die Systematik der Norm nicht berücksichtige und die Unterteilung des Sitzzuteilungsverfahrens in zwei Stufen außer Betracht lasse. Weil es bei der Erhöhung nach § 6 Abs. 5 BWahlG darum gehe, die Sitzzahl zu bestimmen, die im Rahmen der zweiten Verteilung ober- und unterverteilt werde, müsse sich die Formulierung „bis zu drei Sitze“ auf die Gesamtzahl der Sitze beziehen.</t>
+          <t>aa) Der Grundsatz, dass niemand wegen derselben Tat mehrmals bestraft werden darf (ne bis in idem), beschreibt das Prinzip des Strafklageverbrauchs, das Strafgerichte und Strafverfolgungsorgane als Verfahrenshindernis von Amts wegen in jedem Stadium des Strafverfahrens zu beachten haben (vgl. BVerfGE 56, 22 &lt;32&gt;; 162, 358 &lt;371 f. Rn. 46&gt;). Soweit dieser Grundsatz eine erneute Strafverfolgung aufgrund der allgemeinen Strafgesetze betrifft, ist er durch Art. 103 Abs. 3 GG zum verfassungsrechtlichen Verbot erhoben worden (vgl. BVerfGE 3, 248 &lt;251 f.&gt;; 12, 62 &lt;66&gt;; 23, 191 &lt;202&gt;; 56, 22 &lt;32&gt;). Dabei gestaltet Art. 103 Abs. 3 GG das zunächst abstrakte Prinzip des Strafklageverbrauchs als grundrechtsgleiches Recht aus. Er gewährt dem Einzelnen Schutz, den dieser als individuelle Rechtsposition geltend machen kann (vgl. BVerfGE 56, 22 &lt;32&gt;; 162, 358 &lt;371 Rn. 46&gt;; BVerfGK 13, 7 &lt;11&gt;; vgl. auch bereits BVerfGE 3, 248 &lt;252&gt;).</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -1358,14 +1358,14 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>dd) Auch § 6 Abs. 6 BWahlG sei hinreichend bestimmt. Bei welcher Partei ein Überhangmandat auftrete, entscheide sich im Rahmen der durch § 6 Abs. 6 Satz 1 BWahlG angeordneten Verteilung. Man müsse sich dazu des Unterschieds zwischen den Sitzzahlen in § 6 Abs. 6 Satz 1 und § 6 Abs. 6 Satz 2 BWahlG vergewissern: In § 6 Abs. 6 Satz 1 BWahlG seien die Sitze, die zur Anrechnung der bis zu drei ausgleichslosen Überhangmandate führten, nicht enthalten. § 6 Abs. 6 Satz 2 BWahlG hingegen umfasse die drei Überhangmandate.</t>
+          <t>Dieser Schutz kommt Verurteilten wie Freigesprochenen gleichermaßen zu (1) und steht bereits der erneuten Strafverfolgung entgegen (2).</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -1374,14 +1374,14 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ee) Falsch sei zudem die Annahme, das Gesetz lasse im Rahmen des § 48 Abs. 1 Satz 2 BWahlG unterschiedliche Auslegungen zu, welchem Land die ausgleichslosen Überhangmandate zuzuordnen seien. Die Zuordnung ergebe sich aus einem Vergleich der gemäß § 6 Abs. 6 Satz 1 einerseits und § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG andererseits auf die Landeslisten der Parteien mit Überhängen entfallenden Sitzzahlen.</t>
+          <t>(1) Träger des grundrechtsgleichen Rechts aus Art. 103 Abs. 3 GG sind nicht nur Verurteilte, sondern auch Freigesprochene (vgl. BVerfGE 12, 62 &lt;66&gt;; 162, 358 &lt;371 Rn. 46&gt;; BVerfGK 9, 22 &lt;26&gt;).</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -1390,14 +1390,14 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Die Antragstellerinnen und Antragsteller haben auf die Stellungnahmen des Deutschen Bundestages und der Bundesregierung erwidert:</t>
+          <t>Der Wortlaut des Art. 103 Abs. 3 GG ließe zwar eine Auslegung dahingehend zu, dass diese Bestimmung nur nach einer vorangegangenen Verurteilung greift. Eine solche Beschränkung des grundrechtsgleichen Rechts auf Verurteilte hat jedoch weder der historische Verfassungsgeber vorgesehen (a), noch wird Art. 103 Abs. 3 GG in der Praxis der Strafgerichte und Strafverfolgungsbehörden in diesem Sinne verstanden (b). Sie widerspräche zudem dem Zweck des grundrechtsgleichen Rechts (c).</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -1406,14 +1406,14 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1. Die Ausführungen zur Verfassungsmäßigkeit der ausgleichslosen Überhangmandate überzeugten nicht.</t>
+          <t>(a) Die Entstehungsgeschichte der Norm streitet für die Einbeziehung des Freispruchs in den Schutzgehalt des Art. 103 Abs. 3 GG.</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -1422,14 +1422,14 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>a) Der Gestaltungsspielraum des Gesetzgebers sei nicht dadurch eingeschränkt, dass er sich für ein Wahlsystem entschieden habe, das den Grundcharakter einer Verhältniswahl trage, sondern durch die verfassungsrechtlichen Vorgaben aus Art. 38 Abs. 1 Satz 1 GG und Art. 21 Abs. 1 GG. Wahlgleichheit und Chancengleichheit seien nicht nur dann verletzt, wenn das Anfallen von Überhangmandaten den Grundcharakter der Bundestagswahl als Verhältniswahl aufhebe. Eine Verletzung liege vielmehr auch vor, wenn ein Eingriff in diese formal zu verstehenden Grundsätze nicht gerechtfertigt sei.</t>
+          <t>Die Materialien lassen erkennen, dass im Parlamentarischen Rat Einigkeit dahingehend bestand, dass die Aufnahme des Grundsatzes ne bis in idem in das Grundgesetz Schutz bereits vor der mehrfachen Verfolgung und damit auch nach Freisprüchen bieten sollte. Dem steht nicht entgegen, dass sich der Parlamentarische Rat letztlich für die Formulierung entschied, dass eine „mehrfache Bestrafung“ verboten sein solle.</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -1438,14 +1438,14 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>b) Während die Überhangmandate nach altem Recht eine Nebenfolge des Wahlsystems gewesen seien, setze die Gesetzesänderung sie als bewusste Gestaltungsressource zur Verkleinerung des Bundestages ein. Dies sei verfassungswidrig. Dass das Bundesverfassungsgericht Einschränkungen der Wahlgleichheit im „System“ der personalisierten Verhältniswahl in geringem Umfang durch das Element der Personenwahl als gerechtfertigt angesehen habe, führe nicht dazu, dass sich jede Beeinträchtigung von Wahlgrundsätzen und anderen Verfassungsgütern innerhalb dieses „Systems“ rechtfertigen lasse. Nach der Reformkonzeption diene die Regelung nicht der Personalisierung, sondern der Verkleinerung des Bundestages. Dieses Anliegen könne die verfahrensgegenständliche Regelung nicht rechtfertigen. Ein substanzieller Effekt der Überhangmandate auf die Bundestagsgröße sei nicht dargelegt. Die Überhangmandate mit dem höchsten Ausgleichsbedarf seien immer die der CSU, weil sie mit dem geringsten bundesweiten Zweitstimmenergebnis ausgeglichen werden müssten. Trotzdem blieben bei der vorgelegten Beispielrechnung nur zwei Überhangmandate der CSU und ein Überhangmandat der CDU unausgeglichen.</t>
+          <t>Am Ende der Beratung in der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege äußerte der Ausschussvorsitzende Zinn sich zwar ablehnend zu dem ursprünglichen Formulierungsvorschlag „Niemand darf mehrmals strafrechtlich verfolgt werden“. Den Unterschied zwischen „bestrafen“ und „verfolgen“ thematisierte aber weder der Vorschlag noch die Erwiderung. Zinn wandte sich insoweit vielmehr allein gegen die Formulierung „strafrechtlich“, die er anstelle von „aufgrund der allgemeinen Strafgesetze“ für zu weitreichend hielt (vgl. Wortprotokoll der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1449 &lt;1472&gt;). Damit bezog er sich auf die zuvor debattierte Begrenzung des grundgesetzlichen Verbotes auf Kriminalstrafen und das Bestreben, eine Formulierung zu finden, nach der sonstige Strafen des Disziplinar-, Ordnungs-, Polizei- oder auch des Steuerrechts weiter zulässig bleiben sollten (vgl. Wortprotokolle der 7. und 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 6. und 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1347 &lt;1433 ff.&gt; und S. 1449 &lt;1465 f.&gt;). Auch zu Beginn der 8. Ausschusssitzung hatte Zinn nicht zwischen „bestrafen“ und „verfolgen“ differenziert, vielmehr – insoweit unerwidert – betont, Grundgedanke des in Rede stehenden Grundsatzes ne bis in idem sei, „daß niemand wegen derselben Straftat wiederholt verfolgt werden darf“ (Wortprotokoll der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1449 &lt;1465&gt;). Für die Einbeziehung des Freispruchs in das Verbot des Art. 103 Abs. 3 GG spricht auch die Erörterung in der vorangehenden 7. Ausschusssitzung. Zur Darstellung der zahlreichen Problemlagen zwischen Kriminalstrafen, die vom grundgesetzlichen Verbot erfasst sein sollten, und anderen Strafen, die möglich bleiben sollten, wurde gerade ein Beispiel mit strafrechtlichem Freispruch gebildet (vgl. Wortprotokoll der 7. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 6. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1347 &lt;1436&gt;).</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -1454,14 +1454,14 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2. Die Ausführungen des Deutschen Bundestages und der Bundesregierung zur Bestimmtheit der verfahrensgegenständlichen Normen verkennten den verfassungsrechtlichen Maßstab. Soweit sie argumentierten, Gegenstand und Zweck der Sitzzuteilungsregelungen bedingten eine gehobene Komplexität, sei unklar, inwiefern dies die Unbestimmtheit von § 6 BWahlG rechtfertige. Diese folge daraus, dass wesentliche Schritte des Berechnungsverfahrens im Gesetzeswortlaut nicht geregelt würden. Eine Flexibilität in der Auslegung sei vor allem dann notwendig, wenn eine Vielzahl im Einzelnen nicht vorhersehbarer Lebenssachverhalte erfasst werden müsse, was hier nicht der Fall sei. Gerade weil es sich beim Sitzzuteilungsverfahren um mathematische Rechenoperationen handele, eigne es sich für absolut präzise Regelungen. Im Übrigen verabsolutierten Bundestag und Bundesregierung die genetische Auslegung.</t>
+          <t>Der historische Hintergrund nach dem Ende der nationalsozialistischen Herrschaft stützt dieses Verständnis. Die Aufnahme des Grundsatzes ne bis in idem in das Grundgesetz sollte der uferlosen Durchbrechung des Prinzips der Rechtskraft entgegenwirken, die in der nationalsozialistischen Zeit Platz gegriffen hatte (vgl. Entwurf eines Grundgesetzes des Verfassungskonvents der Ministerpräsidentenkonferenz der westlichen Besatzungszonen auf Herrenchiemsee vom 10. bis 23. August 1948 - Darstellender Teil, S. 56; Wortprotokoll der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1449 &lt;1465 ff.&gt;; BVerfGE 56, 22 &lt;32&gt;; BGHSt 5, 323 &lt;329 f.&gt;). Diese Durchbrechungen richteten sich gerade (auch) gegen Freigesprochene. Die Willkürherrschaft des Nationalsozialismus war namentlich dadurch gekennzeichnet, dass „der Freispruch des Richters dem Freigesprochenen die Freiheit nicht mehr verschaffte“ (vgl. Bader, Die deutschen Juristen, 1947, S. 14). Auch wenn in den Beratungen des Parlamentarischen Rates ausdrücklich nur die sogenannte Urteilsergänzung erwähnt wurde (vgl. Wortprotokoll der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1449 &lt;1472&gt;), bestehen keine Anhaltspunkte dafür, das verfassungsrechtliche Verbot der Rechtskraftdurchbrechung auf diese Variante zu beschränken (vgl. BGHSt 5, 323 &lt;330&gt;).</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -1470,14 +1470,14 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>3. Schließlich sei das Gesetz weniger als zehn Monate vor der Wahl des 20. Deutschen Bundestages in Kraft getreten und missachte folglich den von der Venedig-Kommission für Änderungen des Wahlrechts empfohlenen Zeitraum von mindestens einem Jahr vor einer Wahl. Die Verstöße gegen das Gebot der Normenklarheit seien nicht zuletzt dieser kurzfristigen Änderung geschuldet.</t>
+          <t>Dem Verfassungsgeber stand vielmehr der Grundsatz ne bis in idem in seiner breiten, maßgeblich durch das Reichsgericht geprägten Gestalt vor Augen (vgl. BVerfGE 3, 248 &lt;252&gt;; 9, 89 &lt;95 f.&gt;; 12, 62 &lt;66&gt;; 56, 22 &lt;27 f., 34&gt;). Die Reichsstrafprozessordnung von 1877 und insbesondere auch die Weimarer Reichsverfassung enthielten zwar noch keine ausdrückliche Verankerung des Grundsatzes ne bis in idem, setzten dessen Existenz aber als selbstverständlich voraus (vgl. BVerfGE 3, 248 &lt;251&gt;; BGHSt 5, 323 &lt;328&gt;). Dementsprechend ging das Reichsgericht von Anfang an von der Geltung dieses Grundsatzes aus, den es als Mehrfachverfolgungsverbot verstand (vgl. RGSt 2, 347 &lt;348&gt;; 56, 161 &lt;166&gt;; 70, 26 &lt;30&gt;; 72, 99 &lt;102&gt;; BVerfGE 3, 248 &lt;251&gt;) und auch nach Freisprüchen anwandte (vgl. RGSt 2, 347 &lt;348&gt;). Auf diesen vorkonstitutionellen Stand des Prozessrechts und seine Auslegung durch die herrschende Rechtsprechung nimmt Art. 103 Abs. 3 GG Bezug. Der Grundsatz ne bis in idem sollte insoweit durch die Aufnahme in Art. 103 Abs. 3 GG inhaltlich nicht verändert werden (vgl. BVerfGE 3, 248 &lt;252&gt;; 9, 89 &lt;96&gt;; 12, 62 &lt;66&gt;; 23, 191 &lt;202 f.&gt;; 56, 22 &lt;27 f., 34&gt;).</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -1486,14 +1486,14 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1. Der Deutsche Bundestag hat hierauf im Wesentlichen erwidert:</t>
+          <t>Schließlich hatten zum Zeitpunkt der Beratungen des Parlamentarischen Rates die meisten Landesverfassungen den Grundsatz ne bis in idem aufgenommen und dabei in ähnlicher Weise gefasst (vgl. Art. 104 Abs. 2 der Verfassung des Freistaats Bayern vom 2. Dezember 1946; Art. 4 Abs. 3 der Verfassung für Württemberg-Baden vom 28. November 1946; Art. 17 Abs. 3 der Verfassung für Württemberg-Hohenzollern vom 18. Mai 1947; Art. 7 Abs. 2 der Verfassung der Freien Hansestadt Bremen vom 21. Oktober 1947; Art. 22 Abs. 3 der Verfassung des Landes Hessen vom 1. Dezember 1946; Art. 6 Abs. 4 Satz 1 der Verfassung für Rheinland-Pfalz vom 18. Mai 1947). Es ist nicht erkennbar, dass dabei der Ausschluss von Freisprüchen in Betracht gezogen worden wäre. Auch deshalb ist nicht anzunehmen, dass der Parlamentarische Rat den grundgesetzlichen Schutz auf Verurteilte beschränken wollte.</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -1502,14 +1502,14 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>a) Die Rechtsprechung des Bundesverfassungsgerichts zur Einbettung der Überhangmandate in das vom Gesetzgeber ausgestaltete Wahlsystem habe normativen Gehalt. Das Gericht leite aus dem Grundcharakter des Wahlsystems als Verhältniswahl Grenzen für Überhangmandate ab.</t>
+          <t>(b) Die strafrechtliche Praxis unter dem Grundgesetz versteht Art. 103 Abs. 3 GG als verfassungsrechtliche Verankerung des Grundsatzes ne bis in idem und wendet ihn auf Schuld- und Freisprüche gleichermaßen an, ohne dies auch nur im Ansatz zu problematisieren. Das verfassungsrechtliche Schrifttum übernimmt dieses Verständnis als Schutzgehalt des Art. 103 Abs. 3 GG.</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
@@ -1518,14 +1518,14 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>b) Soweit die Antragstellerinnen und Antragsteller argumentierten, dass die Sitzzuteilungsregelungen hochgradig bestimmt sein müssten, zugleich aber Überhangmandate nur als Nebenfolge einer gesetzgeberischen Entscheidung zulässig seien, postulierten sie einen kaum überwindbaren Gegensatz. Unter diesen Voraussetzungen sei es für den Gesetzgeber bei der Zulassung von Überhangmandaten kaum möglich, die Grenze von einer halben Fraktionsstärke hinreichend sicher einzuhalten.</t>
+          <t>Der in Art. 103 Abs. 3 GG verankerte Grundsatz ne bis in idem ist strafrechtshistorisch eng mit der Unschuldsvermutung verknüpft (vgl. Nolte/Aust, in: v. Mangoldt/Klein/Starck, GG, Bd. 3, 7. Aufl. 2018, Art. 103 Rn. 176 f. und 231; Nolte, in: Merten/Papier, HGR, Bd. V, 2013, § 135 Rn. 4 f.; Schulze-Fielitz, in: Dreier, GG, Bd. 3, 3. Aufl. 2018, Art. 103 Abs. 3 Rn. 1). Er versteht sich als in der Aufklärung wiedergewonnenes Gegenprinzip zum Inquisitionsprozess des gemeinen Rechts (vgl. Schulze-Fielitz, in: Dreier, GG, Bd. 3, 3. Aufl. 2018, Art. 103 Abs. 3 Rn. 1). Dieser war von einem absoluten Wahrheitsanspruch einerseits und der bloßen Inquisitenstellung des Einzelnen andererseits geprägt. Dies zeigte sich insbesondere in der verfahrensrechtlichen Möglichkeit der absolutio ab instantia, die lediglich eine vorläufige Einstellung des Verfahrens bedeutete und grundsätzlich bei neuen Erkenntnissen die jederzeitige Wiederaufnahme erlaubte. Demgegenüber bestand eine zentrale Bedeutung des Anklageprozesses darin, die prinzipielle Unendlichkeit des gemeinrechtlichen Inquisitionsgrundsatzes abzulösen und ein Strafverfahren unbedingt zum Abschluss zu bringen. Gerade bei Unerweislichkeit der Schuld sollte der Strafprozess nicht nur vorläufig eingestellt, sondern dauerhaft abgeschlossen werden. Der Freispruch erhielt materiellen Gehalt, indem er „bestätigte“, dass die den Prozess leitende Unschuldsvermutung nicht widerlegt wurde. Der Grundsatz ne bis in idem zielt daher insbesondere auf den Schutz des – aus Mangel an Beweisen – Freigesprochenen ab. Er sichert die vom Rechtsstaat getroffene „Fundamentalentscheidung“ (vgl. Leitmeier, StV 2021, S. 341 &lt;343&gt;), bei nicht behebbaren Zweifeln an der Schuld nach dem Grundsatz in dubio pro reo zu verfahren und dabei zugunsten des tatsächlich Unschuldigen in Kauf zu nehmen, sich auch – zugunsten eines tatsächlich Schuldigen – irren zu können (vgl. Leitmeier, StV 2021, S. 341 &lt;343&gt;; Swoboda, HRRS 2009, S. 188 &lt;196 f.&gt;). Deshalb ist in der strafrechtlichen Praxis der Grundsatz ne bis in idem stets auch auf Freisprüche bezogen worden (vgl. BGHSt 5, 323 &lt;330&gt;; 38, 37 &lt;42 f.&gt;; BGH, NStZ-RR 2004, S. 238 &lt;240&gt;; NStZ-RR 2016, S. 47 &lt;49&gt;).</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
@@ -1534,14 +1534,14 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>c) Der postulierte Widerspruch zwischen der Personalisierung des Deutschen Bundestages einerseits und der Dämpfung seines Wachstums andererseits bestehe nicht. Wenn ein potenziell überhängendes Wahlkreismandat ausgleichslos bleibe, sei der Bundestag relativ personalisierter und zugleich kleiner als bei einem vollständigen Ausgleich. Die konkrete Dämpfungswirkung von bis zu drei ausgleichslosen Überhangmandaten hänge vom jeweiligen Wahlergebnis ab. Soweit die Antragstellerinnen und Antragsteller meinten, die ausgleichslosen Überhangmandate seien nicht stets die mit dem höchsten Ausgleichsbedarf, sei der gewählte Vergleichsmaßstab der bundesweiten Zweitstimmenverteilung verfehlt. Die Regelungen der Sitzzuteilung stellten auf eine landesbezogene Betrachtung ab.</t>
+          <t>(c) Das den Freispruch einschließende Verständnis des Art. 103 Abs. 3 GG trägt seinem grundrechtsgleichen Charakter Rechnung. Jedes Strafverfahren stellt unabhängig von seinem Ausgang eine erhebliche Belastung für den Einzelnen dar. Zweck des grundrechtsgleichen Schutzes ist die Zusicherung, dass jeder wegen derselben Tat diesen Belastungen nur einmal ausgesetzt sein soll (vgl. BVerfGE 56, 22 &lt;31&gt;; BVerfGK 4, 49 &lt;53&gt;). Art. 103 Abs. 3 GG bezweckt die Verhinderung von Grundrechtseingriffen durch das Strafverfahren, verbürgt also die „Einmaligkeit der Strafverfolgung“ (vgl. BGHSt 38, 54 &lt;57&gt;; Appel, Verfassung und Strafe, 1998, S. 133; Schmidt-Aßmann, in: Dürig/Herzog/Scholz, GG, Art. 103 Abs. 3 Rn. 301 &lt;Dez. 1992&gt;), nicht nur die „Einmaligkeit der Sühne“. Der Einzelne soll darauf vertrauen können, wegen eines konkreten individualisierten Sachverhalts nicht erneut vom Staat belangt und mit den Belastungen eines Strafverfahrens überzogen zu werden (vgl. BVerfGE 56, 22 &lt;31&gt;).</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
@@ -1550,14 +1550,14 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>d) Der Deutsche Bundestag vertrete nicht, dass für das Sitzzuteilungsverfahren ein erhöhtes Maß an Auslegungsbedürftigkeit zulässig sei. Es gelte der Bestimmtheitsmaßstab, den die Rechtsprechung aus den einschlägigen verfassungsrechtlichen Anforderungen hergeleitet habe und der demjenigen für Grundrechtseingriffe entspreche. Es seien vielmehr die Antragstellerinnen und Antragsteller, die in Abweichung von diesen Anforderungen ein erhöhtes Maß an Bestimmtheit forderten.</t>
+          <t>(2) Auch aus Entstehungsgeschichte und Zweckrichtung ergibt sich, dass Art. 103 Abs. 3 GG über seinen Wortlaut hinaus nicht allein vor einer Verurteilung, sondern auch bereits vor allen Maßnahmen schützt, deren Zweck die mögliche Verurteilung ist (vgl. BVerfGE 12, 62 &lt;66&gt;; 23, 191 &lt;202&gt;; 65, 377 &lt;381&gt;; 162, 358 &lt;371 Rn. 46&gt;; BVerfGK 4, 49 &lt;52&gt;; 13, 7 &lt;11&gt;). Art. 103 Abs. 3 GG enthält ein Mehrfachverfolgungsverbot, kein bloßes Mehrfachbestrafungsverbot.</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
@@ -1566,14 +1566,14 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2. Die Bundesregierung hat auf die Replik im Wesentlichen erwidert:</t>
+          <t>Aufgabe des Strafprozesses ist es, den Strafanspruch des Staates um des Schutzes der Rechtsgüter Einzelner und der Allgemeinheit willen in einem justizförmigen Verfahren durchzusetzen und hierdurch einen gerechten Schuldausgleich zu bewirken (vgl. BVerfGE 133, 168 &lt;198 f. Rn. 55 f.&gt;). Darf der Täter aber nicht erneut bestraft werden, kann ein gleichwohl geführtes Strafverfahren diese Funktion nicht erfüllen. Ohne die Möglichkeit einer Bestrafung entfällt die Legitimationsgrundlage dafür, den Einzelnen mit den Belastungen eines Strafverfahrens zu überziehen. Ein um seiner selbst willen geführtes Strafverfahren, an dessen Ende kein Strafausspruch erfolgen darf, würde den Einzelnen zum bloßen Objekt der Strafverfolgung herabsetzen (vgl. BVerfGE 133, 168 &lt;197 ff. Rn. 53 ff.&gt;). Strafprozessrechtlich stellt Art. 103 Abs. 3 GG deshalb ein Verfahrenshindernis dar, das als solches bereits der erneuten Einleitung eines Strafverfahrens entgegensteht (vgl. BVerfGE 56, 22 &lt;32&gt;; 162, 358 &lt;371 f. Rn. 46&gt;; BVerfGK 13, 7 &lt;11&gt;).</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
@@ -1582,14 +1582,14 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>a) Im Hinblick auf die verfassungsrechtliche Zulässigkeit ausgleichsloser Überhangmandate ließen die Antragstellerinnen und Antragsteller die Rechtsprechung des Bundesverfassungsgerichts nahezu vollständig außer Betracht. Soweit sie meinten, die Bundesregierung begründe die Zulässigkeit der bis zu drei Überhangmandate mit „vermeintlichen Systemargumenten“, verkennten sie, dass auch die Rechtsprechung eine wahlsystemische Begründung enthalte. Zudem erzwinge der Gesetzgeber ausgleichslose Überhänge nicht, sondern nehme sie in begrenztem Umfang hin.</t>
+          <t>bb) Gegenüber dem Gesetzgeber entfaltet Art. 103 Abs. 3 GG keine andere Wirkung, wenn dieser die gesetzlichen Voraussetzungen für eine erneute Strafverfolgung durch die Wiederaufnahme eines Strafverfahrens schafft (vgl. BVerfGE 15, 303 &lt;307&gt;).</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
@@ -1598,14 +1598,14 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>b) Die Komplexität von § 6 BWahlG beruhe nicht nur darauf, dass schwierige mathematische Operationen in Gesetzessprache ausgedrückt werden müssten. Sie sei auch auf die Verbindung von Personen- und Verhältniswahl und die damit erforderliche Verrechnung von Erst- und Zweitstimmen zurückzuführen sowie darauf, dass die Norm die einzelnen Berechnungsschritte hinreichend dicht steuern müsse.</t>
+          <t>Der Parlamentarische Rat hatte bei der Entscheidung für Art. 103 Abs. 3 GG nicht nur die Urteile und Verfolgungsmaßnahmen der nationalsozialistischen Willkürherrschaft im Blick, sondern auch die ausdrücklich geschaffenen Rechtsbehelfe zur Durchbrechung der Rechtskraft von Strafurteilen (vgl. Entwurf eines Grundgesetzes des Verfassungskonvents der Ministerpräsidentenkonferenz der westlichen Besatzungszonen auf Herrenchiemsee vom 10. bis 23. August 1948 - Darstellender Teil, S. 56; Wortprotokoll der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1449 &lt;1465 ff.&gt;; BVerfGE 56, 22 &lt;32&gt;). Art. 103 Abs. 3 GG sollte als grundrechtsgleiches Recht daher ebenso wie die Grundrechte des ersten Abschnitts des Grundgesetzes gemäß Art. 1 Abs. 3 GG unmittelbar gerade auch den Gesetzgeber binden.</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
@@ -1614,14 +1614,14 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>c) Mit Blick auf den von der Venedig-Kommission empfohlenen Abstand von mindestens einem Jahr zwischen der Änderung des Wahlrechts und dem Wahltermin sei zu beachten, dass der Wahltermin erst am 8. Dezember 2020 auf den 26. September 2021 festgelegt worden sei. Im Zeitpunkt der dritten Lesung des verfahrensgegenständlichen Gesetzes im Deutschen Bundestag am 8. Oktober 2020 sei eine Terminierung der Bundestagswahl noch bis zum 24. Oktober 2021 möglich gewesen. Auch wenn man auf den Zeitpunkt des Inkrafttretens des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 am 19. November 2020 abstelle, sei die Vorgeschichte der Gesetzesänderung zu berücksichtigen.</t>
+          <t>Das in Art. 103 Abs. 3 GG gegenüber den Strafverfolgungsorganen statuierte Verbot mehrfacher Strafverfolgung wäre praktisch wirkungslos, wenn die einfachgesetzliche Ausgestaltung als Wiederaufnahmeverfahren eine erneute Strafverfolgung und gegebenenfalls Verurteilung ermöglichen könnte (vgl. BVerfGE 15, 303 &lt;307&gt;; BGHSt 5, 323 &lt;331&gt;; Remmert, in: Dürig/Herzog/Scholz, GG, Art. 103 Abs. 3 Rn. 44 &lt;Nov. 2018&gt;). Ungeachtet der strafprozessrechtlichen Frage, ob ein Urteil bereits mit der Entscheidung über den Wiederaufnahmeantrag aufgehoben oder ob nur der aus dem ersten Urteil folgende Strafklageverbrauch beseitigt wird (vgl. hierzu etwa Schuster, in: Löwe/Rosenberg, StPO, Bd. 9/1, 27. Aufl. 2022, § 370 Rn. 31 ff.), ermöglicht das Rechtsinstitut der Wiederaufnahme die erneute Strafverfolgung wegen derselben Tat unter Durchbrechung der Rechtskraft eines früheren Urteils. Soll Art. 103 Abs. 3 GG als individuelles grundrechtsgleiches Recht vor einer erneuten Verurteilung gerade auch wegen der Belastungen schützen, die mit einer erneuten Strafverfolgung verbunden sind, muss es auch die gesetzlichen Regelungen erfassen, die dies strafprozessual ermöglichen (vgl. BGHSt 5, 323 &lt;331&gt;).</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
@@ -1630,14 +1630,14 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>In der mündlichen Verhandlung am 18. April 2023 haben die Beteiligten ihr Vorbringen vertieft und ergänzt. Als sachkundige Auskunftspersonen sind zu den Maßstäben des Gebots der Normenklarheit Prof. Dr. Emanuel Towfigh und Prof. (em.) Dr. Martin Morlok sowie zur Subsumtion der verfahrensgegenständlichen Normen Ministerialrat Dr. Henner Jörg Boehl sowie die Bundeswahlleiterin Dr. Ruth Brand und ihr Vorgänger im Amt, Dr. Georg Thiel, angehört worden. Zu wahlmathematischen Fragen hinsichtlich der Möglichkeit eines negativen Stimmgewichts, Beeinträchtigungen der Erfolgswertgleichheit und der Auswirkungen des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 auf die Größe des Deutschen Bundestages hat Prof. (em.) Dr. Friedrich Pukelsheim Stellung genommen.</t>
+          <t>b) Das Mehrfachverfolgungsverbot des Art. 103 Abs. 3 GG trifft eine Vorrangentscheidung zugunsten der Rechtssicherheit gegenüber der materialen Gerechtigkeit (aa). Sie steht einer Relativierung des Verbots durch Abwägung mit anderen Rechtsgütern von Verfassungsrang nicht offen (bb), so dass dem Gesetzgeber bei der Ausgestaltung des Wiederaufnahmerechts insoweit kein Gestaltungsspielraum zukommt (cc).</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
@@ -1646,14 +1646,14 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Der Normenkontrollantrag gemäß Art. 93 Abs. 1 Nr. 2 GG, § 13 Nr. 6, § 76 Abs. 1 BVerfGG ist zulässig, insbesondere liegt das erforderliche objektive Klarstellungsinteresse vor (vgl. BVerfGE 6, 104 &lt;110&gt;; 96, 133 &lt;137&gt;; 106, 244 &lt;250&gt;; 119, 394 &lt;409&gt;; 127, 293 &lt;319&gt;; stRspr).</t>
+          <t>aa) Art. 103 Abs. 3 GG gewährt dem Prinzip der Rechtssicherheit Vorrang vor dem Prinzip der materialen Gerechtigkeit.</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
@@ -1662,14 +1662,14 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Bei einem Antrag nach § 76 Abs. 1 Nr. 1 BVerfGG wird das objektive Klarstellungsinteresse schon dadurch indiziert, dass ein auf das Grundgesetz in besonderer Weise verpflichtetes Organ oder ein Organteil von der Unvereinbarkeit der Norm mit höherrangigem Bundesrecht und daher von deren Nichtigkeit überzeugt ist und eine diesbezügliche Feststellung beim Bundesverfassungsgericht beantragt (vgl. BVerfGE 96, 133 &lt;137&gt;; 106, 244 &lt;250 f.&gt;; 119, 394 &lt;409&gt;; 127, 293 &lt;319&gt;; stRspr). Das objektive Klarstellungsinteresse bleibt so lange bestehen, wie die zur Prüfung gestellte Norm Rechtswirkungen entfaltet, und entfällt lediglich dann, wenn von ihr unter keinem denkbaren Gesichtspunkt mehr Rechtswirkungen ausgehen können (vgl. BVerfGE 97, 198 &lt;213 f.&gt;; 100, 249 &lt;257&gt;; 110, 33 &lt;45&gt;; 113, 167 &lt;193&gt;; 119, 394 &lt;410&gt;; 127, 293 &lt;319&gt;; stRspr).</t>
+          <t>Die Figur der Rechtskraft prägt alle rechtsstaatlichen Entscheidungen (vgl. BVerfGE 2, 380 &lt;392 ff., 403 ff.&gt;; 60, 253 &lt;269 ff.&gt;). Sie entfaltet insbesondere dann ihre Bedeutung, wenn die Sachentscheidung materiell-rechtlich unrichtig ist oder durch Veränderungen der tatsächlichen Grundlagen unrichtig geworden ist (vgl. BVerfGE 2, 380 &lt;403 ff.&gt;; 20, 230 &lt;235&gt;; 35, 41 &lt;58&gt;; 117, 302 &lt;315&gt;). Für Entscheidungen der Exekutive bestehen unterschiedlich ausgeprägte Möglichkeiten der nachträglichen Aufhebung oder Änderung, um den Einklang zwischen Verwaltungsentscheidung und gesetzlicher Grundlage (wieder) herzustellen (vgl. etwa §§ 48 ff., § 51 Verwaltungsverfahrensgesetz; §§ 44 ff. Sozialgesetzbuch X: Sozialverwaltungsverfahren und Sozialdatenschutz). Unabhängig davon kann die Rechtskraft staatlicher Akte, insbesondere von Gerichtsentscheidungen, im Interesse des Rechtsfriedens und der Rechtssicherheit grundsätzlich ungeachtet ihrer inhaltlichen Richtigkeit nicht mehr durchbrochen werden (vgl. BVerfGE 2, 380 &lt;403 ff.&gt;). Wirkt die Rechtskraft einer Entscheidung zugunsten eines Adressaten, wird ihre Bedeutung durch den Aspekt des Vertrauensschutzes verstärkt (vgl. Sommermann, in: v. Mangoldt/Klein/ Starck, GG, Bd. 2, 7. Aufl. 2018, Art. 20 Rn. 304). In diesen Fällen steht sie im Spannungsverhältnis zum Gebot materialer Richtigkeit und Gerechtigkeit (vgl. BVerfGE 22, 322 &lt;329&gt;; BVerfG, Beschluss der 2. Kammer des Zweiten Senats vom 14. September 2006 - 2 BvR 123/06 u.a. -, juris, Rn. 17; Beschluss der 3. Kammer des Zweiten Senats vom 13. Februar 2019 - 2 BvR 2136/17 -, Rn. 20).</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
@@ -1678,14 +1678,14 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Davon ausgehend ist das objektive Klarstellungsinteresse gegeben. Der verfahrensgegenständliche Art. 1 Nr. 3 bis 5 BWahlGÄndG entfaltet jedenfalls so lange Rechtswirkung, wie der auf seiner Grundlage gewählte 20. Deutsche Bundestag besteht (vgl. BVerfGE 151, 152 &lt;162 Rn. 27&gt; – Wahlrechtsausschluss Europawahl - Eilantrag). Hinzu kommt, dass der Deutsche Bundestag in seiner 66. Sitzung am 10. November 2022 entsprechend der Beschlussempfehlung des Wahlprüfungsausschusses vom 7. November 2022 (BTDrucks 20/4000) beschlossen hat, die Wahl zum 20. Deutschen Bundestag am 26. September 2021 im Land Berlin teilweise zu wiederholen (vgl. BT-Plenarprotokoll 20/66, S. 7672 ff.). Dieser Beschluss ist Gegenstand mehrerer Wahlprüfungsbeschwerden vor dem Bundesverfassungsgericht nach Art. 41 Abs. 2 GG, § 13 Nr. 3, § 48 BVerfGG. Gemäß § 44 Abs. 2 Satz 1 BWahlG findet die Wiederholungswahl nach denselben Vorschriften wie die Hauptwahl statt. Ihre tatsächlichen und rechtlichen Bedingungen sollen so weit wie möglich denjenigen entsprechen, die bereits für die Hauptwahl galten (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 44 Rn. 7). In der Folge hätte eine Wiederholung der Wahl des 20. Deutschen Bundestages grundsätzlich nach den Normen des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 stattzufinden (vgl. BVerfG, Beschluss des Zweiten Senats vom 22. März 2023 - 2 BvF 1/21 -, Rn. 12). Auch unter diesem Gesichtspunkt ist nicht ausgeschlossen, dass von der zur Prüfung gestellten Norm noch Rechtswirkungen ausgehen können.</t>
+          <t>Da sowohl das Prinzip der materialen Gerechtigkeit als auch das Prinzip der Rechtssicherheit mit Verfassungsrang ausgestattet sind, ist es grundsätzlich Sache des Gesetzgebers, welchem der beiden Prinzipien im konkreten Fall der Vorzug gegeben werden soll (vgl. BVerfGE 3, 225 &lt;237&gt;; 15, 313 &lt;319&gt;; 22, 322 &lt;329&gt;; 131, 20 &lt;46 f.&gt; m.w.N.). Etwas anderes gilt jedoch, wenn das Grundgesetz diese Entscheidung bereits selbst getroffen hat (vgl. für Art. 117 Abs. 1 GG BVerfGE 3, 225 &lt;238 f.&gt;). Eine solche Entscheidung beinhaltet Art. 103 Abs. 3 GG. Indem Art. 103 Abs. 3 GG bestimmt, dass wegen derselben Tat keine erneute Bestrafung erfolgen darf, hat das Grundgesetz für den Anwendungsbereich dieser Bestimmung, mithin den Bereich strafgerichtlicher Urteile, bereits entschieden, dass dem Prinzip der Rechtssicherheit Vorrang vor dem Prinzip der materialen Gerechtigkeit zukommt.</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
@@ -1694,14 +1694,14 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Der nach Art. 93 Abs. 1 Nr. 2 GG, § 13 Nr. 6, § 76 Abs. 1 BVerfGG zulässige Normenkontrollantrag ist nicht begründet. Im Verfahren der abstrakten Normenkontrolle werden die zur Überprüfung gestellten Normen ohne Bindung an die erhobenen Rügen unter allen verfassungsrechtlichen Gesichtspunkten geprüft (vgl. BVerfGE 37, 363 &lt;396 f.&gt;; 86, 148 &lt;211&gt;; 93, 37 &lt;65&gt;; 97, 198 &lt;214&gt;; 101, 239 &lt;257&gt;; 112, 226 &lt;254&gt;; stRspr). Diese Prüfung ergibt, dass Art. 1 Nr. 3 bis 5 BWahlGÄndG sowohl mit dem verfassungsrechtlichen Bestimmtheitsgebot (I.) als auch mit den Grundsätzen der Gleichheit und der Unmittelbarkeit der Wahl sowie der Chancengleichheit der Parteien vereinbar ist (II.). Auch mit Blick auf den Zeitpunkt des Inkrafttretens der zur Überprüfung gestellten Normen ergeben sich keine verfassungsrechtlichen Bedenken (III.).</t>
+          <t>bb) Die in Art. 103 Abs. 3 GG zugunsten der Rechtssicherheit getroffene Vorrangentscheidung ist absolut. Damit ist das grundrechtsgleiche Recht des Art. 103 Abs. 3 GG abwägungsfest. Zwar folgt dies noch nicht zwingend aus dessen Wortlaut (1) oder Entstehungsgeschichte (2). Jedoch ergibt sich aus der Systematik (3) und dem Sinn und Zweck (4) der Bestimmung, dass diese Entscheidung des Grundgesetzes strikte Geltung beansprucht. Nichts anderes folgt aus der bisherigen Rechtsprechung des Bundesverfassungsgerichts (5).</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
@@ -1710,14 +1710,14 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1. a) Nach dem allgemeinen, im Rechtsstaatsprinzip (Art. 20 Abs. 3 GG) gründenden Gebot hinreichender Bestimmtheit der Gesetze ist der Gesetzgeber gehalten, Vorschriften so bestimmt zu fassen, wie dies nach der Eigenart der zu ordnenden Lebenssachverhalte mit Rücksicht auf den Normzweck möglich ist (vgl. BVerfGE 49, 168 &lt;181&gt;; 59, 104 &lt;114&gt;; 78, 205 &lt;212&gt;; 103, 332 &lt;384&gt;; 134, 141 &lt;184 Rn. 126&gt;; 145, 20 &lt;69 f. Rn. 125&gt;; 149, 293 &lt;323 Rn. 77&gt;; stRspr). Die Betroffenen müssen die Rechtslage erkennen und ihr Verhalten danach ausrichten können (vgl. BVerfGE 103, 332 &lt;384&gt;; 108, 52 &lt;75&gt;; 110, 33 &lt;53 f.&gt;; 113, 348 &lt;375 f.&gt;; 131, 88 &lt;123&gt;; 149, 293 &lt;323 Rn. 77&gt;; stRspr). Die Anforderungen an die Bestimmtheit und Klarheit der Norm dienen ferner dazu, die Verwaltung zu binden und ihr Verhalten nach Inhalt, Zweck und Ausmaß zu begrenzen sowie die Gerichte in die Lage zu versetzen, die Verwaltung anhand rechtlicher Maßstäbe zu kontrollieren (vgl. BVerfGE 56, 1 &lt;12&gt;; 110, 33 &lt;54&gt;; 113, 348 &lt;376 f.&gt;; 120, 378 &lt;407&gt;; 149, 293 &lt;323 Rn. 77&gt;; stRspr). Insoweit steht das verfassungsrechtliche Gebot der Bestimmtheit und Klarheit der Normen im Zusammenhang mit dem Prinzip der Gewaltenteilung (vgl. BVerfGE 8, 274 &lt;325&gt; m.w.N.).</t>
+          <t>(1) Der ebenso knappe wie strikte Wortlaut spricht zunächst dafür, dass der von Art. 103 Abs. 3 GG gewährte Schutz absolut ist (vgl. Sodan, in: ders., GG, 4. Aufl. 2018, Art. 103 Rn. 31; Neumann, in: Festschrift für Heike Jung, 2007, S. 655 &lt;661&gt;). Allerdings weisen auch einige andere Grundrechte und grundrechtsgleiche Rechte keine ausdrücklichen Vorbehalte oder Einschränkungen auf. Gleichwohl ist allgemein anerkannt, dass sie verfassungsimmanenten Schranken unterliegen.</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
@@ -1726,14 +1726,14 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>aa) Bei dem Gebot hinreichender Bestimmtheit und Klarheit der Gesetze handelt es sich um ein einheitliches Postulat, das verschiedene Aspekte in sich vereint. Demgemäß ist der Maßstab hierfür einheitlich zu bestimmen; eine Trennung zwischen Bestimmtheits- und Klarheitsgebot dahingehend, dass eine Norm zwar noch hinreichend bestimmt sein kann, dennoch aber gegen das Gebot der Normenklarheit verstößt, kommt grundsätzlich nicht in Betracht. Dieser Sichtweise steht der Beschluss des Ersten Senats vom 10. November 2020 (BVerfGE 156, 11 – Antiterrordateigesetz II) nicht entgegen. Zwar wurde dort ausdrücklich zwischen dem Gebot der Bestimmtheit, das in erster Linie den Rechtsanwender in den Blick nimmt, und dem Gebot der Normenklarheit, das vor allem auf den Normbetroffenen bezogen ist, unterschieden und vor diesem Hintergrund die eigenständige Bedeutung des Gebots der Normenklarheit hervorgehoben. Nach der dort vorgenommenen Differenzierung geht es bei der Bestimmtheit vornehmlich darum, dass Regierung und Verwaltung im Gesetz die Normanwendung steuernde und begrenzende Handlungsmaßstäbe vorfinden und die Gerichte eine wirksame Rechtskontrolle vornehmen können, während bei der Normenklarheit die inhaltliche Verständlichkeit der Regelung im Vordergrund steht, insbesondere damit sich Bürgerinnen und Bürger auf mögliche belastende Maßnahmen einstellen können, die andernfalls ohne ihr Wissen und ohne die Erreichbarkeit gerichtlicher Kontrolle erfolgen könnten (vgl. BVerfGE 156, 11 &lt;45 f. Rn. 86 ff.&gt;; 162, 1 &lt;125 Rn. 272&gt; – Bayerisches Verfassungsschutzgesetz). Auf die vorliegende Konstellation ist dies indes nicht übertragbar. Denn hier geht es – anders als in der Entscheidung des Ersten Senats – gerade nicht um heimliche Eingriffe des Staates in die Grundrechte von Bürgerinnen und Bürgern, die tief in die Privatsphäre der Betroffenen eindringen und von diesen weitgehend weder wahrgenommen noch angegriffen werden können. Der Gehalt solcher Regelungen kann daher nur sehr eingeschränkt im Wechselspiel von Anwendungspraxis und gerichtlicher Kontrolle konkretisiert werden. Weil die Grundrechte hier ohne Wissen der Bürgerinnen und Bürger und oft ohne die Erreichbarkeit gerichtlicher Kontrolle durch die Verwaltung, durch Polizei und Nachrichtendienste eingeschränkt werden, muss der Inhalt der den Eingriffen zugrundeliegenden Normen verständlich und ohne größere Schwierigkeiten durch Auslegung zu konkretisieren sein (vgl. BVerfGE 156, 11 &lt;45 f. Rn. 87 f.&gt;; 162, 1 &lt;125 f. Rn. 272 f.&gt;). Demgegenüber regeln die hier zur Überprüfung gestellten Vorschriften die Umrechnung von bei der Wahl zum Deutschen Bundestag abgegebenen Stimmen in Parlamentssitze. In Rede steht daher kein heimlicher Grundrechtseingriff. Auch betreffen die angegriffenen Bestimmungen nicht die Wahlhandlung als solche. Vielmehr beziehen sie sich auf den der Stimmabgabe nachgelagerten Vorgang der Sitzverteilung durch Ermittlung und Feststellung des Wahlergebnisses, der den Wahlorganen (§ 8 BWahlG) anvertraut ist. Dieser Vorgang unterliegt – entsprechend dem verfassungsrechtlichen Gebot der Öffentlichkeit der Wahl aus Art. 38 in Verbindung mit Art. 20 Abs. 1 und 2 GG (vgl. BVerfGE 123, 39 &lt;68 ff.&gt;) – dem Öffentlichkeitsgrundsatz (§ 10 Abs. 1 BWahlG, § 54 Bundeswahlordnung &lt;BWO&gt;; vgl. Thum, in: Schreiber, BWahlG, 11. Aufl. 2021, § 10 Rn. 1 ff.), der die Ordnungsgemäßheit und Nachvollziehbarkeit der Wahlvorgänge sichert und damit eine wesentliche Voraussetzung für begründetes Vertrauen der Bürgerinnen und Bürger in den korrekten Ablauf der Wahl schafft (vgl. BVerfGE 123, 39 &lt;68&gt;). Zu diesem Zweck veröffentlicht der Bundeswahlleiter im Zuge der Mitteilung der endgültigen Ergebnisse der Wahl auch die Schritte zur Sitzberechnung und Verteilung der Mandate.</t>
+          <t>(2) Auch die Entstehungsgeschichte lässt unterschiedliche Folgerungen zu. Einerseits erfolgte die explizite Verankerung des Grundsatzes ne bis in idem in Art. 103 Abs. 3 GG als Reaktion auf die Unterordnung der Rechtskraft unter andere Ziele in der nationalsozialistischen Zeit (vgl. oben Rn. 64). Andererseits nimmt Art. 103 Abs. 3 GG auf den bei Inkrafttreten des Grundgesetzes geltenden Stand des Prozessrechts und seiner Auslegung durch die herrschende Rechtsprechung Bezug (vgl. oben Rn. 65). In der Rechtsprechung des Reichsgerichts kam dem Grundsatz ne bis in idem eine der Auslegung der konkreten Prozessrechtsnormen dienende Funktion zu. Er wurde dabei in unterschiedlichem Umfang als verwirklicht oder eingeschränkt angesehen (vgl. RGSt 2, 211 ff.; 2, 347 ff.; 4, 243 ff.; 9, 344 ff.; 51, 241 ff.; 72, 99 ff.).</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
@@ -1742,14 +1742,14 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>bb) Welcher Grad an Bestimmtheit geboten ist, lässt sich nicht generell und abstrakt festlegen, sondern hängt von der Eigenart des Regelungsgegenstands und dem Zweck der betreffenden Norm ab (vgl. BVerfGE 103, 111 &lt;135&gt;; 131, 316 &lt;343&gt;; jeweils m.w.N.). Dabei kann auch der Kreis der Normanwender und Normbetroffenen von Bedeutung sein (vgl. BVerfGE 128, 282 &lt;318&gt;; 149, 293 &lt;324 Rn. 77&gt;; jeweils m.w.N.). Die Anforderungen erhöhen sich insbesondere dann, wenn die Unsicherheit in der Beurteilung der Gesetzeslage die Betätigung von Grundrechten erschwert. Sie sind hingegen geringer bei Normen, die nicht oder nicht intensiv in Grundrechte eingreifen, und bei Normen, die nicht von solcher Art sind, dass Adressaten und Betroffene sich bei der Wahrnehmung von Grundrechten auf ihren Inhalt im Detail vorausschauend einrichten können müssen (vgl. BVerfGE 131, 88 &lt;123&gt; m.w.N.).</t>
+          <t>(3) Bei systematischer Betrachtung erscheint Art. 103 Abs. 3 GG jedoch abwägungsfest.</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
@@ -1758,14 +1758,14 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>cc) Grundsätzlich fehlt es an der notwendigen Bestimmtheit nicht schon deshalb, weil eine Norm auslegungsbedürftig ist (vgl. BVerfGE 45, 400 &lt;420&gt;; 83, 230 &lt;145&gt;; 128, 282 &lt;317&gt;; 131, 316 &lt;343&gt;; 134, 141 &lt;184 Rn. 127&gt;; 149, 160 &lt;203 Rn. 120&gt;; 149, 293 &lt;324 Rn. 78&gt;; stRspr). Dem Bestimmtheitserfordernis ist vielmehr genügt, wenn von der Norm aufgeworfene Auslegungsprobleme mit herkömmlichen juristischen Methoden bewältigt werden können (vgl. BVerfGE 83, 130 &lt;145&gt;; 117, 71 &lt;111&gt;; 134, 141 &lt;184 f. Rn. 127&gt;; 149, 293 &lt;324 Rn. 78&gt;; stRspr). Der Bestimmtheitsgrundsatz fordert nicht, dass der Inhalt gesetzlicher Vorschriften dem Bürger grundsätzlich ohne Zuhilfenahme juristischer Fachkunde erkennbar sein muss (vgl. BVerfGE 110, 3 &lt;64&gt;; 131, 88 &lt;Rn. 123&gt;). Die bei der Auslegung verbleibenden Unsicherheiten dürfen indes nicht so weit gehen, dass die Norm nicht praktikabel ist (vgl. BVerfGE 25, 216 &lt;226 f.&gt;). Insbesondere darf die Vorhersehbarkeit und Justiziabilität des Handelns der durch sie ermächtigten Stellen nicht gefährdet sein (vgl. BVerfGE 118, 168 &lt;188&gt;; 120, 274 &lt;316&gt;; 133, 277 &lt;356 Rn. 181&gt;; 145, 20 &lt;69 f. Rn. 125&gt;; stRspr).</t>
+          <t>Art. 103 Abs. 3 GG stellt eine besondere Ausprägung des im Rechtsstaatsprinzip wurzelnden Vertrauensschutzes dar, die ausschließlich für strafrechtliche Verfahren gilt. Als Sonderregelung mit eigenständigem Gehalt geht Art. 103 Abs. 3 GG in seinem Schutzgehalt über die allgemeinen Prinzipien hinaus, die ihrerseits bereits das Vertrauen in eine rechtskräftige Entscheidung schützen und eine übermäßige Beeinträchtigung der Interessen des Einzelnen verhindern. Dieser weiterreichende Vertrauensschutz beruht darauf, dass ihm unbedingter Vorrang gegenüber den grundsätzlich berechtigten Korrekturinteressen zukommt, die der Gesetzgeber ansonsten wie in anderen Sachbereichen auch (vgl. oben Rn. 77) berücksichtigen könnte.</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -1774,14 +1774,14 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>dd) Auch Verweisungen sind mit dem Gebot hinreichender Bestimmtheit und Klarheit der Normen nicht grundsätzlich unvereinbar. Verweisungen sind als vielfach übliche und teilweise notwendige gesetzestechnische Methode anerkannt, sofern die Verweisungsnorm hinreichend klar erkennen lässt, welche Vorschriften im Einzelnen gelten sollen (vgl. BVerfGE 143, 38 &lt;55 f. Rn. 42&gt; m.w.N.).</t>
+          <t>Art. 103 Abs. 3 GG korrespondiert in Bezug auf diese Unbedingtheit mit Art. 103 Abs. 2 GG. Auch diese Norm stellt eine auf das Strafrecht beschränkte Sonderregelung zu allgemeinen verfassungsrechtlichen Prinzipien dar. Als Spezialfall des allgemeinen Rückwirkungsverbots und anders als dieses verbietet Art. 103 Abs. 2 GG dem Strafgesetzgeber ausnahmslos, rückwirkende Strafgesetze zu erlassen. Dieses besondere Rückwirkungsverbot wirkt somit absolut und ist einer Abwägung nicht zugänglich (vgl. BVerfGE 30, 367 &lt;385&gt;; 95, 96 &lt;132&gt;; 109, 133 &lt;171 f.&gt;). Ein gleichlaufendes Verständnis des Art. 103 Abs. 3 GG als abwägungsfestes Recht komplementiert diesen materiell-rechtlichen Schutz des Einzelnen im Bereich des Strafrechts auf der verfahrensrechtlichen Ebene.</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -1790,14 +1790,14 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>b) Die dargelegten Anforderungen an die Bestimmtheit und Klarheit von Gesetzen gelten auch für wahlrechtliche Normen (vgl. BVerfGE 131, 316 &lt;343 f.&gt;). Etwas anderes ergibt sich nicht aus der Feststellung des Bundesverfassungsgerichts, dass Rechtsklarheit im Wahlrecht in besonderem Maße geboten ist (vgl. BVerfGE 79, 161 &lt;168&gt;). Diese erfolgte mit Blick auf eine Regelungslücke des Wahlgesetzes. Insofern führte der Zweite Senat aus, der Gesetzgeber werde mit Blick auf die im Wahlrecht in besonderem Maße gebotene Rechtsklarheit zu erwägen haben, diese zu schließen. Besondere Bestimmtheitsanforderungen an wahlrechtliche Normen jenseits des Vorliegens einer Regelungslücke sind dem nicht zu entnehmen. Gleiches gilt, soweit der Zweite Senat den Gesetzgeber wiederholt aufgefordert hat, das für den Wähler kaum noch nachzuvollziehende Regelungsgeflecht der Berechnung der Sitzzuteilung im Deutschen Bundestag auf eine normenklare und verständliche Grundlage zu stellen (vgl. BVerfGE 121, 266 &lt;316&gt;; 122, 304 &lt;311&gt;; BVerfG, Beschlüsse des Zweiten Senats vom 9. Februar 2009 - 2 BvC 11/04 -, Rn. 17; vom 18. Februar 2009 - 2 BvC 6/03 -, Rn. 19 sowie - 2 BvC 9/04 -, Rn. 27; vom 26. Februar 2009 - 2 BvC 6/04 -, Rn. 20 sowie - 2 BvC 1/04 -, Rn. 21; vom 25. Februar 2010 - 2 BvC 6/07 -, Rn. 18.). Dieser Appell erfolgte jeweils unter Verweis auf die anstehende Neuregelung des Sitzzuteilungsverfahrens durch den Gesetzgeber, die durch die Entscheidung des Bundesverfassungsgerichts zum negativen Stimmgewicht (BVerfGE 121, 266) notwendig geworden war und die der Gesetzgeber mit dem Neunzehnten Gesetz zur Änderung des Bundeswahlgesetzes vom 25. November 2011 (BGBl I S. 2313) vornahm. Dass an wahlrechtliche Normen ein über das allgemeine Gebot hinreichender Bestimmtheit und Klarheit der Gesetze hinausgehender Maßstab anzulegen wäre, ist der Aufforderung des Bundesverfassungsgerichts dagegen nicht zu entnehmen. Insbesondere lässt sich ein allgemeingültiger verfassungsrechtlicher Maßstab für den maximal zulässigen Grad an Komplexität, den eine wahlrechtliche Vorschrift erreichen darf, nicht entwickeln, zumal die Anforderungen an die Bestimmtheit und Klarheit einer das Wahlgeschehen betreffenden Norm auch davon abhängen, ob sie die Wahlhandlung selbst oder die nachfolgende Ergebnisermittlung betrifft.</t>
+          <t>Art. 103 Abs. 2 und 3 GG stehen den Freiheitsrechten nahe, die nicht nur innerhalb eines Strafverfahrens zu beachten sind, sondern den Grundrechtsträger bereits vor einem Strafverfahren schützen, ohne dass es zur Verwirklichung dieses Schutzes noch einer gesetzlichen Umsetzung bedürfte. Darin unterscheiden sich Art. 103 Abs. 2 und 3 GG von den Rechten, die – wie beispielsweise Art. 103 Abs. 1 GG – auf die Gewährleistung von Rechtsschutz gerichtet sind. Der für alle Verfahrensarten geltende Anspruch auf rechtliches Gehör bedarf einer verfahrensrechtlichen Ausgestaltung durch den Gesetzgeber (vgl. BVerfGE 75, 302 &lt;313 f.&gt;; 89, 28 &lt;35 f.&gt;; 119, 292 &lt;296&gt;).</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -1806,14 +1806,14 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2. Davon ausgehend genügt Art. 1 Nr. 3 bis 5 BWahlGÄndG den Anforderungen des Bestimmtheitsgebots. Dies gilt für die dadurch geänderten § 6 Abs. 5 (a) und Abs. 6 BWahlG (b) ebenso wie für § 48 Abs. 1 BWahlG (c). Auch mit Blick auf die Klarheit der Norm stellt der Umstand, dass wahlberechtigte Bürgerinnen und Bürger allein auf Grundlage des Gesetzestextes ohne Zuhilfenahme weiterer Informationsquellen nicht in der Lage sein dürften, die Regelungen der § 6 Abs. 5 und 6, § 48 BWahlG im Einzelnen zu erfassen, keinen Verfassungsverstoß dar (d).</t>
+          <t>Entsprechendes gilt auch für andere in der Verfassung wurzelnde Rechte im Strafverfahren, die im Gegensatz zu Art. 103 Abs. 3 GG keine ausdrückliche Verankerung im Grundgesetz erfahren haben. Dies sind namentlich die Unschuldsvermutung (vgl. BVerfGE 38, 105 &lt;111&gt;; 122, 248 &lt;271 f.&gt;; 133, 168 &lt;200 f. Rn. 59&gt;) und das Recht auf ein faires Verfahren (vgl. BVerfGE 38, 105 &lt;111&gt;; 122, 248 &lt;271 f.&gt;; 133, 168 &lt;200 f. Rn. 59&gt;) einschließlich seiner Bestandteile wie dem Grundsatz nemo tenetur (vgl. BVerfGE 38, 105 &lt;113 f.&gt;; 55, 144 &lt;150 f.&gt;; 56, 37 &lt;43&gt;; 110, 1 &lt;31&gt;; 133, 168 &lt;201 Rn. 60&gt;; BVerfG, Beschluss der 3. Kammer des Zweiten Senats vom 25. Januar 2022 - 2 BvR 2462/18 -, Rn. 50 ff.), der Beweisregel in dubio pro reo (vgl. BVerfGK 1, 145 &lt;149&gt;; BVerfG, Beschluss der 1. Kammer des Zweiten Senats vom 20. Juni 2007 - 2 BvR 965/07 -, Rn. 3; vgl. auch BVerfGE 9, 167 &lt;169&gt;; 35, 311 &lt;320&gt;; 74, 358 &lt;371&gt;; 133, 168 &lt;199 Rn. 56&gt;; 140, 317 &lt;345 Rn. 57&gt;) und dem Grundsatz der Waffengleichheit (vgl. BVerfGE 110, 226 &lt;253&gt;; 133, 168 &lt;200 Rn. 59&gt;; BVerfG, Beschluss der 3. Kammer des Zweiten Senats vom 12. November 2020 - 2 BvR 1616/18 -, Rn. 32). Sie sichern die Subjektstellung des Beschuldigten während des Verfahrens und sind damit naturgemäß in ihrer Reichweite von der Ausgestaltung des Verfahrens selbst abhängig. Deshalb enthalten sie keine in allen Einzelheiten bestimmten Ge- und Verbote, sondern bedürfen hinsichtlich ihrer Auswirkungen auf das Verfahrensrecht der Konkretisierung je nach den sachlichen Gegebenheiten, vornehmlich durch den Gesetzgeber (vgl. BVerfGE 74, 358 &lt;371 f.&gt;; 133, 168 &lt;202 Rn. 61&gt; m.w.N.). Demgegenüber will Art. 103 Abs. 3 GG nach rechtskräftigem Abschluss des Verfahrens verhindern, dass der Betroffene erneut mit einem solchen Verfahren belastet und in die Rolle des Beschuldigten zurückversetzt wird.</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -1822,14 +1822,14 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>a) § 6 Abs. 5 BWahlG lässt sich bei methodengerechter Auslegung entnehmen, wie die Sitzzahl des Deutschen Bundestages zu erhöhen ist und welche Folgen sich daraus für die Gesamtzahl der Sitze ergeben.</t>
+          <t>(4) Auch Sinn und Zweck des Art. 103 Abs. 3 GG sprechen dafür, dass die Norm absolute Geltung beansprucht. Sowohl die individuelle als auch die gesellschaftliche Zweckrichtung des Art. 103 Abs. 3 GG verlangen die verbindliche Entscheidung zugunsten der Rechtssicherheit. Dies lässt eine Relativierung seines Schutzes nicht zu.</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -1838,14 +1838,14 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>aa) § 6 Abs. 5 Satz 1 BWahlG regelt hinreichend bestimmt, wie und bis zu welchem Punkt die Sitzzahl des Deutschen Bundestages zu erhöhen ist. Soweit er vorschreibt, dass die Sitzzahl so lange erhöht wird, bis „jede Partei bei der zweiten Verteilung der Sitze nach Absatz 6 Satz 1 mindestens die Gesamtzahl der ihren Landeslisten nach den Sätzen 2 und 3 zugeordneten Sitze erhält“, wird deutlich, dass in einem iterativen Prozess die Sitzzahl des Deutschen Bundestages so lange zu erhöhen ist, bis bei der tatsächlichen Verteilung nach § 6 Abs. 6 Satz 1 BWahlG jede Partei die Gesamtzahl der Sitze erhält, die ihren Landeslisten nach § 6 Abs. 5 Satz 2 und 3 BWahlG zugeordnet sind. Für jede Landesliste muss der höhere Wert aus den folgenden Optionen erreicht werden: entweder die Zahl der im Land von Wahlbewerbern der Partei in den Wahlkreisen errungenen Sitze oder der auf ganze Sitze aufgerundete Mittelwert zwischen dieser Zahl der Direktmandate und den Sitzen, die nach der ersten Verteilung nach § 6 Abs. 2 und 3 BWahlG für die Landesliste der Partei ermittelt wurden (§ 6 Abs. 5 Satz 2 BWahlG). Mindestens muss aber für eine Partei insgesamt im Bundestag die Zahl der Sitze erreicht sein, die für diese Partei bei der ersten Verteilung nach § 6 Abs. 2 und 3 BWahlG ermittelt wurde (§ 6 Abs. 5 Satz 3 BWahlG). Die von den Antragstellerinnen und Antragstellern behauptete Undurchführbarkeit der Rechenoperation zur Sitzzahlerhöhung besteht bei methodengerechter Auslegung der Norm daher nicht.</t>
+          <t>Der Zweck des Art. 103 Abs. 3 GG als Individualrecht besteht zunächst darin, den staatlichen Strafanspruch um der Rechtssicherheit des Einzelnen willen zu begrenzen (vgl. BVerfGE 56, 22 &lt;31 f.&gt;; vgl. auch bereits BVerfGE 3, 248 &lt;253 f.&gt;). Der Einzelne soll darauf vertrauen dürfen, dass er nach einem Urteil wegen des abgeurteilten Sachverhalts nicht nochmals belangt werden kann (vgl. BVerfGE 56, 22 &lt;31&gt;). Das grundrechtsgleiche Recht dient damit – ebenso wie Art. 103 Abs. 2 GG (vgl. BVerfGE 109, 133 &lt;171 f.&gt;) – zugleich der Freiheit und der Menschenwürde des Betroffenen. Es verhindert, dass der Einzelne – gegebenenfalls im Rahmen eines Prozesses „ad infinitum“ (vgl. Marxen/Tiemann, ZIS 2008, S. 188 &lt;190&gt;; Arnemann, NJW-Spezial 2021, S. 440) – zum bloßen Objekt der Ermittlung der materiellen Wahrheit herabgestuft wird. Deshalb unterliegt die Strafverfolgung einem geregelten Verfahren, nach dessen Abschluss mittels eines Sachurteils eine weitere Strafverfolgung wegen derselben Tat ausscheidet. Art. 103 Abs. 3 GG beschränkt damit die Durchsetzung des Legalitätsprinzips (vgl. BVerfGE 56, 22 &lt;31 f.&gt;). Diese Selbstbeschränkung des Staates folgt dem rechtsstaatlichen Grundprinzip, mit der Rechtskraft einer Entscheidung Rechtssicherheit des Einzelnen zu schaffen, und konkretisiert es für das Strafrecht als einen der intensivsten Bereiche staatlicher Macht. Wäre dem Gesetzgeber vorbehalten, die Abwägung zwischen Rechtssicherheit und staatlichem Strafanspruch anders zu treffen, könnte Art. 103 Abs. 3 GG selbst das Vertrauen des Angeklagten in den Bestand des in seiner Sache ergangenen Strafurteils und damit Rechtssicherheit für den Einzelnen nicht begründen.</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -1854,14 +1854,14 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>(1) Schon der Wortlaut von § 6 Abs. 5 Satz 1 BWahlG („so lange erhöht, bis“) spricht dafür, dass die beschriebene Rechenoperation ein schrittweises Vorgehen verlangt, nämlich eine iterative – probeweise – Erhöhung der Gesamtsitzzahl (vgl. für eine entsprechende Bestimmung im Gesetz über die Wahlen zum Landtag des Landes Hessen HessStGH, Urteil vom 11. Januar 2021 - P.St. 2733, P.St. 2738 -, juris, Rn. 150), bis die Bedingung des § 6 Abs. 5 Satz 1 BWahlG erreicht ist, bis also jede Partei bei der zweiten Verteilung nach § 6 Abs. 6 Satz 1 BWahlG die Zahl der ihren Landeslisten nach § 6 Abs. 5 Satz 2 und 3 BWahlG zugeordneten Sitze erhält. Die Erhöhung wird dabei so lange vorgenommen, bis diese Bedingung eintritt (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 22 ff.; Wissenschaftliche Dienste des Deutschen Bundestages, WD 3-3000-222/20, S. 6).</t>
+          <t>Daneben dient die Rechtskraft einer Entscheidung auch dem Rechtsfrieden (vgl. BVerfGE 2, 380 &lt;403&gt;; 56, 22 &lt;31&gt;; 115, 51 &lt;62&gt;). Es besteht ein vom Einzelnen unabhängiges Bedürfnis der Gesellschaft an einer endgültigen Feststellung der Rechtslage (vgl. Greco, Strafprozesstheorie und materielle Rechtskraft, 2015, S. 346 ff. m.w.N.). Daher hat sich die moderne rechtsstaatliche Ordnung gegen die Erreichung des Ideals absoluter Wahrheit und für die in einem rechtsförmigen Verfahren festzustellende, stets nur relative Wahrheit entschieden. Auch das Strafrecht gebietet keine Erforschung der Wahrheit „um jeden Preis“ (vgl. BGHSt 14, 358 &lt;365&gt;; 31, 304 &lt;309&gt;). Insoweit sichert die Rechtskraft den dauerhaften Geltungsanspruch gerichtlicher Entscheidungen. Rechtsmittel tragen dem Umstand Rechnung, dass jede Entscheidung fehlerhaft und daher korrekturbedürftig sein kann; sie erhöhen damit die Richtigkeitsgewähr. Die Möglichkeit, ein Verfahren durch Rechtsmittel unaufhörlich weiterzuführen, beziehungsweise die Möglichkeit der Wiederaufnahme, es von Neuem zu beginnen, würde jedoch fortwährende Zweifel an der Richtigkeit des Urteilsspruchs zulassen und damit das Vertrauen in die Effektivität der Streitentscheidung durch die Rechtsprechung beeinträchtigen.</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -1870,14 +1870,14 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>(2) Auch die Systematik der Absätze 5 und 6 spricht für dieses Verständnis. Ihr Zusammenspiel ergibt, dass § 6 Abs. 5 Satz 1 BWahlG zum einen eine Erhöhung der Gesamtsitzzahl vorschreibt („die Zahl der nach Absatz 1 Satz 3 verbleibenden Sitze wird […] erhöht“) und zum anderen deren Endpunkt festlegt („bis jede Partei bei der zweiten Verteilung nach Absatz 6 Satz 1 mindestens die Gesamtzahl der ihren Landeslisten nach den Sätzen 2 und 3 zugeordneten Sitze erhält“).</t>
+          <t>(5) Die bisherige Rechtsprechung des Bundesverfassungsgerichts bestätigt das Verständnis des Art. 103 Abs. 3 GG als absolutes und abwägungsfestes Verbot.</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -1886,14 +1886,14 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Dabei folgt aus der Normsystematik auch das Verfahren der Sitzzahlerhöhung. Da sich die zweite Verteilung gemäß § 6 Abs. 6 Satz 1 BWahlG nach dem in § 6 Abs. 2 Satz 2 bis 7 für die erste Verteilung geregelten Divisorverfahren mit Standardrundung richtet, ist dieses Verfahren auch im Rahmen der Sitzzahlerhöhung nach § 6 Abs. 5 BWahlG zugrunde zu legen. Nur auf diese Weise ist zu ermitteln, bei welcher Sitzzahl die unter Anwendung dieses Verfahrens vorzunehmende zweite Verteilung den gesetzlich bestimmten Anforderungen genügt (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 22, 24). Dafür ist die Gesamtsitzzahl schrittweise, in sich wiederholenden Rechengängen zu erhöhen und jedes Mal unter Anwendung des Divisorverfahrens mit Standardrundung zu prüfen, ob die durch § 6 Abs. 6 in Verbindung mit § 6 Abs. 5 BWahlG vorgegebenen Anforderungen bei der Verteilung erfüllt sind (vgl. Bundeswahlleiter, Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 451 f.; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 22, 24).</t>
+          <t>Das Bundesverfassungsgericht hat bisher Art. 103 Abs. 3 GG nicht mit anderen Verfassungswerten abgewogen und auch nicht zum Ausdruck gebracht, dass das Schutzgut des Art. 103 Abs. 3 GG mit anderen Verfassungsgütern abgewogen werden könnte. Vielmehr befassen sich die zu dieser Verfassungsnorm ergangenen Entscheidungen mit der Bestimmung ihres Schutzgehalts. Während Ausgangspunkt hierfür das vorgefundene Gesamtbild des Strafprozessrechts ist (vgl. BVerfGE 3, 248 &lt;252&gt;; 9, 89 &lt;96&gt;; 12, 62 &lt;66&gt;; 65, 377 &lt;384&gt;), werden strafrechtsdogmatische Weiterentwicklungen nicht von vornherein ausgeschlossen. Das Bundesverfassungsgericht hat sie zum Anlass für korrespondierende „Grenzkorrekturen“ des Schutzgehalts des Art. 103 Abs. 3 GG genommen (vgl. BVerfGE 56, 22 &lt;34&gt;). Diese Grenzkorrekturen nimmt es selbst vor, so dass angegriffene Entscheidungen verfassungsrechtlich vollständig an Art. 103 Abs. 3 GG zu überprüfen sind (vgl. BVerfGE 56, 22 &lt;27 ff.&gt;).</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -1902,14 +1902,14 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>(3) Diesen Regelungsgehalt von § 6 Abs. 5 Satz 1 BWahlG bestätigt die Begründung des Gesetzentwurfs. Dort heißt es (BTDrucks 19/22504, S. 8): „Absatz 5 regelt, wie bisher, die Erhöhung der Gesamtsitzzahl für die endgültige Sitzverteilung in der zweiten Stufe der Sitzverteilung nach Absatz 6. Nach Satz 1 wird die Gesamtsitzzahl so weit erhöht, bis jede Partei bei der bundesweiten Oberverteilung nach Absatz 6 Satz 1 die Summe der Sitze, die den Landeslisten dieser Partei nach Maßgabe des Absatzes 5 Sätze 2 und 3 zugeordnet sind, erhält“. Die Formulierung „wie bisher“ verweist darauf, dass der Gesetzgeber das bisherige Verfahren der Sitzzahlerhöhung nach dem BWahlG 2013 grundsätzlich beibehalten wollte (vgl. auch BTDrucks 19/22504, S. 1, 5). Bei diesem wurde die Gesamtsitzzahl schrittweise erhöht, bis bei der Verteilung auf die Landeslisten nach § 6 Abs. 6 Satz 1 BWahlG 2013 die Bedingung des § 6 Abs. 5 Satz 1 Halbsatz 2 BWahlG 2013 erreicht war (vgl. BTDrucks 17/11819, S. 5; Lang, GreifRecht 2019, S. 76 &lt;81&gt;; Strelen, in: Schreiber, BWahlG, 10. Aufl. 2017, § 6 Rn. 1c, 26, 26c; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 22).</t>
+          <t>Auch die Formulierung, die vorkonstitutionelle Auslegung des Grundsatzes ne bis in idem sei als „immanente Schranke“ des Art. 103 Abs. 3 GG anzusehen (vgl. BVerfGE 3, 248 &lt;252 f.&gt;), stellt die absolute Wirkung der Norm nicht in Abrede. Sie bringt vielmehr zum Ausdruck, dass mit Art. 103 Abs. 3 GG eine vornehmlich durch die Rechtsprechung des Reichsgerichts normativ vorgeprägte prozessrechtliche Garantie in das Grundgesetz aufgenommen wurde und sich daher der Gehalt dieser Bestimmung aus dieser Vorprägung erschließt (vgl. BVerfGE 3, 248 &lt;251&gt;). Dem Einwand, dass damit eine „Versteinerung“ des Gewährleistungsgehalts des Art. 103 Abs. 3 GG drohe (vgl. Zehetgruber, JR 2020, S. 157 &lt;160&gt;), begegnet der Zweite Senat durch ein enges Verständnis des Schutzgehalts des Art. 103 Abs. 3 GG, das lediglich Grenzkorrekturen im Randbereich erlaubt (vgl. BVerfGE 56, 22 &lt;34&gt;).</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
@@ -1918,14 +1918,14 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>(4) Diese Auslegung entspricht schließlich auch dem Sinn und Zweck der Regelung. Diese wurde im Grundsatz bereits durch das Zweiundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 3. Mai 2013 (BGBl I S. 1082) geschaffen und sollte in Reaktion auf das Urteil des Bundesverfassungsgerichts vom 25. Juli 2012 (BVerfGE 131, 316) die Entstehung ausgleichsloser Überhangmandate vermeiden (vgl. BTDrucks 17/11819, S. 1). Während sich der Gesetzgeber zunächst für einen Vollausgleich aller potenziellen Überhangmandate entschied (vgl. BTDrucks 17/11819, S. 5 f.), ließ er mit der erneuten Änderung durch das verfahrensgegenständliche Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 wieder bis zu drei unausgeglichene Überhangmandate mit dem Ziel zu, das Anwachsen des Deutschen Bundestages zu dämpfen (vgl. BTDrucks 19/22504, S. 1, 5, 6). Dies ändert aber nichts daran, dass sowohl das Bundeswahlgesetz 2013 als auch das Bundeswahlgesetz in der hier zur Überprüfung gestellten Fassung mit der Wechselbezüglichkeit von § 6 Abs. 5 und 6 BWahlG darauf abzielen, eine Erhöhung der Sitzzahl nur so lange stattfinden zu lassen, bis der jeweils gewünschte Ausgleichseffekt erzielt ist (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 22 ff.).</t>
+          <t>cc) Auch gegenüber dem das Wiederaufnahmerecht gestaltenden Gesetzgeber, der ebenso wie die Strafverfolgungsorgane dem Normbefehl des Art. 103 Abs. 3 GG unterliegt (vgl. oben Rn. 72 ff.), stellt Art. 103 Abs. 3 GG ein absolutes und abwägungsfestes Verbot dar. Zwar obliegt dem Gesetzgeber grundsätzlich die Ausgestaltung der aus dem Rechtsstaatprinzip folgenden Grundsätze. Er kann dabei im Regelfall zwischen dem Prinzip der materialen Gerechtigkeit und der Rechtssicherheit abwägen. Bei der Ausgestaltung des Wiederaufnahmerechts kommt ihm jedoch ein Gestaltungsspielraum nur zu, soweit nicht das abwägungsfeste Verbot des Art. 103 Abs. 3 GG greift.</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
@@ -1934,14 +1934,14 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>bb) Auch § 6 Abs. 5 Satz 2 und 3 BWahlG genügen den vorgenannten Bestimmtheitsanforderungen. Sie regeln eindeutig, welche Sitzzahl jeder Landesliste beziehungsweise Partei bei der Erhöhung der Gesamtsitzzahl des Deutschen Bundestages nach § 6 Abs. 5 Satz 1 BWahlG zu berücksichtigen ist, und legen damit „Mindestsitzzahlen“ (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 28) der Parteien fest. Der Regelung lässt sich mit hinreichender Bestimmtheit entnehmen, dass bei der Sitzzahlerhöhung pro Land entweder sämtliche Direktmandate einer Partei oder der (höhere) Mittelwert aus den Direktmandaten und den auf die jeweilige Landesliste dieser Partei entfallenden Mandaten anzusetzen und diese Zahlen zu addieren, mindestens aber die (Gesamt-)Summe der für jede Partei bei der ersten (fiktiven) Verteilung ermittelten Sitze in Ansatz zu bringen sind.</t>
+          <t>c) Als abwägungsfestes Verbot ist das grundrechtsgleiche Recht des Art. 103 Abs. 3 GG in Abgrenzung zu den allgemeinen rechtsstaatlichen Garantien eng auszulegen (aa). Soweit dieser Schutzgehalt reicht, ist dem Gesetzgeber die Eröffnung einer Wiederaufnahme zum Nachteil des Grundrechtsträgers aufgrund neuer Tatsachen oder Beweismittel versagt (bb).</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -1950,14 +1950,14 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>(1) Gemäß § 6 Abs. 5 Satz 2 BWahlG wird jeder Landesliste zunächst die Zahl der im Land von Wahlbewerbern der Partei in den Wahlkreisen nach § 5 BWahlG errungenen Sitze, das heißt die Zahl ihrer Direktmandate, garantiert (§ 6 Abs. 5 Satz 2 Alternative 1 BWahlG). Alternativ wird der auf ganze Sitze aufgerundete Mittelwert zwischen der Zahl der von der jeweiligen Partei erzielten Direktmandate und den für die Landesliste nach der ersten Verteilung (§ 6 Abs. 2 und 3 BWahlG) ermittelten Sitze in Ansatz gebracht (§ 6 Abs. 5 Satz 2 Alternative 2 BWahlG). Garantiert wird jeweils der höhere Wert der beiden Alternativen, wobei die erste Alternative in den Fällen einschlägig ist, in denen eine Landesliste ebenso viele Direktmandate wie oder mehr Direktmandate als Listenmandate errungen hat, die zweite Alternative dagegen in den Fällen, in denen die Anzahl der Listenmandate die der Direktmandate übersteigt (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 28). Darüber hinaus bestimmt § 6 Abs. 5 Satz 3 BWahlG, dass jede Partei mindestens die bei der ersten Verteilung (§ 6 Abs. 2 und 3 BWahlG) für ihre Landeslisten ermittelten Sitze erhält. Nach der Entwurfsbegründung zielt dies auf den Fall, dass die Summe der nach § 6 Abs. 5 Satz 2 BWahlG ermittelten Sitze die Summe der in der ersten Verteilung für die Landeslisten der jeweiligen Partei ermittelten Sitze unterschreitet (vgl. BTDrucks 19/22504, S. 8).</t>
+          <t>aa) Art. 103 Abs. 3 GG umfasst nur eine eng umgrenzte Einzelausprägung des Vertrauensschutzes in rechtskräftige Entscheidungen (1). Er schützt den Einzelnen allein vor erneuter Strafverfolgung aufgrund der allgemeinen Strafgesetze (2), wenn wegen derselben Tat (3) bereits durch ein deutsches Gericht (4) ein rechtskräftiges Strafurteil (5) ergangen ist.</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
@@ -1966,14 +1966,14 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>(2) Verfassungsrechtliche Bedenken hinsichtlich der Bestimmtheit dieser Regelungen bestehen nicht. Dies gilt auch in Bezug auf § 6 Abs. 5 Satz 3 BWahlG. Insoweit lässt bereits der Wortlaut der Norm, der von „Landeslisten“ im Plural spricht, erkennen, dass auf die Gesamtzahl der bei der ersten Verteilung für eine Partei ermittelten Sitze abzustellen ist. Dem entspricht die Begründung des Gesetzentwurfs, die explizit jeweils auf die „Summe“ der Sitze Bezug nimmt (vgl. BTDrucks 19/22504, S. 8). Der Regelungszweck bestätigt diese Auslegung. § 6 Abs. 5 Satz 3 BWahlG soll verhindern, dass es bei Parteien, die wenige Direktmandate gewonnen haben, aufgrund von § 6 Abs. 5 Satz 2 BWahlG zu einer übermäßigen Reduzierung der Sitzansprüche und damit zu zusätzlichen Proporzverzerrungen kommt (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 29). Dieses Ziel ist nur erreichbar, wenn im Rahmen des § 6 Abs. 5 Satz 3 BWahlG alle für eine Partei bei der ersten Verteilung nach § 6 Abs. 2 und 3 BWahlG ermittelten Sitze garantiert werden.</t>
+          <t>(1) Die Bestimmung des Art. 103 Abs. 3 GG ist auch im Hinblick auf seinen engen Schutzgehalt mit Art. 103 Abs. 2 GG vergleichbar. Art. 103 Abs. 2 GG enthält ein absolutes und striktes Verbot, das der Abwägung nicht zugänglich ist (vgl. BVerfGE 30, 367 &lt;385&gt;; 95, 96 &lt;132&gt;; 109, 133 &lt;171 f.&gt;). Für den Bereich des materiellen Strafrechts fasst Art. 103 Abs. 2 GG Einzelausprägungen des Rechtsstaatsprinzips enger. Dies gilt insbesondere für den Gesetzesvorbehalt (vgl. BVerfGE 47, 109 &lt;120&gt;; 75, 329 &lt;340 ff.&gt;; 78, 374 &lt;381 f.&gt;; 87, 399 &lt;411&gt;; 126, 170 &lt;194 f.&gt;), das Bestimmtheitsgebot (vgl. BVerfGE 25, 269 &lt;285&gt;; 78, 374 &lt;382&gt;; 126, 170 &lt;194 ff.&gt;; 143, 38 &lt;53 f. Rn. 38&gt;; 159, 223 &lt;292 ff. Rn. 152 ff.&gt; – Bundesnotbremse I &lt;Ausgangs- und Kontaktbeschränkungen&gt;) und das Rückwirkungsverbot (vgl. BVerfGE 25, 269 &lt;286&gt;; 30, 367 &lt;385&gt;; 46, 188 &lt;192 f.&gt;; 81, 132 &lt;135&gt;; 95, 96 &lt;131&gt;; 109, 133 &lt;172&gt;; 156, 354 &lt;388 f. Rn. 104 f.&gt; – Vermögensabschöpfung). Gerade mit dem absoluten Rückwirkungsverbot erfüllt Art. 103 Abs. 2 GG seine rechtsstaatliche und grundrechtliche Gewährleistungsfunktion durch eine strikte Formalisierung (vgl. BVerfGE 95, 96 &lt;96 LS 1 und 131&gt;). Nichts anderes gilt für Art. 103 Abs. 3 GG. Auch dieses Recht fasst den Vertrauensschutz, der auf den Bestand rechtskräftiger Entscheidungen als Ausprägung des Rechtsstaatsprinzips gerichtet ist, als Einzelausprägung für den Bereich des Strafrechts enger als in anderen Rechtsbereichen. Art. 103 Abs. 3 GG erfüllt seine Gewährleistungsfunktion ebenso wie Art. 103 Abs. 2 GG durch eine strikte Formalisierung.</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
@@ -1982,14 +1982,14 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>cc) Auch § 6 Abs. 5 Satz 4 BWahlG genügt bei methodengerechter Auslegung den Bestimmtheitsanforderungen.</t>
+          <t>(2) Das Mehrfachverfolgungsverbot des Art. 103 Abs. 3 GG bezieht sich nur auf die Anwendung der allgemeinen Strafgesetze, das heißt des Kriminalstrafrechts (vgl. BVerfGE 21, 378 &lt;383 f.&gt;; 21, 391 &lt;401 f.&gt;; 27, 180 &lt;185&gt;; 43, 101 &lt;105&gt;; 66, 337 &lt;356 f.&gt;).</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -1998,14 +1998,14 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>(1) Gemäß § 6 Abs. 5 Satz 4 BWahlG bleiben bei der Sitzzahlerhöhung in den Wahlkreisen errungene Sitze, die nicht nach § 6 Abs. 4 Satz 1 BWahlG von der Zahl der für die Landesliste ermittelten Sitze abgezogen werden können, bis zu einer Zahl von drei unberücksichtigt. Folglich geht es um Direktmandate einer Partei, welche die Zahl der in dem jeweiligen Land nach Zweitstimmen errungenen Mandate übersteigen. Es handelt sich demgemäß um Quasi-Überhangmandate (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 25, der von „drohenden Überhangmandaten“ spricht).</t>
+          <t>Art. 103 Abs. 3 GG knüpft an das mit einer Strafe verbundene autoritative Unwerturteil über die schuldhafte Verletzung eines allgemein gewährleisteten Rechtsgutes und die Störung des allgemeinen Rechtsfriedens an (vgl. BVerfGE 21, 391 &lt;403&gt;; 43, 101 &lt;105&gt;). Die Gewährleistung betrifft staatliche Maßnahmen, die eine missbilligende hoheitliche Reaktion auf ein rechtswidriges, schuldhaftes Verhalten darstellen und wegen dieses Verhaltens auf die Verhängung eines Übels gerichtet sind, das dem Schuldausgleich dient (vgl. BVerfGK 14, 357 &lt;364&gt;; 16, 98 &lt;107&gt;). Nicht erfasst sind somit Maßnahmen der Strafvollstreckung (vgl. BVerfGE 117, 71 &lt;115&gt;) sowie Maßregeln der Besserung und Sicherung (vgl. BVerfGE 55, 28 &lt;30&gt;; BVerfGK 14, 357 &lt;364&gt;; 16, 98 &lt;107&gt;).</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -2014,14 +2014,14 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>(2) Entgegen der Auffassung der Antragstellerinnen und Antragsteller fehlt es in § 6 Abs. 5 Satz 4 BWahlG hinsichtlich des Tatbestandsmerkmals „bis zu einer Zahl von drei“ nicht an der notwendigen Bestimmtheit. Die Auslegung ergibt, dass § 6 Abs. 5 Satz 4 BWahlG lediglich für bis zu drei Überhangmandate insgesamt gilt, ohne dass es auf deren Identifizierbarkeit ankommt.</t>
+          <t>Dabei erstreckt sich Art. 103 Abs. 3 GG jedoch nicht auf alle Sanktionen, die sich unter den Begriff der Strafe fassen lassen, sondern ausdrücklich nur auf solche, die aufgrund der allgemeinen Strafgesetze ergehen (vgl. auch Remmert, in: Dürig/Herzog/Scholz, GG, Art. 103 Abs. 3 Rn. 57 &lt;Nov. 2018&gt;). Nach dem dokumentierten Willen des Verfassungsgebers (vgl. Wortprotokoll der 8. Sitzung des Ausschusses für Verfassungsgerichtshof und Rechtspflege vom 7. Dezember 1948, abgedruckt in: Büttner/Wettengel, Der Parlamentarische Rat, Bd. 13/2, 2002, S. 1449 &lt;1465 f. und 1472&gt;) ist hierunter allein das „eigentliche“ Strafrecht im Sinne des Strafgesetzbuches und seiner Nebengesetze im Gegensatz zum Dienst-, Disziplinar-, Ordnungs-, Polizei- und Berufsstrafrecht zu verstehen (vgl. BVerfGE 21, 378 &lt;383 f.&gt;; 21, 391 &lt;401, 403 f.&gt;; 27, 180 &lt;185&gt;; 28, 264 &lt;276 f.&gt;; 43, 101 &lt;105&gt;; 66, 337 &lt;357&gt;). Insbesondere ist damit die Verfolgung von Ordnungswidrigkeiten vom Verbot des Art. 103 Abs. 3 GG ausgenommen (vgl. BVerfGE 21, 378 &lt;388&gt;; 43, 101 &lt;105&gt;; BVerfG, Beschluss der 2. Kammer des Zweiten Senats vom 31. Mai 1990 - 2 BvR 1722/89 -, juris; vgl. zum Streitstand im Schrifttum Remmert, in: Dürig/Herzog/Scholz, GG, Art. 103 Abs. 3 Rn. 58 m.w.N. &lt;Nov. 2018&gt;). Dies gilt ungeachtet dessen, dass ihre Ahndung durch Geldbußen einen Strafcharakter aufweist und daher insbesondere von Art. 103 Abs. 2 GG erfasst wird (vgl. BVerfGE 81, 132 &lt;135&gt;; 87, 399 &lt;411&gt;; BVerfGK 11, 337 &lt;349&gt;). Ebenso wenig erstreckt sich Art. 103 Abs. 3 GG auf verwaltungsrechtliche Sanktionen (vgl. BVerfGE 20, 365 &lt;372&gt;).</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
@@ -2030,14 +2030,14 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>(a) Zwar ist den Antragstellerinnen und Antragstellern zuzugestehen, dass sich aus dem Wortlaut der Norm allein nicht erschließt, ob die Zahl „bis zu drei“ pro Landesliste, pro Partei oder auf alle Landeslisten aller Parteien bezogen zu verstehen ist (vgl. auch Pukelsheim/Bischof, DVBl 2021, S. 417 &lt;420&gt;). Der Wortlaut eines Gesetzes bildet aber regelmäßig nur den Ausgangspunkt seiner Auslegung (vgl. BVerfGE 133, 168 &lt;205 Rn. 66&gt; m.w.N.).</t>
+          <t>(3) Art. 103 Abs. 3 GG verbietet die erneute Strafverfolgung nur, wenn ein Strafurteil dieselbe Tat, also den geschichtlichen – und damit zeitlich und hinsichtlich des Sachverhalts begrenzten – Vorgang zum Gegenstand hat, welchen Anklage und Eröffnungsbeschluss umreißen und innerhalb dessen der Angeklagte als Täter oder Teilnehmer einen Straftatbestand verwirklicht haben soll (vgl. BVerfGE 23, 191 &lt;202&gt;; 45, 434 &lt;435&gt;; 56, 22 &lt;28&gt;; BVerfGK 5, 7 &lt;8&gt;; 7, 417 &lt;418&gt;; BVerfG, Beschluss der 2. Kammer des Zweiten Senats vom 15. Oktober 2014 - 2 BvR 920/14 -, Rn. 26).</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -2046,14 +2046,14 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>(b) Die systematische Auslegung ergibt, dass gemäß § 6 Abs. 5 Satz 4 BWahlG nur insgesamt bis zu drei Quasi-Überhangmandate nicht ausgeglichen werden sollen.</t>
+          <t>(4) Der Schutz des Art. 103 Abs. 3 GG wird dabei allein durch Strafurteile deutscher Gerichte ausgelöst (vgl. BVerfGE 12, 62 &lt;66&gt;; 75, 1 &lt;15 f.&gt;; BVerfGK 13, 7 &lt;11 f.&gt;; 19, 265 &lt;273&gt;). Bei transnationalen Konstellationen ist darauf abzustellen, inwieweit aufgrund des Völker- oder des Unionsrechts die Mehrfachverfolgung ausgeschlossen ist (vgl. insoweit etwa BVerfGK 13, 7 &lt;11 f.&gt;; 19, 265 &lt;273&gt;).</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
@@ -2062,14 +2062,14 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>(aa) Bei der systematischen Auslegung ist darauf abzustellen, dass einzelne Rechtssätze, die der Gesetzgeber in einen sachlichen Zusammenhang gestellt hat, grundsätzlich so zu interpretieren sind, dass sie logisch miteinander vereinbar sind; es ist davon auszugehen, dass der Gesetzgeber sachlich Zusammenhängendes so geregelt hat, dass die gesamte Regelung einen durchgehenden, verständlichen und widerspruchsfreien Sinn ergibt (vgl. BVerfGE 48, 246 &lt;257&gt;; 124, 25 &lt;40 f.&gt;). Gerade die Stellung einer Vorschrift im Gesetz und ihr sachlich-logischer Zusammenhang mit anderen Vorschriften können den Sinn und Zweck der Norm freilegen (vgl. BVerfGE 35, 263 &lt;279&gt;; 48, 246 &lt;255 f.&gt;).</t>
+          <t>(5) Art. 103 Abs. 3 GG entfaltet seine Wirkung nur nach Strafverfahren, die durch ein rechtskräftiges Sachurteil abgeschlossen wurden (a). Vertrauensschutz, der durch andere Entscheidungen begründet wird, die zum rechtskräftigen Abschluss eines Strafverfahrens führen, ist nicht vom engen Schutzgehalt des Art. 103 Abs. 3 GG erfasst, sondern besteht nach allgemeinen Grundsätzen (b).</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
@@ -2078,14 +2078,14 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>(bb) Demgemäß ist vorliegend in Rechnung zu stellen, dass § 6 Abs. 5 Satz 4 BWahlG auf die Sitzzahlerhöhung nach § 6 Abs. 5 Satz 1 BWahlG („Bei der Erhöhung“) Bezug nimmt. Diese ist auf die Feststellung der Gesamtzahl der Sitze im Deutschen Bundestag gerichtet, die im Rahmen der zweiten Verteilung nach § 6 Abs. 6 BWahlG konkret zur Verfügung stehen müssen. Dafür wird nach § 6 Abs. 5 Satz 1 BWahlG die Zahl der nach § 6 Abs. 1 Satz 3 BWahlG verbleibenden Sitze so lange erhöht, bis jede Partei in der zweiten Verteilung nach § 6 Abs. 6 Satz 1 BWahlG mindestens die ihren Landeslisten zugeordneten Mindestsitze (§ 6 Abs. 5 Satz 2 und 3 BWahlG) erhält. Vor diesem Hintergrund liegt es auf der Hand, auch die Zahl der bei dieser Erhöhung nicht zu berücksichtigenden Sitze im Sinne von § 6 Abs. 5 Satz 4 BWahlG auf die Gesamtzahl der zur Verfügung zu stellenden Sitze zu beziehen (vgl. auch Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 25).</t>
+          <t>(a) Das Mehrfachverfolgungsverbot des Art. 103 Abs. 3 GG wird nur durch Strafurteile ausgelöst, die aufgrund einer Hauptverhandlung in der Sache ergangen sind. Diese Begrenzung des Schutzgehalts liegt in der Funktion des strafrechtlichen Hauptverfahrens begründet (vgl. BVerfGE 3, 248 &lt;251 f.&gt;; 65, 377 &lt;383&gt;) und findet ihre Bestätigung in der Entstehungsgeschichte der Bestimmung.</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -2094,14 +2094,14 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Für die Auffassung der Antragstellerinnen und Antragsteller, dass sich die Zahl von bis zu drei nicht zu berücksichtigenden Quasi-Überhangmandaten auch auf die Summe der den Landeslisten einer Partei zugeordneten Sitze beziehen kann, mithin pro Partei verstanden werden könnte, gibt es in § 6 Abs. 5 Satz 4 BWahlG keinen Anhaltspunkt. Etwas anderes folgt auch nicht aus § 6 Abs. 5 Satz 3 BWahlG, wonach „jede Partei“ mindestens die bei der ersten Verteilung ermittelten Sitze erhält. § 6 Abs. 5 Satz 3 BWahlG betrifft die Zahl der einer Partei mindestens garantierten Sitze, deren Summe die Gesamtzahl der Sitze bildet, die es im Wege der Sitzzahlerhöhung gemäß § 6 Abs. 5 Satz 1 BWahlG zu erreichen gilt. § 6 Abs. 5 Satz 4 BWahlG bezieht sich demgegenüber auf das Verfahren der Sitzzahlerhöhung in seiner Gesamtheit. Die Norm nimmt damit gerade nicht die Zahl der den einzelnen Parteien garantierten Sitze in den Blick. Dem steht auch der Hinweis der Antragstellerinnen und Antragsteller nicht entgegen, dass § 6 Abs. 5 Satz 1 und 3 BWahlG jeweils auf den „Landeslisten“ zugeordnete Sitze der Parteien Bezug nehmen. In beiden Vorschriften stellen sich diese Sitze lediglich als Rechengröße dar, um daraus die Gesamtzahl der im Wege der Sitzzahlerhöhung gemäß § 6 Abs. 5 Satz 1 BWahlG zur Verfügung zu stellenden Sitze zu ermitteln. Wenn aber § 6 Abs. 5 Satz 4 BWahlG bestimmt, dass „dabei“ bis zu drei Quasi-Überhangmandate außer Betracht bleiben, kann dies nur auf den Prozess der Sitzzahlerhöhung insgesamt bezogen sein.</t>
+          <t>Zentrales Anliegen des Strafprozesses ist die Ermittlung des wahren Sachverhalts (vgl. BVerfGE 57, 250 &lt;275&gt;; 118, 212 &lt;231&gt;; 122, 248 &lt;270&gt;; 130, 1 &lt;26&gt;; 133, 168 &lt;199 Rn. 56&gt;). Die Hauptverhandlung bildet das Kernstück des Strafprozesses. In ihr soll der Sachverhalt endgültig aufgeklärt und festgestellt werden. Gemäß § 244 Abs. 2 StPO hat das Gericht zur Erforschung der Wahrheit die Beweisaufnahme von Amts wegen auf alle Tatsachen und Beweismittel zu erstrecken, die für die Entscheidung von Bedeutung sind. Die Hauptverhandlung bietet nach allgemeiner Prozesserfahrung die größtmögliche Gewähr für die Erforschung der Wahrheit und zugleich für die bestmögliche Verteidigung des Angeklagten und damit für ein gerechtes Urteil (vgl. BVerfGE 65, 377 &lt;383&gt;). Sie schafft die prozessual vorgesehenen Voraussetzungen dafür, Feststellungen zur Schuld zu treffen und gegebenenfalls die Unschuldsvermutung zu widerlegen (vgl. BVerfGE 74, 358 &lt;372 f.&gt;). Aus dem Inbegriff der Hauptverhandlung schöpft das Gericht seine Überzeugung über die Tatsachen, die es als erwiesen erachtet und auf die es das Urteil stützt (vgl. § 261, § 264 Abs. 1, § 267 Abs. 1 StPO). Um des Schutzes der Rechtsgüter Einzelner und der Allgemeinheit willen ist der Strafprozess als justizförmiges Verfahren ausgestaltet (vgl. BVerfGE 133, 168 &lt;199 Rn. 56&gt;). Die Wahrheitsfindung erfolgt rechtsgeleitet und stellt die weitestgehende Form rechtsstaatlicher Sachverhaltsermittlung und Urteilsfindung dar. Die Unschuldsvermutung erzwingt ein prozessordnungsgemäßes Verfahren zum Beweis des Gegenteils. Erst auf dieser Grundlage können Feststellungen zur Schuld erfolgen (vgl. BVerfGE 74, 358 &lt;371&gt;). In diesem rechtsstaatlichen Rahmen ist der Staat von Verfassungs wegen gehalten, eine funktionstüchtige Strafrechtspflege zu gewährleisten, ohne die der Gerechtigkeit nicht zum Durchbruch verholfen werden kann (vgl. BVerfGE 33, 367 &lt;383&gt;; 46, 214 &lt;222&gt;; 122, 248 &lt;272&gt;; 130, 1 &lt;26&gt;; 133, 168 &lt;199 f. Rn. 57&gt;). Diese besondere Ausgestaltung des strafgerichtlichen Hauptverfahrens mit der Hauptverhandlung vermittelt dem auf ihm gründenden Urteil die Legitimation, die Grundlage für seine Rechtskraft ist und den damit verbundenen uneingeschränkten Eintritt des Strafklageverbrauchs im Sinne des Art. 103 Abs. 3 GG rechtfertigt (vgl. BVerfGE 3, 248 &lt;253 f.&gt;; 65, 377 &lt;383&gt;; vgl. auch BVerfGE 23, 191 &lt;202&gt;).</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -2110,14 +2110,14 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Gegen dieses Ergebnis spricht auch nicht, dass § 6 Abs. 5 Satz 4 BWahlG bei der Beschreibung der Mandate, die unberücksichtigt bleiben, den Begriff der „Landesliste“ – anders als § 6 Abs. 5 Satz 1 und 3 BWahlG – in der Einzahl verwendet. Soweit die Antragstellerinnen und Antragsteller meinen, dies lege nahe, dass die Zahl „bis zu drei“ auf die einzelne Landesliste einer Partei bezogen sei, lassen sie unberücksichtigt, dass § 6 Abs. 5 Satz 4 BWahlG den Begriff Landesliste hier unter Bezugnahme auf § 6 Abs. 4 BWahlG verwendet. Dieser bestimmt, dass von der für jede Landesliste ermittelten Sitzzahl (§ 6 Abs. 2 und 3 BWahlG) die Zahl der von der Partei im jeweiligen Land errungenen Direktmandate abgerechnet wird (Satz 1) und diese Mandate einer Partei auch dann erhalten bleiben, wenn ihre Zahl die Zahl der Listenmandate übersteigt (Satz 2). Gemäß § 6 Abs. 4 BWahlG werden die Direktmandate folglich im Rahmen der jeweiligen Landesliste angerechnet. Deshalb verwendet die Regelung den Begriff der Landesliste in der Einzahl. § 6 Abs. 5 Satz 4 BWahlG nimmt auf diese Formulierung des § 6 Abs. 4 BWahlG Bezug und benutzt daher den Begriff der Landesliste ebenfalls in der Einzahl. Dass die einzelne Landesliste damit zugleich Bezugspunkt der Nichtberücksichtigung von bis zu drei Quasi-Überhangmandaten sein soll, ergibt sich daraus nicht.</t>
+          <t>Aus diesen Gründen kam der Grundsatz ne bis in idem bereits in seiner durch das Reichsgericht geprägten Gestalt, auf die der Verfassungsgeber bei der Schaffung des Art. 103 Abs. 3 GG maßgeblich abstellte, nur bei Strafurteilen uneingeschränkt zur Anwendung (vgl. BVerfGE 3, 248 &lt;251&gt; m.w.N.; 65, 377 &lt;382 f.&gt;).</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -2126,14 +2126,14 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Soweit die Antragstellerinnen und Antragsteller schließlich einwenden, dass mehrere Parteien nach der ersten Verteilung über Quasi-Überhangmandate verfügten und anhand des Wortlauts von § 6 Abs. 5 Satz 4 BWahlG nicht entschieden werden könne, welche dieser Mandate bis zu einer Zahl von drei nicht ausgeglichen werden sollen, verkennen sie, dass es im Rahmen der Sitzzahlerhöhung einer konkreten Zuordnung der nicht zu berücksichtigenden Quasi-Überhangmandate nicht bedarf. Vielmehr geht es lediglich um die Ermittlung der Gesamtzahl der Sitze für die zweite Verteilung gemäß § 6 Abs. 6 BWahlG. Bei welchen Parteien nicht ausgeglichene Überhangmandate entstehen, entscheidet sich erst im Rahmen dieser zweiten Verteilung. Der Zuordnung der unausgeglichenen Überhangmandate zu den jeweiligen Landeslisten kommt schließlich Relevanz im Falle des Nachrückens für ausscheidende Abgeordnete nach § 48 Abs. 1 Satz 2 BWahlG zu (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 25, 31, 34, 36).</t>
+          <t>(b) Die weiteren Entscheidungsformen, mit denen ein Strafverfahren seinen Abschluss finden kann, begründen ebenfalls schutzwürdiges Vertrauen. Der Schutz rührt jedoch nicht unmittelbar aus Art. 103 Abs. 3 GG her, sondern wurzelt verfassungsrechtlich im allgemeinen rechtsstaatlichen Gebot des Vertrauensschutzes. Dies betrifft sowohl Strafbefehle (aa) als auch Verfahrenseinstellungen der Staatsanwaltschaft (bb) und verfahrensbeendende Gerichtsentscheidungen (cc).</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -2142,14 +2142,14 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>(c) Auch die genetische Auslegung bestätigt, dass gemäß § 6 Abs. 5 Satz 4 BWahlG bei der Sitzzahlerhöhung bis zu drei Quasi-Überhangmandate insgesamt hinzunehmen sind.</t>
+          <t>(aa) Strafbefehle unterfallen nicht dem Schutz des Art. 103 Abs. 3 GG. Einfachgesetzliche Regelungen – wie insbesondere § 373a StPO – sind vielmehr am allgemeinen Prozessgrundsatz ne bis in idem als Ausfluss des rechtsstaatlichen Vertrauensschutzgebotes zu messen.</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -2158,14 +2158,14 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>(aa) In der Begründung des Gesetzentwurfs wird zu § 6 Abs. 5 Satz 4 BWahlG ausgeführt (BTDrucks 19/22504, S. 8 f.; ähnlich auch S. 6): „Die erhöhte Gesamtsitzzahl fällt […] im Ergebnis um so viele Sitze zu niedrig für eine vollständige Anrechnung aller Wahlkreismandate aus, dass bei der endgültigen Verteilung nach Absatz 6 im Ergebnis bis zu drei Überhangmandate entstehen“. Dies setzt voraus, dass auch im Rahmen der der zweiten Verteilung vorgeschalteten Erhöhung nach § 6 Abs. 5 BWahlG nur bis zu drei Quasi-Überhangmandate insgesamt nicht berücksichtigt werden.</t>
+          <t>Das Strafbefehlsverfahren (§§ 407 ff. StPO) dient vornehmlich der Vereinfachung und Beschleunigung des Strafverfahrens. Im Gegensatz zum Urteilsverfahren fehlt dem Gericht die Möglichkeit, den Unrechts- und Schuldgehalt der Tat frei und umfassend zu ermitteln und so das öffentliche Interesse an einer gerechten Entscheidung uneingeschränkt zu wahren (vgl. BVerfGE 3, 248 &lt;253&gt;; 65, 377 &lt;383&gt;). Insoweit steht ein Strafbefehl, gegen den nicht rechtzeitig Einspruch erhoben worden ist, einem Urteil nicht im Sinne des § 410 Abs. 3 StPO gleich (vgl. bereits BVerfGE 3, 248 &lt;254&gt;). Aufgrund dessen hat schon das Reichsgericht dem Strafbefehl nur einen eingeschränkten Strafklageverbrauch zuerkannt und eine Verurteilung im ordentlichen Verfahren wegen einer bereits von einem Strafbefehl erfassten Tat dann für zulässig gehalten, wenn die Bestrafung unter einem rechtlichen Gesichtspunkt erfolgte, der nicht schon im Strafbefehl gewürdigt wurde und eine erhöhte Strafbarkeit begründete (vgl. BVerfGE 3, 248 &lt;251&gt; m.w.N.). Diese vorkonstitutionelle Rechtsprechung hat das Bundesverfassungsgericht im Hinblick auf die Entstehungsgeschichte der Bestimmung als immanente Schranke des Art. 103 Abs. 3 GG angesehen (vgl. BVerfGE 3, 248 &lt;252 f.&gt;; 65, 377 &lt;382 ff.&gt;).</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -2174,14 +2174,14 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>(bb) Von dieser Auslegung sind auch die Sachverständigen im Rahmen der Anhörung vor dem Ausschuss für Inneres und Heimat ausgegangen. Trotz zum Teil geäußerter Bedenken, dass das Tatbestandsmerkmal „bis zu einer Zahl von drei“ in § 6 Abs. 5 Satz 4 BWahlG unterschiedlich verstanden werden könne (vgl. Behnke, BTAusschussdrucks 19&lt;4&gt;584 D, S. 8 f.; Schönberger, BTAusschussdrucks 19&lt;4&gt;584 B, S. 5), haben sie im Ergebnis einhellig ausgeführt, dass insbesondere die Begründung des Gesetzentwurfs dafür spreche, dass bis zu drei Quasi-Überhangmandate insgesamt bei der Sitzzahlerhöhung hinzunehmen seien (vgl. Behnke, BTAusschussdrucks 19&lt;4&gt;58 D, S. 8; Schönberger, BTAusschussdrucks 19&lt;4&gt;584 B, S. 5; Pukelsheim, BTAusschussdrucks 19&lt;4&gt;584 A neu, S. 2 sowie Anlage 4; Vehrkamp, BTAusschussdrucks 19&lt;4&gt;584 C, S. 3, 4 f.; Vosgerau, BTAusschussdrucks 19&lt;4&gt;584 F, S. 2; Grzeszick, BTAusschussdrucks 19&lt;4&gt;584 E, S. 6).</t>
+          <t>(bb) Einstellungsentscheidungen der Staatsanwaltschaft vermitteln dem Betroffenen nach allgemeinen rechtsstaatlichen Grundsätzen ein schutzwürdiges Vertrauen in den Bestand der getroffenen Entscheidung, bewirken aber keinen umfassenden Strafklageverbrauch im Sinne des Art. 103 Abs. 3 GG (vgl. BVerfG, Beschluss der 1. Kammer des Zweiten Senats vom 19. Mai 2022 - 2 BvR 1110/21 -, Rn. 50; BGHSt 54, 1 &lt;6 ff. Rn. 14 ff.&gt;). Art. 103 Abs. 3 GG bezieht sich nur auf Entscheidungen staatlicher Gerichte im Sinne des Art. 92 GG, wie sich aus der Verortung der Norm im „Abschnitt IX. Die Rechtsprechung“ des Grundgesetzes ergibt. Auch enthalten Einstellungsentscheidungen der Staatsanwaltschaft keine der Rechtskraft fähigen Feststellungen zur Schuld des Betroffenen.</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -2190,14 +2190,14 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>(cc) Die Beschlussempfehlung des Ausschusses für Inneres und Heimat bestätigt, dass der Änderung von § 6 Abs. 5 Satz 4 BWahlG diese Vorstellung zugrunde lag (vgl. BTDrucks 19/23187, S. 6, 7, 8). Auch wenn angemerkt wurde, dass eine klarere Formulierung wünschenswert gewesen wäre, wurde eindeutig von bis zu drei unausgeglichenen Überhangmandaten insgesamt ausgegangen (vgl. BTDrucks 19/23187, S. 7).</t>
+          <t>Dem steht nicht entgegen, dass dem in Art. 50 GRCh in Verbindung mit Art. 54 SDÜ geregelten unionsrechtlichen Grundsatz ne bis in idem unter bestimmten Voraussetzungen auch staatsanwaltschaftliche Einstellungsentscheidungen unterfallen können (vgl. BVerfG, Beschluss der 1. Kammer des Zweiten Senats vom 19. Mai 2022 - 2 BvR 1110/21 -, Rn. 37 ff. m.w.N. zur Rechtsprechung des Gerichtshofs der Europäischen Union). Art. 103 Abs. 3 GG regelt den Schutzgehalt des Grundsatzes ne bis in idem gerade nicht umfassend, sondern beschränkt das Verbot der Mehrfachverfolgung auf Strafverfahren vor deutschen Gerichten, die mit einem Sachurteil beendet worden sind. Daher besteht hier kein Anlass, das grundrechtsgleiche Recht des Art. 103 Abs. 3 GG im Lichte der EU-Grundrechtecharta auszulegen (vgl. BVerfGE 152, 152 &lt;177 ff. Rn. 60 ff.&gt; – Recht auf Vergessen I). Vielmehr regeln Art. 50 GRCh und Art. 103 Abs. 3 GG jeweils für ihren eigenen Anwendungsbereich Ausprägungen dieses allgemeinen Prinzips, das unter dem Grundgesetz ergänzend durch das allgemeine rechtsstaatliche Vertrauensschutzgebot verwirklicht wird. Ein hinreichendes Schutzniveau des Grundsatzes ne bis in idem bei staatsanwaltschaftlichen Verfahrenseinstellungen ist somit insgesamt gewährleistet.</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -2206,14 +2206,14 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>(dd) Schließlich belegen zahlreiche Beiträge in der parlamentarischen Debatte diese Regelungskonzeption des Gesetzgebers (vgl. BT-Plenarprotokoll 19/177, S. 22326; 19/183, S. 23042, 23048, 23051). Dass dort auch andere Auffassungen vertreten wurden (vgl. BT-Plenarprotokoll 19/177, S. 22327, 22328; 19/183, S. 23044), steht dem nicht entgegen. Für die Frage nach Regelungskonzeption und Zweck eines Gesetzes kommt den Gesetzesmaterialien, in denen sich regelmäßig die im Verfahren als wesentlich erachteten Vorstellungen der am Gesetzgebungsverfahren beteiligten Organe und Personen finden, zwar eine nicht unerhebliche Indizwirkung zu (vgl. BVerfGE 149, 126 &lt;154 f. Rn. 74&gt; m.w.N.; BVerfG, Beschluss des Zweiten Senats vom 20. Juni 2023 - 2 BvE 1/17 -, Rn. 45 – Organstreit Finanzierungsausschluss NPD). Nicht entscheidend sind dabei aber die subjektiven Vorstellungen einzelner Mitglieder der beteiligten Organe (vgl. BVerfGE 157, 223 &lt;263 f. Rn. 106&gt; m.w.N. – Berliner Mietendeckel; BVerfG, Beschluss des Zweiten Senats vom 20. Juni 2023 - 2 BvE 1/17 -, Rn. 45). Bei der ausschließlich von Abgeordneten der damaligen Oppositionsfraktionen geäußerten Auffassung, dass sich die Formulierung „bis zu einer Zahl von drei“ in § 6 Abs. 5 Satz 4 BWahlG auch auf jede einzelne Landesliste beziehen könne (vgl. BT-Plenarprotokoll 19/177, S. 22327, 22328; 19/183, S. 23044), handelt es sich um eine solche subjektive Bewertung einzelner Abgeordneter der Parlamentsminderheit.</t>
+          <t>(cc) Auch gerichtliche Einstellungsentscheidungen sind nicht vom Schutzgehalt des Art. 103 Abs. 3 GG erfasst. Sie enthalten weder in Form eines Prozessurteils (vgl. § 260 Abs. 3 StPO) noch eines Beschlusses (vgl. § 153 Abs. 2 Satz 1, § 153a Abs. 2 Satz 1, § 206a Abs. 1, § 206b Satz 1 StPO) rechtskräftige Feststellungen zur Schuld der betroffenen Person. Daher schaffen sie zwar nach Maßgabe des allgemeinen Grundsatzes ne bis in idem einen Vertrauenstatbestand in den Bestand der Verfahrenseinstellung, entfalten jedoch keine absolute Sperrwirkung nach Art. 103 Abs. 3 GG (vgl. BGHSt 48, 331 &lt;334 ff.&gt;).</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
@@ -2222,14 +2222,14 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>(d) Des Weiteren sprechen Sinn und Zweck der Regelung für das gefundene Auslegungsergebnis. Ziel des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 ist es nach der Entwurfsbegründung, einer stetigen Erhöhung der Sitzzahl des Deutschen Bundestages durch Vollausgleich von Überhangmandaten zu begegnen, um dessen Arbeits- und Funktionsfähigkeit zu erhalten. Dieses Ziel soll erreicht werden, indem ausgehend vom System der personalisierten Verhältniswahl in begrenztem Umfang auf den Ausgleich von Überhangmandaten verzichtet und ein „angemessener Ausgleich zwischen dem Anliegen möglichst proportionaler Abbildung des Zweitstimmenergebnisses im Deutschen Bundestag und dem mit der Personalwahl verbundenen Belang uneingeschränkten Erhalts von Wahlkreismandaten“ im Sinne der Rechtsprechung des Bundesverfassungsgerichts angestrebt wird (vgl. BTDrucks 19/22504, S. 6). Diesbezüglich hat das Bundesverfassungsgericht festgestellt, dass im System der personalisierten Verhältniswahl ein solcher Ausgleich dann noch als gewahrt angesehen werden kann, wenn die Zahl unausgeglichener Überhangmandate etwa die Hälfte der für die Bildung einer Fraktion erforderlichen Zahl von Abgeordneten (vgl. § 10 Abs. 1 GO-BT) nicht überschreitet (vgl. BVerfGE 131, 316 &lt;369&gt;). Vor diesem Hintergrund ist davon auszugehen, dass der Gesetzentwurf darauf abzielt, zur Reduzierung der Bundestagsgröße unausgeglichene Überhangmandate nur unterhalb dieser Schwelle zuzulassen (vgl. BTDrucks 19/22504, S. 6). Dies lässt sich mit der Auslegung, dass bei der Erhöhung der Bundestagsgröße gemäß § 6 Abs. 5 Satz 4 BWahlG bis zu drei Quasi-Überhangmandate insgesamt nicht berücksichtigt und damit im Rahmen der zweiten Verteilung zu echten Überhangmandaten werden, sicher erreichen. Anders wäre es, wenn bis zu drei Quasi-Überhangmandate pro Partei beziehungsweise pro Landesliste einer jeden Partei nicht berücksichtigt würden. In letzterem Fall ließe die Norm offensichtlich das Anfallen von Überhangmandaten in einem Umfang zu, der den Grundcharakter der Wahl als Verhältniswahl aufheben und Bedenken gegen deren Verfassungskonformität begründen würde (vgl. BVerfGE 131, 316 &lt;368 ff.&gt;); im ersteren Fall wäre dies jedenfalls nicht ausgeschlossen.</t>
+          <t>Ebenso wenig haben Gerichtsbeschlüsse, die aufgrund der Ablehnung eines hinreichenden Tatverdachts zur Verfahrensbeendigung führen (vgl. § 174 Abs. 1, § 204 StPO), das Mehrfachverfolgungsverbot des Art. 103 Abs. 3 GG zur Folge. Auch sie enthalten keine rechtskräftigen Schuldfeststellungen, sondern beruhen auf einer bloßen Verdachtsprüfung, die außerhalb einer Hauptverhandlung im schriftlichen Verfahren erfolgt (vgl. BGHSt 48, 331 &lt;336&gt;). Sie bewirken daher keinen umfassenden Strafklageverbrauch, der Art. 103 Abs. 3 GG unterfiele, sondern gewähren lediglich schutzwürdiges Vertrauen in den Bestand der gerichtlichen Entscheidung. Die insoweit in der Strafprozessordnung geregelten Möglichkeiten zur Wiederaufnahme des Verfahrens aufgrund neuer Tatsachen oder Beweismittel (vgl. § 211, § 174 Abs. 2 StPO) sind somit nicht an Art. 103 Abs. 3 GG, sondern am allgemeinen Prozessgrundsatz ne bis in idem zu messen.</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -2238,14 +2238,14 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>(e) Vor diesem Hintergrund spricht auch das Gebot verfassungskonformer Auslegung für ein Verständnis von § 6 Abs. 5 Satz 4 BWahlG im Sinne einer Nichtberücksichtigung von bis zu drei Quasi-Überhangmandaten insgesamt. Danach ist diejenige Auslegung der Norm vorzuziehen, die mit dem Grundgesetz in Einklang steht (vgl. BVerfGE 148, 69 &lt;130 f. Rn. 150&gt; m.w.N.). Selbst wenn vorliegend mehrere Auslegungsvarianten in Betracht kämen, spräche dies für eine Auslegung im dargestellten Sinn, da diese verlässlich ausschließt, dass Überhangmandate in einem Umfang entstehen können, der den Grundcharakter der Wahl als einer Verhältniswahl missachtet (vgl. auch Behnke, BTAusschussdrucks 19&lt;4&gt;584 D, S. 8).</t>
+          <t>Dem steht nicht entgegen, dass das Bundesverfassungsgericht in zwei Kammerbeschlüssen festgehalten hat, ein Nichteröffnungsbeschluss nach § 204 StPO (vgl. BVerfGK 4, 49 &lt;52 f.&gt;) beziehungsweise ein Verwerfungsbeschluss gemäß § 174 Abs. 2 StPO (vgl. BVerfGK 9, 22 &lt;25 f.&gt;) gewährten Schutz vor erneuter Strafverfolgung, und dabei auch auf die „Garantiefunktion des Art. 103 Abs. 3 GG“ (BVerfGK 9, 22 &lt;25&gt;) beziehungsweise auf dessen „Ausstrahlungswirkung“ (BVerfGK 4, 49 &lt;52&gt;) hingewiesen hat. Denn in der Sache haben beide Kammern lediglich auf den allgemeinen Grundsatz ne bis in idem abgestellt und auch nur einen eingeschränkten Strafklageverbrauch infolge der in Rede stehenden Gerichtsbeschlüsse angenommen. Eine Verletzung von Art. 103 Abs. 3 GG selbst war gerade nicht Gegenstand der Entscheidungen.</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -2254,14 +2254,14 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>(f) Schließlich spricht auch das Verständnis, das die Wahlorgane § 6 Abs. 5 Satz 4 BWahlG in der Praxis zugrunde gelegt haben, für eine Bestimmung des Regelungsgehalts der Norm im Sinne einer Beschränkung auf drei unausgeglichene Quasi-Überhangmandate insgesamt.</t>
+          <t>bb) Im Rahmen dieses begrenzten Schutzgehalts verbietet Art. 103 Abs. 3 GG dem Gesetzgeber die Wiederaufnahme von Strafverfahren zum Nachteil des Grundrechtsträgers nicht generell (1), jedenfalls aber die Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel (2).</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -2270,14 +2270,14 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>(aa) Für die Beantwortung der Frage, welche Regelungskonzeption einem Gesetz zugrunde liegt, kommt dem Verständnis der Vorschrift in der Praxis – zumal wenn es sich um ein einheitliches, über einen längeren Zeitraum unverändertes Verständnis handelt – eine gewisse Indizwirkung zu (vgl. BVerfGE 122, 248 &lt;283 f.&gt; [Sondervotum]; vgl. für die Berücksichtigung der Praxis bei der Auslegung von Wahlrechtsnormen BVerfGE 95, 335 &lt;347 f.&gt;; 121, 266 &lt;309&gt;). Soweit – wie vorliegend – zu beurteilen ist, ob ein Gesetz den Anforderungen des Bestimmtheitsgebots genügt, die Normanwender in ihm mithin hinreichend steuernde und begrenzende Handlungsmaßstäbe vorfinden, liegt der Rückgriff auf deren Auslegungs- und Anwendungspraxis besonders nahe (vgl. zu Divergenzen in der Judikatur als Indiz für die Unbestimmtheit einer Norm BVerfGE 92, 1 &lt;18&gt;).</t>
+          <t>(1) Die Wiederaufnahme eines Strafverfahrens kann auch darauf gerichtet sein, ein mit rechtsstaatlichen Grundsätzen nicht zu vereinbarendes Urteil aufzuheben, ohne dass eine Änderung des materiellen Ergebnisses im Vordergrund steht. Ist dies der Fall, ist Art. 103 Abs. 3 GG nicht berührt (a). Auch Regelungen, die aus anderen Gründen auf die Aufhebung eines Strafurteils zielen, verbietet Art. 103 Abs. 3 GG nicht (b).</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -2286,14 +2286,14 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>(bb) Die Feststellung, wie viele Sitze auf die einzelnen Landeslisten entfallen und welche Bewerber gewählt sind, obliegt gemäß § 42 BWahlG in Verbindung mit § 78 Abs. 2 BWO dem Bundeswahlausschuss nach Prüfung der Wahlunterlagen durch den Bundeswahlleiter, der gemäß § 9 Abs. 2 Satz 1 BWahlG auch Vorsitzender des Bundeswahlausschusses ist. Bereits die von dem Bundeswahlleiter veröffentlichte Musterberechnung zur Sitzverteilung nach dem Fünfundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 mit dem Ergebnis der Bundestagswahl 2017 hat gezeigt, dass er § 6 Abs. 5 Satz 4 BWahlG dahingehend auslegt, dass im Rahmen der Erhöhung der Sitzzahl des Deutschen Bundestages nach § 6 Abs. 5 BWahlG bis zu drei Quasi-Überhangmandate insgesamt unberücksichtigt bleiben (vgl. Bundeswahlleiter, Musterberechnung: Sitzverteilung nach dem 25. BWahlGÄndG mit dem Ergebnis der Bundestagswahl 2017, 2020, S. 8). Auch der Ermittlung der Sitzverteilung für den 20. Deutschen Bundestag wurde diese Auslegung zugrunde gelegt (vgl. Bundeswahlleiter, Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 421). Zweifel, ob die Norm auch anders verstanden werden könnte, hat der Bundeswahlleiter weder anlässlich dieser Berechnungen noch im Rahmen der mündlichen Verhandlung zum Ausdruck gebracht.</t>
+          <t>(a) Wird durch eine Wiederaufnahme ein Urteil korrigiert, ohne den materiellen Entscheidungsinhalt zu ändern, ist der Schutzgehalt des Art. 103 Abs. 3 GG noch nicht berührt. Dementsprechend verstößt die Wiederaufnahme des Verfahrens nicht gegen Art. 103 Abs. 3 GG, wenn sie darauf beschränkt ist, die materielle Rechtsgrundlage eines Strafurteils auszuwechseln, weil das Bundesverfassungsgericht sie für nichtig erklärt hat, und dabei alle sonstigen Urteilsbestandteile unberührt lässt (vgl. BVerfGE 15, 303 &lt;307&gt;). Ob eine solche beschränkte Wiederaufnahme eines Strafverfahrens, durch die im Beschlusswege ohne Erneuerung der Hauptverhandlung und ohne Anhörung des Verurteilten das ursprüngliche Urteil geändert wird, nach den Vorschriften der Strafprozessordung und des § 79 BVerfGG erfolgen darf, ist nicht unmittelbar vom Bundesverfassungsgericht zu prüfen (vgl. BVerfGE 15, 303 &lt;306&gt; m.w.N.). Erfolgt auf der Grundlage der bestehenden einfachgesetzlichen Vorschriften eine solche beschränkte Wiederaufnahme, so liegt darin keine von Art. 103 Abs. 3 GG verbotene nochmalige Bestrafung, wenn die tatsächlichen Feststellungen des Urteils, die rechtliche Beurteilung der Tat im Übrigen, die Art und Höhe der Strafe und die Vollstreckungsvoraussetzungen unverändert bleiben (vgl. BVerfGE 15, 303 &lt;308&gt;).</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -2302,14 +2302,14 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>(3) Soweit § 6 Abs. 5 Satz 4 BWahlG weiter bestimmt, dass die Quasi-Überhangmandate bei der Erhöhung „unberücksichtigt bleiben“, genügt auch dies den dargelegten Bestimmtheitsanforderungen. Die Regelung sieht vor, dass bis zu drei Quasi-Überhangmandate bei der Berechnung der Sitzzahlerhöhung außer Betracht zu lassen und nicht lediglich – wie von den Antragstellerinnen und Antragstellern erörtert – von der gemäß § 6 Abs. 5 Satz 1 BWahlG ermittelten Gesamtsitzzahl in Abzug zu bringen sind. Letzteres führte dazu, dass sich die Größe des Deutschen Bundestages im Vergleich zu seiner Sitzzahl bei einem Vollausgleich lediglich um maximal drei Sitze verringerte. Eine derart geringfügige Reduzierung des Anwachsens der Größe des Deutschen Bundestages trägt dem im Fünfundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 zum Ausdruck kommenden Willen des Gesetzgebers erkennbar nicht Rechnung.</t>
+          <t>(b) Wiederaufnahmeregelungen, die nicht in erster Linie auf die Änderung des materiellen Entscheidungsinhalts zielen, sondern vorrangig auf die Aufhebung eines Strafurteils gerichtet sind, sind ebenfalls nicht vom Verbot des Art. 103 Abs. 3 GG umfasst.</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
@@ -2318,14 +2318,14 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>§ 6 Abs. 5 Satz 4 BWahlG normiert zudem ausdrücklich, dass Quasi-Überhangmandate „bei der Erhöhung“ der Sitzzahlen bis zu einer Zahl von drei unberücksichtigt bleiben. Daraus folgt, dass diese Mandate bereits im Prozess der Berechnung der erhöhten Gesamtsitzzahl des Deutschen Bundestages gemäß § 6 Abs. 5 Satz 1 BWahlG nicht in Ansatz zu bringen sind. Voraussetzungen und Grenzen des Erhöhungsprozesses ergeben sich aus § 6 Abs. 5 Satz 2 bis 4 BWahlG. Demnach endet die Erhöhung in dem Moment, in dem bei der zweiten Verteilung nach § 6 Abs. 6 Satz 1 BWahlG jede Partei die ihr garantierten Mindestsitze (§ 6 Abs. 2 Satz 2 und 3 BWahlG) erhält und zugleich die Summe der verbleibenden Quasi-Überhangmandate nicht mehr als drei beträgt. Dass bis zu drei Quasi-Überhangmandate bei der Erhöhung „unberücksichtigt“ bleiben, besagt folglich, dass sie in die Erhöhung der Gesamtsitzzahl des Deutschen Bundestages nicht einbezogen, mithin nicht ausgeglichen werden (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 25). Dieses Verständnis hat auch in der Begründung des Entwurfs zum Fünfundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 einen deutlichen Niederschlag gefunden (vgl. BTDrucks 19/22504, S. 1, 6, 8 f.) und entspricht der Vorgehensweise, die die im Innenausschuss des Deutschen Bundestages zu der Gesetzesänderung angehörten Sachverständigen erläutert haben (vgl. Pukelsheim, BTAusschussdrucks 19&lt;4&gt;584 A neu, Anlage 5, S. 2, 6, 10, 14, 18; Behnke, BTAusschussdrucks 19&lt;4&gt;584 D, S. 7).</t>
+          <t>Dies betrifft insbesondere die Wiederaufnahme von Strafverfahren gemäß § 362 Nr. 1–4 StPO (vgl. Schulze-Fielitz, in: Dreier, GG, Bd. 3, 3. Aufl. 2018, Art. 103 Abs. 3 Rn. 32 und 35; Nolte/Aust, in: v. Mangoldt/Klein/Starck, GG, Bd. 3, 7. Aufl. 2018, Art. 103 Rn. 222 f.; vgl. auch Kunig/Saliger, in: v. Münch/Kunig, GG, Bd. 2, 7. Aufl. 2021, Art. 103 Rn. 78; Degenhart, in: Sachs, GG, 9. Aufl. 2021, Art. 103 Rn. 84; Radtke, in: Epping/Hillgruber, BeckOK GG, Art. 103 Rn. 47 f. &lt;Aug. 2022&gt;; a.A. Sodan, in: ders., GG, 4. Aufl. 2018, Art. 103 Rn. 31 f.; Brade, AöR 146 &lt;2021&gt;, S. 130 &lt;167, 170&gt;; zweifelnd Neumann, in: Festschrift für Heike Jung, 2007, S. 655 &lt;666&gt;; Höfling/Burkiczak, in: Friauf/Höfling, GG, Bd. 5, Art. 103 Rn. 173 ff. &lt;IV/09&gt;; Remmert, in: Dürig/Herzog/Scholz, GG, Art. 103 Abs. 3 Rn. 62 &lt;Nov. 2018&gt;). Diese Bestimmungen stellen immanente Schranken des Art. 103 Abs. 3 GG dar (vgl. BVerfGE 3, 248 &lt;252 f.&gt;; 65, 377 &lt;384&gt;). Inwieweit sie den allgemeinen verfassungsrechtlichen Vorgaben, insbesondere dem Grundsatz der Verhältnismäßigkeit genügen (zu § 362 Nr. 1–2 StPO vgl. Grünewald, ZStW 120 &lt;2008&gt;, S. 545 &lt;574 f.&gt;; Greco, Strafprozesstheorie und materielle Rechtskraft, 2015, S. 985 ff.; zu § 362 Nr. 4 StPO vgl. Knoche, DRiZ 1971, S. 299 &lt;299&gt;; Loos, in: Festschrift für Hans-Ludwig Schreiber, 2003, S. 277 &lt;280 f.&gt;; Bohn, Die Wiederaufnahme des Strafverfahrens zuungunsten des Angeklagten vor dem Hintergrund neuer Beweise, 2016, S. 51; Eschelbach, in: KMR-StPO, § 362 Rn. 84 ff. &lt;Aug. 2005&gt;), bedarf hier keiner Entscheidung.</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -2334,14 +2334,14 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>dd) Schließlich ist § 6 Abs. 5 Satz 5 BWahlG ein hinreichend bestimmter Normbefehl zu entnehmen. Demnach erhöht sich die Gesamtzahl der Sitze im Sinne von § 1 Abs. 1 BWahlG um die „Unterschiedszahl“. Soweit die Antragstellerinnen und Antragsteller rügen, aus dem Wortlaut ergebe sich nicht, welche Unterschiedszahl gemeint sei, überzeugt dies nicht. Ernstliche Zweifel, dass der Begriff der „Unterschiedszahl“ in § 6 Abs. 5 Satz 5 BWahlG die Differenz zwischen der gesetzlichen Regelgröße des Deutschen Bundestages einerseits und der erhöhten Mandatszahl aufgrund der Sitzzahlerhöhung andererseits bezeichnet, bestehen nicht. § 6 Abs. 5 Satz 5 BWahlG soll sicherstellen, dass sich die Gesamtgröße des Deutschen Bundestages um die Zahl erhöht, die erforderlich ist, um den Parteien bei der zweiten Verteilung nach § 6 Abs. 6 BWahlG sämtliche, sich aus § 6 Abs. 5 Satz 1 bis 4 BWahlG ergebenden Sitze zuweisen zu können. Diese Zahl wird in § 6 Abs. 5 Satz 5 BWahlG mit dem Begriff der „Unterschiedszahl“ bezeichnet.</t>
+          <t>§ 362 Nr. 1–3 StPO ermöglicht die Wiederaufnahme, wenn durch anderweitiges Urteil festgestellt (§ 364 StPO) ist, dass in der Hauptverhandlung eine Urkundenfälschung, eine strafbewehrte Falschaussage durch Zeugen oder Sachverständige oder eine Amtspflichtverletzung durch einen Richter oder Schöffen begangen wurde. Die Wiederaufnahme erfolgt bei einer Amtspflichtverletzung (§ 362 Nr. 3 StPO) unabhängig von der inhaltlichen Richtigkeit des Urteils. Auch in den Fällen eines erwiesenermaßen falschen Beweises (§ 362 Nr. 1 und 2 StPO) steht nicht die Korrektur des Ergebnisses im Vordergrund. Die Wiederaufnahme entfällt in letzteren Fällen nur dann, wenn ausgeschlossen ist, dass diese Handlungen Einfluss auf die Entscheidung gehabt haben (§ 370 Abs. 1, 2. Alt. StPO). Ziel der Wiederaufnahme ist in allen diesen Fällen nicht notwendig ein im Ergebnis anderes Urteil, sondern primär die Wiederholung des fehlerbehafteten Verfahrens.</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -2350,14 +2350,14 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>b) Auch die Regelung der zweiten (tatsächlichen) Sitzzuteilung in § 6 Abs. 6 BWahlG genügt bei methodengerechter Auslegung den Bestimmtheitsanforderungen.</t>
+          <t>Die Wiederaufnahmemöglichkeit entfaltet damit Vorwirkungen auf das eigentliche Strafverfahren. Wahrheits- und Rechtspflichten im gerichtlichen Verfahren werden dadurch neben ihrer Strafbewehrung verstärkt. Eine Manipulation des Verfahrens kann nicht dadurch lohnenswert erscheinen, dass ein – für den Angeklagten möglicherweise günstiges – rechtskräftiges Urteil erreicht wird. Bereits der Entwurf der Deutschen Strafprozessordnung von 1873, der § 362 Nr. 1–3 StPO entsprechende Wiederaufnahmegründe vorsah, wurde damit begründet, dass niemand die „Früchte seiner strafbaren Handlungen genießen“ solle. Es verstoße gegen die Fundamentalsätze des Strafrechts, wenn man zulassen wollte, dass „der Verbrecher der verwirkten Strafe durch die Begehung eines neuen Verbrechens entzogen werde“, unabhängig davon durch wen es begangen werde (vgl. Motive zu dem Entwurf einer Deutschen Strafprozessordnung nach den Beschlüssen der von dem Bundesrath eingesetzten Kommission, 1873, S. 174; vgl. auch Frank, Die Wiederaufnahme zuungunsten des Angeklagten im Strafverfahren, 2022, S. 177 f.).</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
@@ -2366,14 +2366,14 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>aa) Dies gilt zunächst für § 6 Abs. 6 Satz 1 BWahlG. Danach werden die nach Absatz 5 zu vergebenden Sitze bundesweit nach der Zahl der zu berücksichtigenden Zweitstimmen in dem in § 6 Abs. 2 Satz 2 bis 7 BWahlG beschriebenen Divisorverfahren mit Standardrundung nach Sainte-Laguë/Schepers auf die nach § 6 Abs. 3 BWahlG zu berücksichtigenden Parteien verteilt. Soweit die Antragstellerinnen und Antragsteller geltend machen, dabei sei unklar, was mit den „nach § 6 Abs. 5 BWahlG zu vergebenden Sitze[n]“ gemeint sei, ist dem nicht zu folgen. Sie räumen selbst zutreffend ein, dass damit die erhöhte Sitzzahl ohne Überhangmandate bezeichnet sein dürfte.</t>
+          <t>Ein Urteil mit einem solch schwerwiegenden Mangel verfehlt die Anforderungen an ein justizförmiges, rechtsgeleitetes Verfahren. Die Wahrung dieser Anforderungen ist jedoch unverzichtbare rechtsstaatliche Voraussetzung für einen gerechten Schuldspruch (vgl. BVerfGE 133, 168 &lt;199 ff. Rn. 56 ff.&gt;). Die Möglichkeit, ein unter solchen Mängeln gefundenes Urteil aufzuheben und das Verfahren zu wiederholen, sichert den Geltungsanspruch des Urteils und damit die rechtsstaatliche Autorität des Strafverfahrens ab.</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -2382,14 +2382,14 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>§ 6 Abs. 6 Satz 1 BWahlG regelt im Rahmen der zweiten (tatsächlichen) Mandatszuteilung die bundesweite Verteilung der nach § 6 Abs. 5 BWahlG zu vergebenden Sitze auf die nach § 6 Abs. 3 BWahlG zu berücksichtigenden Parteien und bestimmt, dass diese nach der Zahl der Zweitstimmen erfolgt. Da aufgrund § 6 Abs. 5 Satz 4 BWahlG im Rahmen der Sitzzahlerhöhung kein vollständiger Ausgleich von Quasi-Überhangmandaten stattfindet, sondern bis zu drei Quasi-Überhangmandate nicht ausgeglichen werden, kann es sich bei der nach § 6 Abs. 6 Satz 1 BWahlG proportional nach dem Zweitstimmenergebnis auf die Parteien zu verteilenden Sitzzahl nur um die nach § 6 Abs. 5 Satz 1 bis 4 BWahlG ermittelte Sitzzahl (ohne die drei unausgeglichenen Überhangmandate) handeln (vgl. auch Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 30 f.). Dies wird durch § 6 Abs. 6 Satz 4 BWahlG bestätigt. Danach verbleiben den Parteien die in den Wahlkreisen errungenen Sitze auch dann, wenn sie die nach § 6 Abs. 6 Satz 1 BWahlG ermittelte Zahl übersteigen. Ein dahingehender Regelungsbedarf besteht aber nur, wenn bei der Berechnung nach § 6 Abs. 6 Satz 1 BWahlG unausgeglichene Überhangmandate nicht berücksichtigt werden. Dem entspricht die Anwendung der Norm durch den Bundeswahlleiter (vgl. Bundeswahlleiter, Musterberechnung: Sitzverteilung nach dem 25. BWahlGÄndG mit dem Ergebnis der Bundestagswahl 2017, 2020, S. 8 f.; ders., Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 421 f., 451).</t>
+          <t>Auch § 362 Nr. 4 StPO hat nicht eine Änderung des Freispruchs zum eigentlichen, vorrangigen Ziel. Vielmehr hat die Norm den Zweck, ein Verhalten zu verhindern, das die Autorität des rechtsstaatlichen Strafverfahrens infrage stellen würde (vgl. Frister, in: SK-StPO, 5. Aufl. 2018, § 362 Rn. 1; Tiemann, in: KK-StPO, 9. Aufl. 2023, § 362 Rn. 1a, 26; Kaspar, in: Satzger/Schluckebier/Widmaier, StPO, 5. Aufl. 2023, § 362 Rn. 7; Weiler, in: Dölling/Duttge/ Rössner, Gesamtes Strafrecht, 5. Aufl. 2022, § 362 StPO Rn. 6; a.A. Kubiciel, GA 2021, S. 380 &lt;392&gt;; Schöch, in: Festschrift für Manfred Maiwald, 2010, S. 769 &lt;779 f.&gt;). In den Motiven zur Strafprozessordnung von 1877 wurde der entsprechende Wiederaufnahmetatbestand damit begründet, dass das allgemeine Rechtsbewusstsein leicht irregeführt werden könne, wenn ein Freigesprochener sich folgenlos öffentlich der Straftat rühmen könnte (vgl. Motive zum Entwurf einer Strafprozessordnung von 1874, abgedruckt in: Hahn, Die gesammten Materialien zu den Reichs-Justizgesetzen, Bd. 3, Erste Abteilung, 1880, S. 265). Er solle nicht in aller Öffentlichkeit die kriminelle Tat schildern, das Opfer und dessen Angehörige verhöhnen, mit dem Freispruch prahlen und den Staat lächerlich machen dürfen (vgl. Marxen/Tiemann, ZIS 2008, S. 188 &lt;189&gt; m.w.N.; Tiemann, in: KK-StPO, 9. Aufl. 2023, § 362 Rn. 1a, 11). Der Grundsatz des akkusatorischen Strafverfahrens, das mit einem Freispruch endet, wenn die Unschuldsvermutung nicht widerlegt werden kann, wäre verkannt, wenn ein Freigesprochener beanspruchte, in seinen sozialen Bezügen nicht als unschuldig, sondern als Täter wahrgenommen zu werden.</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
@@ -2398,14 +2398,14 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>bb) (1) Soweit § 6 Abs. 6 Satz 2 BWahlG sodann bestimmt, dass in den Parteien die Sitze nach der Zahl der zu berücksichtigenden Zweitstimmen in dem in § 6 Abs. 2 Satz 2 bis 7 BWahlG beschriebenen Berechnungsverfahren auf die Landeslisten verteilt werden, ist – anders als in § 6 Abs. 6 Satz 1 BWahlG – die Zahl der Sitze inklusive möglicher unausgeglichener Überhangmandate zugrunde zu legen (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 31 f.; Pukelsheim/Bischof, DVBl 2021, S. 417 &lt;421&gt;). Dies folgt aus § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG, wonach bei der Unterverteilung auf die Landeslisten der Parteien jeder Landesliste mindestens die nach § 6 Abs. 5 Satz 2 BWahlG für sie ermittelte Sitzzahl zugeteilt wird. Diese Mindestsitze sichern sämtliche Direktmandate, und zwar auch dann, wenn diese den Zweitstimmenanteil trotz Sitzzahlerhöhung übersteigen (vgl. Bundeswahlleiter, Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 422; ders., Musterberechnung: Sitzverteilung nach dem 25. BWahlGÄndG mit dem Ergebnis der Bundestagswahl 2017, 2020, S. 9; Grzeszick, BTAusschussdrucks 19&lt;4&gt;584 E, S. 9 f.). Demgemäß werden nach § 6 Abs. 6 Satz 2 BWahlG insgesamt bis zu drei Sitze mehr an die Landeslisten verteilt als im Rahmen der Oberverteilung auf die Parteien nach § 6 Abs. 6 Satz 1 BWahlG (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 32).</t>
+          <t>(2) Demgegenüber verbietet Art. 103 Abs. 3 GG dem Gesetzgeber die Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel, die vorrangig auf eine inhaltlich „richtigere“ Entscheidung zielt (a). Weder ein zwischenzeitlich gewandeltes Verfassungsverständnis (b) noch grundrechtlich geschützte Belange der Opfer und Opferangehörigen (c) führen zu einem anderen Ergebnis.</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
@@ -2414,14 +2414,14 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>(2) Soweit die Antragstellerinnen und Antragsteller einen Wechsel der Bezugsgröße in Satz 1 und 2 des § 6 Abs. 6 BWahlG rügen, der im Widerspruch zum Gesetzeswortlaut stehe, scheinen sie davon auszugehen, dass durch die Formulierung „die Sitze“ in § 6 Abs. 6 Satz 2 BWahlG die Sitzzahl des § 6 Abs. 6 Satz 1 BWahlG in Bezug genommen sei (vgl. auch Pukelsheim/Bischof, DVBl 2021, S. 417 &lt;421&gt;). Dies ergibt sich aber aus dem Wortlaut der Norm nicht. § 6 Abs. 6 Satz 1 BWahlG spricht von den „nach Absatz 5 zu vergebenden Sitzen“. In § 6 Abs. 6 Satz 2 BWahlG heißt es hingegen allgemein „die Sitze“, nicht aber zum Beispiel „diese Sitze“. Daher führt das alleinige Abstellen auf den Wortlaut nicht zu einem eindeutigen Ergebnis. Die Diskrepanz der Sitzzahlen nach § 6 Abs. 6 Satz 1 und § 6 Abs. 6 Satz 2 BWahlG ist nach Systematik und Telos der Regelung gerade intendiert (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 31 f.). Sie dient der Umsetzung der gesetzgeberischen Grundentscheidung, bis zu drei ausgleichslose Überhangmandate zuzulassen. Dazu ist für die Oberverteilung auf die Parteien allein auf die Sitze abzustellen, die proportional zu verteilen sind. Die anschließende Unterverteilung auf die Landeslisten der jeweiligen Partei muss hingegen auch die Sitze berücksichtigen, die als ausgleichslose Überhangmandate zu Proporzverzerrungen führen, da andernfalls nicht alle von den Parteien gewonnenen Sitze umfasst wären.</t>
+          <t>(a) Die Korrektur eines Strafurteils mit dem Ziel, eine inhaltlich „richtigere“ und damit materiell gerechtere Entscheidung herbeizuführen, lässt sich mit der von Art. 103 Abs. 3 GG getroffenen unbedingten Vorrangentscheidung zugunsten der Rechtssicherheit gegenüber der materialen Gerechtigkeit nicht vereinbaren.</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
@@ -2430,14 +2430,14 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>(3) Entgegen den Bedenken der Antragstellerinnen und Antragsteller ist § 6 Abs. 6 Satz 2 BWahlG im Wege der Auslegung auch hinreichend bestimmt zu entnehmen, wie die Unterverteilung auf die Landeslisten zu erfolgen hat.</t>
+          <t>Bereits das Reichsgericht, auf dessen Rechtsprechung zum Grundsatz ne bis in idem Art. 103 Abs. 3 GG inhaltlich Bezug nimmt (vgl. oben Rn. 65), ging davon aus, dass die Einleitung einer neuen Strafverfolgung auch dann ausgeschlossen sein sollte, wenn Tatsachen oder Beweise, die erst „nach eingetretener Rechtskraft des Urteiles zum Vorschein gekommen sind, vorher aber nicht bekannt und nicht zur Sprache gebracht worden waren, die That unter einem anderen rechtlichen Gesichtspunkte strafbar erscheinen lassen“ (vgl. RGSt 2, 347 &lt;348&gt;). Es knüpfte an die der Reichsstrafprozessordnung von 1877 zugrundeliegenden Gesetzesmaterialien an, die betonten, „aufgrund neuer Thatsachen aber [lasse] der Entwurf die Wiederaufnahme des Urtheils zum Nachtheil des Angeklagten in keinem Fall zu“ (vgl. Motive zu dem Entwurf einer Deutschen Strafprozessordnung nach den Beschlüssen der von dem Bundesrath eingesetzten Kommission, 1873, S. 174).</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
@@ -2446,14 +2446,14 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>(a) § 6 Abs. 6 Satz 2 BWahlG regelt durch den Verweis auf das Berechnungsverfahren nach § 6 Abs. 2 Satz 2 bis 7 BWahlG zunächst, dass die Unterverteilung innerhalb der Parteien nach dem Divisorverfahren mit Standardrundung nach Sainte-Laguë/Schepers stattfindet. Zugleich bestimmt § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG, dass jeder Landesliste mindestens die nach § 6 Abs. 5 Satz 2 BWahlG für sie ermittelte Sitzzahl zugeteilt wird. In der Folge ist der Zuteilungsdivisor so zu bestimmen, dass die Landeslisten, bei denen nach der ersten Verteilung neben Direktmandaten (auch) Listenmandate anfallen, sämtliche Direktmandate und jedenfalls die Hälfte der nach Anrechnung dieser Direktmandate verbleibenden Listenmandate erhalten. Dafür ist der anfängliche Divisor, der durch Teilung der zu berücksichtigenden Zweitstimmen durch die Zahl der zu verteilenden Sitze bestimmt wird, iterativ zu verändern, bis diese Bedingung erfüllt ist (vgl. Bundeswahlleiter, Musterberechnung: Sitzverteilung nach dem 25. BWahlGÄndG mit dem Ergebnis der Bundestagswahl 2017, 2020, S. 9; ders., Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 422, 453 ff.).</t>
+          <t>Der Zweck einer Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel erschöpft sich darin, eine mögliche Diskrepanz zwischen dem Inhalt eines Strafurteils und der materiell-rechtlichen Wirklichkeit, die sich nachträglich offenbart, zu beseitigen. Soweit eine solche Wiederaufnahme vorgesehen ist, gibt der Gesetzgeber der materialen Gerechtigkeit Vorrang vor der Rechtssicherheit. Dies läuft Art. 103 Abs. 3 GG zuwider.</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
@@ -2462,14 +2462,14 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>(b) Diese Auslegung der Norm entspricht sowohl ihrem Sinn und Zweck als auch ihrer Entstehungsgeschichte. Die Mindestsitzzahlgarantie des § 6 Abs. 6 Satz 2 Halbsatz 2 in Verbindung mit Abs. 5 Satz 2 BWahlG ist darauf gerichtet, durch die vorrangige Verteilung von Sitzen an Landeslisten mit Direktmandaten eine länderübergreifende Kompensation von Quasi-Überhangmandaten einer Partei zu ermöglichen und dadurch die Sitzansprüche bei Überhängen zu reduzieren, zugleich aber zu verhindern, dass einer Landesliste gar keine beziehungsweise weniger Sitze zugeteilt werden, als ihr nach § 6 Abs. 5 Satz 2 BWahlG zustehen (vgl. BTDrucks 19/22504, S. 6 f.; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 28, 32). Um dies zu erreichen, bestimmt § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG eine zusätzliche Bedingung für die Wahl des Zuteilungsdivisors im Rahmen der Unterverteilung der Sitze auf die Landeslisten. Damit orientiert sich die Norm an der Technik der Vorgängerregelung, welche für die Unterverteilung der Sitze auf die Landeslisten der Parteien ebenfalls das Divisorverfahren mit Standardrundung vorsah und als zusätzliche Bedingung formulierte, dass jede Landesliste mindestens die Zahl der in den Wahlkreisen des Landes von der Partei errungenen Sitze erhalten sollte (§ 6 Abs. 6 Satz 2 BWahlG 2013). Auch nach der Vorgängerregelung musste bei der Verteilung der Sitze auf die Landeslisten der Parteien nach dem Divisorverfahren mit Standardrundung der Divisor so gewählt werden, dass die Partei die ihr zustehende Zahl an Sitzen und zusätzlich jede Landesliste mindestens so viele Sitze erhielt, wie sie Wahlkreise gewonnen hatte (vgl. Strelen, in: Schreiber, BWahlG, 10. Aufl. 2017, § 6 Rn. 26c).</t>
+          <t>Die Rechtssicherheit, die durch das justizförmig zustande gekommene Urteil geschaffen wurde, erstreckt sich darauf, dass sie nicht durch das Auftauchen neuer Tatsachen oder Beweismittel infrage gestellt wird (vgl. auch BVerfGE 56, 22 &lt;31&gt;; 65, 377 &lt;383 und 385&gt;). Der Rechtsstaat nimmt die Möglichkeit einer im Einzelfall vielleicht unrichtigen Entscheidung vielmehr um der Rechtssicherheit willen in Kauf (vgl. BVerfGE 2, 380 &lt;403&gt;), namentlich auch dann, wenn diese Unrichtigkeit auf nachträglich hervortretenden Umständen beruht (vgl. BVerfGE 56, 22 &lt;31&gt;). Diese ziehen die Rechtsförmigkeit und Rechtsstaatlichkeit des vorausgegangenen Strafverfahrens nicht in Zweifel und begründen daher auch keinen schwerwiegenden Mangel der ergangenen Entscheidung. Deshalb zielt die Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel nicht darauf, den Geltungsanspruch der ergangenen Entscheidung zu stärken, sondern stellt diese, im Gegenteil, zur Disposition. Aber gerade im Falle eines Freispruchs bedarf es der Autorität eines rechtskräftigen Urteils. Aufgabe und Funktion eines Urteils und dessen Rechtskraft bestehen darin, die Rechtslage zu dem für das Gericht maßgeblichen Zeitpunkt durch die Rechtsbeständigkeit des Inhalts der Entscheidung verbindlich festzustellen und hierdurch Rechtssicherheit und Rechtsfrieden zu schaffen (vgl. BVerfGE 47, 146 &lt;161&gt;).</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
@@ -2478,14 +2478,14 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>cc) Schließlich genügen auch § 6 Abs. 6 Satz 3 und 4 BWahlG im Ergebnis den Bestimmtheitsanforderungen.</t>
+          <t>(b) Art. 103 Abs. 3 GG hat auch nicht aufgrund einer gewandelten Verfassungswirklichkeit eine veränderte Bedeutung erhalten, in deren Folge dem Gesetzgeber die Gestaltung einer – womöglich eng umgrenzten – Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel offen stünde.</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
@@ -2494,14 +2494,14 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>(1) Gemäß § 6 Abs. 6 Satz 3 BWahlG ist von der nach § 6 Abs. 6 Satz 2 BWahlG für jede Landesliste einer Partei ermittelten Gesamtzahl der Sitze die Anzahl der von ihr in dem jeweiligen Land erzielten Direktmandate abzuziehen. Die Norm ordnet mithin die für die personalisierte Verhältniswahl typusbestimmende Anrechnung der Direktmandate auf die Ergebnisse der Verhältniswahl an (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 33). Zweifel hinsichtlich ihrer Bestimmtheit bestehen nicht.</t>
+          <t>Zwar sind das Straf- und das Strafprozessrecht fortwährend Änderungen unterworfen. Insbesondere die Zulassung der Verständigung hat dabei auch Einfluss auf die Wahrheitsfindungsfunktion des Strafprozesses erlangt (vgl. BVerfGE 133, 168 &lt;204 ff. Rn. 65 ff.&gt;). An den verfassungsrechtlichen Vorgaben für das Strafverfahren vermögen diese oder auch andere Entwicklungen jedoch nichts zu ändern (vgl. BVerfGE 133, 168 &lt;225 ff. Rn. 100 ff.&gt;).</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
@@ -2510,14 +2510,14 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>(2) Sodann bestimmt § 6 Abs. 6 Satz 4 BWahlG, dass die in den Wahlkreisen errungenen Sitze einer Partei auch dann verbleiben, wenn sie die nach § 6 Abs. 6 Satz 1 BWahlG ermittelte Zahl übersteigen. Dies ist bei methodengerechter Auslegung dahingehend zu verstehen, dass die von einer Partei in den Wahlkreisen eines Landes errungenen Direktmandate ihr auch dann verbleiben, wenn sie die Zahl der Mandate übersteigen, die der entsprechenden Landesliste unter Zugrundelegung der erhöhten Gesamtsitzzahl (§ 6 Abs. 6 Satz 1 BWahlG) ohne Berücksichtigung der Landesmindestsitzzahl (§ 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG) zustehen.</t>
+          <t>Nichts anderes gilt für die Weiterentwicklung kriminaltechnischer Methoden und Aufklärungsmöglichkeiten. Sie können neue Ausprägungen grundrechtlicher Schutzbedarfe hervorbringen (vgl. BVerfGE 65, 1 &lt;42&gt;; 109, 279 &lt;309&gt;; 112, 304 &lt;316&gt;; 113, 29 &lt;45 f.&gt;; 120, 274 &lt;305 f.&gt;; 120, 378 &lt;398 f.&gt;; 154, 152 &lt;215 ff. Rn. 87 ff.&gt; – BND - Ausland-Ausland-Fernmeldeaufklärung; BVerfG, Urteil des Ersten Senats vom 16. Februar 2023 - 1 BvR 1547/19 u.a. -, Rn. 52 ff. – Automatisierte Datenanalyse). Eine Zurücknahme verfassungsrechtlichen Schutzes gegenüber staatlichen Eingriffen folgt daraus jedoch nicht.</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
@@ -2526,14 +2526,14 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>(a) Zwar ließe sich § 6 Abs. 6 Satz 4 BWahlG allein nach seinem Wortlaut aufgrund der Bezugnahme auf die bundesweite Oberverteilung der Sitze auf die Parteien gemäß § 6 Abs. 6 Satz 1 BWahlG auch dahingehend verstehen, dass nur Fälle erfasst sind, in denen die Zahl der Direktmandate, die eine Partei bundesweit errungen hat, die Zahl der Sitze übersteigt, die der Partei nach ihrem bundesweiten Zweitstimmenergebnis unter Berücksichtigung der Sitzzahlerhöhung zustehen.</t>
+          <t>Erst recht nehmen die verfassungsrechtlichen Vorgaben gegenüber dem Gesetzgeber nicht deshalb ab, weil eine gefestigte demokratische und rechtsstaatliche Entwicklung in der Bundesrepublik Deutschland dazu geführt hätte, dass eine Abkehr oder Aufweichung der verfassungsrechtlichen Grundsätze nicht mehr zu befürchten sind (vgl. dagegen Hoven, JZ 2021, S. 1154 &lt;1160&gt;). Die Gewährleistungen der im Grundgesetz garantierten Grundrechte stehen „nicht unter dem Vorbehalt einer realen Gefahr für die freiheitlich-demokratische Grundordnung“ (vgl. Pohlreich, HRRS 2023, S. 140 &lt;143&gt;).</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -2542,14 +2542,14 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>(b) Der Rückgriff auf die übrigen Auslegungsmethoden zeigt jedoch, dass im Rahmen von § 6 Abs. 6 Satz 4 BWahlG keine bundesweite, sondern eine landeslistenbezogene Betrachtung vorzunehmen ist.</t>
+          <t>(c) Eine Ausweitung des gesetzgeberischen Gestaltungsspielraums zur Regelung der Wiederaufnahme von Strafverfahren kann auch nicht auf die Belange von Opfern und deren Angehörigen gestützt werden.</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
@@ -2558,14 +2558,14 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>(aa) Dafür spricht zunächst die systematische Auslegung. § 6 Abs. 6 Satz 4 BWahlG schließt unmittelbar an § 6 Abs. 6 Satz 3 BWahlG an, nach dem von der für jede Landesliste ermittelten Sitzzahl die Zahl der von der Partei in den Wahlkreisen des Landes errungenen Sitze abgerechnet werden. § 6 Abs. 6 Satz 3 BWahlG nimmt die Anrechnung der Direktmandate auf die Listenmandate einer Partei folglich bezogen auf die einzelnen Landeslisten vor. § 6 Abs. 6 Satz 4 BWahlG will in unmittelbarem Zusammenhang damit sicherstellen, dass die in den Wahlkreisen eines Landes errungenen Direktmandate der Partei auch dann verbleiben, wenn diese Anrechnung nicht vollständig möglich ist (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 25). Auch § 6 Abs. 6 Satz 5 BWahlG spricht für ein landeslistenbezogenes Verständnis von § 6 Abs. 6 Satz 4 BWahlG, indem er bestimmt, dass sich in diesem Fall die Gesamtzahl der Sitze im Sinne von § 1 Abs. 1 BWahlG um die Unterschiedszahl erhöht und eine erneute Berechnung nach § 6 Abs. 6 Satz 1 BWahlG nicht stattfindet. Mit der Formulierung „in diesem Fall“ knüpft er unmittelbar daran an, dass eine Differenz im Sinne von § 6 Abs. 6 Satz 4 BWahlG vorliegt. Es geht § 6 Abs. 6 Satz 5 BWahlG mithin darum, dass die bei der Sitzzahlerhöhung gemäß § 6 Abs. 5 BWahlG nicht berücksichtigten bis zu drei Quasi-Überhangmandate tatsächlich zu Überhangmandaten werden und die Gesamtzahl der Sitze entsprechend ansteigt (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 34 f.). Dies lässt sich aber nur erreichen, wenn die in § 6 Abs. 6 Satz 5 BWahlG genannte „Unterschiedszahl“ nicht lediglich den Fall einer bundesweiten Differenz zwischen Direktmandaten und Listenmandaten einer Partei bezeichnet, sondern die Differenz zwischen den Sitzzahlen, die der jeweiligen Landesliste nach § 6 Abs. 6 Satz 1 BWahlG zustehen, und der Zahl der von der entsprechenden Partei in dem Land darüber hinausgehend errungenen Direktmandate.</t>
+          <t>Zwar kann nach der Kammerrechtsprechung aus der staatlichen Schutzpflicht aus Art. 2 Abs. 2 Satz 1 und 2 in Verbindung mit Art. 1 Abs. 1 Satz 2 GG ein Anspruch gegen den Staat auf effektive Strafverfolgung dort folgen, wo der Einzelne nicht in der Lage ist, erhebliche Straftaten gegen seine höchstpersönlichen Rechtsgüter abzuwehren, und ein Verzicht auf die effektive Verfolgung solcher Taten zu einer Erschütterung des Vertrauens in das Gewaltmonopol des Staates und einem allgemeinen Klima der Rechtsunsicherheit und Gewalt führen kann (vgl. BVerfG, Beschluss der 1. Kammer des Zweiten Senats vom 26. Juni 2014 - 2 BvR 2699/10 -, Rn. 10; Beschluss der 3. Kammer des Zweiten Senats vom 6. Oktober 2014 - 2 BvR 1568/12 -, Rn. 11; Beschluss der 3. Kammer des Zweiten Senats vom 19. Mai 2015 - 2 BvR 987/11 -, Rn. 20; Beschluss der 2. Kammer des Zweiten Senats vom 15. Januar 2020 - 2 BvR 1763/16 -, Rn. 35 f.; Beschluss der 2. Kammer des Zweiten Senats vom 21. Dezember 2022 - 2 BvR 378/20 -, Rn. 53). Der Anspruch auf effektive Strafverfolgung verbürgt jedoch kein bestimmtes Ergebnis, sondern verpflichtet die Strafverfolgungsorgane grundsätzlich nur zu einem (effektiven) Tätigwerden (vgl. BVerfG, Beschluss der 2. Kammer des Zweiten Senats vom 21. Dezember 2022 - 2 BvR 378/20 -, Rn. 56). Die Gründe für eine Wiederaufnahme zulasten des Angeklagten aufgrund neuer Tatsachen oder Beweismittel wurzeln jedoch nicht in gravierenden Mängeln der Strafverfolgung an sich und insbesondere nicht in der Nichtverfolgung einer Straftat. Ein Freispruch steht vielmehr am Ende eines Strafverfahrens, das gerade nicht eingestellt, sondern durchgeführt worden ist. Das Vertrauen der Opfer und deren Angehöriger in die rechtsförmige und effektive Strafverfolgung kann daher durch Freisprüche grundsätzlich nicht erschüttert werden.</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
@@ -2574,14 +2574,14 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>(bb) Auch die genetische und die teleologische Auslegung sprechen für das dargelegte Verständnis von § 6 Abs. 6 Satz 4 BWahlG.</t>
+          <t>Insbesondere der Verweis auf die fortlaufende Verbesserung der Ermittlungsmethoden stellt die Rechtsstaatlichkeit früherer Strafverfolgung nicht infrage. Wird die Aufklärung ungelöster Fälle mithilfe früher nicht verfügbarer Erkenntnismittel möglich, bestätigt dies vielmehr die rechtsstaatliche Unbedenklichkeit der früheren, wenn auch in der Sache unvollständigen Ergebnisse. Technischen Fortschritt unterstellt, kann eine spätere und daher mit moderneren Methoden geführte Aufklärung die Chance besserer Erkenntnisse in sich tragen. Sie kann aber auch durch den Umstand belastet sein, dass nicht alle für das zuerst geführte Verfahren relevanten Beweismittel auch im zweiten Verfahren noch zur Verfügung stehen oder ebenso ertragreich sind, wie sie es im ersten Verfahren waren. Dem steht indes das weit gewichtigere Ziel zeitnaher Aufklärung und Verurteilung von Straftaten gegenüber. Letzteres liegt nicht nur im Interesse des Angeklagten und der Allgemeinheit, sondern insbesondere auch der Opfer und ihrer Angehörigen. Auch der Vertreter des WEISSER RING e.V. hat in der mündlichen Verhandlung erläutert, dass eine generelle Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel nicht dem Anliegen der Opferschutzorganisation entspreche. Ein Strafprozess, der wegen des grundsätzlich stets möglichen Auftauchens neuer Tatsachen oder Beweismittel faktisch nie ende, würde für die Opfer beziehungsweise für ihre Hinterbliebenen eine erhebliche seelische Belastung darstellen, die das Bedürfnis an einer inhaltlich richtigen Aufklärung und Urteilsfindung immer weiter zurücktreten lasse, je mehr Zeit nach der Tat verstrichen sei.</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
@@ -2590,14 +2590,14 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Zum einen knüpft die Formulierung des § 6 Abs. 6 Satz 3 bis 5 BWahlG erkennbar an entsprechende Regelungen in früheren Bundeswahlgesetzen an. Schon § 6 BWahlG 1956 (BGBl I S. 383) bestimmte:</t>
+          <t>Ohnehin geht der Anspruch auf effektive Strafverfolgung nicht über die Erzwingung einer Anklage und die Verfahrensrechte als Nebenkläger hinaus. Die inhaltliche Korrektur eines Strafurteils, namentlich eine Verurteilung anstelle eines Freispruchs, ist hiervon nicht umfasst (vgl. BVerfG, Beschluss der 1. Kammer des Zweiten Senats vom 26. Juni 2014 - 2 BvR 2699/10 -, Rn. 14; Beschluss der 3. Kammer des Zweiten Senats vom 6. Oktober 2014 - 2 BvR 987/11 -, Rn. 15; Beschluss der 3. Kammer des Zweiten Senats vom 19. Mai 2015 - 2 BvR 1568/12 -, Rn. 24; Beschluss der 2. Kammer des Zweiten Senats vom 15. Januar 2020 - 2 BvR 1763/16 -, Rn. 42; Beschluss der 2. Kammer des Zweiten Senats vom 21. Dezember 2022 - 2 BvR 378/20 -, Rn. 56 f.). Der Staat ist nur zur Strafverfolgung selbst, nicht auch zu ihrem Erfolg im Sinne der Ermittlung der absoluten Wahrheit verpflichtet, erst recht nicht im Wege der Wiederaufnahme bereits rechtskräftig abgeschlossener Verfahren.</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
@@ -2606,14 +2606,14 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Zum anderen soll durch § 6 Abs. 6 Satz 4 BWahlG nach der Vorstellung des Gesetzgebers die Zuteilung der gemäß § 6 Abs. 5 Satz 4 BWahlG aus dem Ausgleich ausgenommenen bis zu drei Überhangmandate garantiert werden (vgl. BTDrucks 19/22504, S. 9). Dies setzt voraus, dass § 6 Abs. 6 Satz 4 BWahlG nicht lediglich den Fall einer bundesweiten Differenz von Direkt- und Listenmandaten einer Partei erfasst, sondern auch solche Überhangkonstellationen, die auf einer Differenz von Direkt- und Listenmandaten einer Partei in einem Land beruhen.</t>
+          <t>2. Die hier mittelbar angegriffene Norm des § 362 Nr. 5 StPO verstößt danach gegen Art. 103 Abs. 3 GG. Sie erlaubt für den Bereich des Strafrechts (a) eine erneute Strafverfolgung derselben Tat, über die bereits ein rechtskräftiges Strafurteil ergangen ist (b), in erster Linie mit dem Ziel der inhaltlichen Korrektur des Urteils (c), und läuft damit dem Schutzgehalt des Art. 103 Abs. 3 GG zuwider (d).</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -2622,14 +2622,14 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>(c) Zuzugestehen ist dabei, dass § 6 Abs. 6 Satz 4 BWahlG in seinem Regelungsgehalt nicht über § 6 Abs. 6 Satz 2 BWahlG hinausgeht. Durch die dortige Regelung, wonach jeder Landesliste mindestens die nach § 6 Abs. 5 Satz 2 BWahlG für sie ermittelte Sitzzahl zugeteilt wird, ist gewährleistet, dass jeder Partei sämtliche Direktmandate unabhängig davon zugeteilt werden, ob deren Zahl die der Partei bundesweit zugeteilte Zahl an Sitzen gemäß § 6 Abs. 6 Satz 1 BWahlG übersteigt. Weitergehende Gewährleistungen enthält § 6 Abs. 6 Satz 4 BWahlG nicht. Dies führt jedoch nicht zu einer anderen möglichen Auslegung der Regelung und demzufolge nicht zur Unbestimmtheit.</t>
+          <t>a) Die Regelung des § 362 Nr. 5 StPO betrifft das Strafrecht. Nicht nur der Tatbestand des Mordes nach § 211 StGB, sondern auch die darüber hinaus von § 362 Nr. 5 StPO erfassten Verbrechen nach dem Völkerstrafgesetzbuch sind allgemeine Strafgesetze im Sinne des Art. 103 Abs. 3 GG (vgl. entsprechend zu Art. 103 Abs. 2 GG BVerfG, Beschluss der 4. Kammer des Zweiten Senats vom 12. Dezember 2000 - 2 BvR 1290/99 -, Rn. 18 ff.).</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
@@ -2638,14 +2638,14 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>c) Davon ausgehend genügt auch § 48 Abs. 1 Satz 2 BWahlG den Anforderungen des Bestimmtheitsgebots. Die Regelung steht in unmittelbarem Zusammenhang mit § 48 Abs. 1 Satz 1 BWahlG. Danach wird, wenn ein gewählter Bewerber stirbt oder dem Landeswahlleiter schriftlich die Ablehnung des Erwerbs der Mitgliedschaft erklärt oder wenn ein Abgeordneter stirbt oder sonst nachträglich aus dem Deutschen Bundestag ausscheidet, der Sitz aus der Landesliste derjenigen Partei besetzt, für die der gewählte Bewerber oder ausgeschiedene Abgeordnete bei der Wahl angetreten ist. Gemäß § 48 Abs. 1 Satz 2 BWahlG gilt dies nicht, solange die Partei in dem betreffenden Land Mandate gemäß § 6 Abs. 6 Satz 4 BWahlG innehat. Die Regelung schließt die Listennachfolge in unausgeglichene Überhangmandate aus. Entgegen den Bedenken der Antragstellerinnen und Antragsteller ist dabei § 48 Abs. 1 Satz 2 BWahlG hinreichend deutlich zu entnehmen, wann eine solche Überhangsituation vorliegt (aa) und in welchem Land sie besteht (bb).</t>
+          <t>Das Völkerstrafgesetzbuch sieht für die in ihm geregelten Delikte die Verhängung von Kriminalstrafen vor, die ein autoritatives Unwerturteil über die schuldhafte Verletzung eines allgemein gewährleisteten Rechtsgutes und die Störung des allgemeinen Rechtsfriedens beinhalten. Auch weist es keine Besonderheiten auf, die eine gegenüber dem übrigen Strafrecht abweichende Behandlung rechtfertigten. Es besteht vielmehr eine systematische und inhaltliche Nähe zwischen den beiden Regelungskomplexen, die einer unterschiedlichen Sperrwirkung von Verurteilungen, die auf ihrer Grundlage ergangen sind, entgegensteht. Das Völkerstrafgesetzbuch verzichtet weitgehend auf einen allgemeinen Teil und verweist deshalb in § 2 VStGB auf die allgemeinen Bestimmungen des Strafgesetzbuches. Das Delikt des Völkermordes war vor seiner Neuregelung in § 6 VStGB im Jahr 2002 in dem bereits 1954 eingeführten § 220a StGB geregelt (vgl. BGBl II 1954 S. 729 und BGBl I 2002 S. 2254). Nach dem in § 1 Satz 1 VStGB normierten Weltrechtsprinzip ist zudem das deutsche Strafrecht im Übrigen anwendbar. Für Tötungen und Körperverletzungen folgt dies nach der Rechtsprechung des Bundesgerichtshofs aus einer Annexkompetenz. Damit kann nach den auch in diesen Fällen geltenden allgemeinen Konkurrenzregeln (vgl. BGHSt 55, 157 &lt;173 Rn. 50&gt;; 64, 89 &lt;107 Rn. 70&gt;) insbesondere eine Verurteilung wegen Völkermordes nach § 6 VStGB in Tateinheit mit Mord nach § 211 StGB erfolgen (vgl. BGHSt 45, 64 &lt;69 f.&gt;; 64, 89 &lt;107 f. Rn. 71&gt;).</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
@@ -2654,14 +2654,14 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>aa) (1) § 48 Abs. 1 Satz 2 BWahlG nimmt hinsichtlich des Ausschlusses der Listennachfolge ausdrücklich auf Mandate im Sinne von § 6 Abs. 6 Satz 4 BWahlG Bezug. Dies sind auf der Grundlage der vorstehenden Auslegung der Norm die von einer Partei in den Wahlkreisen eines Landes errungenen Sitze, die die Zahl der Sitze übersteigen, die der entsprechenden Landesliste der Partei unter Zugrundelegung der erhöhten Gesamtsitzzahl (§ 6 Abs. 6 Satz 1 BWahlG) ohne Berücksichtigung der Landesmindestsitzzahl (§ 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG) zustehen. Im Ergebnis sind dies die unausgeglichenen Überhangmandate.</t>
+          <t>b) § 362 Nr. 5 StPO stellt ferner auf ein rechtskräftiges Strafurteil eines deutschen Gerichts ab, worunter auch der Freispruch fällt. Die Norm ermöglicht mit der Wiederaufnahme des Verfahrens zuungunsten des Freigesprochenen eine erneute Strafverfolgung wegen derselben – bereits abgeurteilten – Tat.</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
@@ -2670,14 +2670,14 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>(2) Dies entspricht auch der genetischen sowie teleologischen Auslegung von § 48 Abs. 1 Satz 2 BWahlG. Die Begründung des Gesetzentwurfs stellt darauf ab, dass zukünftig wieder bis zu drei (echte) Überhangmandate auftreten können. Dadurch werde die in § 48 Abs. 1 Satz 2 BWahlG 2008 getroffene Regelung erneut erforderlich. Sie führe dazu, dass die Nachbesetzung aus der Landesliste nicht zur Anwendung gelange, wenn der Abgeordnete aus einem Land komme, in dem die betroffene Partei über unausgeglichene Überhangmandate im Sinne des § 6 Abs. 6 Satz 4 BWahlG verfüge (vgl. BTDrucks 19/22504, S. 9). Folglich ist § 48 Abs. 1 Satz 2 BWahlG 2008 darauf gerichtet, die Vorgaben des Beschlusses des Bundesverfassungsgerichts vom 26. Februar 1998 (BVerfGE 97, 317) umzusetzen. Danach kommt bei dem Ausscheiden eines Wahlkreisabgeordneten aus dem Bundestag eine Listennachfolge nicht in Betracht, solange die Partei in dem betroffenen Land über mehr Direktmandate verfügt, als ihr Listensitze zustehen (vgl. BVerfGE 97, 317 &lt;322 ff.&gt;). Der Gesetzgeber verfolgt mit § 48 Abs. 1 Satz 2 BWahlG erkennbar den Zweck, entsprechend der Rechtsprechung des Bundesverfassungsgerichts ein Nachrücken aus der Landesliste auszuschließen, solange in dem Land ein unausgeglichener Überhang an Wahlkreismandaten gegenüber den der Landesliste nach Zweitstimmen zustehenden Sitzen besteht (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 36).</t>
+          <t>c) Grund für die Wiederaufnahme gemäß § 362 Nr. 5 StPO sind neue Tatsachen oder Beweismittel. Zweck dieser Wiederaufnahme ist in erster Linie die inhaltliche Korrektur des Freispruchs. Bereits der Untertitel des Einführungsgesetzes – „Gesetz zur Herstellung materieller Gerechtigkeit“ – verweist auf diesen Zweck der Einführung des neuen Wiederaufnahmegrundes (BGBl I 2021 S. 5252). Auch in der Gesetzesbegründung wird auf keinen anderen Zweck als die Korrektur des „unbefriedigenden“ beziehungsweise „schlechterdings unerträglichen“ Ergebnisses verwiesen, das bestünde, wenn eine Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel weiterhin ausgeschlossen wäre (vgl. BTDrucks 19/30399, S. 1, 9). Der Bestand des Freispruchs soll entfallen, wenn „nach Abschluss des Gerichtsverfahrens neue, belastende Beweismittel aufgefunden werden, aus denen sich mit einer hohen Wahrscheinlichkeit die strafrechtliche Verantwortlichkeit eines zuvor Freigesprochenen ergibt“ (vgl. BTDrucks 19/30399, S. 1 und ähnlich S. 9 f.). Der „Widerspruch der Rechtskraft zur materiellen Gerechtigkeit [soll] aufgelöst“ werden (vgl. BTDrucks 19/30399, S. 2 und ähnlich S. 9 f.). Ziel des Gesetzes ist nichts anderes als die Ermöglichung der Wiederaufnahme aufgrund neuer Tatsachen oder Beweismittel (vgl. BTDrucks 19/30399, S. 6).</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
@@ -2686,14 +2686,14 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>bb) Entgegen den Bedenken der Antragstellerinnen und Antragsteller ergibt die Auslegung von § 48 Abs. 1 Satz 2 BWahlG auch hinreichend bestimmt, welcher Landesliste die bis zu drei unausgeglichenen Überhangmandate zuzuordnen sind. Dem steht nicht entgegen, dass der Wortlaut der Norm dem Rechtsanwender hierfür keine Kriterien an die Hand gibt. Ungeachtet dessen ist nach der Gesamtkonzeption der Regelung davon auszugehen, dass die unausgeglichenen Überhangmandate den Landeslisten einer Partei dadurch zugeordnet werden, dass die Zahl der Sitze, die einer Partei nach § 6 Abs. 6 Satz 1 BWahlG bundesweit zustehen, mit der Zahl der Sitze verglichen wird, die ihren Landeslisten nach § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG zufallen. Ein Überhangmandat liegt bei den Landeslisten vor, bei denen nur aufgrund der Mindestsitzzahlgarantie nach § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG alle Wahlkreismandate erhalten bleiben (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 36).</t>
+          <t>d) § 362 Nr. 5 StPO unterläuft somit die in Art. 103 Abs. 3 GG getroffene – abwägungsfeste – Vorrangentscheidung zugunsten der Rechtssicherheit gegenüber der materialen Gerechtigkeit. Die Neuregelung ist mit dem Mehrfachverfolgungsverbot des Art. 103 Abs. 3 GG nicht zu vereinbaren.</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
@@ -2702,14 +2702,14 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>(1) Für dieses Normverständnis spricht zunächst die genetische Auslegung.</t>
+          <t>Zudem verletzt die Anwendung des § 362 Nr. 5 StPO auf Verfahren, die bereits vor Inkrafttreten dieser Bestimmung durch rechtskräftigen Freispruch abgeschlossen waren, das Rückwirkungsverbot aus Art. 103 Abs. 3 in Verbindung mit Art. 20 Abs. 3 GG.</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>
@@ -2718,14 +2718,14 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Im Verlauf des Gesetzgebungsverfahrens hat der Sachverständige Grzeszick für die Zuordnung der Überhangmandate auf die Landeslisten eine entsprechende Vergleichsrechnung vorgeschlagen. Demnach entstünden die unausgeglichenen Überhangmandate bei den Landeslisten, bei denen nach Verteilung der Sitze nach § 6 Abs. 6 Satz 2 Halbsatz 1 BWahlG weniger Sitze anfielen als gemäß § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG (vgl. Grzeszick, BTAusschussdrucks 19&lt;4&gt;584 E, S. 9 f.). Soweit die Antragstellerinnen und Antragsteller diesen Vorschlag für unklar halten, weil er zwei verschiedene Rechenwege zulasse, überzeugt dies nicht. Der Sachverständige hat in der Anhörung keinen Zweifel daran gelassen, wie die von ihm vorgeschlagene Vergleichsrechnung durchzuführen sei (vgl. Ausschuss für Inneres und Heimat, Protokoll Nr. 19/100, S. 28 f.). Darüber hinaus lässt die von den Antragstellerinnen und Antragstellern alternativ erwogene Zuordnung der Überhangmandate zu den Landeslisten nach dem Durchschnitt von Zweitstimmen pro Sitz außer Betracht, dass im Rahmen der zweiten Verteilung die Unterverteilung auf die Landeslisten nicht streng proportional nach Zweitstimmen erfolgt, sondern unter Berücksichtigung garantierter Mindestsitzzahlen.</t>
+          <t>1. Verfassungsrechtlicher Maßstab für die Zulässigkeit einer Rechtsänderung, die an Sachverhalte der Vergangenheit anknüpft und zugleich Rechtsfolgen in die Vergangenheit erstreckt, ist – wegen des Schwergewichts der Regelung auf der Rechtsfolgenseite – vorrangig das Rechtsstaatsprinzip des Art. 20 Abs. 3 GG in Verbindung mit den von der Rechtsfolgenanordnung berührten Grundrechten oder grundrechtsgleichen Rechten (vgl. BVerfGE 72, 200 &lt;257&gt;; 156, 354 &lt;404 f. Rn. 139&gt;).</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
@@ -2734,14 +2734,14 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Der Vorschlag des Sachverständigen ist im weiteren Gesetzgebungsverfahren aufgegriffen worden. So verweist die CDU/CSU-Bundestagsfraktion in der Begründung der Beschlussempfehlung des federführenden Ausschusses für Inneres und Heimat darauf, dass für die Zuordnung der Überhangmandate zu einer Landesliste im Rahmen des § 48 Abs. 1 Satz 2 BWahlG eine „am Normzweck ausgerichtete Vergleichsberechnung“ durchzuführen sei; dafür sei bei einer Partei mit Überhangmandaten die Sitzzahl fiktiv so lange zu erhöhen, bis alle Mindestsitzansprüche dem Zweitstimmenergebnis bis auf die Anzahl der Überhangmandate entsprächen (vgl. BTDrucks 19/23187, S. 6). Abweichende Stellungnahmen zum Verfahren der Zuordnung von Überhangmandaten zu den Landeslisten im Rahmen von § 48 Abs. 1 Satz 2 BWahlG sind weder der Beschlussempfehlung noch den Äußerungen in der parlamentarischen Debatte zu entnehmen (vgl. BT-Plenarprotokoll 19/177, S. 22326 ff.; 19/183, S. 23041 ff.). Dies spricht dafür, dass es sich bei der Begründung der Beschlussempfehlung des federführenden Ausschusses für Inneres und Heimat durch die CDU/CSU-Fraktion, die den Gesetzentwurf mit eingebracht hat, um Ausführungen von maßgeblich am Gesetzgebungsverfahren Beteiligten handelt, denen bei der Ermittlung des gesetzgeberischen Willens eine nicht unerhebliche Indizwirkung zukommt (vgl. BVerfGE 149, 126 &lt;154 f. Rn. 74&gt; m.w.N.).</t>
+          <t>a) Das Bundesverfassungsgericht unterscheidet dabei in ständiger Rechtsprechung zwischen Gesetzen mit „echter“ und solchen mit „unechter“ Rückwirkung. Eine Rechtsnorm entfaltet „echte“ Rückwirkung in Form einer Rückbewirkung von Rechtsfolgen, wenn ihre Rechtsfolge mit belastender Wirkung für vor dem Zeitpunkt ihrer Verkündung bereits abgeschlossene Tatbestände gelten soll. Demgegenüber ist von einer „unechten“ Rückwirkung in Form einer tatbestandlichen Rückanknüpfung auszugehen, wenn eine Norm auf gegenwärtige, noch nicht abgeschlossene Sachverhalte und Rechtsbeziehungen für die Zukunft einwirkt und damit zugleich die betroffene Rechtsposition entwertet (vgl. BVerfGE 101, 239 &lt;263&gt;; 123, 186 &lt;257&gt;; 148, 217 &lt;255 Rn. 136&gt;), etwa wenn belastende Rechtsfolgen einer Norm erst nach ihrer Verkündung eintreten, tatbestandlich aber von einem bereits ins Werk gesetzten Sachverhalt ausgelöst werden (vgl. BVerfGE 63, 343 &lt;356&gt;; 72, 200 &lt;242&gt;; 97, 67 &lt;79&gt;; 105, 17 &lt;37 f.&gt;; 127, 1 &lt;17&gt;; 132, 302 &lt;318 Rn. 43&gt;; 148, 217 &lt;255 Rn. 136&gt;).</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
@@ -2750,14 +2750,14 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Dem steht nicht entgegen, dass der Sachverständige Pukelsheim in der Anhörung vor dem Ausschuss für Inneres und Heimat die Auffassung vertreten hat, gemäß § 48 Abs. 1 Satz 2 BWahlG finde keine Listennachfolge statt, wenn der ausgeschiedene Abgeordnete aus einem Land komme, in dem in der ersten Verteilung Quasi-Überhangmandate angefallen seien (vgl. Pukelsheim, BTAusschussdrucks 19&lt;4&gt;584 A neu, Anlage 4, Fn. 1). Dieser Vorschlag, der im weiteren Gesetzgebungsverfahren nicht aufgegriffen wurde, lässt außer Betracht, dass es sich bei den Quasi-Überhangmandaten um eine rein rechnerische Größe handelt und sie zudem im Rahmen der Sitzzahlerhöhung weitgehend ausgeglichen werden. Tatsächlich entstehen Überhangmandate erst im Rahmen der zweiten Verteilung nach § 6 Abs. 6 BWahlG. Nur insoweit ist aber eine Listennachfolge nach der Rechtsprechung des Bundesverfassungsgerichts ausgeschlossen. Eine Auslegung, welche für § 48 Abs. 1 Satz 2 BWahlG darauf abstellte, ob in einem Land im Rahmen der ersten Verteilung Quasi-Überhangmandate angefallen sind, dehnte den Kreis der von einer Listennachfolge ausgeschlossenen Landeslisten systemwidrig aus.</t>
+          <t>b) Eine Rückbewirkung von Rechtsfolgen („echte“ Rückwirkung) ist grundsätzlich verfassungsrechtlich unzulässig (vgl. BVerfGE 13, 261 &lt;271&gt;; 95, 64 &lt;87&gt;; 122, 374 &lt;394&gt;; 131, 20 &lt;39&gt;; 141, 56 &lt;73 Rn. 43&gt;; 156, 354 &lt;405 Rn. 140&gt; m.w.N.). Dieses grundsätzliche Verbot der Rückbewirkung von Rechtsfolgen schützt das Vertrauen in die Verlässlichkeit und Berechenbarkeit der unter der Geltung des Grundgesetzes geschaffenen Rechtsordnung und der auf ihrer Grundlage erworbenen Rechte (vgl. BVerfGE 101, 239 &lt;262&gt;; 132, 302 &lt;317 Rn. 41&gt;; 135, 1 &lt;21 Rn. 60&gt;; 156, 354 &lt;405 Rn. 140&gt;). Die Kategorie der „echten“ Rückwirkung – verstanden als zeitliche Rückbewirkung von Rechtsfolgen auf abgeschlossene Tatbestände – findet ihre Rechtfertigung darin, dass mit ihr eine Fallgruppe gekennzeichnet ist, in welcher der Vertrauensschutz regelmäßig Vorrang hat, weil der in der Vergangenheit liegende Sachverhalt mit dem Eintritt der Rechtsfolge kraft gesetzlicher Anordnung einen Grad der Abgeschlossenheit erreicht hat, über den sich der Gesetzgeber vorbehaltlich besonders schwerwiegender Gründe nicht mehr hinwegsetzen darf (vgl. BVerfGE 127, 1 &lt;19&gt;; 156, 354 &lt;406 Rn. 142&gt;).</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
@@ -2766,14 +2766,14 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>(2) Auch das konkrete Berechnungsverfahren zur Bestimmung der Länder, in denen unausgeglichene Überhangmandate auftreten und eine Listennachfolge gemäß § 48 Abs. 1 Satz 2 BWahlG daher ausgeschlossen ist, ergibt sich im Wege der systematischen Auslegung. § 48 Abs. 1 Satz 2 BWahlG steht in unmittelbarem Zusammenhang mit der zweiten Verteilung gemäß § 6 Abs. 6 BWahlG, in der die Sitze zunächst bundesweit auf die Parteien (Satz 1) und sodann in den Parteien auf die Landeslisten (Satz 2) verteilt werden. Für beide Verteilungen wird auf das Divisorverfahren mit Standardrundung verwiesen, welches in § 6 Abs. 2 Satz 2 bis 7 BWahlG geregelt ist. Dies spricht dafür, dieses Verfahren auch für die Bestimmung der von einer Listennachfolge ausgeschlossenen Länder nach § 48 Abs. 1 Satz 2 BWahlG zur Anwendung zu bringen, indem die auf diesem Wege ermittelten Sitzzahlen nach § 6 Abs. 6 Satz 1 BWahlG einerseits und § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG andererseits verglichen werden.</t>
+          <t>Das Rückwirkungsverbot findet im Grundsatz des Vertrauensschutzes indes nicht nur seinen Grund, sondern auch seine Grenze (vgl. BVerfGE 13, 261 &lt;271 f.&gt;; 88, 384 &lt;404&gt;; 101, 239 &lt;266&gt;; 126, 369 &lt;393&gt;; 135, 1 &lt;21 Rn. 61&gt;; 156, 354 &lt;406 Rn. 142&gt; m.w.N.). Eine Ausnahme vom Grundsatz der Unzulässigkeit echter Rückwirkungen ist anerkanntermaßen gegeben, wenn die Betroffenen schon im Zeitpunkt, auf den die Rückwirkung bezogen wird, nicht auf den Fortbestand einer gesetzlichen Regelung vertrauen durften, sondern mit deren Änderung rechnen mussten (vgl. BVerfGE 13, 261 &lt;272&gt;; 30, 367 &lt;387&gt;; 88, 384 &lt;404&gt;; 95, 64 &lt;86 f.&gt;; 122, 374 &lt;394&gt;; 135, 1 &lt;22 Rn. 62&gt;; 156, 354 &lt;406 f. Rn. 143&gt; m.w.N.). Vertrauensschutz kommt insbesondere dann nicht in Betracht, wenn die Rechtslage so unklar und verworren war, dass eine Klärung erwartet werden musste (vgl. BVerfGE 13, 261 &lt;272&gt;; 30, 367 &lt;388&gt;; 88, 384 &lt;404&gt;; 122, 374 &lt;394&gt;; 135, 1 &lt;22 Rn. 62&gt;; 156, 354 &lt;407 Rn. 143&gt; m.w.N.), oder wenn das bisherige Recht in einem Maße systemwidrig und unbillig war, dass ernsthafte Zweifel an seiner Verfassungsmäßigkeit bestanden (vgl. BVerfGE 13, 215 &lt;224&gt;; 30, 367 &lt;388&gt;; 135, 1 &lt;22 Rn. 62&gt;; 156, 354 &lt;407 Rn. 143&gt;). Dasselbe gilt, wenn im Laufe der Zeit (durch Entwicklungen in der Rechtsprechung) ein Zustand allgemeiner und erheblicher Rechtsunsicherheit eingetreten war und für eine Vielzahl Betroffener Unklarheit darüber herrschte, was rechtens sei (vgl. BVerfGE 72, 302 &lt;325 f.&gt;; 131, 20 &lt;41&gt;; 156, 354 &lt;407 Rn. 143&gt;). Der Vertrauensschutz muss ferner zurücktreten, wenn überragende Belange des Gemeinwohls, die dem Prinzip der Rechtssicherheit vorgehen, eine rückwirkende Beseitigung erfordern (vgl. BVerfGE 13, 261 &lt;272&gt;; 18, 429 &lt;439&gt;; 88, 384 &lt;404&gt;; 101, 239 &lt;263 f.&gt;; 122, 374 &lt;394 f.&gt;; 135, 1 &lt;22 Rn. 62&gt;; 156, 354 &lt;407 Rn. 143&gt;), wenn der Bürger sich nicht auf den durch eine ungültige Norm erzeugten Rechtsschein verlassen durfte (vgl. BVerfGE 13, 261 &lt;272&gt;; 18, 429 &lt;439&gt;; 50, 177 &lt;193 f.&gt;; 101, 239 &lt;263 f.&gt;; 135, 1 &lt;22 Rn. 62&gt;; 156, 354 &lt;407 Rn. 143&gt;) oder wenn durch die sachlich begründete rückwirkende Gesetzesänderung kein oder nur ganz unerheblicher Schaden verursacht wird (sogenannter Bagatellvorbehalt; vgl. BVerfGE 30, 367 &lt;389&gt;; 72, 200 &lt;258&gt;; 95, 64 &lt;87&gt;; 101, 239 &lt;263 f.&gt;; 135, 1 &lt;22 f. Rn. 62&gt;; 156, 354 &lt;407 Rn. 143&gt;).</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
@@ -2782,14 +2782,14 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>(3) Dieses Auslegungsergebnis entspricht auch Sinn und Zweck der Regelung. § 48 Abs. 1 Satz 2 BWahlG soll sicherstellen, dass entsprechend der Rechtsprechung des Bundesverfassungsgerichts ein Nachrücken in den Überhang nicht stattfindet (vgl. BVerfGE 97, 317). Demgemäß ist es erforderlich, aber auch ausreichend, die Listennachfolge so lange auszuschließen, wie die betroffene Partei in dem jeweiligen Land über mindestens eines der insgesamt bis zu drei unausgeglichenen Überhangmandate verfügt, die im Rahmen der zweiten Verteilung auftreten können.</t>
+          <t>2. Soweit § 362 Nr. 5 StPO die Wiederaufnahme auch für Verfahren ermöglicht, die bereits zum Zeitpunkt seines Inkrafttretens rechtskräftig abgeschlossen waren (a), liegt darin eine „echte“ Rückwirkung (b), die auch nicht ausnahmsweise zulässig ist (c).</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
@@ -2798,14 +2798,14 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>(4) Schließlich spricht auch die Anwendung der Norm durch die Wahlorgane für das gefundene Auslegungsergebnis. Nach deren Praxis erfolgt die Feststellung, auf welche Landeslisten die bis zu drei Überhangmandate entfallen, dadurch, dass für jede Landesliste mit drohendem Überhang die Zweitstimmen durch die Mindestsitzzahl abzüglich 0,5 beziehungsweise bei zwei oder drei verbleibenden Überhängen zusätzlich durch die Mindestsitzzahl abzüglich 1,5 und 2,5 dividiert werden. Bei den bis zu drei Landeslisten mit dem kleinsten Quotienten verbleibt der Überhang (vgl. Bundeswahlleiter, Musterberechnung: Sitzverteilung nach dem 25. BWahlGÄndG mit dem Ergebnis der Bundestagswahl 2017, 2020, S. 15; ders., Wahl zum 20. Deutschen Bundestag am 26. September 2021, Heft 3, S. 432; soweit der Bundeswahlleiter jeweils von der zweiten Unterverteilung auf die Landeslisten „gemäß § 6 Absatz 2 Satz 2 BWG“ spricht, handelt es sich erkennbar um ein Versehen). Die Bundeswahlleiterin hat im Rahmen der mündlichen Verhandlung nachvollziehbar ausgeführt, dass es nach Inkrafttreten des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 keine Zweifel gegeben habe, dass für die Zuordnung der Überhangmandate zu einer konkreten Landesliste das beschriebene Verfahren anzuwenden sei.</t>
+          <t>a) Die Regelung des § 362 Nr. 5 StPO erfasst auch Freisprüche, die bereits vor ihrem Inkrafttreten am 30. Dezember 2021 in Rechtskraft erwachsen sind. Eine andere Auslegung der ohne Übergangsbestimmungen erlassenen Norm kommt angesichts des deutlich erkennbaren Willens des Gesetzgebers nicht in Betracht. Gerade den streitgegenständlichen Fall und die vom Vater des Opfers mit initiierte Petition an den Deutschen Bundestag nimmt die Gesetzesbegründung ausdrücklich in Bezug (vgl. BTDrucks 19/30399, S. 10; siehe insoweit auch BVerfGE 162, 358 &lt;374 f. Rn. 56&gt;). Zudem sieht die Gesetzesbegründung insbesondere dann eine „unerträgliche“ Situation, deren Beseitigung das Gesetz bezweckt, wenn neue technische Ermittlungsmethoden die Überführung eines in der Vergangenheit Freigesprochenen ermöglichen würden (vgl. BTDrucks 19/30399, S. 2, 10). Insbesondere auf den Nachweis von DNA-Spuren weist der Gesetzentwurf hin (vgl. BTDrucks 19/30399, S. 1 f., 9 f.). Dies umfasst in erster Linie Verfahren, in denen der Freispruch zu einer Zeit erging, in der diese Analysemethoden noch nicht die heutige Qualität aufwiesen.</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
@@ -2814,14 +2814,14 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>d) Eine andere verfassungsrechtliche Bewertung folgt auch nicht daraus, dass wahlberechtigte Bürgerinnen und Bürger allein auf Grundlage des Gesetzestextes ohne Zuhilfenahme weiterer Informationsquellen nicht in der Lage sein dürften, die Regelungen der § 6 Abs. 5 und 6, § 48 BWahlG im Einzelnen zu erfassen.</t>
+          <t>b) Die Erstreckung auf Freisprüche, die bereits vor Inkrafttreten des § 362 Nr. 5 StPO rechtskräftig geworden sind, stellt eine „echte“ Rückwirkung im Sinne einer Rückbewirkung von Rechtsfolgen dar.</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
@@ -2830,14 +2830,14 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>aa) Besondere, über die Bestimmtheit der Norm hinausgehende Klarheitsanforderungen ergeben sich nicht aus ihrem Adressatenkreis. Die §§ 6, 48 BWahlG sind primär an die Wahlorgane als Rechtsanwender gerichtet, nicht hingegen unmittelbar an die wahlberechtigten Bürgerinnen und Bürger. Diesen wird durch die Vorschriften weder ein bestimmtes Verhalten abverlangt noch sind sie in sonstiger Weise belastenden Maßnahmen ausgesetzt. Vielmehr geben §§ 6, 48 BWahlG den Wahlorganen, die mit der Ermittlung und Feststellung des Wahlergebnisses betraut sind (§§ 37 ff. BWahlG, §§ 67 ff. BWO), vor, wie aufgrund der abgegebenen Stimmen zu berechnen ist, wie viele Sitze auf die einzelnen Landeslisten entfallen und welche Bewerberinnen und Bewerber gewählt sind. Eigenständige Regelungsspielräume verbleiben den Wahlorganen dabei nicht.</t>
+          <t>Das Prinzip der Rechtskraft dient gerade dazu, einer Entscheidung abschließenden Charakter zu verleihen und eine erneute Infragestellung zu verhindern. Insbesondere im Strafverfahren enthält ein Freispruch den abschließenden Aussagegehalt, dass sich der Tatverdacht, der dem Strafverfahren zugrunde lag, nicht bestätigt hat. Der geregelte Lebenssachverhalt, an den eine gesetzliche Neuregelung der Wiederaufnahme Rechtsfolgen knüpft, ist das Verfahren, nicht der zugrundeliegende, den Verfahrensgegenstand prägende tatsächliche Sachverhalt (vgl. BVerfGE 63, 343 &lt;360&gt;). Erfolgt die Wiederaufnahme aufgrund einer Norm, die erst nachträglich in Kraft tritt, ändert sie die Rechtsfolgen eines Freispruchs. Den zuvor bestehenden Vorbehalten, die in den bisherigen Wiederaufnahmegründen zum Ausdruck kommen, fügt die Neuregelung einen weiteren Vorbehalt hinzu (vgl. auch BVerfGE 2, 380 &lt;403&gt;; Kaspar, GA 2022, S. 21 &lt;34&gt;).</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
@@ -2846,14 +2846,14 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>bb) Das Gebot hinreichender Bestimmtheit und Klarheit der Gesetze verlangt darüber hinaus nur das Maß an Bestimmtheit und Klarheit, welches nach der Eigenart der zu ordnenden Lebenssachverhalte mit Rücksicht auf den Normzweck möglich ist (vgl. BVerfGE 49, 168 &lt;181&gt;; 59, 104 &lt;114&gt;; 78, 205 &lt;212&gt;; 103, 332 &lt;384&gt;; 134, 141 &lt;184 Rn. 126&gt;; 145, 20 &lt;69 f. Rn. 125&gt;; 149, 293 &lt;323 Rn. 77&gt;; stRspr). Deshalb ist es hinnehmbar, eine Norm zur Ergebnisermittlung so zu fassen, dass die damit betrauten Wahlorgane sie bei methodengerechter Auslegung ordnungsgemäß anwenden können, wahlberechtigte Bürgerinnen und Bürger sie aber in der Regel nicht allein aufgrund des Normtextes, sondern erst unter Zuhilfenahme weiterer Informationsquellen im Einzelnen erfassen können.</t>
+          <t>Zudem geht von dem Eintritt der Rechtskraft keine geringere Zäsurwirkung aus als von dem Eintritt der Verfolgungsverjährung. Bereits diese führt nach der Rechtsprechung des Bundesverfassungsgerichts zum Abschluss des betreffenden Vorgangs und begründet schutzwürdiges Vertrauen vor einer Strafverfolgung; rückwirkende Änderungen der Verjährungsvorschriften stellen daher eine „echte“ Rückwirkung dar (vgl. BVerfGE 156, 354 &lt;403 f. Rn. 135 f.&gt;; vgl. auch bereits BVerfGE 25, 269 &lt;286 ff.&gt;; 63, 343 &lt;359 f.&gt;). Dies gilt erst recht für den rechtskräftigen Abschluss eines Strafverfahrens.</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
@@ -2862,14 +2862,14 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>(1) Die Regelung des § 6 BWahlG, die das Sitzzuteilungsverfahren für die Wahl des Deutschen Bundestages betrifft, muss der Entscheidung des Gesetzgebers zum Wahlsystem Rechnung tragen. Gemäß § 1 Abs. 1 Satz 2 BWahlG hat der Gesetzgeber sich in verfassungskonformer Weise (vgl. BVerfGE 6, 84 &lt;90&gt;; 6, 104 &lt;111&gt;; 95, 335 &lt;349 f.&gt;; 121, 266 &lt;296&gt;) für eine mit der Personenwahl verbundene Verhältniswahl entschieden. In einem solchen Wahlsystem ist ein gewisses Maß an Komplexität des Sitzzuteilungsverfahrens nicht zu vermeiden (vgl. Lang, Wahlrecht und Bundesverfassungsgericht, 2014, S. 79). Hinzu kommt, dass der Gesetzgeber sich für einen Ausgleich von Überhangmandaten entschieden hat und deshalb die Sitzzahl des Deutschen Bundestages nicht als absolute Größe im Gesetz festgelegt ist. Vielmehr muss auch die Berechnung der Gesamtsitzzahl des Deutschen Bundestages gesetzlich beschrieben werden. Eine weitere Erhöhung der Komplexität ergibt sich aus der Entscheidung des Gesetzgebers, hierbei auch föderale Gesichtspunkte zu berücksichtigen, mithin die Berechnungsschritte sowohl auf Landes- als auch auf Bundesebene anzusiedeln. Die Entscheidung des Gesetzgebers, das Element der Personenwahl bei der Bundestagswahl zu stärken sowie die Vergrößerung des Bundestages zu begrenzen und dies nicht nur mithilfe eines, sondern zweier Instrumente zu bewirken, steigert die Komplexität erneut. Gleichwohl müssen die Vorschriften des Sitzzuteilungsverfahrens die Wahlorgane hinreichend bestimmt anleiten, was potenziell zulasten der Allgemeinverständlichkeit gehen kann (vgl. Lang, Wahlrecht und Bundesverfassungsgericht, 2014, S. 79; vgl. grundsätzlich zu diesem Zielkonflikt Towfigh, Der Staat 48 &lt;2009&gt;, S. 36 f., 71 f.).</t>
+          <t>c) Die mit der Neuregelung des § 362 Nr. 5 StPO einhergehende „echte“ Rückwirkung ist verfassungsrechtlich nicht ausnahmsweise zulässig. Die Voraussetzungen der in der Rechtsprechung des Bundesverfassungsgerichts anerkannten Ausnahmen liegen nicht vor. Freigesprochene dürfen auf die Rechtskraft des Urteils und die Begrenzung der Rechtskraftdurchbrechung nach alter Rechtslage vertrauen (aa). Auch zwingende Gründe des Gemeinwohls bestehen nicht; insbesondere sind die Maßgaben, die der Senat für die Beurteilung der rückwirkenden Regelung der Vermögensabschöpfung herangezogen hat (BVerfGE 156, 354), nicht auf die Einführung des neuen Wiederaufnahmegrundes zulasten des Angeklagten übertragbar (bb).</t>
         </is>
       </c>
       <c r="B153" t="inlineStr"/>
@@ -2878,14 +2878,14 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>(2) Das Gebot hinreichender Bestimmtheit und Klarheit der Gesetze führt nicht dazu, dass der Gesetzgeber in seinem Spielraum gemäß Art. 38 Abs. 3 GG zur Auswahl des Wahlsystems (vgl. BVerfGE 95, 335 &lt;349&gt;) eingeschränkt wäre. Es verpflichtet ihn nicht, das Bundestagswahlrecht in der Sache möglichst einfach zu konzipieren, um es im Gesetz dann auch einfach darstellen zu können. Insbesondere ist der Gesetzgeber unter dem Gesichtspunkt des Gebots der Bestimmtheit und Normenklarheit nicht daran gehindert, sich – wie geschehen – für ein personalisiertes Verhältniswahlrecht mit zwei Stimmen, für die grundsätzliche Verrechnung von Wahlkreismandaten mit den von der jeweiligen Partei gewonnenen Listenmandaten, für die Garantie des über die Erststimme gewonnenen Wahlkreismandats, für den grundsätzlichen Ausgleich nicht durch Listenmandate gedeckter Wahlkreismandate und für eine Begrenzung des Anwachsens des Bundestages mit den Mitteln dreier nicht ausgeglichener Überhangmandate sowie einer begrenzten länderübergreifenden Verrechnung von Direktmandaten zu entscheiden. Angesichts der hohen Komplexität des vom Gesetzgeber gemäß Art. 38 Abs. 3 GG festgelegten Wahlsystems sind die darauf bezogenen Vorschriften notwendigerweise kompliziert. Eine verfassungsrechtliche Anforderung, das bestimmte (vgl. Rn. 86 ff.) Sitzzuteilungsverfahren klarer zu fassen, könnte daher allein auf eine andere Formulierung, nicht aber – wie das Sondervotum meint (vgl. dort Rn. 20) – auf den Inhalt der Wahlrechtsregelung gerichtet sein. Auch wenn verständlichere Gesetzesfassungen uneingeschränkt wünschenswert sind, führt eine unzureichende Umsetzung dieses Anliegens nicht zu einem Verfassungsverstoß.</t>
+          <t>aa) Freigesprochene dürfen darauf vertrauen, dass die Rechtskraft des Freispruchs nur aufgrund der bisherigen Rechtslage durchbrochen werden kann. Der Grundsatz ne bis in idem erkennt die Schutzwürdigkeit des Vertrauens in ein freisprechendes Strafurteil an, und Art. 103 Abs. 3 GG verleiht diesem Vertrauensschutz Verfassungsrang.</t>
         </is>
       </c>
       <c r="B154" t="inlineStr"/>
@@ -2894,14 +2894,14 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>cc) Unabhängig davon ist (weiterhin) sichergestellt, dass sich die Wählerinnen und Wähler über die grundsätzlichen Wirkungen ihres Stimmverhaltens für die Sitzberechnung und die Zuteilung der Mandate verlässlich informieren können. Insofern genügen §§ 6, 48 BWahlG in der hier verfahrensgegenständlichen Fassung auch den Anforderungen des Demokratieprinzips, aus dem sich ergibt, dass die Wahl im demokratischen Verfassungsstaat in besonderer Weise die Aufgabe erfüllt, als Integrationsvorgang des Volkes zu wirken (vgl. BVerfGE 6, 84 &lt;92 f.&gt;; 71, 81 &lt;97&gt;; 95, 408 &lt;419&gt;). Diese Integrationsfunktion vermag der Wahlvorgang nur zu erfüllen, wenn für die Wählerinnen und Wähler in groben Zügen erkennbar und verständlich ist, wie die einzelne Wählerstimme in Mandate umgerechnet wird. Die Fassung der Norm gefährdet diese Integrationsfunktion der Wahl jedoch nicht.</t>
+          <t>§ 362 Nr. 5 StPO dient auch nicht dazu, rechtliche Zweifel zu klären. Im Gegenteil besteht über die Rechtskraft eines Freispruchs gerade im Fall neuer Tatsachen oder Beweismittel vollständige Klarheit. Auch die dem Gesetzgebungsverfahren vorangegangenen Reformbestrebungen legten dies als selbstverständlich zugrunde.</t>
         </is>
       </c>
       <c r="B155" t="inlineStr"/>
@@ -2910,14 +2910,14 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>(1) Der Wortlaut der §§ 6, 48 BWahlG mag zwar für interessierte Wählerinnen und Wähler nicht ohne Zuhilfenahme weiterer Informationsquellen klar verständlich sein. Jedoch enthält er keine den wahren Regelungsgehalt verschleiernde Formulierungen. Ihm lassen sich vielmehr durchaus wesentliche Informationen entnehmen, so etwa in § 6 Abs. 1 Satz 1 BWahlG (Verteilung der Sitze auf die Landeslisten nach Zweitstimmen), in § 6 Abs. 6 Satz 3 und 4 BWahlG (Verrechnung von Wahlkreismandaten mit Listenmandaten unter Garantie der Wahlkreismandate) und in § 6 Abs. 5 Satz 4 BWahlG (Hinnahme von bis zu drei nicht ausgeglichenen Überhangmandaten).</t>
+          <t>Die Unverjährbarkeit der von § 362 Nr. 5 StPO erfassten Delikte gebietet keine andere Bewertung. Gerade für unverjährbare Delikte kann erst ein Freispruch die weitere Strafverfolgung ausschließen. Er trifft, anders als das Institut der Verjährung (vgl. BVerfGE 25, 269 &lt;286 f.&gt;; 156, 354 &lt;413 Rn. 158 f.&gt;), eine ausdrückliche staatliche Entscheidung darüber, dass die Voraussetzungen für die Bestrafung eines bestimmten Verhaltens nicht erfüllt sind, und knüpft hieran den Ausschluss erneuter Strafverfolgung. Daher entfaltet ein Freispruch eine noch stärkere Zäsurwirkung als der Eintritt der Verfolgungsverjährung (vgl. Gerson, StV 2022, S. 124 &lt;128 f.&gt;).</t>
         </is>
       </c>
       <c r="B156" t="inlineStr"/>
@@ -2926,14 +2926,14 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>(2) In den Blick zu nehmen sind zudem Normumfeld, Regelungsgeschichte und Verfassungswirklichkeit.</t>
+          <t>Unerheblich ist, ob der Betroffene zum Zeitpunkt seines Freispruchs wusste, dass das Urteil materiell-rechtlich falsch war. In Fortsetzung des Grundsatzes in dubio pro reo schützen der Grundsatz ne bis in idem und Art. 103 Abs. 3 GG den Freigesprochenen gerade unabhängig von dessen materiell-rechtlicher Schuld (vgl. Kaspar, GA 2022, S. 21 &lt;35&gt;). Angesichts der Selbstbelastungsfreiheit und des Rechts auf Schweigen darf dem Freigesprochenen nicht nachträglich angelastet werden, dass er ein unrichtiges, aber für ihn günstiges Urteil nicht korrigiert.</t>
         </is>
       </c>
       <c r="B157" t="inlineStr"/>
@@ -2942,14 +2942,14 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Das Bundeswahlgesetz in der Fassung des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2022 benennt – etwa in § 1 („mit der Personenwahl verbundenen Verhältniswahl“) oder § 4 („zwei Stimmen“) – wesentliche Elemente des Wahlrechtssystems, die in das Verständnis der Sitzberechnung und Mandatszuteilung einfließen. Überdies wurde mit der Vorschrift des Art. 1 Nr. 3 bis 5 BWahlGÄndG nicht etwa ein neues Wahlsystem etabliert. Sie nimmt lediglich begrenzte Korrekturen und Modifikationen an dem in der Bundesrepublik Deutschland seit langem bestehenden System eines personalisierten Verhältniswahlrechts vor. Dabei hat sie das zuvor etablierte Verfahren der Ausgleichsmandate und der damit verbundenen Vergrößerung des Bundestages grundsätzlich beibehalten und nur modifizierend weiterentwickelt. Wählerinnen und Wähler können daher auf Erfahrungen und Praxis vorangehender Wahlen auch für das Verständnis der Neuregelung zurückgreifen. Außerdem wurde die verfahrensgegenständliche Änderung politisch kontrovers diskutiert. In diesem Kontext wurden ausführliche Modellrechnungen angestellt, die der Bundeswahlleiter öffentlich zugänglich gemacht hat. Mit ihnen ist die Sitzberechnung und Mandatszuteilung auch im Einzelnen nachvollziehbar. Entgegen der Auffassung des Sondervotums (vgl. dort Rn. 17) entstehen hierdurch keine Spielräume der Norminterpretation, da die gesetzlichen Vorgaben bestimmt sein müssen und bestimmt sind.</t>
+          <t>bb) Der Vertrauensschutz tritt hier auch nicht wegen zwingender Gründe des Gemeinwohls, die dem Prinzip der Rechtssicherheit vorgehen und eine rückwirkende Beseitigung erfordern, zurück.</t>
         </is>
       </c>
       <c r="B158" t="inlineStr"/>
@@ -2958,14 +2958,14 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Ein Verstoß gegen die Grundsätze der Gleichheit und der Unmittelbarkeit der Wahl sowie die Chancengleichheit der Parteien (1.) liegt nicht vor (2.).</t>
+          <t>Die vom Gesetzgeber mit der Regelung des § 362 Nr. 5 StPO insgesamt beabsichtigte Verwirklichung des Prinzips der materialen Gerechtigkeit verdrängt die zentrale Bedeutung der Rechtssicherheit für den Rechtsstaat nicht. Der Freispruch eines möglicherweise Schuldigen und der Fortbestand dieses Freispruchs trotz abnehmender Zweifel an der Schuld des Freigesprochenen sind unter dem Gesichtspunkt des Gemeinwohls nicht „unerträglich“, sondern vielmehr Folgen einer rechtsstaatlichen Strafrechtsordnung, in der der Zweifelsgrundsatz eine zentrale Rolle spielt.</t>
         </is>
       </c>
       <c r="B159" t="inlineStr"/>
@@ -2974,14 +2974,14 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>1. a) Gemäß Art. 38 Abs. 1 Satz 1 GG werden die Abgeordneten des Deutschen Bundestages in allgemeiner, unmittelbarer, freier, gleicher und geheimer Wahl gewählt. Der Grundsatz der Gleichheit der Wahl sichert dabei die vom Demokratieprinzip vorausgesetzte Egalität der Bürgerinnen und Bürger (vgl. BVerfGE 99, 1 &lt;13&gt;; 121, 266 &lt;295&gt;; 124, 1 &lt;18&gt;; 135, 259 &lt;284 Rn. 44&gt;; 146, 327 &lt;349 Rn. 59&gt;; stRspr). Als eine der wesentlichen Grundlagen der freiheitlich demokratischen Grundordnung im Sinne des Grundgesetzes (vgl. BVerfGE 6, 84 &lt;91&gt;; 11, 351 &lt;360&gt;; 121, 266 &lt;295&gt;; 124, 1 &lt;18&gt;; 135, 259 &lt;284 Rn. 44&gt;; 146, 327 &lt;349 Rn. 59&gt;; stRspr) gebietet er, dass alle Wahlberechtigten das aktive und passive Wahlrecht möglichst in formal gleicher Weise ausüben können, und ist daher im Sinne einer strengen und formalen Gleichheit zu verstehen (vgl. BVerfGE 51, 222 &lt;234&gt;; 78, 350 &lt;357 f.&gt;; 82, 322 &lt;337&gt;; 121, 266 &lt;295&gt;; 135, 259 &lt;284 Rn. 44&gt;; 146, 327 &lt;349 f. Rn. 59&gt;; stRspr).</t>
+          <t>Die Maßstäbe der Entscheidung des Senats zur rückwirkenden Vermögensabschöpfung (BVerfGE 156, 354) können nicht auf die vorliegende Konstellation übertragen werden. Den zwingenden Gemeinwohlgrund, der eine „echte“ Rückwirkung rechtfertigen kann, sah der Senat dort in der Situation, dass der Staat mit der Verfolgungsverjährung darauf verzichtet, gegen den Straftäter mit den Mitteln des Strafrechts vorzugehen. Dies könne den für die Rechtstreue der Bevölkerung abträglichen Eindruck eines erheblichen Vollzugsdefizits begründen. Die Vermögensabschöpfung führe „in normbekräftigender Weise sowohl dem Straftäter als auch der Rechtsgemeinschaft vor Augen […], dass eine strafrechtswidrige Vermögensmehrung von der Rechtsordnung nicht anerkannt wird und deshalb keinen Bestand haben kann“ (BVerfGE 156, 354 &lt;410 Rn. 151&gt;). Raum für diese Ausnahme vom Rückwirkungsverbot eröffne erst der Umstand, dass die Vermögensabschöpfung keine dem Schuldgrundsatz unterliegende Nebenstrafe darstelle, sondern eine Maßnahme eigener Art mit kondiktionsähnlichem, präventiv-ordnendem Charakter. In diesem Fall stehe die Vertrauensschutzposition der Betroffenen zurück, weil sich die Bewertung eines bestimmten Verhaltens als Straftat durch den Eintritt der Verfolgungsverjährung nicht ändere und daher das Vertrauen in den Fortbestand unredlich erworbener Rechte grundsätzlich nicht schutzwürdig sei (vgl. BVerfGE 156, 354 &lt;411 ff. Rn. 152, 155, 157, 161&gt;).</t>
         </is>
       </c>
       <c r="B160" t="inlineStr"/>
@@ -2990,14 +2990,14 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Aus dem Grundsatz der Wahlgleichheit folgt für das Wahlgesetz, dass die Stimme eines jeden Wahlberechtigten grundsätzlich den gleichen Zählwert und die gleiche rechtliche Erfolgschance haben muss. Alle Wählerinnen und Wähler sollen mit der Stimme, die sie abgeben, den gleichen Einfluss auf das Wahlergebnis nehmen können (vgl. BVerfGE 95, 335 &lt;353, 369 f.&gt;; 121, 266 &lt;295&gt;; 124, 1 &lt;18&gt;; 129, 300 &lt;317 f.&gt;; 131, 316 &lt;337&gt;; 146, 327 &lt;350 Rn. 59&gt;; stRspr). Bei der Verhältniswahl verlangt der Grundsatz der Wahlgleichheit darüber hinaus, dass jeder Wähler mit seiner Stimme auch den gleichen Einfluss auf die Zusammensetzung der zu wählenden Volksvertretung haben muss (vgl. BVerfGE 16, 130 &lt;139&gt;; 95, 335 &lt;353, 372&gt;; 131, 316 &lt;338&gt;; 146, 327 &lt;350 Rn. 59&gt;; stRspr). Ziel des Verhältniswahlsystems ist es, dass alle Parteien in einem möglichst den Stimmenzahlen angenäherten Verhältnis in dem zu wählenden Organ vertreten sind. Zur Zählwert- und Erfolgschancengleichheit tritt im Verhältniswahlrecht die Erfolgswertgleichheit hinzu, die verlangt, dass jede gültige Stimme mit gleichem Gewicht bewertet wird, ihr mithin ein anteilsmäßig gleicher Erfolg zukommt (vgl. BVerfGE 120, 82 &lt;103&gt;; 129, 300 &lt;318&gt;; 131, 316 &lt;337 f.&gt;; 135, 259 &lt;284 Rn. 45&gt;; 146, 327 &lt;350 Rn. 59&gt;; stRspr).</t>
+          <t>Die Wiederaufnahme eines bereits mit Urteil abgeschlossenen Strafverfahrens unterscheidet sich hiervon grundlegend. Sie ist auf eine dem Schuldgrundsatz unterliegende Strafe gerichtet. Das Vertrauen gründet hier nicht in dem Eintritt der Verjährung, sondern in einem rechtskräftigen Urteil. Im Fall eines Freispruchs ist dies gerade nicht mit einem Unwerturteil verbunden, vielmehr ist das Vertrauen verfassungsrechtlich geschützt. Die Wiederaufnahme ist auf eine erneute Strafverfolgung gerichtet und stützt sich auf einen Verdacht, nicht aber auf die Feststellung einer rechtswidrigen Tat (vgl. § 73a StGB). Es lässt sich auch nicht feststellen, dass es zur gesellschaftlichen Normstabilisierung der Rückwirkung des § 362 Nr. 5 StPO bedarf. Insbesondere ist nicht zu erkennen, wie der Fortbestand eines Freispruchs, dem stets eine Hauptverhandlung vorausgegangen ist, den Eindruck eines Vollzugsdefizits erwecken könnte.</t>
         </is>
       </c>
       <c r="B161" t="inlineStr"/>
@@ -3006,14 +3006,14 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Die Erfolgswertgleichheit der Wählerstimmen bei der Verhältniswahl verlangt nicht, dass sich – bei einer ex-post-Betrachtung – ergibt, dass jede Wählerin und jeder Wähler zu exakt gleichen Teilen zur Sitzzuteilung beigetragen hat. Die Ermittlung des Anteils, den eine Stimme an den Gesamtstimmen hat, und die verhältnismäßige Verteilung der zur Verfügung stehenden Sitze erfordern ein mathematisches Verfahren, das in keinem Fall zu dem Ergebnis führen kann, dass die vorhandenen Sitze genau dem ermittelten verhältnismäßigen Anteil jeder einzelnen Wählerstimme entsprechend verteilt sind. Soweit dieser Anteil sich nur als Bruchteil einer ganzen Zahl darstellt, kann er schon deshalb nicht auf die Sitzvergabe übertragen werden, weil es Bruchteile von Sitzen nicht gibt.</t>
+          <t>Gemäß § 95 Abs. 3 BVerfGG ist § 362 Nr. 5 StPO für nichtig zu erklären.</t>
         </is>
       </c>
       <c r="B162" t="inlineStr"/>
@@ -3022,14 +3022,14 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>b) Der Grundsatz der Unmittelbarkeit der Wahl fordert, dass die Wählerinnen und Wähler die Abgeordneten selbst auswählen. Er schließt jedes Wahlverfahren aus, bei dem zu den Wählerinnen und Wählern eine weitere Instanz hinzutritt, die nach ihrem eigenen Ermessen die Abgeordneten endgültig auswählt und damit deren direkte Wahl ausschließt (vgl. BVerfGE 7, 63 &lt;68&gt;; 7, 77 &lt;84 f.&gt;; 47, 253 &lt;279 f.&gt;). Der Grundsatz der Unmittelbarkeit der Wahl setzt demgemäß ein Wahlverfahren voraus, in dem die Wählerinnen und Wähler vor dem Wahlakt erkennen können, welche Personen sich um ein Abgeordnetenmandat bewerben und wie sich die eigene Stimmabgabe auf Erfolg oder Misserfolg der Wahlbewerber auswirkt (vgl. BVerfGE 47, 253 &lt;279 ff.&gt;; 95, 335 &lt;350&gt;; 97, 317 &lt;326&gt;; 121, 266 &lt;307&gt;). Für den Grundsatz der Unmittelbarkeit ist nicht entscheidend, dass die Stimme tatsächlich die von den Wählerinnen und Wählern beabsichtigte Wirkung entfaltet. Ausreichend ist die Möglichkeit einer der Intention des jeweiligen Wählers entsprechenden positiven Beeinflussung des Wahlergebnisses (vgl. BVerfGE 121, 266 &lt;307&gt;).</t>
+          <t>Die auf dieser Vorschrift beruhenden Beschlüsse des Oberlandesgerichts und des Landgerichts sind nach § 95 Abs. 2 BVerfGG aufzuheben, und die Sache ist an das Landgericht zurückzuverweisen.</t>
         </is>
       </c>
       <c r="B163" t="inlineStr"/>
@@ -3038,14 +3038,14 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>c) Um die verfassungsrechtlich gebotene Offenheit des Prozesses der politischen Willensbildung zu gewährleisten, ist es unerlässlich, dass die Parteien, soweit irgend möglich, gleichberechtigt am politischen Wettbewerb teilnehmen. Von dieser Einsicht her empfängt der aus Art. 21 Abs. 1 GG abzuleitende Verfassungsgrundsatz der gleichen Wettbewerbschancen der politischen Parteien das ihm eigene Gepräge (vgl. BVerfGE 148, 11 &lt;24 Rn. 42&gt;). Er beinhaltet, dass jeder Partei grundsätzlich die gleichen Möglichkeiten im gesamten Wahlverfahren und damit gleiche Chancen bei der Verteilung der Sitze eingeräumt werden müssen. Das Recht der politischen Parteien auf Chancengleichheit hängt eng mit den Grundsätzen der Allgemeinheit und Gleichheit der Wahl zusammen. Deshalb muss in diesem Bereich – ebenso wie bei der durch die Grundsätze der Allgemeinheit und Gleichheit der Wahl verbürgten gleichen Behandlung der Wählerinnen und Wähler – Gleichheit in einem strikten und formalen Sinn verstanden werden. Wenn die öffentliche Gewalt in den Parteienwettbewerb in einer Weise eingreift, die auf die Chancen der Parteien im politischen Wettbewerb zurückwirkt, sind ihrem Ermessen besonders enge Grenzen gesetzt (vgl. BVerfGE 120, 82 &lt;104 f.&gt;; 129, 300 &lt;319&gt;; 135, 259 &lt;285 Rn. 48&gt;; 146, 327 &lt;350 Rn. 60&gt;).</t>
+          <t>Die Entscheidung über die Auslagenerstattung der kostenrechtlich eigenständigen Verfahren über die Verfassungsbeschwerde sowie den Antrag auf Erlass einer einstweiligen Anordnung (vgl. BVerfGE 89, 91; 141, 56 &lt;81 Rn. 65&gt;) beruht auf § 34a Abs. 2 und 3 BVerfGG. Die Auslagen sind dem Beschwerdeführer zu gleichen Teilen von dem Land Niedersachsen und der Bundesrepublik Deutschland zu erstatten, weil die aufgehobenen Entscheidungen von Gerichten des Landes Niedersachsen getroffen worden sind, der Grund der Aufhebung aber in der Verfassungswidrigkeit einer bundesrechtlichen Vorschrift liegt (vgl. BVerfGE 101, 106 &lt;132&gt;; 131, 239 &lt;267&gt;).</t>
         </is>
       </c>
       <c r="B164" t="inlineStr"/>
@@ -3054,14 +3054,14 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>d) Die Grundsätze der Wahlgleichheit und der Chancengleichheit der Parteien unterliegen keinem absoluten Differenzierungsverbot. Allerdings folgt aus ihrem formalen Charakter, dass dem Gesetzgeber bei der Ordnung des Wahlrechts nur ein eng bemessener Spielraum für Differenzierungen verbleibt. Diese bedürfen zu ihrer Rechtfertigung stets eines besonderen, sachlich legitimierten Grundes. Das bedeutet nicht, dass sich die Differenzierung als von Verfassungs wegen notwendig darstellen muss. Differenzierungen im Wahlrecht können aber nur durch Gründe gerechtfertigt werden, die durch die Verfassung legitimiert und von einem Gewicht sind, das der Wahlgleichheit die Waage halten kann (vgl. BVerfGE 120, 82 &lt;106 f.&gt;; 121, 266 &lt;297&gt;; 129, 300 &lt;320&gt;; 130, 212 &lt;227 f.&gt;; 135, 259 &lt;286 Rn. 51&gt;; 146, 327 &lt;351 Rn. 61&gt;; 162, 207 &lt;238 Rn. 92&gt; – Äußerungsbefugnisse der Bundeskanzlerin; jeweils m.w.N.).</t>
+          <t>Die Entscheidung ist zu C. I. mit 6 : 2 Stimmen, im Übrigen einstimmig ergangen.</t>
         </is>
       </c>
       <c r="B165" t="inlineStr"/>
@@ -3070,1207 +3070,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>Hierzu zählen Gründe, die sich aus der Natur der Wahl einer Volksvertretung ergeben, insbesondere die mit der Wahl verfolgten Ziele. Solche stellen die Sicherung des Charakters der Wahl als eines Integrationsvorgangs bei der politischen Willensbildung des Volkes und die Sicherung der Funktionsfähigkeit der zu wählenden Volksvertretung dar (vgl. BVerfGE 95, 408 &lt;418&gt;; 120, 82 &lt;107&gt;; 121, 266 &lt;297 f.&gt;; 129, 300 &lt;320 f.&gt;; 135, 259 &lt;286 Rn. 52&gt;; 146, 327 &lt;351 Rn. 62&gt;; jeweils m.w.N.). Auch die verfassungslegitime Zielsetzung der personalisierten Verhältniswahl, die darauf abzielt, dem Wähler im Rahmen einer Verhältniswahl die Wahl von Persönlichkeiten zu ermöglichen, stellt einen Grund dar, der zur Rechtfertigung von Eingriffen in die Gleichheit der Wahl und die Chancengleichheit der Parteien in Betracht kommt (vgl. BVerfGE 7, 63 &lt;74 f.&gt;; 16, 130 &lt;140&gt;; 95, 335 &lt;358 ff.&gt;; 131, 316 &lt;363, 365 ff.&gt;).</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr"/>
-      <c r="C166" t="n">
-        <v>165</v>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>Es ist grundsätzlich Aufgabe des Gesetzgebers, die verfolgten Zwecke mit dem Gebot der Wahlgleichheit und der Chancengleichheit der Parteien zum Ausgleich zu bringen. Das Bundesverfassungsgericht prüft lediglich, ob die verfassungsrechtlichen Grenzen eingehalten sind, nicht aber, ob der Gesetzgeber zweckmäßige oder rechtspolitisch erwünschte Lösungen gefunden hat (vgl. BVerfGE 51, 222 &lt;237 f.&gt;; 95, 408 &lt;420&gt;; 121, 266 &lt;303 f.&gt;; 131, 316 &lt;338 f.&gt;; 146, 327 &lt;352 Rn. 63&gt;). Es kann, sofern die differenzierende Regelung an einem Ziel orientiert ist, das der Gesetzgeber bei der Ausgestaltung des Wahlrechts verfolgen darf, einen Verstoß gegen den Grundsatz der Gleichheit der Wahl oder der Chancengleichheit der Parteien nur feststellen, wenn die Regelung zur Erreichung dieses Ziels nicht geeignet ist oder das Maß des zur Erreichung dieses Ziels Erforderlichen überschreitet (vgl. BVerfGE 6, 84 &lt;94&gt;; 51, 222 &lt;238&gt;; 95, 408 &lt;420&gt;; 120, 82 &lt;107&gt;; 121, 266 &lt;304&gt;; 129, 300 &lt;321&gt;; 131, 316 &lt;339&gt;; 135, 259 &lt;287 Rn. 53&gt;; 146, 327 &lt;352 f. Rn. 64&gt;; 162, 207 &lt;238 Rn. 92&gt;).</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr"/>
-      <c r="C167" t="n">
-        <v>166</v>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>e) Dies ändert nichts daran, dass dem Gesetzgeber für Differenzierungen im Rahmen der Wahlgleichheit nur ein eng bemessener Spielraum verbleibt (vgl. BVerfGE 95, 408 &lt;418&gt;; 129, 300 &lt;322&gt;; 135, 259 &lt;289 Rn. 57&gt;; 146, 327 &lt;352 Rn. 63&gt;). Da gerade bei der Wahlgesetzgebung die Gefahr besteht, dass die jeweilige Parlamentsmehrheit sich statt von gemeinwohlbezogenen Erwägungen von dem Ziel des eigenen Mandatserhalts leiten lässt, unterliegt die Ausgestaltung des Wahlrechts hinsichtlich der Beachtung der verfassungsrechtlichen Vorgaben strikter verfassungsgerichtlicher Kontrolle (vgl. BVerfGE 120, 22 &lt;105&gt;; 129, 300 &lt;322 f.&gt;; 130, 212 &lt;229&gt;; 135, 259 &lt;287&gt;). Das Gericht prüft daher in vollem Umfang, ob eine Regelung, die in die Wahlgleichheit und die Chancengleichheit der Parteien eingreift, durch einen Grund gerechtfertigt ist, der von der Verfassung legitimiert und von einem Gewicht ist, das den genannten Grundsätzen die Waage halten kann, sowie ob die getroffene Regelung zur Erreichung des angestrebten Ziels geeignet und erforderlich ist.</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr"/>
-      <c r="C168" t="n">
-        <v>167</v>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>2. Nach diesen Maßstäben verstößt das durch das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 modifizierte Sitzzuteilungsverfahren nicht gegen die Grundsätze der Gleichheit und der Unmittelbarkeit der Wahl sowie der Chancengleichheit der Parteien. Dies gilt, soweit es das Anfallen von Überhangmandaten ohne Ausgleich zulässt (a), ebenso wie mit Blick darauf, dass es eine teilweise Verrechnung von Direktmandaten, die eine Partei in einem Land errungen hat, mit Listenmandaten derselben Partei in einem anderen Land erlaubt (b). Verfassungsrechtlich relevante Effekte des negativen Stimmgewichts sind mit dem zur Überprüfung gestellten Sitzzuteilungsverfahren nicht verbunden (c).</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr"/>
-      <c r="C169" t="n">
-        <v>168</v>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>a) Das Bundesverfassungsgericht geht in ständiger Rechtsprechung davon aus, dass die Bundestagswahl unbeschadet der Direktwahl der Wahlkreiskandidaten den Grundcharakter einer Verhältniswahl trägt (vgl. BVerfGE 6, 84 &lt;90&gt;; 16, 130 &lt;139&gt;; 95, 335 &lt;357 f.&gt;; 121, 266 &lt;297&gt;; 131, 316 &lt;359&gt;). Daran ist auch mit Blick auf die Neuregelung der Sitzverteilung durch das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 festzuhalten. Der gemäß § 6 Abs. 5 und 6 BWahlG durchzuführende Verhältnisausgleich unterliegt daher uneingeschränkt den allgemeinen Anforderungen an Durchbrechungen des Gebots der Erfolgswertgleichheit im Verhältniswahlrecht (vgl. BVerfGE 1, 208 &lt;246 f.&gt;; 6, 84 &lt;90&gt;; 95, 335 &lt;386&gt;; 131, 316 &lt;361&gt;). Indem § 6 Abs. 6 Satz 3 BWahlG die Zuteilung von bis zu drei Überhangmandaten ohne Ausgleich erlaubt, werden Wählerstimmen im Sitzzuteilungsverfahren ungleich behandelt und es wird in die Wahlgleichheit sowie die Chancengleichheit der Parteien eingegriffen (aa). Dies ist durch die verfassungslegitime Zielsetzung der personalisierten Verhältniswahl, den Wählerinnen und Wählern im Rahmen einer Verhältniswahl die Wahl von Persönlichkeiten zu ermöglichen, jedoch gerechtfertigt (bb).</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr"/>
-      <c r="C170" t="n">
-        <v>169</v>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>aa) (1) Mit dem Anfall von Überhangmandaten erhalten die abgegebenen Stimmen einen unterschiedlichen Erfolgswert. Aufgrund des durch die Anrechnung der Wahlkreismandate auf die Listenmandate einer Partei herbeigeführten Verhältnisausgleichs kann grundsätzlich jeder Wähler nur einmal (mit seiner Zweitstimme) Einfluss auf die proportionale Zusammensetzung des Parlaments nehmen. Die Erststimme bleibt demgegenüber grundsätzlich ohne Auswirkung auf die Verteilung der Mandate auf die politischen Parteien (vgl. BVerfGE 79, 161 &lt;167&gt;; 131, 316 &lt;362&gt;). Fällt jedoch ein Überhang an, so tragen Wählerinnen und Wähler mit ihrer Erststimme zum Gewinn von Wahlkreismandaten bei, die nicht mehr mit Listenmandaten verrechnet werden können und die deshalb den auf der Grundlage des Zweitstimmenergebnisses ermittelten Proporz durchbrechen. Damit gewinnt neben der Zweitstimme auch die Erststimme Einfluss auf die politische Zusammensetzung des Bundestages. Da diese Wirkung nur bei denjenigen Wählerinnen und Wählern eintritt, die ihre Erststimme einem erfolgreichen Wahlkreisbewerber gegeben haben, dessen Partei in dem betreffenden Land einen Überhang erzielt, ist die Erfolgswertgleichheit beeinträchtigt. Zwar hat jeder Wähler gleichermaßen die Chance, zur Gruppe derjenigen zu gehören, deren Stimmen stärkeren Einfluss auf die politische Zusammensetzung des Parlaments nehmen. Jedoch ist – schon ex ante betrachtet – gerade nicht gewährleistet, dass alle Wählerinnen und Wähler durch ihre Stimmabgabe gleichen Einfluss auf die Sitzverteilung nehmen können (vgl. BVerfGE 131, 316 &lt;362 f.&gt;). Unausgeglichene Überhangmandate stellen daher einen Eingriff in den Grundsatz der Gleichheit der Wahl gemäß Art. 38 Abs. 1 Satz 1 GG dar.</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr"/>
-      <c r="C171" t="n">
-        <v>170</v>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>(2) Auch die Chancengleichheit der politischen Parteien aus Art. 21 Abs. 1 GG wird durch Überhangmandate beeinträchtigt. Sie ist nur gewahrt, wenn jede Partei, ungeachtet der den mit einem Sitzzuteilungsverfahren nach dem Verteilungsprinzip der Verhältniswahl unausweichlich verbundenen Rundungsabweichungen, annähernd dieselbe Stimmenzahl benötigt, um ein Mandat zu erringen. Bei einer Partei, die einen Überhang erzielt, entfallen jedoch auf jeden ihrer Sitze weniger Zweitstimmen als bei einer Partei, der dies nicht gelingt (vgl. BVerfGE 131, 316 &lt;363&gt; m.w.N.).</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr"/>
-      <c r="C172" t="n">
-        <v>171</v>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>(3) Die unterschiedliche Behandlung der Wählerstimmen in Fällen fehlender Anrechenbarkeit auf erlangte Listenmandate schlägt sich nach Maßgabe des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 in der Zusammensetzung des Parlaments nieder, weil ein vollständiger Ausgleich oder eine vollständige Verrechnung der überhängenden Mandate nicht mehr stattfindet. Im Rahmen der Erhöhung der Sitzzahl des Deutschen Bundestages gemäß § 6 Abs. 5 BWahlG bleiben in den Wahlkreisen errungene Sitze, die nicht nach § 6 Abs. 4 Satz 1 BWahlG von der Zahl der für die Landesliste ermittelten Sitze abgerechnet werden können, bis zu einer Zahl von drei unberücksichtigt (§ 6 Abs. 5 Satz 4 BWahlG). In der Folge kann es dazu kommen, dass bis zu drei Wahlkreismandate nicht gemäß § 6 Abs. 6 Satz 3 BWahlG auf die für die jeweilige Landesliste derselben Partei ermittelte Sitzzahl angerechnet werden können. Das Gesetz bestimmt für diesen Fall, dass die Direktmandate der Partei verbleiben und sich die Gesamtzahl der Parlamentssitze um die Unterschiedszahl erhöht, ohne dass der Proporz wiederhergestellt wird (§ 6 Abs. 6 Satz 5 BWahlG).</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr"/>
-      <c r="C173" t="n">
-        <v>172</v>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>bb) Der mit der gesetzlich vorgesehenen Zuteilung von bis zu drei Überhangmandaten verbundene Eingriff in die Wahlgleichheit und die Chancengleichheit der Parteien ist mit Blick auf die in der Entscheidung des Bundesverfassungsgerichts vom 25. Juli 2012 (BVerfGE 131, 316) entwickelten Maßstäbe (1) gerechtfertigt (2).</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr"/>
-      <c r="C174" t="n">
-        <v>173</v>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>(1) Die mit der ausgleichslosen Zuteilung von Überhangmandaten verbundene Differenzierung des Erfolgswertes der Wählerstimmen kann verfassungsrechtlich in begrenztem Umfang durch das besondere Anliegen einer mit der Personenwahl verbundenen Verhältniswahl gerechtfertigt sein (vgl. BVerfGE 131, 316 &lt;365 ff.&gt;). Dies hat das Bundesverfassungsgericht bereits vor Einführung der Ausgleichsmandate festgestellt.</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr"/>
-      <c r="C175" t="n">
-        <v>174</v>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>(a) Danach ist die Zielsetzung der personalisierten Verhältniswahl, die darin besteht, den Wählerinnen und Wählern die Möglichkeit zu geben, auch im Rahmen der Verhältniswahl Persönlichkeiten zu wählen, von der Verfassung gedeckt (vgl. BVerfGE 131, 316 &lt;365&gt;). Auf diese Weise möchte der Gesetzgeber die Verbindung zwischen den Wählerinnen und Wählern und den Abgeordneten stärken und zugleich in gewissem Umfang der dominierenden Stellung der Parteien bei der politischen Willensbildung des Volkes (Art. 21 Abs. 1 Satz 1 GG) ein Korrektiv im Sinne der Unabhängigkeit der Abgeordneten (Art. 38 Abs. 1 Satz 2 GG) entgegensetzen. Durch die Wahl der Wahlkreiskandidaten soll annähernd die Hälfte der Abgeordneten in einer engeren persönlichen Beziehung zu ihrem Wahlkreis stehen (vgl. BVerfGE 7, 63 &lt;74&gt;; 16, 130 &lt;140&gt;; 41, 399 &lt;423&gt;; 95, 335 &lt;352, 358, 360&gt;; 131, 316 &lt;365 f.&gt;). Dieses Ziel kann nur verwirklicht werden, wenn der erfolgreiche Kandidat sein Wahlkreismandat auch dann erhält, wenn das nach dem Proporz ermittelte Sitzkontingent der Landesliste seiner Partei zur Verrechnung nicht ausreicht (vgl. BVerfGE 95, 335 &lt;394&gt;; 131, 316 &lt;366&gt;).</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr"/>
-      <c r="C176" t="n">
-        <v>175</v>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>Dieses Anliegen ist hinreichend gewichtig, um die ausgleichslose Zuteilung von Überhangmandaten in begrenztem Umfang zu rechtfertigen (vgl. BVerfGE 7, 63 &lt;74 f.&gt;; 16, 130 &lt;140&gt;; 95, 335 &lt;360&gt;; 131, 316 &lt;366&gt;). Der Gesetzgeber hat sich für ein Wahlsystem entschieden, das sowohl dem Anliegen einer Personenwahl als auch dem Ziel der Verhältniswahl, alle Parteien in einem möglichst den Stimmenzahlen angenäherten Verhältnis im Parlament abzubilden, Rechnung tragen will. Beide von der Verfassung legitimierten Ziele lassen sich innerhalb dieses Wahlsystems nicht in voller Reinheit verwirklichen. So trifft es zwar zu, dass die durch den Anfall von Überhangmandaten bewirkte Differenzierung des Erfolgswertes der Wählerstimmen mit einer personalisierten Verhältniswahl nicht zwangsläufig verbunden ist, weil der als Ergebnis des unvollständig durchgeführten Verhältnisausgleichs gestörte Proporz etwa durch Zuteilung von Ausgleichsmandaten wiederhergestellt werden könnte (vgl. BVerfGE 95, 335 &lt;394 f.&gt;; 131, 316 &lt;366&gt;). Allerdings erforderte eine vollständige Verwirklichung des Ziels der Verhältniswahl eine im Einzelnen nicht vorhersehbare Erhöhung der Sitzzahl des Bundestages. Dies stünde im Widerspruch zu der Zielsetzung, die Abgeordneten des Deutschen Bundestages annähernd zur Hälfte personenbezogen zu legitimieren. Zugleich wären Beeinträchtigungen des föderalen Proporzes zu erwarten. Das Anliegen der Personenwahl und das mit der Verhältniswahl verfolgte Ziel weitgehender Proportionalität stehen mithin in einem Spannungsverhältnis, das sich nur durch einen vom Gesetzgeber vorzunehmenden Ausgleich beider Prinzipien auflösen lässt. Im Rahmen des ihm insoweit zukommenden Gestaltungsspielraums darf der Gesetzgeber das Anliegen einer proportionalen Verteilung der Gesamtzahl der Sitze grundsätzlich zurückstellen und Überhangmandate ohne Wiederherstellung des Proporzes zulassen (vgl. BVerfGE 131, 316 &lt;366 f.&gt;).</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr"/>
-      <c r="C177" t="n">
-        <v>176</v>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>(b) Das Ausmaß der mit der ausgleichslosen Zuteilung von Überhangmandaten verbundenen Differenzierung des Erfolgswertes der Wählerstimmen muss sich jedoch innerhalb des gesetzgeberischen Konzepts einer personalisierten Verhältniswahl halten (vgl. BVerfGE 95, 408 &lt;421&gt;; 131, 316 &lt;367&gt;). Die Zuteilung zusätzlicher Bundestagssitze außerhalb des Proporzes darf nicht dazu führen, dass der Grundcharakter der Wahl als einer am Ergebnis der für die Parteien abgegebenen Stimmen orientierten Verhältniswahl aufgehoben wird (vgl. BVerfGE 95, 335 &lt;361, 365 f.&gt;; 131, 316 &lt;367&gt;). Es ist in erster Linie Aufgabe des Gesetzgebers, die Zahl hinnehmbarer Überhangmandate festzulegen (vgl. BVerfGE 131, 316 &lt;367&gt;). Dabei hat er jedoch zu beachten, dass Überhangmandate nur in eng begrenztem Umfang mit dem Charakter der Wahl als Verhältniswahl vereinbar sind. Fallen sie regelmäßig in größerer Zahl an, widerspricht dies der Grundentscheidung des Gesetzgebers für die personalisierte Verhältniswahl (vgl. BVerfGE 95, 335 &lt;365 f.&gt;; 131, 316 &lt;368&gt;). Der Zweite Senat des Bundesverfassungsgerichts hat einen angemessenen Ausgleich zwischen dem Anliegen möglichst proportionaler Abbildung des Zweitstimmenergebnisses im Deutschen Bundestag und dem mit der Personenwahl verbundenen Belang uneingeschränkten Erhalts von Wahlkreismandaten dann nicht mehr als gewahrt angesehen, wenn die Zahl der Überhangmandate etwa die Hälfte der für die Bildung einer Fraktion erforderlichen Zahl überschreitet (vgl. BVerfGE 131, 316 &lt;368 ff.&gt;).</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr"/>
-      <c r="C178" t="n">
-        <v>177</v>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>(2) Nach diesen Maßstäben, an denen der Senat festhält, ist die durch die Zuteilung von bis zu drei unausgeglichenen Überhangmandaten bewirkte Beeinträchtigung der Wahlgleichheit und der Chancengleichheit der Parteien durch das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 gerechtfertigt. Mit der Neuregelung des Sitzzuteilungsverfahrens verfolgt der Gesetzgeber das verfassungslegitime Ziel einer Stärkung des Elements der Personenwahl (a). Die Zulassung von bis zu drei Überhangmandaten ist zudem geeignet und erforderlich, dieses Ziel zu erreichen, insbesondere können Überhangmandate nicht in einem Umfang anfallen, der den Grundcharakter der Wahl als Verhältniswahl aufhebt (b). Auch darf der Gesetzgeber den Anfall von bis zu drei Überhangmandaten ohne Ausgleich bewusst in Kauf nehmen (c).</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr"/>
-      <c r="C179" t="n">
-        <v>178</v>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>(a) Mit der Zulassung von bis zu drei Überhangmandaten strebt der Gesetzgeber weiterhin das verfassungslegitime Ziel an, das Element der Personenwahl bei der Wahl zum Deutschen Bundestag zu stärken (aa). Vor diesem Hintergrund kann dahinstehen, ob Befürchtungen, der Deutsche Bundestag könne infolge einer weiteren Vergrößerung die Grenzen seiner Arbeits- und Handlungsfähigkeit erreichen (vgl. BTDrucks 19/22504, S. 1, 5), eigenständig die durch die Zulassung von Überhangmandaten bewirkten Gleichheitsbeeinträchtigungen rechtfertigen können (bb).</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr"/>
-      <c r="C180" t="n">
-        <v>179</v>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>(aa) § 6 BWahlG in der Fassung des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 dient unverändert der Umsetzung der Grundentscheidung des Gesetzgebers für eine mit der Personenwahl verbundene Verhältniswahl (§ 1 Abs. 1 Satz 2 BWahlG), da die Sitze auf die Parteien und in den Parteien auf die Landeslisten grundsätzlich nach dem Zweitstimmenergebnis verteilt werden (§ 6 Abs. 6 Satz 1 und 2 Halbsatz 1 BWahlG). Das Element der Personenwahl findet darin Ausdruck, dass 299 Abgeordnete und somit die Hälfte der Ausgangsgröße von 598 Abgeordneten (§ 1 Abs. 1 Satz 1 BWahlG) mit der Erststimme auf der Grundlage von Kreiswahlvorschlägen nach den Grundsätzen der Mehrheitswahl gewählt werden (§ 1 Abs. 2, § 4 Halbsatz 1, § 5 BWahlG; vgl. dazu BVerfGE 131, 316 &lt;357&gt;). Die Zuteilung dieser Mandate wird durch § 6 Abs. 4 Satz 2, § 6 Abs. 6 Satz 2 Halbsatz 2 in Verbindung mit § 6 Abs. 5 Satz 2 sowie § 6 Abs. 6 Satz 4 BWahlG garantiert. Um eine übermäßige Proporzverzerrung durch den Anfall von Überhangmandaten zu verhindern und den verfassungsrechtlichen Anforderungen der Erfolgswertgleichheit möglichst Rechnung zu tragen, sieht § 6 Abs. 5 BWahlG eine die Überhänge ausgleichende Erhöhung der Sitzzahl des Deutschen Bundestages vor. Dabei findet im Unterschied zum Bundeswahlgesetz 2013 jedoch kein vollständiger Ausgleich der rechnerisch anfallenden Überhangmandate mehr statt. Vielmehr werden gemäß § 6 Abs. 5 Satz 4 BWahlG bis zu drei der Quasi-Überhangmandate aus der ersten Verteilung nicht ausgeglichen. Sie bleiben in der zweiten Verteilung nach § 6 Abs. 6 BWahlG erhalten und werden als echte Überhangmandate zugeteilt. Im Ergebnis sichert das Sitzzuteilungsverfahren nach § 6 Abs. 5 und 6 BWahlG damit weiterhin den Erhalt aller Direktmandate als Ausdruck des Elements der Personenwahl.</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr"/>
-      <c r="C181" t="n">
-        <v>180</v>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>Die Begründung des Entwurfs des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 verweist dementsprechend darauf, dass am System der personalisierten Verhältniswahl festgehalten werde, und bekennt sich ausdrücklich zum Grundcharakter der Verhältniswahl (vgl. BTDrucks 19/22504, S. 1). Die Proporzbeeinträchtigung, die durch den Anfall von bis zu drei Überhangmandaten in Kauf genommen werde, führe nicht dazu, dass der Ausgleich zwischen dem Anliegen der Personenwahl und dem mit der Verhältniswahl verfolgten Ziel weitgehender Proportionalität nicht mehr als gewahrt anzusehen sei (vgl. BTDrucks 19/22504, S. 6). Damit liegt dem Gesetzentwurf erkennbar die Vorstellung zugrunde, der proporzverzerrende Anfall von Überhangmandaten sei dem Anliegen der personalisierten Verhältniswahl geschuldet (vgl. auch BTDrucks 19/23187, S. 2, 6 f.).</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr"/>
-      <c r="C182" t="n">
-        <v>181</v>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>Die Zulassung von bis zu drei unausgeglichenen Überhangmandaten stellt sich als Weiterentwicklung der Reaktion des Gesetzgebers auf die Rechtsprechung des Bundesverfassungsgerichts dar, wonach dieser verpflichtet ist, bei der Umsetzung der mit der Personenwahl verfolgten engen Bindung zwischen Wählerschaft und Abgeordneten Vorkehrungen gegen einen übermäßigen Anfall von Überhangmandaten zu treffen (vgl. BVerfGE 131, 316 &lt;370 ff.&gt;). Während das Bundeswahlgesetz 2011 keinerlei Regelung zum Ausgleich von Überhangmandaten traf, sah der Gesetzgeber unter Hinweis auf die Senatsentscheidung vom 25. Juli 2012 (BVerfGE 131, 316) in § 6 Abs. 5 BWahlG 2013 einen Vollausgleich vor (vgl. BTDrucks 17/11819, S. 5 f.). In der Folge wuchs der Deutsche Bundestag 2017 auf 709 Abgeordnete an. Um einer weiteren Vergrößerung des Parlaments entgegenzusteuern, ergänzte der Gesetzgeber die zunächst zur Erfüllung des verfassungsrechtlichen Regelungsauftrags gefundene Lösung um die verfahrensgegenständliche Neuregelung und nahm den Vollausgleich partiell zurück (vgl. BTDrucks 19/22504, S. 1, 5, 6). Dies ändert nichts daran, dass mit dem etablierten Wahlsystem am Grundcharakter einer personalisierten Verhältniswahl festgehalten wird.</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr"/>
-      <c r="C183" t="n">
-        <v>182</v>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>Zwar weicht es von dem Ziel, exakt die Hälfte der Abgeordneten des Deutschen Bundestages im Wege der Personenwahl zu bestimmen, ab, denn die zum Ausgleich von Proporzverzerrungen durchgeführte Erhöhung der Sitzzahl des Deutschen Bundestages (§ 6 Abs. 5 BWahlG) führt dazu, dass sich das Verhältnis von Wahlkreismandaten und Listenmandaten zugunsten der Listenmandate verschiebt. Dies ändert aber nichts daran, dass weiterhin jedenfalls ein maßgeblicher Anteil der Abgeordneten des Deutschen Bundestages direkt in den Wahlkreisen gewählt und damit dem Element der Personenwahl Rechnung getragen wird. Dabei wirkt die Zulassung von bis zu drei Überhangmandaten der Verschiebung des Verhältnisses von Direkt- und Listenmandaten, die mit dem Ausgleich von Quasi-Überhangmandaten verbunden ist, entgegen. Dies dient dem verfassungslegitimen Ziel, das Element der Personenwahl zu stärken.</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr"/>
-      <c r="C184" t="n">
-        <v>183</v>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>(bb) Vor diesem Hintergrund kann dahinstehen, ob die hinter der Begrenzung des Anwachsens der Bundestagsgröße stehenden Befürchtungen, der Deutsche Bundestag könne die Grenzen seiner Arbeits- und Handlungsfähigkeit erreichen (vgl. BTDrucks 19/22504, S. 1, 5), für sich genommen die durch die Zulassung von Überhangmandaten bewirkten Gleichheitsbeeinträchtigungen rechtfertigen können. Bei der Sicherung der Arbeits- und Funktionsfähigkeit des Parlaments handelt es sich um einen verfassungsrechtlichen Belang von höchstem Rang (vgl. BVerfGE 95, 335 &lt;404&gt;), der dem Grunde nach der Wahlgleichheit und der Chancengleichheit der Parteien die Waage halten kann. Ob dieser Belang aber bei einer Fortsetzung des Vollausgleichs von Überhangmandaten überhaupt tangiert wäre, bedarf angesichts des Rückgriffs auf den verfassungsrechtlich legitimierten Belang der Stärkung des Elements der Personenwahl keiner Entscheidung.</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr"/>
-      <c r="C185" t="n">
-        <v>184</v>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>(b) Die Zulassung von bis zu drei ausgleichslosen Überhangmandaten ist geeignet und erforderlich, das Ziel der Aufrechterhaltung und Stärkung des Elements der Personenwahl zu erreichen. Die Neuregelung bewegt sich innerhalb des dem Gesetzgeber eröffneten Gestaltungskorridors zur Schaffung eines personalisierten Verhältniswahlrechts (vgl. auch Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 26, 58).</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr"/>
-      <c r="C186" t="n">
-        <v>185</v>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>(aa) Der Senat hält daran fest, dass ein angemessener Ausgleich zwischen dem Anliegen möglichst proportionaler Abbildung des Zweitstimmenergebnisses im Deutschen Bundestag und dem mit der Personenwahl verbundenen Belang des uneingeschränkten Erhalts von Wahlkreismandaten und des annähernd ausgeglichenen Verhältnisses von Wahlkreismandaten und Listenmandaten dann nicht mehr gewahrt ist, wenn die Zahl der Überhangmandate etwa die Hälfte der für die Bildung einer Fraktion erforderlichen Zahl von Abgeordneten überschreitet (vgl. BVerfGE 131, 316 &lt;369 f.&gt;). Ausgehend von § 10 Abs. 1 Satz 1 GO-BT in der Fassung der Bekanntmachung vom 2. Juli 1980 (BGBl I S. 1237) sind dies 15 Abgeordnete (vgl. bereits BVerfGE 131, 316 &lt;369 f.&gt;). Diese Grenze ist durch die zur Überprüfung gestellte Neuregelung des § 6 Abs. 5 und 6 BWahlG bei Weitem nicht überschritten, da bundesweit höchstens drei unausgeglichene Überhangmandate anfallen können. Dies begrenzt das Gewicht der damit einhergehenden Gleichheitsbeeinträchtigung deutlich.</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr"/>
-      <c r="C187" t="n">
-        <v>186</v>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>(bb) Der Erforderlichkeit der Regelung steht auch nicht entgegen, dass der Gesetzgeber die mit der Personalisierung verfolgten Zwecke ebenso gut ohne Beeinträchtigung der Erfolgswertgleichheit durch einen Vollausgleich aller Überhangmandate erreichen könnte. Zwar ist die durch den Anfall von Überhangmandaten bewirkte Differenzierung des Erfolgswertes der Wählerstimmen mit einer personalisierten Verhältniswahl nicht zwangsläufig verbunden, weil der gestörte Proporz durch Zuteilung von Ausgleichsmandaten wiederhergestellt werden könnte (vgl. BVerfGE 95, 335 &lt;394 f.&gt;; 131, 316 &lt;366&gt;). Allerdings erforderte eine vollständige Verwirklichung des Ziels der Verhältniswahl eine im Einzelnen nicht vorhersehbare Erhöhung der Sitzzahl des Bundestages, wodurch das Ziel, die Abgeordneten des Deutschen Bundestages annäherungsweise zur Hälfte personenbezogen zu legitimieren, nicht erreicht werden könnte (vgl. BVerfGE 131, 316 &lt;366&gt;). Demnach stellt der Vollausgleich kein gegenüber der begrenzten Zulassung von Überhangmandaten ebenso wirksames Mittel zur Stärkung des Elements der Personenwahl dar. Im Fall eines Vollausgleichs blieben zwar alle Direktmandate erhalten. Es veränderte sich aber das Verhältnis zwischen in den Wahlkreisen direkt gewählten Abgeordneten und solchen, die über die Landeslisten der Parteien in den Deutschen Bundestag einziehen. Das Element der Personenwahl würde dadurch relativ geschwächt (vgl. auch Möllers, RuP 2012, S. 1 &lt;7 f.&gt; m.w.N.). In einer solchen Situation obliegt es dem Gesetzgeber, sich innerhalb der aus der Grundentscheidung für das System der personalisierten Verhältniswahl ergebenden verfassungsrechtlichen Grenzen zu entscheiden, inwieweit durch einen Vollausgleich von Überhangmandaten dem Proportionalitätsprinzip Rechnung getragen oder durch eine annähernd gleiche Zahl an Direkt- und Listenmandaten das Element der Personenwahl gestärkt wird.</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr"/>
-      <c r="C188" t="n">
-        <v>187</v>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>(c) Der Verfassungsmäßigkeit der vorliegend zur Überprüfung gestellten Regelung steht nicht entgegen, dass der Gesetzgeber die Entstehung von bis zu drei Überhangmandaten in Kauf nimmt. Die Argumentation der Antragstellerinnen und Antragsteller, der Gesetzgeber dürfe Überhangmandate nur als Nebenfolge seiner Wahlsystementscheidung hinnehmen, geht fehl.</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr"/>
-      <c r="C189" t="n">
-        <v>188</v>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>(aa) Zwar hat das Bundesverfassungsgericht ausgeführt, dass die mit der Zulassung von Überhangmandaten verbundene Differenzierung der Wahlgleichheit und der Chancengleichheit der Parteien nur insoweit mit dem Grundsatz der gleichen Wahl vereinbar ist, als sie sich als notwendige Folge des besonderen Charakters der personalisierten Verhältniswahl darstellt (vgl. BVerfGE 16, 130 &lt;140&gt;; 95, 335 &lt;358&gt;). Daraus ergibt sich jedoch nicht, dass Überhangmandate nur eine Nebenfolge der Wahlsystementscheidung des Gesetzgebers sein dürften. Der Gesetzgeber ist im Rahmen des ihm durch Art. 38 Abs. 3 GG übertragenen Gestaltungsauftrags befugt, ein Wahlsystem zu schaffen, das sowohl dem Anliegen einer Personenwahl als auch dem Ziel der Verhältniswahl, alle Parteien in einem den Stimmenzahlen entsprechenden Verhältnis im Parlament abzubilden, möglichst Rechnung trägt. Beide von der Verfassung legitimierten Ziele lassen sich innerhalb eines Wahlsystems nicht in voller Reinheit verwirklichen. Sie stehen in einem Spannungsverhältnis, das sich nur durch einen vom Gesetzgeber vorzunehmenden Ausgleich beider Prinzipien auflösen lässt. Im Rahmen des ihm insoweit zukommenden Gesetzgebungsauftrags darf der Gesetzgeber das Anliegen einer proportionalen Verteilung der Gesamtzahl der Sitze zurückstellen und Überhangmandate ohne Wiederherstellung des Proporzes zulassen, solange sich die damit verbundene Differenzierung des Erfolgswertes der Wählerstimmen innerhalb des gesetzgeberischen Konzepts hält (vgl. BVerfGE 95, 408 &lt;421&gt;; 131, 316 &lt;366 f.&gt;). Ob es sich dabei um eine bewusst herbeigeführte Konsequenz oder nur um eine ungewollte Nebenfolge der gesetzgeberischen Systementscheidung handelt, ist ohne Belang.</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr"/>
-      <c r="C190" t="n">
-        <v>189</v>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>(bb) Auch soweit das Bundesverfassungsgericht in der Vergangenheit auf das Vorliegen eines „zwingenden Grundes“ als Voraussetzung für die Rechtfertigung von Differenzierungen der Wahlgleichheit abgestellt hat (vgl. BVerfGE 6, 84 &lt;92&gt;; 51, 222 &lt;236&gt;; 95, 408 &lt;418&gt;; 129, 300 &lt;320&gt;), bedeutet dies nicht, dass sich die Differenzierung von Verfassungs wegen als notwendig darstellen muss. Dies ändert nichts daran, dass Differenzierungen im Wahlrecht durch Gründe gerechtfertigt sein können, die durch die Verfassung legitimiert und von einem Gewicht sind, das der Wahlgleichheit die Waage halten kann (vgl. BVerfGE 162, 207 &lt;238 Rn. 92&gt;). Dabei ist nicht erforderlich, dass die Verfassung diese Zwecke zu verwirklichen gebietet (vgl. BVerfGE 120, 82 &lt;107&gt; m.w.N.). Gleiches gilt für Differenzierungen der Chancengleichheit der Parteien (vgl. BVerfGE 162, 207 &lt;238 Rn. 92&gt;).</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr"/>
-      <c r="C191" t="n">
-        <v>190</v>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>(cc) Zudem hat der Gesetzgeber den Anfall von Überhangmandaten bereits in der Vergangenheit hingenommen, wenn Wahlkreismandate auf die für die jeweilige Landesliste ermittelte Sitzzahl nicht angerechnet werden konnten, und sich nicht veranlasst gesehen, das Entstehen von Überhangmandaten zu neutralisieren (vgl. nur BVerfGE 95, 335 &lt;356 f.&gt;). Das Bundesverfassungsgericht hat dies unter dem Aspekt einer bewussten Inkaufnahme von Überhangmandaten nicht beanstandet. Vielmehr hat es festgestellt, dass das Anliegen der Personenwahl und das mit der Verhältniswahl verfolgte Ziel weitgehender Proportionalität in einem Spannungsverhältnis stehen, welches sich nur durch einen vom Gesetzgeber vorzunehmenden Ausgleich beider Prinzipien auflösen lässt. Im Rahmen des ihm insoweit zukommenden Gestaltungsspielraums darf der Gesetzgeber Überhangmandate ohne Wiederherstellung des Proporzes in begrenztem Umfang zulassen. Dabei ist es im Rahmen der sich aus seiner Wahlsystementscheidung ergebenden Grenzen seine Sache, die Zahl hinnehmbarer Überhangmandate konkret festzulegen (vgl. BVerfGE 131, 316 &lt;366 f.&gt;).</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr"/>
-      <c r="C192" t="n">
-        <v>191</v>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>b) Soweit es die zur Überprüfung gestellte Änderung des Bundeswahlgesetzes nach § 6 Abs. 6 Satz 2 Halbsatz 2 in Verbindung mit Abs. 5 Satz 2 BWahlG erlaubt, Direktmandate einer Partei mit Listenmandaten derselben Partei in einem anderen Land zu verrechnen, ist damit eine Beeinträchtigung der Wahlgleichheit verbunden (aa). Diese ist jedoch durch das verfassungslegitime Anliegen einer Stärkung der Personenwahl ebenfalls gerechtfertigt (bb).</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr"/>
-      <c r="C193" t="n">
-        <v>192</v>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>aa) Gemäß § 6 Abs. 5 Satz 2 BWahlG wird im Rahmen der Sitzzahlerhöhung jeder Landesliste der höhere Wert aus entweder der Zahl der im Land von Wahlbewerbern der Partei in den Wahlkreisen nach § 5 BWahlG errungenen Sitze oder dem auf ganze Sitze aufgerundeten Mittelwert zwischen diesen und den für die Landesliste der Partei nach der ersten Verteilung nach § 6 Abs. 2 und 3 BWahlG ermittelten Sitze zugeordnet. Dies stellt die Mindestsitzzahl dar, die jeder Landesliste im Rahmen der tatsächlichen zweiten Verteilung gemäß § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG zugeteilt wird. In der Konsequenz kann dieser Verrechnungsmechanismus dazu führen, dass einer Partei in einem Land mit relativ schwachen Erststimmenergebnissen Listenmandate, die ihr nach ihrem Zweitstimmenergebnis im Land zustünden, nicht zugeteilt, sondern diese zur Verrechnung von Quasi-Überhangmandaten derselben Partei in anderen Ländern verwendet werden.</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr"/>
-      <c r="C194" t="n">
-        <v>193</v>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>Die länderübergreifende Verrechnung von Direkt- und Listenmandaten hat eine Beeinträchtigung der Erfolgswertgleichheit der Stimmen der Wählerinnen und Wähler, die die zur Kompensation herangezogene Landesliste gewählt haben, zur Folge (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 60 m.w.N.). Entgegen einer dazu vertretenen Auffassung (vgl. Grzeszick, BTAusschussdrucks 19&lt;4&gt;584 E, S. 5) wird die Erfolgswertgleichheit im System der Verhältniswahl nicht ausschließlich parteiübergreifend, mithin zwischen den Wählerinnen und Wählern verschiedener Parteien, gewährleistet. Die Erfolgswertgleichheit verlangt, dass jede gültig abgegebene Stimme bei dem anzuwendenden Rechenverfahren mit gleichem Gewicht bewertet wird und ihr ein anteilsmäßig gleicher Erfolg zukommt (vgl. BVerfGE 95, 335 &lt;353&gt;; 131, 316 &lt;338&gt;; 146, 327 &lt;350 Rn. 59&gt;; jeweils m.w.N.). Sie ist Ausfluss der Gleichheit der Staatsbürger und gilt daher absolut und nicht nur relativ im Vergleich zwischen verschiedenen Parteien. Durch die Regelung des § 6 Abs. 6 Satz 2 Halbsatz 2 in Verbindung mit Abs. 5 Satz 2 BWahlG wird sie beeinträchtigt, weil den Stimmen derjenigen Wähler, die mit ihrer Zweitstimme die Landesliste einer Partei wählen, deren Mandate zur Kompensation von Quasi-Überhangmandaten derselben Partei in einem anderen Land herangezogen werden, ein geringerer Erfolgswert zukommt als den Stimmen derjenigen Wähler, die für eine andere Landesliste dieser Partei abgegeben worden sind, deren Mandate nicht zu Kompensationszwecken verrechnet werden (vgl. BTDrucks 19/22504, S. 7; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 60 m.w.N.). Darüber hinaus sinkt der Erfolgswert der Stimmen, die für die zu Kompensationszwecken herangezogene Landesliste abgegeben worden sind, auch im Vergleich zu den für die Landeslisten anderer Parteien in diesem Land abgegebenen Stimmen (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 60 m.w.N.). Ebenso berührt ist die passive Wahlgleichheit in Form der Chancengleichheit der betroffenen Wahlbewerber, denen trotz der rechnerisch ausreichenden Zahl an Zweitstimmen für die Landesliste ihrer Partei kein Mandat zugeteilt wird (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 60 m.w.N.).</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr"/>
-      <c r="C195" t="n">
-        <v>194</v>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>bb) Der mit der internen Verrechnung von Direktmandaten und Listenmandaten verbundene Eingriff in die Wahlgleichheit ist jedoch zur Aufrechterhaltung und Stärkung des Elements der Personenwahl bei der Wahl des Deutschen Bundestages gerechtfertigt.</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr"/>
-      <c r="C196" t="n">
-        <v>195</v>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>(1) Die Möglichkeit der länderübergreifenden Verrechnung von Direkt- und Listenmandaten dient dem Ziel, die Zuweisung sämtlicher Direktmandate zu gewährleisten, und stärkt damit das Element der Personenwahl.</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr"/>
-      <c r="C197" t="n">
-        <v>196</v>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>(2) Sie ist zur Erreichung dieses Ziels auch geeignet und erforderlich. Die Möglichkeit der länderübergreifenden Verrechnung von Direkt- und Listenmandaten derselben Partei trägt zur Erhaltung aller von einer Partei bundesweit gewonnenen Wahlkreismandate und einer annähernd gleichen Zahl von Direkt- und Listenmandaten bei. Mildere, die Wahlgleichheit weniger einschränkende Instrumente, die dieses Ziel ebenso gut erreichten, stehen nicht zur Verfügung. Würde auf die Möglichkeit der länderübergreifenden Verrechnung verzichtet, könnten Überhangsituationen nicht kompensiert werden und fielen Überhangmandate in einem größeren Ausmaß an. Würden diese nicht ausgeglichen, hätte das in die Gleichheit der Wahl eingreifende Proporzverzerrungen zur Folge, die nicht weniger gewichtig wären als die Eingriffe in die Erfolgswertgleichheit, die mit dem vorliegend zu beurteilenden Verrechnungsmodell verbunden sind. Erfolgte hingegen ein Vollausgleich der Quasi-Überhangmandate, würde das Ziel, die Abgeordneten des Deutschen Bundestages annähernd zur Hälfte personenbezogen zu legitimieren (vgl. BVerfGE 131, 316 &lt;366&gt;), in geringerem Umfang erreicht. Gleiches gälte, wenn an dem Modell des teilweisen Ausgleichs festgehalten und die Sitzzahl des Deutschen Bundestages so lange erhöht würde, bis nicht mehr als drei Überhangmandate verblieben. Ohne das Element der internen Verrechnung stiege die Zahl der auszugleichenden Quasi-Überhangmandate. Damit nähme die Größe des Bundestages zu (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 28), sodass sich das Verhältnis von Wahlkreisabgeordneten und Abgeordneten, die über die Landeslisten der Parteien in den Deutschen Bundestag einziehen, zulasten Ersterer verschöbe. Vor diesem Hintergrund hat der Gesetzgeber mit der Verrechnungsklausel des § 6 Abs. 5 Satz 2 BWahlG den ihm eingeräumten Spielraum zur Ausgestaltung des Bundestagswahlrechts nicht überschritten.</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr"/>
-      <c r="C198" t="n">
-        <v>197</v>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>(3) Dem steht nicht entgegen, dass nach den Ausführungen des Sachverständigen Pukelsheim in der mündlichen Verhandlung die Mindestsitzgarantie nach dem Bundeswahlgesetz 2013 zu einer gegenüber der Garantie von Mindestsitzen nach dem Fünfundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 geringeren Beeinträchtigung der Erfolgswertgleichheit führte (vgl. auch Pukelsheim/ Bischof, DVBl 2021, S. 417 &lt;425&gt;; Pukelsheim, BTAusschussdrucks 19&lt;4&gt;584 A neu, Anlage 1). Denn die mit dem Fünfundzwanzigsten Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 eingeführte parteiinterne Verrechnung von Listen- mit Direktmandaten führt zu einer geringeren Zahl an auszugleichenden Mandaten und vermindert den Umfang der Sitzzahlerhöhung gemäß § 6 Abs. 5 BWahlG (vgl. Pukelsheim/ Bischof, DVBl 2021, S. 417 &lt;419&gt;). Dies dient dem Ziel eines ausgeglichenen Verhältnisses von Direkt- und Listenmandaten. Der Verrechnungsmechanismus des § 6 Abs. 5 Satz 2 BWahlG stärkt dadurch das Element der Persönlichkeitswahl und genügt damit den verfassungsrechtlichen Rechtfertigungsanforderungen, auch wenn damit ein im Vergleich zu den Regelungen des Bundeswahlgesetzes 2013 stärkerer Eingriff in die Erfolgswertgleichheit der abgegebenen Stimmen verbunden ist.</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr"/>
-      <c r="C199" t="n">
-        <v>198</v>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>(4) Soweit gegen die parteiinterne Verrechnung von Listen- mit Direktmandaten eingewandt wird, dass Gerechtigkeits- und Fairnessvorstellungen von Wählerinnen und Wählern verletzt würden, wenn ihre beziehungsweise die für ihre Landesliste abgegebene Zweitstimme für ein Direktmandat in einem anderen Land bezahle, statt zur Wahl der Personen auf der gewählten Landesliste beizutragen (vgl. Behnke, ZParl 2012, S. 675 &lt;684 f.&gt;; ders., ZParl 2019, S. 630 &lt;643 ff.&gt;), folgt daraus nichts anderes. Die Entscheidung des Wahlgesetzgebers für eine mit der Personenwahl verbundene Verhältniswahl (§ 1 Abs. 1 Satz 2 BWahlG) verlangt eine Anrechnung der Direktmandate auf Sitze, die sich nach der Verhältniswahl berechnen. Dabei ist die Priorisierung der Direktmandate dem System der personalisierten Verhältniswahl in der Ausgestaltung des Bundeswahlgesetzes auch in der Fassung des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 immanent. Dieses Wahlsystem ist darauf angelegt, die Ergebnisse der vorgeschalteten Personenwahl zu erhalten (vgl. BVerfGE 131, 316 &lt;359&gt;; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 19 ff.). Vor diesem Hintergrund ist mit der länderübergreifenden Verrechnung von Direkt- und Listenmandaten ein wahlsystemwidriger Effekt nicht verbunden.</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr"/>
-      <c r="C200" t="n">
-        <v>199</v>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>(5) Allerdings kann das Verrechnungsmodell nicht sicherstellen, dass die einzelnen Landesverbände der Parteien im Bundestag in der Stärke vertreten sind, wie dies dem Anteil der auf sie entfallenden Zweitstimmen entspricht. Vielmehr nimmt die Regelung eine Verzerrung des föderalen Proporzes in Kauf (vgl. BTDrucks 19/22504, S. 7; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 60 m.w.N.). Dieser Effekt tritt aber auch dann auf, wenn Überhangmandate ohne Verrechnung oder Ausgleich zugeteilt werden, denn in diesem Fall erzielt jede hiervon begünstigte Landesliste eine Überrepräsentation gegenüber anderen Landeslisten (vgl. BVerfGE 95, 335 &lt;401 f.&gt;). Zwar wird diese föderale Proporzverzerrung durch den Verrechnungsmechanismus des § 6 Abs. 5 Satz 2 BWahlG verschärft, weil er nicht nur zu einer Überrepräsentation der Landeslisten mit Überhangmandaten, sondern zugleich dazu führt, dass andere Landeslisten derselben Partei mit Blick auf die erzielten Wahlergebnisse bei der Sitzzuteilung benachteiligt werden (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 60 m.w.N.). Bei der Gewichtung des Anliegens einer föderalen Zuordnung der Stimmen ist aber zu berücksichtigen, dass es bei der Wahl zum Deutschen Bundestag um die Wahl des unitarischen Vertretungsorgans des Bundesvolkes geht (vgl. BVerfGE 121, 266 &lt;305&gt; m.w.N.). Vor diesem Hintergrund ist der Gesetzgeber bei der Ausgestaltung des Wahlrechts zum Deutschen Bundestag berechtigt, aber nicht verpflichtet, föderalen Belangen Rechnung zu tragen (vgl. BVerfGE 6, 84 &lt;99&gt;; 16, 130 &lt;143&gt;; 95, 335 &lt;402&gt;; 121, 266 &lt;305&gt; m.w.N.). Ebenso steht es ihm im Rahmen seines Regelungsauftrags gemäß Art. 38 Abs. 3 GG frei, föderalen Belangen ein größeres oder geringeres Gewicht beizumessen (vgl. BVerfGE 131, 316 &lt;345&gt;). Dass er diesen Spielraum vorliegend überschritten hätte, ist nicht ersichtlich.</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr"/>
-      <c r="C201" t="n">
-        <v>200</v>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>(6) Hinzu kommt, dass das Gewicht der Beeinträchtigung sowohl der Erfolgswertgleichheit als auch des föderalen Proporzes begrenzt ist. Den Landeslisten ist nach § 6 Abs. 6 Satz 2 Halbsatz 2 in Verbindung mit Abs. 5 Satz 2 BWahlG garantiert, dass sie mindestens einen Teil der ihnen nach dem Zweitstimmenergebnis im Land zustehenden Mandate erhalten, nämlich jedenfalls die Hälfte der nach Anrechnung der Direktmandate verbleibenden Listenmandate (vgl. Pukelsheim/Bischof, DVBl 2021, S. 417 &lt;419 f.&gt;; Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 28). Es kann also nicht dazu kommen, dass eine Landesliste entgegen dem Votum der Wählerinnen und Wähler im betreffenden Land gar keine Sitze erhält, weil die ihr nach dem Zweitstimmenergebnis zustehenden Sitze vollständig zur Anrechnung von Direktmandaten derselben Partei in anderen Ländern verwendet werden (vgl. BTDrucks 19/22504, S. 7).</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr"/>
-      <c r="C202" t="n">
-        <v>201</v>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>(7) Soweit unterschiedlich beurteilt wird, in welchem Umfang die Verrechnung von Listenmandaten mit Direktmandaten derselben Partei in einem anderen Land dazu beiträgt, das Anwachsen der Größe des Deutschen Bundestages zu bremsen (vgl. Pukelsheim/ Bischof, DVBl 2021, S. 417 &lt;419, 425&gt; m.w.N.; Behnke, BTAusschussdrucks 19&lt;4&gt;584 D, S. 21), kann dahinstehen, ob die mit der Verrechnung einhergehenden Beeinträchtigungen des Proporzes unter dem Gesichtspunkt der Sicherung der Arbeits- und Funktionsfähigkeit des Parlaments (vgl. BVerfGE 95, 335 &lt;404&gt;) gerechtfertigt werden können. Sie sind bereits durch das verfassungsrechtlich anerkannte Ziel, das Element der Personenwahl bei der Wahl des Deutschen Bundestages aufrechtzuerhalten und zu stärken, hinreichend legitimiert. Auf die Frage, ob und inwiefern die Neuregelung der Sitzzuteilung der Sicherung der Arbeits- und Funktionsfähigkeit des Deutschen Bundestages dient, kommt es daher nicht an.</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr"/>
-      <c r="C203" t="n">
-        <v>202</v>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>c) Mit dem zur Überprüfung gestellten Sitzzuteilungsverfahren ist ein verfassungsrechtlich relevanter Effekt des negativen Stimmgewichts, der die Grundsätze der Wahlgleichheit und der Chancengleichheit der Parteien sowie der Unmittelbarkeit der Wahl verletzte (aa), nicht verbunden (bb).</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr"/>
-      <c r="C204" t="n">
-        <v>203</v>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>aa) Die Mandatszuteilung darf grundsätzlich nicht dazu führen, dass die Sitzzahl einer Partei erwartungswidrig mit der auf diese oder eine konkurrierende Partei entfallenden Stimmenzahl korreliert (Effekt des negativen Stimmgewichts; vgl. BVerfGE 131, 316 &lt;346 f.&gt;). Dies ist der Fall, wenn ein Zweitstimmengewinn zu einem Sitzverlust der betroffenen Partei führen kann und dieser auch einen Sitzanteilsverlust für diese Partei bedeutet. Gleiches gilt, wenn ein Zweitstimmenverlust zu einem Sitzgewinn der betroffenen Partei führen kann und dieser einen Sitzanteilsgewinn dieser Partei nach sich zieht.</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr"/>
-      <c r="C205" t="n">
-        <v>204</v>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>(1) Der Effekt des negativen Stimmgewichts beeinträchtigt die Wahlgleichheit und die Chancengleichheit der Parteien (vgl. BVerfGE 121, 266 &lt;299 f.&gt;; 131, 316 &lt;347&gt;). Die Erfolgswertgleichheit beinhaltet, dass eine Stimme für die Partei, für die sie abgegeben wurde, positive Wirkung entfalten können muss. Ein Wahlsystem, das darauf ausgelegt ist oder doch jedenfalls in typischen Konstellationen zulässt, dass ein Zuwachs an Stimmen zu Mandatsverlusten führt oder dass für den Wahlvorschlag einer Partei insgesamt mehr Mandate erzielt werden, wenn auf ihn weniger oder auf einen konkurrierenden Vorschlag mehr Stimmen entfallen, führt zu willkürlichen Ergebnissen und lässt den demokratischen Wettbewerb um Zustimmung bei den Wahlberechtigten widersinnig erscheinen (vgl. BVerfGE 121, 266 &lt;299&gt;). Ein Berechnungsverfahren, das dazu führt, dass eine Wählerstimme für eine Partei Wirkung gegen diese Partei entfaltet, widerspricht Sinn und Zweck einer demokratischen Wahl (vgl. BVerfGE 121, 266 &lt;300&gt;; 131, 316 &lt;347&gt;). Der Effekt des negativen Stimmgewichts beeinträchtigt neben der Erfolgswertgleichheit auch die Erfolgschancengleichheit. Diese erlaubt zwar, dass – wie zum Beispiel im Mehrheitswahlrecht – Stimmen nicht gewertet werden, nicht aber, dass einer Wahlstimme neben der Chance, zum beabsichtigten Erfolg beizutragen, auch die Gefahr innewohnt, dem eigenen Wahlziel zu schaden (vgl. BVerfGE 121, 266 &lt;300 f.&gt;).</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr"/>
-      <c r="C206" t="n">
-        <v>205</v>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>(2) Der Effekt des negativen Stimmgewichts beeinträchtigt zudem den Grundsatz der Unmittelbarkeit der Wahl, weil die Wählerinnen und Wähler nicht erkennen können, ob sich ihre Stimme stets für die präferierte Partei und deren Wahlbewerber positiv auswirkt oder ob sie durch ihre Stimme den Misserfolg eines Kandidaten oder der präferierten Partei verursachen. Gesetzliche Regelungen, die derartige Unwägbarkeiten nicht nur in seltenen und unvermeidbaren Ausnahmefällen hervorrufen, sind mit dem Grundsatz der Unmittelbarkeit der Wahl nicht zu vereinbaren (vgl. BVerfGE 121, 266 &lt;307 f.&gt;; 131, 316 &lt;347&gt;).</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr"/>
-      <c r="C207" t="n">
-        <v>206</v>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>bb) Davon ausgehend sind die zur Überprüfung gestellten Normen unter dem Gesichtspunkt des negativen Stimmgewichts von Verfassungs wegen nicht zu beanstanden. Ungeachtet der unterschiedlichen Auffassungen zu der Frage, inwieweit sich aufgrund des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 Fälle des negativen Stimmgewichts überhaupt ergeben können (1), ist davon auszugehen, dass dieser Effekt jedenfalls nicht in verfassungsrechtlich relevanter Weise auftreten kann (2).</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr"/>
-      <c r="C208" t="n">
-        <v>207</v>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>(1) Die Frage, ob sich nach den Regelungen des § 6 Abs. 5 und 6 BWahlG der Effekt des negativen Stimmgewichts überhaupt ergeben kann, ist sowohl im Gesetzgebungsverfahren (a) als auch in der Literatur (b) unterschiedlich beurteilt und in der mündlichen Verhandlung durch den Sachverständigen Pukelsheim bejaht worden (c).</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr"/>
-      <c r="C209" t="n">
-        <v>208</v>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>(a) (aa) Im Gesetzgebungsverfahren hat die Sachverständige Schönberger die Auffassung vertreten, der Effekt des negativen Stimmgewichts sei evident. Die Zulassung unausgeglichener Überhangmandate habe zur Folge, dass das Weniger an Zweitstimmen für eine Partei, das zur Entstehung eines unausgeglichenen Überhangmandats führe, automatisch eine geringere Mandatszahl für andere, konkurrierende Parteien und somit eine erwartungswidrige Korrelation mit der Sitzzahl einer anderen Partei bewirke (vgl. Schönberger, BTAusschussdrucks 19&lt;4&gt;584 B, S. 6). In einer Nachwahlkonstellation bestehe die Möglichkeit, ein Direktmandat zu einem Überhangmandat zu machen, indem weniger Zweitstimmen für die entsprechende Partei abgegeben würden, und dadurch die Mandatszahl konkurrierender Parteien zu reduzieren (vgl. Schönberger, Ausschuss für Inneres und Heimat, Protokoll Nr. 19/100, S. 11).</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr"/>
-      <c r="C210" t="n">
-        <v>209</v>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>(bb) Der Sachverständige Grzeszick hat im Gesetzgebungsverfahren hingegen kein unzulässiges negatives Stimmgewicht erkannt. Zwar könne der den Überhangmandaten eigene Effekt, dass durch mehr Zweitstimmen für eine Partei in einem Land ein Überhangmandat zum Listensitz werden könne, diesen Zweitstimmen die positive Sitzrelevanz nehmen. Er verkehre das Mehr an Zweitstimmen aber nicht in ihr Gegenteil, denn dazu sei ein Sitzverlust nötig. Entsprechendes gelte für den umgekehrten Effekt, dass ein Weniger an Zweitstimmen sich nicht nachteilig auf die Sitzzahl auswirke, soweit dadurch ein unausgeglichenes Überhangmandat entstehe. Zudem habe das Bundesverfassungsgericht in seinem Urteil vom 25. Juli 2012 (BVerfGE 131, 316) bis zu 15 ausgleichslose Überhangmandate für verfassungsgemäß, den Effekt des negativen Stimmgewichts aber zugleich für verfassungswidrig erklärt. Bedingte bereits die proportionale Besserstellung einer Partei durch Überhangmandate ein unzulässiges negatives Stimmgewicht, sei die Entscheidung widersprüchlich (vgl. Grzeszick, BTAusschussdrucks 19&lt;4&gt;584 E, S. 8; ders., Ausschuss für Inneres und Heimat, Protokoll Nr. 19/100, S. 18 f.). Der „Dresdener Nachwahleffekt“ der föderalen Verschiebung könne nicht mehr vorkommen. Dies werde zum einen durch die festen Kontingente in der ersten Verteilung verhindert, zum anderen durch die Garantie des § 6 Abs. 6 Satz 2 Halbsatz 2 BWahlG. Jedenfalls sei nach der Rechtsprechung des Bundesverfassungsgerichts nur ein Effekt relevant, der nicht nur ganz außergewöhnlich auftrete (vgl. Grzeszick, Ausschuss für Inneres und Heimat, Protokoll Nr. 19/100, S. 19). Dies sei hier nicht der Fall.</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr"/>
-      <c r="C211" t="n">
-        <v>210</v>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>(cc) Der Sachverständige Vehrkamp vertrat in der Anhörung des Bundestagsausschusses für Inneres und Heimat die Auffassung, das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 ermögliche das Auftreten negativer Stimmgewichte, wenn sich bei einer Nachwahl ein durch Zweitstimmen gedecktes Direktmandat in ein durch Zweitstimmen nicht gedecktes Überhangmandat verwandele (vgl. Vehrkamp, Ausschuss für Inneres und Heimat, Protokoll Nr. 19/100, S. 10).</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr"/>
-      <c r="C212" t="n">
-        <v>211</v>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>(b) (aa) In der Literatur gehen Pukelsheim und Bischof davon aus, dass mit dem Auftreten negativer Stimmgewichte zu rechnen sei. Eine Partei könne bei mehr Zweitstimmen schlechter dastehen, da diese tendenziell zu einem Abbau von Überhangmandaten führten. Umgekehrt könnten weniger Zweitstimmen bewirken, dass sich Proporzmandate zu Überhangmandaten wandelten. Konstellationen, in denen das negative Stimmgewicht sichtbar werde, dürften jedoch eine nur marginale Rolle spielen (vgl. Pukelsheim/Bischof, DVBl 2021, S. 417 &lt;424&gt;).</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr"/>
-      <c r="C213" t="n">
-        <v>212</v>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>(bb) Boehl vertritt hingegen die Ansicht, der Effekt des negativen Stimmgewichts trete aufgrund des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 nicht auf, weil die Sitzverteilung im Ausgangspunkt nach voneinander getrennten Sitzkontingenten der Länder erfolge und sich Zweitstimmenverluste nicht zugunsten einer anderen Landesliste der gleichen Partei auswirken könnten. Wenn weniger Wählerinnen und Wähler einer Landesliste ihre Zweitstimme gäben, könne dies allenfalls deren Sitzzahl zugunsten der Landeslisten anderer Parteien in diesem Land vermindern. In einer Überhangsituation bleibe hingegen die Sitzzahl der Partei gleich, weil sie in diesem Fall durch die Zahl der Direktmandate bestimmt werde und nicht von der Zweitstimmenzahl abhänge. Diese Folgen stellten aber keinen paradoxen Effekt dar.</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr"/>
-      <c r="C214" t="n">
-        <v>213</v>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>Grundlage der Sitzzahlerhöhung seien die Mandatszahlen, die sich in der ersten Verteilung unter Ausschluss des Effekts des negativen Stimmgewichts ergäben. Durch die Sitzzahlerhöhung könne daher kein negatives Stimmgewicht in die zweite Verteilung und das Endergebnis transportiert werden. Nach der Sitzzahlerhöhung würden die Sitze auf die Parteien exakt nach deren Zweitstimmenverhältnis verteilt.</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr"/>
-      <c r="C215" t="n">
-        <v>214</v>
-      </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>Auch die bis zu drei Überhangmandate könnten nicht zu negativen Stimmgewichten führen. Überhangmandate seien zwar notwendige, aber keine hinreichende Bedingung für das Entstehen von negativem Stimmgewicht. Wenn sich weniger Zweitstimmen für eine Landesliste auf die Sitzzahl einer anderen Landesliste der gleichen Partei nicht positiv auswirken könnten, sei für die Annahme eines negativen Stimmgewichts kein Raum (vgl. Boehl, in: Schreiber, BWahlG, 11. Aufl. 2021, § 6 Rn. 65).</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr"/>
-      <c r="C216" t="n">
-        <v>215</v>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>(c) In der mündlichen Verhandlung hat der Sachverständige Pukelsheim die Auffassung vertreten, dass unter den Vorgaben des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 Konstellationen existierten, in denen ein negatives Stimmgewicht auftrete. Er hat dabei auf ein Szenario verwiesen, in dem mehr Zweitstimmen für eine Partei dazu führen könnten, dass ein nicht auszugleichendes Überhangmandat dieser Partei zu einem über den Mindestsitzanspruch der Partei gemäß § 6 Abs. 5 Satz 3 BWahlG garantierten Mandat werde. Dies bewirke keinen Sitzgewinn für die Partei selbst, führe über das Ausgleichsverfahren aber zu zusätzlichen Sitzen für die konkurrierenden Parteien. Zur Frage nach Ausmaß und Wahrscheinlichkeit des Effekts des negativen Stimmgewichts gab der Sachverständige Pukelsheim an, dies nicht belastbar beantworten zu können.</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr"/>
-      <c r="C217" t="n">
-        <v>216</v>
-      </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>(2) Davon ausgehend ergibt sich aus den zur Überprüfung gestellten Normen kein verfassungsrechtlich relevanter Effekt des negativen Stimmgewichts.</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr"/>
-      <c r="C218" t="n">
-        <v>217</v>
-      </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>(a) Die wesentliche Ursache für das Auftreten des negativen Stimmgewichts unter dem Bundeswahlgesetz in der Fassung des Neunzehnten Gesetzes zur Änderung des Bundeswahlgesetzes vom 25. November 2011 (BGBl I S. 2313) bestand in der Bestimmung der Ländersitzkontingente nach der Wählerzahl (vgl. BVerfGE 131, 316 &lt;347 ff.&gt;). Diese Ursache ist bereits durch das Zweiundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 3. Mai 2013 (BGBl I S. 1082) entfallen. Gemäß dem bei der nachfolgenden Gesetzesänderung unangetastet gebliebenen § 6 Abs. 2 Satz 1 BWahlG wird das Ländersitzkontingent in der ersten Verteilung nach dem Bevölkerungsanteil bestimmt. Die Abgabe oder Nichtabgabe einer Stimme wirkt sich damit auf die Höhe der Sitzkontingente der Länder nicht aus. Sitzplatzverschiebungen zwischen den Ländern in Abhängigkeit von der Wählerzahl sind ausgeschlossen. Auch ist die Möglichkeit der Listenverbindungen entfallen, die nach dem Bundeswahlgesetz in der Fassung des Siebzehnten Gesetzes zur Änderung des Bundeswahlgesetzes vom 11. März 2005 (BGBl I S. 674) im Zusammenhang mit Überhangmandaten den Effekt des negativen Stimmgewichts auslösten (vgl. BVerfGE 121, 266 &lt;298 ff., 305&gt;).</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr"/>
-      <c r="C219" t="n">
-        <v>218</v>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>(b) Die in Abweichung hierzu durch das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 eröffnete Möglichkeit der ausgleichslosen Zuteilung von bis zu drei Überhangmandaten löst den Effekt des negativen Stimmgewichts jedenfalls nicht in verfassungsrechtlich relevanter Weise aus.</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr"/>
-      <c r="C220" t="n">
-        <v>219</v>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>(aa) Zwar geht mit der Zulassung ausgleichsloser Überhangmandate einher, dass ein Zuwachs an Zweitstimmen für eine Partei dazu führen kann, dass ein ausgleichsloses Überhangmandat wegfällt. Ein derartiger Stimmenzuwachs führte aber nicht dazu, dass die betroffene Partei erwartungswidrig Mandate verlöre. Vielmehr bliebe die Zahl der auf sie entfallenden Mandate gleich, und es würde lediglich ein ausgleichsloses Überhangmandat durch ein mit Zweitstimmen unterlegtes Direktmandat ersetzt. Ein widersinniger, dem Sinn und Zweck einer demokratischen Wahl widersprechender Effekt (vgl. BVerfGE 121, 266 &lt;299 ff.&gt;; 131, 316 &lt;346 f.&gt;) zum Nachteil der von dem Zweitstimmenzuwachs betroffenen Partei wäre damit nicht verbunden.</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr"/>
-      <c r="C221" t="n">
-        <v>220</v>
-      </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>Allerdings hat der Sachverständige Pukelsheim in der mündlichen Verhandlung ausgeführt, dass der durch den Zweitstimmenzuwachs mögliche Verlust eines Überhangmandats zugunsten eines mit Zweitstimmen unterlegten Direktmandats über das Ausgleichsverfahren zu zusätzlichen Sitzen für konkurrierende Parteien führen kann. Dabei handelt es sich jedoch um eine bloß mittelbare Auswirkung des Zweitstimmenzuwachses einer Partei, die keine durchgreifenden verfassungsrechtlichen Bedenken begründet.</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr"/>
-      <c r="C222" t="n">
-        <v>221</v>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>So ist diese Auswirkung zunächst nicht mit einem eigenständigen Eingriff in den Grundsatz der Wahlgleichheit verbunden. Zwar hat die durch einen Zweitstimmenzuwachs verursachte Umwandlung eines ausgleichslosen Überhangmandats in ein ausgleichspflichtiges, mit Zweitstimmen unterlegtes Direktmandat im Ergebnis eine relative Besserstellung konkurrierender Parteien durch die Zuteilung von Ausgleichsmandaten zur Folge. Ursache hierfür ist aber der im Verfahren der Sitzzahlerhöhung gemäß § 6 Abs. 5 BWahlG angelegte Ausgleichsmechanismus. Dieser zielt gerade darauf, den durch die Garantie des Erhalts aller Direktmandate verursachten Eingriff in die Erfolgswertgleichheit jeder abgegebenen Stimme zu korrigieren. Werden zusätzliche Ausgleichsmandate vergeben, hat dies einen geringeren Eingriff in die Erfolgswertgleichheit aller abgegebenen Stimmen zur Folge.</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr"/>
-      <c r="C223" t="n">
-        <v>222</v>
-      </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>Ebenso wenig liegt ein Eingriff in den Grundsatz der Unmittelbarkeit der Wahl vor. Da das Mehr an Zweitstimmen nicht zu einer Verminderung der Sitzzahl der präferierten Partei führt, fehlt es an einem inversen, der Erwartungshaltung der Wählerinnen und Wähler widersprechenden Effekt. Die mittelbare Konsequenz der Zuteilung weiterer Ausgleichsmandate an konkurrierende Parteien genügt hierfür nicht. Sie ist im System der Verhältniswahl angelegt und jedenfalls durch das Ziel der Wiederherstellung der Wahlgleichheit gerechtfertigt.</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr"/>
-      <c r="C224" t="n">
-        <v>223</v>
-      </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>Hinzu kommt, dass es sich bei der durch einen Zuwachs an Zweitstimmen bedingten Ersetzung eines unausgeglichenen Überhangmandats um einen äußerst seltenen und daher verfassungsrechtlich unbedenklichen Ausnahmefall handeln dürfte (vgl. BVerfGE 121, 266 &lt;307 f.&gt;; 131, 316 &lt;347&gt;). Voraussetzung wäre, dass ein echtes Überhangmandat betroffen ist, dessen Zahl gemäß § 6 Abs. 5 Satz 4 BWahlG auf höchstens drei begrenzt ist. Dass ein solcher Fall über seltene Ausnahmefälle hinaus eintreten könnte, ist nicht ersichtlich. Auch der Sachverständige Pukelsheim hat in der mündlichen Verhandlung keine Angaben zur Wahrscheinlichkeit des Eintritts einer solchen Konstellation machen können.</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr"/>
-      <c r="C225" t="n">
-        <v>224</v>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>(bb) Umgekehrt kann der Verlust von Zweitstimmen dazu führen, dass die von der betroffenen Partei in dem Land gewonnenen Wahlkreismandate nicht mehr vollständig auf die ihr nach der Landesliste zustehenden Mandate angerechnet werden können, sodass ein unausgeglichenes Überhangmandat anfällt. Auch in diesem Fall bliebe die Zahl der auf die betroffene Partei entfallenden Mandate gleich. Ein erwartungswidriger Effekt in dem Sinne, dass das Weniger an Zweitstimmen zu einem Mehr an Mandaten der betroffenen Partei führte, träte nicht ein.</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr"/>
-      <c r="C226" t="n">
-        <v>225</v>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>Allenfalls könnten Mandate konkurrierender Parteien entfallen, da das auf diese Weise entstandene echte Überhangmandat nicht mehr am Ausgleichsmechanismus gemäß § 6 Abs. 5 Satz 2 und 3 BWahlG teilnähme. Verfassungsrechtliche Bedenken hiergegen bestehen nicht. Der Wegfall von Ausgleichsmandaten bei der Umwandlung eines nicht mehr durch Zweitstimmen gedeckten Direktmandats in ein unausgeglichenes Überhangmandat ist Folge der durch den Gesetzgeber im Rahmen des ihm durch Art. 38 Abs. 3 GG eingeräumten Gesetzgebungsauftrags getroffenen Wahlsystementscheidung. Ist er – wie dargestellt (s.o. Rn. 174 ff.) – befugt, eine begrenzte Zahl an echten Überhangmandaten zuzulassen, stellt sich die hierauf bezogene Nichtzuteilung von Ausgleichsmandaten nicht als widersinniger, dem Sinn und Zweck einer demokratischen Wahl widersprechender Effekt (vgl. BVerfGE 121, 266 &lt;300&gt;; 131, 316 &lt;346 f.&gt;) dar. Auch insoweit liegt daher ein verfassungsrechtlich relevantes negatives Stimmgewicht nicht vor.</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr"/>
-      <c r="C227" t="n">
-        <v>226</v>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>Die zu überprüfenden Normen sind schließlich nicht deshalb verfassungsrechtlich zu beanstanden, weil sie weniger als ein Jahr vor der Wahl des 20. Deutschen Bundestages in Kraft getreten sind. Weder der Verhaltenskodex für Wahlen der Europäischen Kommission für Demokratie durch Recht (Venedig-Kommission, 1.) noch die Rechtsprechung des Europäischen Gerichtshofs für Menschenrechte zu Art. 3 des 1. Zusatzprotokolls zur Konvention zum Schutz der Menschenrechte und Grundfreiheiten (ZP I EMRK, 2.) haben zur Folge, dass durch den Zeitpunkt des Inkrafttretens des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes vom 14. November 2020 die Stabilität des Wahlrechts in verfassungswidriger Weise beeinträchtigt worden ist (3.). Sonstige verfassungsrechtliche Bedenken sind nicht ersichtlich (4.).</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr"/>
-      <c r="C228" t="n">
-        <v>227</v>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>1. a) Nach Ziffer II. 2. b der Leitlinien des Verhaltenskodex für Wahlen der Venedig-Kommission (Verhaltenskodex für Wahlen – Leitlinien und erläuternder Bericht – CDL-AD &lt;2002&gt; 23rev2-cor) sollen die Grundelemente des Wahlrechts bis ein Jahr vor einer Wahl nicht mehr verändert werden. In dem erläuternden Bericht wird ausgeführt:</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="n">
-        <v>228</v>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>b) Nach diesen Erwägungen soll durch die Stabilität des Wahlrechts die Glaubwürdigkeit des für die Demokratie konstitutiven Wahlprozesses gewährleistet werden. Die Wählerinnen und Wähler sollen darauf vertrauen können, dass ihre Stimme dasjenige Element ist, das über die Zusammensetzung des Parlaments entscheidet, und dieses nicht durch Manipulationen des Wahlrechts zugunsten der herrschenden Mehrheit unterlaufen wird. Hierbei soll bereits der Anschein von Manipulationen verhindert werden (vgl. BVerfGE 151, 152 &lt;171 Rn. 50&gt;).</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr"/>
-      <c r="C230" t="n">
-        <v>229</v>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>c) Indes begreift die Venedig-Kommission die zur Wahrung hinreichender Stabilität des Wahlrechts aufgestellte Jahresfrist nicht als unverrückbar. Vielmehr hat sie in einer gemeinsamen Stellungnahme mit dem Büro für demokratische Institutionen und Menschenrechte (ODIHR) der Organisation für Sicherheit und Zusammenarbeit in Europa (OSZE) ausgeführt, dass Abweichungen von der Jahresfrist zulässig und mit dem Grundsatz der Stabilität des Wahlrechts vereinbar sein können, etwa wenn die Änderungen eher technischer Art sind oder auf Empfehlungen fundierter Sachverständigengutachten zurückgehen. Allerdings müsse sichergestellt sein, dass der Wahlleitung und den politischen Entscheidungsträgern eine angemessene Zeit verbleibt, um die Wahlen ordnungsgemäß zu organisieren (vgl. Venedig-Kommission, OSZE/ODIHR: Armenia, Joint Urgent Opinion on Amendments to the Electoral Code and Related Legislation, CDL-PI &lt;2021&gt; 006, Rn. 22).</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr"/>
-      <c r="C231" t="n">
-        <v>230</v>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>2. Nach der Rechtsprechung des Europäischen Gerichtshofs für Menschenrechte können Beeinträchtigungen der Stabilität des Wahlrechts Art. 3 ZP I EMRK verletzen (vgl. EGMR, Georgian Labour Party v. Georgia, Urteil vom 8. Juli 2008, Nr. 9103/04, §§ 88 f.; &lt;GK&gt;, Tănase v. Moldova, Urteil vom 27. April 2010, Nr. 7/08, § 179; Ekoglasnost c. Bulgarie, Urteil vom 6. November 2012, Nr. 30386/05, §§ 68 ff.). Dieser verpflichtet die Vertragsstaaten, in angemessenen Zeitabständen freie und geheime Wahlen unter Bedingungen abzuhalten, welche die freie Äußerung der Meinung des Volkes bei der Wahl der gesetzgebenden Körperschaften gewährleisten. Der Gerichtshof hat ausgeführt, die Stabilität des Wahlrechts sei von besonderer Bedeutung für die Achtung der in Art. 3 ZP I EMRK garantierten Rechte. Wenn ein Staat die grundlegenden Wahlvorschriften zu häufig oder „am Vorabend“ einer Wahl ändere, könne er die Achtung der Öffentlichkeit vor den Garantien, die die Freiheit der Wahl gewährleisten, oder ihr Vertrauen in deren Existenz untergraben (vgl. EGMR, Ekoglasnost c. Bulgarie, Urteil vom 6. November 2012, Nr. 30386/05, § 68). Nach der Rechtsprechung des Europäischen Gerichtshofs für Menschenrechte ist bei der Anwendung von Art. 3 ZP I EMRK indes jedes Wahlgesetz im Lichte der politischen Entwicklung des betreffenden Landes zu beurteilen (vgl. EGMR, Georgian Labour Party v. Georgia, Urteil vom 8. Juli 2008, Nr. 9103/04, § 89).</t>
-        </is>
-      </c>
-      <c r="B232" t="inlineStr"/>
-      <c r="C232" t="n">
-        <v>231</v>
-      </c>
-      <c r="D232" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>3. Demgemäß ist vorliegend der Zeitpunkt des Inkrafttretens der zur Überprüfung gestellten Änderung des Bundeswahlgesetzes verfassungsrechtlich nicht zu beanstanden.</t>
-        </is>
-      </c>
-      <c r="B233" t="inlineStr"/>
-      <c r="C233" t="n">
-        <v>232</v>
-      </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>a) Zwar stehen die Europäische Menschenrechtskonvention und ihre Zusatzprotokolle – soweit sie für die Bundesrepublik Deutschland in Kraft getreten sind – innerhalb der deutschen Rechtsordnung (nur) im Rang eines Bundesgesetzes (vgl. BVerfGE 74, 358 &lt;370&gt;; 111, 307 &lt;316 f.&gt;; 128, 326 &lt;367&gt;; 141, 1 &lt;19 Rn. 45&gt;; 148, 296 &lt;350 f. Rn. 127&gt;; 151, 1 &lt;26 f. Rn. 61&gt; – Wahlrechtsausschluss Bundestagswahl). Gleichwohl besitzen sie verfassungsrechtliche Bedeutung als Auslegungshilfe für die Bestimmung des Inhalts und der Reichweite der Gewährleistungen des Grundgesetzes (vgl. BVerfGE 74, 358 &lt;370&gt;; 83, 119 &lt;128&gt;; 111, 307 &lt;317, 329&gt;; 120, 180 &lt;200 f.&gt;; 128, 326 &lt;367 f.&gt;; 148, 296 &lt;351 Rn. 128&gt;; 151, 1 &lt;27 Rn. 62&gt;). Ihre Heranziehung ist Ausdruck der Völkerrechtsfreundlichkeit des Grundgesetzes, das einer Einbindung der Bundesrepublik Deutschland in inter- und supranationale Zusammenhänge sowie deren Weiterentwicklung nicht entgegensteht, sondern diese voraussetzt und erwartet (vgl. BVerfGE 151, 1 &lt;27 Rn. 62&gt;). Allerdings zielt die Heranziehung als Auslegungshilfe nicht auf eine schematische Parallelisierung einzelner verfassungsrechtlicher Begriffe (vgl. BVerfGE 137, 273 &lt;320 f. Rn. 128&gt;; 141, 1 &lt;30 Rn. 72&gt;; 148, 296 &lt;353 Rn. 131&gt;; 151, 1 &lt;27 Rn. 63&gt;). Vielmehr gilt auch für die völkerrechtsfreundliche Auslegung des Grundgesetzes, dass Ähnlichkeiten im Normtext nicht über Unterschiede, die sich aus dem Kontext der Rechtsordnungen ergeben, hinwegtäuschen dürfen (vgl. BVerfGE 148, 296 &lt;353 Rn. 131&gt;; 151, 1 &lt;27 f. Rn. 63&gt;). Im Rahmen der Heranziehung der Europäischen Menschenrechtskonvention als Auslegungshilfe berücksichtigt das Bundesverfassungsgericht Entscheidungen des Europäischen Gerichtshofs für Menschenrechte, und zwar auch dann, wenn sie nicht denselben Streitgegenstand wie das verfassungsgerichtliche Verfahren betreffen. Dies beruht auf der Orientierungs- und Leitungsfunktion, die der Rechtsprechung des Europäischen Gerichtshofs für Menschenrechte für die Auslegung der Europäischen Menschenrechtskonvention auch über den konkret entschiedenen Einzelfall hinaus zukommt (vgl. BVerfGE 128, 326 &lt;368&gt;; 148, 296 &lt;351 f. Rn. 129&gt;; 151, 1 &lt;28 Rn. 64&gt;).</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr"/>
-      <c r="C234" t="n">
-        <v>233</v>
-      </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>Stellungnahmen von Ausschüssen und vergleichbaren Organen internationaler Organisationen kommt im innerstaatlichen Bereich keine unmittelbare Bindungswirkung zu (vgl. BVerfGE 151, 1 &lt;29 Rn. 65&gt; m.w.N.; 151, 152 &lt;170 Rn. 48&gt;). Der Venedig-Kommission ist nach Art. 1 ihres Statuts vom 21. Februar 2002 (Committee of Ministers’ Resolution &lt;2002&gt; 3: Revised Statute of the European Commission for Democracy through Law &lt;21 February 2002&gt;) eine (lediglich) beratend-kooperative Funktion zugewiesen (vgl. BVerfGE 151, 152 &lt;170 Rn. 48&gt; m.w.N.).</t>
-        </is>
-      </c>
-      <c r="B235" t="inlineStr"/>
-      <c r="C235" t="n">
-        <v>234</v>
-      </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
-        <is>
-          <t>b) Davon ausgehend genügen die zur Überprüfung gestellten Änderungen des Bundeswahlgesetzes den Anforderungen an die Stabilität des Wahlrechts.</t>
-        </is>
-      </c>
-      <c r="B236" t="inlineStr"/>
-      <c r="C236" t="n">
-        <v>235</v>
-      </c>
-      <c r="D236" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
-        <is>
-          <t>aa) Zwar traten die antragsgegenständlichen Regelungen des Fünfundzwanzigsten Gesetzes zur Änderung des Bundeswahlgesetzes am 19. November 2020 in Kraft (Art. 2 Abs. 1 BWahlGÄndG). Der Termin für die Wahl zum 20. Deutschen Bundestag wurde mit Anordnung vom 8. Dezember 2020 (BGBl I S. 2769) auf den 26. September 2021 bestimmt. Danach lagen zwischen dem Abschluss des Gesetzgebungsverfahrens und dem Termin der Bundestagswahl nur etwas über zehn Monate. Auch betrifft das zu überprüfende Gesetz das Sitzzuteilungsverfahren, auf dessen Änderung die Jahresfrist der Venedig-Kommission ausdrücklich Anwendung finden soll (vgl. Venedig-Kommission, Auslegungserklärung über die Stabilität des Wahlrechts, CDL-AD &lt;2005&gt; 043, II. Nr. 3 und 4).</t>
-        </is>
-      </c>
-      <c r="B237" t="inlineStr"/>
-      <c r="C237" t="n">
-        <v>236</v>
-      </c>
-      <c r="D237" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>bb) Allerdings liegt der Anschein einer manipulativen Verfestigung existierender Regierungsmehrheiten durch das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 fern. Dies folgt schon daraus, dass die zur Überprüfung gestellte Neufassung des Bundeswahlgesetzes nichts daran geändert hat, dass die Sitze – wie bereits nach § 6 BWahlG 2013 – gemäß § 6 Abs. 5 und 6 BWahlG grundsätzlich nach der Zahl der zu berücksichtigenden Zweitstimmen im Divisorverfahren mit Standardrundung vergeben werden. Sofern die Neuregelung die Zuteilung von bis zu drei unausgeglichenen Überhangmandaten ermöglicht hat, kommt dies zwar tendenziell den Parteien zugute, deren Fraktionen den antragsgegenständlichen Gesetzentwurf – noch außerhalb der Jahresfrist (vgl. BTDrucks 19/22504) – in den Deutschen Bundestag eingebracht haben. Eine grundlegende Veränderung des politischen Wettbewerbs um Wählerstimmen ist mit der Neuregelung aber nicht verbunden. Hinzu kommt, dass die Wahlrechtsänderung das Ergebnis einer Debatte war, die bereits in der 18. Legislaturperiode des Deutschen Bundestages intensiv geführt worden war (vgl. nur Wissenschaftliche Dienste des Deutschen Bundestages, WD 3-3000-055/16). Das Fünfundzwanzigste Gesetz zur Änderung des Bundeswahlgesetzes vom 14. November 2020 wurde weder überraschend noch „am Vorabend“ der Wahl des 20. Deutschen Bundestages beschlossen. Schließlich betraf es im Wesentlichen lediglich die Regelungen der Sitzzuteilung. Die Vorbereitung der Wahl des 20. Deutschen Bundestages einschließlich der Aufstellung der Kandidatinnen und Kandidaten war von den Änderungen nicht betroffen. Die Wahlrechtsänderung ist daher nicht geeignet, das Vertrauen der Wählerinnen und Wähler in die Beachtung der Garantien, die die Freiheit der Wahl gewährleisten, und in das Unterbleiben von Manipulationen der Wahl zugunsten der herrschenden Mehrheit zu erschüttern.</t>
-        </is>
-      </c>
-      <c r="B238" t="inlineStr"/>
-      <c r="C238" t="n">
-        <v>237</v>
-      </c>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>4. Vor diesem Hintergrund kann dahinstehen, ob und gegebenenfalls durch welche Vorschriften des Grundgesetzes der Grundsatz der Stabilität des Wahlrechts auch unmittelbar verfassungsrechtlich gewährleistet ist. Der Zeitpunkt der Änderung des Bundeswahlgesetzes stellt diesen Grundsatz aus den dargelegten Gründen nicht infrage. Dass sein verfassungsrechtlich garantierter Gewährleistungsgehalt über das vorstehend Ausgeführte hinausgehen könnte, ist nicht ersichtlich.</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr"/>
-      <c r="C239" t="n">
-        <v>238</v>
-      </c>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>Die Entscheidung ist mit 5:3 Stimmen ergangen.</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr"/>
-      <c r="C240" t="n">
-        <v>239</v>
-      </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/11/fs20231129_2bvf000121.html?nn=68020</t>
+          <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update queries and URLs in notebooks for improved clarity and accuracy
</commit_message>
<xml_diff>
--- a/04_bverfg_rag/bverfg_urteil.xlsx
+++ b/04_bverfg_rag/bverfg_urteil.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D165"/>
+  <dimension ref="A1:F165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,6 +446,16 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Aktenzeichen</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>az_rn</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>url</t>
         </is>
       </c>
@@ -462,6 +472,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -478,6 +498,16 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -494,6 +524,16 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -510,6 +550,16 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 4</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -526,6 +576,16 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -542,6 +602,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 6</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -558,6 +628,16 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 7</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -574,6 +654,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 8</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -590,6 +680,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 9</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -606,6 +706,16 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 10</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -622,6 +732,16 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 11</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -638,6 +758,16 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 12</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -654,6 +784,16 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 13</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -670,6 +810,16 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 14</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -686,6 +836,16 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 15</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -702,6 +862,16 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 16</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -718,6 +888,16 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 17</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -734,6 +914,16 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 18</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -750,6 +940,16 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 19</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -766,6 +966,16 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 20</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -782,6 +992,16 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 21</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -798,6 +1018,16 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 22</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -814,6 +1044,16 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 23</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -830,6 +1070,16 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 24</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -846,6 +1096,16 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 25</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -862,6 +1122,16 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 26</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -878,6 +1148,16 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 27</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -894,6 +1174,16 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 28</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -910,6 +1200,16 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 29</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -926,6 +1226,16 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 30</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -942,6 +1252,16 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 31</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -958,6 +1278,16 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 32</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -974,6 +1304,16 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 33</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -990,6 +1330,16 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 34</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1006,6 +1356,16 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 35</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1022,6 +1382,16 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 36</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1038,6 +1408,16 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 37</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1054,6 +1434,16 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 38</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1070,6 +1460,16 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 39</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1086,6 +1486,16 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 40</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1102,6 +1512,16 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 41</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1118,6 +1538,16 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 42</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1134,6 +1564,16 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 43</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1150,6 +1590,16 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 44</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1166,6 +1616,16 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 45</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1182,6 +1642,16 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 46</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1198,6 +1668,16 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 47</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1214,6 +1694,16 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 48</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1230,6 +1720,16 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 49</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1246,6 +1746,16 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 50</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1262,6 +1772,16 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 51</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1278,6 +1798,16 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 52</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1294,6 +1824,16 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 53</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1310,6 +1850,16 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 54</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1326,6 +1876,16 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 55</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1342,6 +1902,16 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 56</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1358,6 +1928,16 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 57</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1374,6 +1954,16 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 58</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1390,6 +1980,16 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 59</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1406,6 +2006,16 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 60</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1422,6 +2032,16 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 61</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1438,6 +2058,16 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 62</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1454,6 +2084,16 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 63</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1470,6 +2110,16 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 64</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1486,6 +2136,16 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 65</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1502,6 +2162,16 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 66</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1518,6 +2188,16 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 67</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1534,6 +2214,16 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 68</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1550,6 +2240,16 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 69</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1566,6 +2266,16 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 70</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1582,6 +2292,16 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 71</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1598,6 +2318,16 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 72</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1614,6 +2344,16 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 73</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1630,6 +2370,16 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 74</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1646,6 +2396,16 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 75</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1662,6 +2422,16 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 76</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1678,6 +2448,16 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 77</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1694,6 +2474,16 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 78</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1710,6 +2500,16 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 79</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1726,6 +2526,16 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 80</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1742,6 +2552,16 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 81</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1758,6 +2578,16 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 82</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1774,6 +2604,16 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 83</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1790,6 +2630,16 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 84</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1806,6 +2656,16 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 85</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1822,6 +2682,16 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 86</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1838,6 +2708,16 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 87</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1854,6 +2734,16 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 88</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1870,6 +2760,16 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 89</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1886,6 +2786,16 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 90</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1902,6 +2812,16 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 91</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1918,6 +2838,16 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 92</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1934,6 +2864,16 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 93</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1950,6 +2890,16 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 94</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1966,6 +2916,16 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 95</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1982,6 +2942,16 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 96</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -1998,6 +2968,16 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 97</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2014,6 +2994,16 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 98</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2030,6 +3020,16 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 99</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2046,6 +3046,16 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 100</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2062,6 +3072,16 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 101</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2078,6 +3098,16 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 102</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2094,6 +3124,16 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 103</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2110,6 +3150,16 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 104</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2126,6 +3176,16 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 105</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2142,6 +3202,16 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 106</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2158,6 +3228,16 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 107</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2174,6 +3254,16 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 108</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2190,6 +3280,16 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 109</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2206,6 +3306,16 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 110</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2222,6 +3332,16 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 111</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2238,6 +3358,16 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 112</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2254,6 +3384,16 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 113</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2270,6 +3410,16 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 114</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2286,6 +3436,16 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 115</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2302,6 +3462,16 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 116</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2318,6 +3488,16 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 117</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2334,6 +3514,16 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 118</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2350,6 +3540,16 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 119</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2366,6 +3566,16 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 120</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2382,6 +3592,16 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 121</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2398,6 +3618,16 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 122</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2414,6 +3644,16 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 123</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2430,6 +3670,16 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 124</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2446,6 +3696,16 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 125</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2462,6 +3722,16 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 126</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2478,6 +3748,16 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 127</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2494,6 +3774,16 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 128</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2510,6 +3800,16 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 129</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2526,6 +3826,16 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 130</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2542,6 +3852,16 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 131</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2558,6 +3878,16 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 132</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2574,6 +3904,16 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 133</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2590,6 +3930,16 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 134</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2606,6 +3956,16 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 135</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2622,6 +3982,16 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 136</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2638,6 +4008,16 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 137</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2654,6 +4034,16 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 138</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2670,6 +4060,16 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 139</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2686,6 +4086,16 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 140</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2702,6 +4112,16 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 141</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2718,6 +4138,16 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 142</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2734,6 +4164,16 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 143</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2750,6 +4190,16 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 144</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2766,6 +4216,16 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 145</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2782,6 +4242,16 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 146</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2798,6 +4268,16 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 147</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2814,6 +4294,16 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 148</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2830,6 +4320,16 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 149</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2846,6 +4346,16 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 150</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2862,6 +4372,16 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 151</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2878,6 +4398,16 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 152</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2894,6 +4424,16 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 153</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2910,6 +4450,16 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 154</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2926,6 +4476,16 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 155</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2942,6 +4502,16 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 156</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2958,6 +4528,16 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 157</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2974,6 +4554,16 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 158</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -2990,6 +4580,16 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 159</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -3006,6 +4606,16 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 160</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -3022,6 +4632,16 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 161</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -3038,6 +4658,16 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 162</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -3054,6 +4684,16 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 163</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>
       </c>
@@ -3069,6 +4709,16 @@
         <v>164</v>
       </c>
       <c r="D165" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2 BvR 900/22, Rn. 164</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
         <is>
           <t>https://www.bundesverfassungsgericht.de/SharedDocs/Entscheidungen/DE/2023/10/rs20231031_2bvr090022.html?nn=68020</t>
         </is>

</xml_diff>